<commit_message>
lots of chnages and updates
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\claude_repos\trigital\nipige_qa_automation\src\resources\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dbt\nipigeautomation\src\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{490DC677-9684-4523-BABB-89A15AAAB416}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10234118-E70A-4085-B825-86FFC29AC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="734" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="734" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Regression" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="RESTUserTest" sheetId="8" r:id="rId5"/>
     <sheet name="SOAPAccountServiceTest" sheetId="11" r:id="rId6"/>
     <sheet name="DatabaseTest" sheetId="10" r:id="rId7"/>
+    <sheet name="DashboardTest" sheetId="12" r:id="rId8"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="178">
   <si>
     <t>TestID</t>
   </si>
@@ -48,9 +49,6 @@
     <t>Login with valid credentials</t>
   </si>
   <si>
-    <t>Login with invalid credentials</t>
-  </si>
-  <si>
     <t>test3210</t>
   </si>
   <si>
@@ -84,9 +82,6 @@
     <t>TC01_ValidLogin</t>
   </si>
   <si>
-    <t>Incorrect user name or password.</t>
-  </si>
-  <si>
     <t>ErrorMessage</t>
   </si>
   <si>
@@ -190,12 +185,6 @@
   </si>
   <si>
     <t>true</t>
-  </si>
-  <si>
-    <t>TC03_LoginCreateAccount</t>
-  </si>
-  <si>
-    <t>Login with valid credentials from Create Account</t>
   </si>
   <si>
     <t>CreateAccountTest</t>
@@ -522,6 +511,63 @@
   </si>
   <si>
     <t>tenant</t>
+  </si>
+  <si>
+    <t>Invalid password!!</t>
+  </si>
+  <si>
+    <t>Invalid password</t>
+  </si>
+  <si>
+    <t>TC03_BlankEmail</t>
+  </si>
+  <si>
+    <t>Blank email</t>
+  </si>
+  <si>
+    <t>Please enter email/username/phone</t>
+  </si>
+  <si>
+    <t>TC04_BlankPassword</t>
+  </si>
+  <si>
+    <t>Blank password</t>
+  </si>
+  <si>
+    <t>Please enter password</t>
+  </si>
+  <si>
+    <t>TC05_BlankRole</t>
+  </si>
+  <si>
+    <t>Blank role</t>
+  </si>
+  <si>
+    <t>Please select login way</t>
+  </si>
+  <si>
+    <t>TC01_DashboardLoad</t>
+  </si>
+  <si>
+    <t>TC04_OrderChartDropdown</t>
+  </si>
+  <si>
+    <t>TC05_TopRevenueDropdown</t>
+  </si>
+  <si>
+    <t>Verify Dashboard Load</t>
+  </si>
+  <si>
+    <t>Verify Order Chart Dropdown</t>
+  </si>
+  <si>
+    <t>Verify Top Revenue Dropdown</t>
+  </si>
+  <si>
+    <t>Verify Dashboard Filters</t>
+  </si>
+  <si>
+    <t>TC03_DashboardFilters</t>
   </si>
 </sst>
 </file>
@@ -574,7 +620,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
@@ -582,6 +628,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -865,107 +920,107 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" t="s">
+        <v>153</v>
+      </c>
+      <c r="C4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B5" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B6" t="s">
+        <v>153</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>128</v>
+      </c>
+      <c r="B7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B4" t="s">
-        <v>157</v>
-      </c>
-      <c r="C4" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>152</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>154</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
         <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>110</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>111</v>
-      </c>
-      <c r="B6" t="s">
-        <v>157</v>
-      </c>
-      <c r="C6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>132</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>156</v>
-      </c>
-      <c r="B8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>158</v>
-      </c>
-      <c r="B9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -988,165 +1043,165 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B64F1D3-BE77-42C5-8522-489964BC065B}">
   <dimension ref="A1:O3"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.26953125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.54296875" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="11" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="9.140625" style="1"/>
+    <col min="15" max="15" width="21.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B2">
         <v>11235</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="L2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="O2" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B3">
         <v>11645</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" s="1" t="s">
+      <c r="I3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="I3" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="J3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="M3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="L3" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="M3" s="1" t="s">
+      <c r="N3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="N3" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="O3" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1162,94 +1217,94 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3637AC5E-DFD7-4094-AEE3-13F4A2BD531E}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.1796875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="55.5703125" customWidth="1"/>
-    <col min="8" max="8" width="41.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.54296875" customWidth="1"/>
+    <col min="8" max="8" width="41.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E1" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="F1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G1" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="H1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B2">
         <v>1337</v>
       </c>
       <c r="C2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="D2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="H2" t="s">
         <v>104</v>
       </c>
-      <c r="F2" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="H2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B3">
         <v>1547</v>
       </c>
       <c r="C3" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D3" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E3" t="s">
+        <v>99</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>107</v>
-      </c>
       <c r="H3" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -1264,298 +1319,348 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A954124-2682-439B-BF75-C124F90C5D43}">
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="44.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.5703125" customWidth="1"/>
-    <col min="5" max="5" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.42578125" customWidth="1"/>
+    <col min="1" max="1" width="24.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.54296875" customWidth="1"/>
+    <col min="5" max="5" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.453125" customWidth="1"/>
     <col min="7" max="7" width="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>131</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="7">
+        <v>1243</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="G2" s="7"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="7">
+        <v>1244</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="G1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2">
-        <v>1243</v>
-      </c>
-      <c r="C2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" t="s">
-        <v>159</v>
-      </c>
-      <c r="E2" t="s">
-        <v>160</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="B4" s="7">
+        <v>1245</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3">
-        <v>1244</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" t="s">
-        <v>159</v>
-      </c>
-      <c r="E3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F3" t="s">
-        <v>162</v>
-      </c>
-      <c r="G3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B4">
-        <v>1245</v>
-      </c>
-      <c r="C4" t="s">
-        <v>54</v>
-      </c>
-      <c r="D4" t="s">
-        <v>159</v>
-      </c>
-      <c r="E4" t="s">
-        <v>160</v>
-      </c>
-      <c r="F4" t="s">
-        <v>162</v>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="B5" s="7">
+        <v>1246</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="B6" s="7">
+        <v>1247</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" display="mailto:freshcart@gmail.com" xr:uid="{994A6811-48D5-46DB-BE82-A65EC3BD9727}"/>
+    <hyperlink ref="D3" r:id="rId2" display="mailto:freshcart@gmail.com" xr:uid="{8654ADCA-0949-49F2-B5FB-F0C018C0203C}"/>
+    <hyperlink ref="D5" r:id="rId3" display="mailto:freshcart@gmail.com" xr:uid="{A6ACEF41-978A-4533-9283-AE91C15012D7}"/>
+    <hyperlink ref="D6" r:id="rId4" display="mailto:freshcart@gmail.com" xr:uid="{9E320769-34D1-4D2D-98B5-979FE79754B5}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9496EF85-5873-4562-AF45-3630E5F53D1F}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.54296875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="43" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>58</v>
-      </c>
-      <c r="G1" t="s">
-        <v>69</v>
-      </c>
-      <c r="H1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>62</v>
       </c>
       <c r="B2">
         <v>1137</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>64</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>68</v>
       </c>
       <c r="F2" s="4"/>
       <c r="G2">
         <v>200</v>
       </c>
       <c r="H2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B3">
         <v>1138</v>
       </c>
       <c r="C3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D3" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F3" s="4"/>
       <c r="G3">
         <v>200</v>
       </c>
       <c r="H3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B4">
         <v>1139</v>
       </c>
       <c r="C4" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D4" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E4" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F4" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G4">
         <v>201</v>
       </c>
       <c r="H4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B5">
         <v>1140</v>
       </c>
       <c r="C5" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D5" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F5" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="G5">
         <v>200</v>
       </c>
       <c r="H5" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B6">
         <v>1141</v>
       </c>
       <c r="C6" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="D6" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="F6" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="G6">
         <v>201</v>
       </c>
       <c r="H6" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B7">
         <v>1142</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="D7" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G7">
         <v>200</v>
       </c>
       <c r="H7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -1567,146 +1672,146 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C41D663D-6548-4F04-A1E9-0786B9531E75}">
   <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="28.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="51.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="51.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="G1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B2">
         <v>1113</v>
       </c>
       <c r="C2" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="F2" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="G2" t="s">
+        <v>135</v>
+      </c>
+      <c r="H2" t="s">
         <v>136</v>
       </c>
-      <c r="G2" t="s">
-        <v>139</v>
-      </c>
-      <c r="H2" t="s">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>140</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>144</v>
       </c>
       <c r="B3">
         <v>1114</v>
       </c>
       <c r="C3" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="G3" t="s">
+        <v>135</v>
+      </c>
+      <c r="H3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>145</v>
-      </c>
-      <c r="D3" t="s">
-        <v>142</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="G3" t="s">
-        <v>139</v>
-      </c>
-      <c r="H3" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>149</v>
       </c>
       <c r="B4">
         <v>1115</v>
       </c>
       <c r="C4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D4" t="s">
+        <v>143</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="G4" t="s">
+        <v>135</v>
+      </c>
+      <c r="H4" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>150</v>
-      </c>
-      <c r="D4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="G4" t="s">
-        <v>139</v>
-      </c>
-      <c r="H4" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>154</v>
       </c>
       <c r="B5">
         <v>1116</v>
       </c>
       <c r="C5" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D5" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="G5" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="H5" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -1722,129 +1827,223 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F66E855F-71DD-4AFC-9C48-E6F935E4E730}">
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="44.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="102.42578125" customWidth="1"/>
+    <col min="1" max="1" width="24.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="102.453125" customWidth="1"/>
     <col min="6" max="6" width="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B2">
         <v>1467</v>
       </c>
       <c r="C2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B3">
         <v>1468</v>
       </c>
       <c r="C3" t="s">
+        <v>112</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>116</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>120</v>
       </c>
       <c r="B4">
         <v>1469</v>
       </c>
       <c r="C4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>121</v>
-      </c>
-      <c r="D4" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>125</v>
       </c>
       <c r="B5">
         <v>1470</v>
       </c>
       <c r="C5" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B6">
         <v>1471</v>
       </c>
       <c r="C6" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B7">
         <v>1472</v>
       </c>
       <c r="C7" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D7" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B8">
         <v>1473</v>
       </c>
       <c r="C8" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D8" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EC53475-F706-43CF-8BD8-C4C2908430C2}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="30.7265625" customWidth="1"/>
+    <col min="2" max="2" width="5.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="6"/>
+    </row>
+    <row r="2" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="B2" s="7">
+        <v>2001</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="D2" s="7"/>
+    </row>
+    <row r="3" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A3" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="B3" s="7">
+        <v>2003</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="D3" s="7"/>
+    </row>
+    <row r="4" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="B4" s="7">
+        <v>2004</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="D4" s="7"/>
+    </row>
+    <row r="5" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="B5" s="7">
+        <v>2005</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="D5" s="7"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="7"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="7"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="7"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added sheet for testing
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -5,30 +5,33 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sriro\Music\nipige_qa_automation\src\resources\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\claude_repos\trigital\nipige_qa_automation\src\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57EE1A2F-AC18-4818-B029-B91DFFF56D05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD9E1556-7960-4039-A5B6-5614B938C703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Regression" sheetId="1" r:id="rId1"/>
-    <sheet name="CreateAccountTest" sheetId="2" r:id="rId2"/>
-    <sheet name="ContactUsTest" sheetId="3" r:id="rId3"/>
-    <sheet name="Admin App" sheetId="5" r:id="rId4"/>
+    <sheet name="InventoryManagement" sheetId="13" r:id="rId2"/>
+    <sheet name="SetupMasters" sheetId="12" r:id="rId3"/>
+    <sheet name="LoginTest" sheetId="5" r:id="rId4"/>
     <sheet name="ServiceTicketTest" sheetId="6" r:id="rId5"/>
-    <sheet name="BulkPromotion" sheetId="7" r:id="rId6"/>
-    <sheet name="RESTUserTest" sheetId="8" r:id="rId7"/>
-    <sheet name="SOAPAccountServiceTest" sheetId="9" r:id="rId8"/>
-    <sheet name="DatabaseTest" sheetId="10" r:id="rId9"/>
+    <sheet name="CreateAccountTest" sheetId="2" r:id="rId6"/>
+    <sheet name="OrderManagementTest" sheetId="11" r:id="rId7"/>
+    <sheet name="ContactUsTest" sheetId="3" r:id="rId8"/>
+    <sheet name="BulkPromotion" sheetId="7" r:id="rId9"/>
+    <sheet name="RESTUserTest" sheetId="8" r:id="rId10"/>
+    <sheet name="SOAPAccountServiceTest" sheetId="9" r:id="rId11"/>
+    <sheet name="DatabaseTest" sheetId="10" r:id="rId12"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="235">
   <si>
     <t>TestName</t>
   </si>
@@ -382,9 +385,6 @@
   </si>
   <si>
     <t>TC02_InvalidTicketID</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Service Ticket Invalid Ticket ID</t>
   </si>
   <si>
     <t>SR9999999999</t>
@@ -723,6 +723,21 @@
   </si>
   <si>
     <t>TC09_AdminInvalidUsernameAndPassword</t>
+  </si>
+  <si>
+    <t>Service Ticket Invalid Ticket ID</t>
+  </si>
+  <si>
+    <t>ServiceTicketTest</t>
+  </si>
+  <si>
+    <t>OrderManagementTest</t>
+  </si>
+  <si>
+    <t>SetupMasters</t>
+  </si>
+  <si>
+    <t>InventoryManagement</t>
   </si>
 </sst>
 </file>
@@ -1099,14 +1114,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.4140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1117,9 +1133,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -1128,20 +1144,20 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>233</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>234</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
@@ -1150,9 +1166,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>231</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
@@ -1161,329 +1177,595 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>232</v>
       </c>
       <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
         <v>8</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
         <v>4</v>
       </c>
       <c r="C8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>14</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B12" t="s">
         <v>4</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:C9" numberStoredAsText="1"/>
+    <ignoredError sqref="A7:C9 A1:C1 A11:C12 A10:B10" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" t="s">
+        <v>149</v>
+      </c>
+      <c r="E1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F1" t="s">
+        <v>151</v>
+      </c>
+      <c r="G1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B2">
+        <v>1137</v>
+      </c>
+      <c r="C2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E2" t="s">
+        <v>156</v>
+      </c>
+      <c r="G2">
+        <v>200</v>
+      </c>
+      <c r="H2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>158</v>
+      </c>
+      <c r="B3">
+        <v>1138</v>
+      </c>
+      <c r="C3" t="s">
+        <v>159</v>
+      </c>
+      <c r="D3" t="s">
+        <v>160</v>
+      </c>
+      <c r="E3" t="s">
+        <v>161</v>
+      </c>
+      <c r="G3">
+        <v>200</v>
+      </c>
+      <c r="H3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B4">
+        <v>1139</v>
+      </c>
+      <c r="C4" t="s">
+        <v>164</v>
+      </c>
+      <c r="D4" t="s">
+        <v>165</v>
+      </c>
+      <c r="E4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F4" t="s">
+        <v>166</v>
+      </c>
+      <c r="G4">
+        <v>201</v>
+      </c>
+      <c r="H4" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>168</v>
+      </c>
+      <c r="B5">
+        <v>1140</v>
+      </c>
+      <c r="C5" t="s">
+        <v>169</v>
+      </c>
+      <c r="D5" t="s">
+        <v>170</v>
+      </c>
+      <c r="E5" t="s">
+        <v>161</v>
+      </c>
+      <c r="F5" t="s">
+        <v>171</v>
+      </c>
+      <c r="G5">
+        <v>200</v>
+      </c>
+      <c r="H5" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>173</v>
+      </c>
+      <c r="B6">
+        <v>1141</v>
+      </c>
+      <c r="C6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D6" t="s">
+        <v>175</v>
+      </c>
+      <c r="E6" t="s">
+        <v>176</v>
+      </c>
+      <c r="F6" t="s">
+        <v>177</v>
+      </c>
+      <c r="G6">
+        <v>201</v>
+      </c>
+      <c r="H6" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>179</v>
+      </c>
+      <c r="B7">
+        <v>1142</v>
+      </c>
+      <c r="C7" t="s">
+        <v>180</v>
+      </c>
+      <c r="D7" t="s">
+        <v>181</v>
+      </c>
+      <c r="E7" t="s">
+        <v>161</v>
+      </c>
+      <c r="G7">
+        <v>200</v>
+      </c>
+      <c r="H7" t="s">
+        <v>162</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:H7" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" t="s">
+        <v>149</v>
+      </c>
+      <c r="E1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F1" t="s">
+        <v>151</v>
+      </c>
+      <c r="G1" t="s">
+        <v>182</v>
+      </c>
+      <c r="H1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B2">
+        <v>1113</v>
+      </c>
+      <c r="C2" t="s">
+        <v>185</v>
+      </c>
+      <c r="D2" t="s">
+        <v>186</v>
+      </c>
+      <c r="E2" t="s">
+        <v>187</v>
+      </c>
+      <c r="F2" t="s">
+        <v>188</v>
+      </c>
+      <c r="G2" t="s">
+        <v>189</v>
+      </c>
+      <c r="H2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>191</v>
+      </c>
+      <c r="B3">
+        <v>1114</v>
+      </c>
+      <c r="C3" t="s">
+        <v>192</v>
+      </c>
+      <c r="D3" t="s">
+        <v>193</v>
+      </c>
+      <c r="E3" t="s">
+        <v>187</v>
+      </c>
+      <c r="F3" t="s">
+        <v>194</v>
+      </c>
+      <c r="G3" t="s">
+        <v>189</v>
+      </c>
+      <c r="H3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>196</v>
+      </c>
+      <c r="B4">
+        <v>1115</v>
+      </c>
+      <c r="C4" t="s">
+        <v>197</v>
+      </c>
+      <c r="D4" t="s">
+        <v>198</v>
+      </c>
+      <c r="E4" t="s">
+        <v>187</v>
+      </c>
+      <c r="F4" t="s">
+        <v>199</v>
+      </c>
+      <c r="G4" t="s">
+        <v>189</v>
+      </c>
+      <c r="H4" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>201</v>
+      </c>
+      <c r="B5">
+        <v>1116</v>
+      </c>
+      <c r="C5" t="s">
+        <v>202</v>
+      </c>
+      <c r="D5" t="s">
+        <v>203</v>
+      </c>
+      <c r="E5" t="s">
+        <v>187</v>
+      </c>
+      <c r="F5" t="s">
+        <v>204</v>
+      </c>
+      <c r="G5" t="s">
+        <v>205</v>
+      </c>
+      <c r="H5" t="s">
+        <v>206</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0800-000000000000}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{00000000-0004-0000-0800-000001000000}"/>
+    <hyperlink ref="E4" r:id="rId3" xr:uid="{00000000-0004-0000-0800-000002000000}"/>
+    <hyperlink ref="E5" r:id="rId4" xr:uid="{00000000-0004-0000-0800-000003000000}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:H5" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B2">
+        <v>1467</v>
+      </c>
+      <c r="C2" t="s">
+        <v>209</v>
+      </c>
+      <c r="D2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>211</v>
+      </c>
+      <c r="B3">
+        <v>1468</v>
+      </c>
+      <c r="C3" t="s">
+        <v>212</v>
+      </c>
+      <c r="D3" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>214</v>
+      </c>
+      <c r="B4">
+        <v>1469</v>
+      </c>
+      <c r="C4" t="s">
+        <v>215</v>
+      </c>
+      <c r="D4" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>216</v>
+      </c>
+      <c r="B5">
+        <v>1470</v>
+      </c>
+      <c r="C5" t="s">
+        <v>217</v>
+      </c>
+      <c r="D5" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>219</v>
+      </c>
+      <c r="B6">
+        <v>1471</v>
+      </c>
+      <c r="C6" t="s">
+        <v>220</v>
+      </c>
+      <c r="D6" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>221</v>
+      </c>
+      <c r="B7">
+        <v>1472</v>
+      </c>
+      <c r="C7" t="s">
+        <v>222</v>
+      </c>
+      <c r="D7" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>224</v>
+      </c>
+      <c r="B8">
+        <v>1473</v>
+      </c>
+      <c r="C8" t="s">
+        <v>225</v>
+      </c>
+      <c r="D8" t="s">
+        <v>210</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:D8" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:O3"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="14.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F1" t="s">
-        <v>20</v>
-      </c>
-      <c r="G1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H1" t="s">
-        <v>22</v>
-      </c>
-      <c r="I1" t="s">
-        <v>23</v>
-      </c>
-      <c r="J1" t="s">
-        <v>24</v>
-      </c>
-      <c r="K1" t="s">
-        <v>25</v>
-      </c>
-      <c r="L1" t="s">
-        <v>26</v>
-      </c>
-      <c r="M1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" t="s">
-        <v>28</v>
-      </c>
-      <c r="O1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B2">
-        <v>11235</v>
-      </c>
-      <c r="C2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F2" t="s">
-        <v>33</v>
-      </c>
-      <c r="G2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I2" t="s">
-        <v>36</v>
-      </c>
-      <c r="J2" t="s">
-        <v>37</v>
-      </c>
-      <c r="K2" t="s">
-        <v>38</v>
-      </c>
-      <c r="L2" t="s">
-        <v>39</v>
-      </c>
-      <c r="M2" t="s">
-        <v>40</v>
-      </c>
-      <c r="N2" t="s">
-        <v>41</v>
-      </c>
-      <c r="O2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B3">
-        <v>11645</v>
-      </c>
-      <c r="C3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F3" t="s">
-        <v>46</v>
-      </c>
-      <c r="G3" t="s">
-        <v>47</v>
-      </c>
-      <c r="H3" t="s">
-        <v>35</v>
-      </c>
-      <c r="I3" t="s">
-        <v>36</v>
-      </c>
-      <c r="J3" t="s">
-        <v>48</v>
-      </c>
-      <c r="K3" t="s">
-        <v>49</v>
-      </c>
-      <c r="L3" t="s">
-        <v>50</v>
-      </c>
-      <c r="M3" t="s">
-        <v>51</v>
-      </c>
-      <c r="N3" t="s">
-        <v>52</v>
-      </c>
-      <c r="O3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-    <hyperlink ref="D3" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
-  </hyperlinks>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90FDD46F-321E-406B-BA60-13EEF3FF3405}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:O3" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G1" t="s">
-        <v>56</v>
-      </c>
-      <c r="H1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B2">
-        <v>1337</v>
-      </c>
-      <c r="C2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F2" t="s">
-        <v>62</v>
-      </c>
-      <c r="G2" t="s">
-        <v>63</v>
-      </c>
-      <c r="H2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>65</v>
-      </c>
-      <c r="B3">
-        <v>1547</v>
-      </c>
-      <c r="C3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D3" t="s">
-        <v>67</v>
-      </c>
-      <c r="E3" t="s">
-        <v>68</v>
-      </c>
-      <c r="F3" t="s">
-        <v>69</v>
-      </c>
-      <c r="G3" t="s">
-        <v>70</v>
-      </c>
-      <c r="H3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
-    <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
-  </hyperlinks>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3361DFF-EE58-48FD-8CE6-2AFDE302B9DA}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:H3" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="39.4140625" customWidth="1"/>
-    <col min="2" max="2" width="4.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.08203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="39.375" customWidth="1"/>
+    <col min="2" max="2" width="5.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.58203125" customWidth="1"/>
+    <col min="7" max="7" width="17.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -1506,7 +1788,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>85</v>
       </c>
@@ -1526,7 +1808,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>90</v>
       </c>
@@ -1549,7 +1831,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>93</v>
       </c>
@@ -1569,7 +1851,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>95</v>
       </c>
@@ -1592,7 +1874,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>97</v>
       </c>
@@ -1609,9 +1891,9 @@
         <v>101</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B7">
         <v>1247</v>
@@ -1629,9 +1911,9 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B8">
         <v>1248</v>
@@ -1652,9 +1934,9 @@
         <v>80</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B9">
         <v>1249</v>
@@ -1675,9 +1957,9 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B10">
         <v>1250</v>
@@ -1717,13 +1999,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:L3"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="28.75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -1761,7 +2043,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>108</v>
       </c>
@@ -1796,34 +2078,312 @@
         <v>116</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>117</v>
       </c>
       <c r="C3" t="s">
-        <v>118</v>
+        <v>230</v>
       </c>
       <c r="E3" t="s">
         <v>89</v>
       </c>
       <c r="F3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:L3" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:L2 A3:B3 D3:L3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:O3"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="14.625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" t="s">
+        <v>24</v>
+      </c>
+      <c r="K1" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" t="s">
+        <v>26</v>
+      </c>
+      <c r="M1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2">
+        <v>11235</v>
+      </c>
+      <c r="C2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J2" t="s">
+        <v>37</v>
+      </c>
+      <c r="K2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L2" t="s">
+        <v>39</v>
+      </c>
+      <c r="M2" t="s">
+        <v>40</v>
+      </c>
+      <c r="N2" t="s">
+        <v>41</v>
+      </c>
+      <c r="O2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3">
+        <v>11645</v>
+      </c>
+      <c r="C3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H3" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" t="s">
+        <v>48</v>
+      </c>
+      <c r="K3" t="s">
+        <v>49</v>
+      </c>
+      <c r="L3" t="s">
+        <v>50</v>
+      </c>
+      <c r="M3" t="s">
+        <v>51</v>
+      </c>
+      <c r="N3" t="s">
+        <v>52</v>
+      </c>
+      <c r="O3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:O3" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F107B412-2D3C-4F87-A9E1-F6E22431D809}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2">
+        <v>1337</v>
+      </c>
+      <c r="C2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" t="s">
+        <v>62</v>
+      </c>
+      <c r="G2" t="s">
+        <v>63</v>
+      </c>
+      <c r="H2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3">
+        <v>1547</v>
+      </c>
+      <c r="C3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F3" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" t="s">
+        <v>70</v>
+      </c>
+      <c r="H3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:H3" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -1837,180 +2397,180 @@
         <v>72</v>
       </c>
       <c r="E1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F1" t="s">
         <v>120</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>121</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>122</v>
       </c>
-      <c r="H1" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C2" t="s">
         <v>124</v>
-      </c>
-      <c r="B2" t="s">
-        <v>124</v>
-      </c>
-      <c r="C2" t="s">
-        <v>125</v>
       </c>
       <c r="D2" t="s">
         <v>89</v>
       </c>
       <c r="E2" t="s">
+        <v>125</v>
+      </c>
+      <c r="F2" t="s">
         <v>126</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>127</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>128</v>
       </c>
-      <c r="H2" t="s">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>130</v>
-      </c>
-      <c r="C3" t="s">
-        <v>131</v>
       </c>
       <c r="D3" t="s">
         <v>89</v>
       </c>
       <c r="E3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F3" t="s">
+        <v>131</v>
+      </c>
+      <c r="G3" t="s">
         <v>132</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
         <v>133</v>
       </c>
-      <c r="H3" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>134</v>
-      </c>
-      <c r="C4" t="s">
-        <v>135</v>
       </c>
       <c r="D4" t="s">
         <v>89</v>
       </c>
       <c r="E4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F4" t="s">
         <v>18</v>
       </c>
       <c r="G4" t="s">
+        <v>135</v>
+      </c>
+      <c r="H4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
         <v>136</v>
       </c>
-      <c r="H4" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>137</v>
-      </c>
-      <c r="C5" t="s">
-        <v>138</v>
       </c>
       <c r="D5" t="s">
         <v>89</v>
       </c>
       <c r="E5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G5">
         <v>8145031601</v>
       </c>
       <c r="H5" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
+        <v>139</v>
+      </c>
+      <c r="C6" t="s">
         <v>140</v>
-      </c>
-      <c r="C6" t="s">
-        <v>141</v>
       </c>
       <c r="D6" t="s">
         <v>89</v>
       </c>
       <c r="E6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F6" t="s">
+        <v>141</v>
+      </c>
+      <c r="G6" t="s">
         <v>142</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
         <v>143</v>
       </c>
-      <c r="H6" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>144</v>
-      </c>
-      <c r="C7" t="s">
-        <v>145</v>
       </c>
       <c r="D7" t="s">
         <v>89</v>
       </c>
       <c r="E7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F7" t="s">
         <v>25</v>
       </c>
       <c r="G7" t="s">
+        <v>145</v>
+      </c>
+      <c r="H7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
         <v>146</v>
       </c>
-      <c r="H7" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>147</v>
-      </c>
-      <c r="C8" t="s">
-        <v>148</v>
       </c>
       <c r="D8" t="s">
         <v>89</v>
       </c>
       <c r="E8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F8" t="s">
         <v>27</v>
       </c>
       <c r="G8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -2022,464 +2582,4 @@
     <ignoredError sqref="A1:H8" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" t="s">
-        <v>150</v>
-      </c>
-      <c r="E1" t="s">
-        <v>151</v>
-      </c>
-      <c r="F1" t="s">
-        <v>152</v>
-      </c>
-      <c r="G1" t="s">
-        <v>104</v>
-      </c>
-      <c r="H1" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>154</v>
-      </c>
-      <c r="B2">
-        <v>1137</v>
-      </c>
-      <c r="C2" t="s">
-        <v>155</v>
-      </c>
-      <c r="D2" t="s">
-        <v>156</v>
-      </c>
-      <c r="E2" t="s">
-        <v>157</v>
-      </c>
-      <c r="G2">
-        <v>200</v>
-      </c>
-      <c r="H2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>159</v>
-      </c>
-      <c r="B3">
-        <v>1138</v>
-      </c>
-      <c r="C3" t="s">
-        <v>160</v>
-      </c>
-      <c r="D3" t="s">
-        <v>161</v>
-      </c>
-      <c r="E3" t="s">
-        <v>162</v>
-      </c>
-      <c r="G3">
-        <v>200</v>
-      </c>
-      <c r="H3" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>164</v>
-      </c>
-      <c r="B4">
-        <v>1139</v>
-      </c>
-      <c r="C4" t="s">
-        <v>165</v>
-      </c>
-      <c r="D4" t="s">
-        <v>166</v>
-      </c>
-      <c r="E4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F4" t="s">
-        <v>167</v>
-      </c>
-      <c r="G4">
-        <v>201</v>
-      </c>
-      <c r="H4" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>169</v>
-      </c>
-      <c r="B5">
-        <v>1140</v>
-      </c>
-      <c r="C5" t="s">
-        <v>170</v>
-      </c>
-      <c r="D5" t="s">
-        <v>171</v>
-      </c>
-      <c r="E5" t="s">
-        <v>162</v>
-      </c>
-      <c r="F5" t="s">
-        <v>172</v>
-      </c>
-      <c r="G5">
-        <v>200</v>
-      </c>
-      <c r="H5" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>174</v>
-      </c>
-      <c r="B6">
-        <v>1141</v>
-      </c>
-      <c r="C6" t="s">
-        <v>175</v>
-      </c>
-      <c r="D6" t="s">
-        <v>176</v>
-      </c>
-      <c r="E6" t="s">
-        <v>177</v>
-      </c>
-      <c r="F6" t="s">
-        <v>178</v>
-      </c>
-      <c r="G6">
-        <v>201</v>
-      </c>
-      <c r="H6" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>180</v>
-      </c>
-      <c r="B7">
-        <v>1142</v>
-      </c>
-      <c r="C7" t="s">
-        <v>181</v>
-      </c>
-      <c r="D7" t="s">
-        <v>182</v>
-      </c>
-      <c r="E7" t="s">
-        <v>162</v>
-      </c>
-      <c r="G7">
-        <v>200</v>
-      </c>
-      <c r="H7" t="s">
-        <v>163</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:H7" numberStoredAsText="1"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" t="s">
-        <v>150</v>
-      </c>
-      <c r="E1" t="s">
-        <v>151</v>
-      </c>
-      <c r="F1" t="s">
-        <v>152</v>
-      </c>
-      <c r="G1" t="s">
-        <v>183</v>
-      </c>
-      <c r="H1" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>185</v>
-      </c>
-      <c r="B2">
-        <v>1113</v>
-      </c>
-      <c r="C2" t="s">
-        <v>186</v>
-      </c>
-      <c r="D2" t="s">
-        <v>187</v>
-      </c>
-      <c r="E2" t="s">
-        <v>188</v>
-      </c>
-      <c r="F2" t="s">
-        <v>189</v>
-      </c>
-      <c r="G2" t="s">
-        <v>190</v>
-      </c>
-      <c r="H2" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>192</v>
-      </c>
-      <c r="B3">
-        <v>1114</v>
-      </c>
-      <c r="C3" t="s">
-        <v>193</v>
-      </c>
-      <c r="D3" t="s">
-        <v>194</v>
-      </c>
-      <c r="E3" t="s">
-        <v>188</v>
-      </c>
-      <c r="F3" t="s">
-        <v>195</v>
-      </c>
-      <c r="G3" t="s">
-        <v>190</v>
-      </c>
-      <c r="H3" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>197</v>
-      </c>
-      <c r="B4">
-        <v>1115</v>
-      </c>
-      <c r="C4" t="s">
-        <v>198</v>
-      </c>
-      <c r="D4" t="s">
-        <v>199</v>
-      </c>
-      <c r="E4" t="s">
-        <v>188</v>
-      </c>
-      <c r="F4" t="s">
-        <v>200</v>
-      </c>
-      <c r="G4" t="s">
-        <v>190</v>
-      </c>
-      <c r="H4" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>202</v>
-      </c>
-      <c r="B5">
-        <v>1116</v>
-      </c>
-      <c r="C5" t="s">
-        <v>203</v>
-      </c>
-      <c r="D5" t="s">
-        <v>204</v>
-      </c>
-      <c r="E5" t="s">
-        <v>188</v>
-      </c>
-      <c r="F5" t="s">
-        <v>205</v>
-      </c>
-      <c r="G5" t="s">
-        <v>206</v>
-      </c>
-      <c r="H5" t="s">
-        <v>207</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0800-000000000000}"/>
-    <hyperlink ref="E3" r:id="rId2" xr:uid="{00000000-0004-0000-0800-000001000000}"/>
-    <hyperlink ref="E4" r:id="rId3" xr:uid="{00000000-0004-0000-0800-000002000000}"/>
-    <hyperlink ref="E5" r:id="rId4" xr:uid="{00000000-0004-0000-0800-000003000000}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:H5" numberStoredAsText="1"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>209</v>
-      </c>
-      <c r="B2">
-        <v>1467</v>
-      </c>
-      <c r="C2" t="s">
-        <v>210</v>
-      </c>
-      <c r="D2" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>212</v>
-      </c>
-      <c r="B3">
-        <v>1468</v>
-      </c>
-      <c r="C3" t="s">
-        <v>213</v>
-      </c>
-      <c r="D3" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>215</v>
-      </c>
-      <c r="B4">
-        <v>1469</v>
-      </c>
-      <c r="C4" t="s">
-        <v>216</v>
-      </c>
-      <c r="D4" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>217</v>
-      </c>
-      <c r="B5">
-        <v>1470</v>
-      </c>
-      <c r="C5" t="s">
-        <v>218</v>
-      </c>
-      <c r="D5" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>220</v>
-      </c>
-      <c r="B6">
-        <v>1471</v>
-      </c>
-      <c r="C6" t="s">
-        <v>221</v>
-      </c>
-      <c r="D6" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>222</v>
-      </c>
-      <c r="B7">
-        <v>1472</v>
-      </c>
-      <c r="C7" t="s">
-        <v>223</v>
-      </c>
-      <c r="D7" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>225</v>
-      </c>
-      <c r="B8">
-        <v>1473</v>
-      </c>
-      <c r="C8" t="s">
-        <v>226</v>
-      </c>
-      <c r="D8" t="s">
-        <v>211</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:D8" numberStoredAsText="1"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
"Complete Bulk Promotion automation for Customer and Order entities"
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\claude_repos\trigital\nipige_qa_automation\src\resources\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sriro\Music\nipige_qa_automation\src\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD9E1556-7960-4039-A5B6-5614B938C703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{608D0EBE-8A00-4AEA-81BF-24BD4AD7EDC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Regression" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="269">
   <si>
     <t>TestName</t>
   </si>
@@ -738,16 +738,126 @@
   </si>
   <si>
     <t>InventoryManagement</t>
+  </si>
+  <si>
+    <t>TC08_Customer_Date</t>
+  </si>
+  <si>
+    <t>Validate Customer Date</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>12-05-2026|19-05-2026</t>
+  </si>
+  <si>
+    <t>TC09_Customer_InvalidEmail</t>
+  </si>
+  <si>
+    <t>Validate Invalid Customer Email</t>
+  </si>
+  <si>
+    <t>invalid@test.com</t>
+  </si>
+  <si>
+    <t>TC10_Customer_InvalidPhone</t>
+  </si>
+  <si>
+    <t>Validate Invalid Customer Phone</t>
+  </si>
+  <si>
+    <t>TC11_Customer_InvalidCustomerNo</t>
+  </si>
+  <si>
+    <t>Validate Invalid Customer Number</t>
+  </si>
+  <si>
+    <t>CKXM99999</t>
+  </si>
+  <si>
+    <t>TC12_Order_City</t>
+  </si>
+  <si>
+    <t>Validate Order City</t>
+  </si>
+  <si>
+    <t>Order</t>
+  </si>
+  <si>
+    <t>TC13_Order_Date</t>
+  </si>
+  <si>
+    <t>Validate Order Date</t>
+  </si>
+  <si>
+    <t>01-01-2026|08-06-2026</t>
+  </si>
+  <si>
+    <t>TC14_Order_OrderAmount</t>
+  </si>
+  <si>
+    <t>Validate Order Amount</t>
+  </si>
+  <si>
+    <t>Order Amount</t>
+  </si>
+  <si>
+    <t>1|100</t>
+  </si>
+  <si>
+    <t>Range</t>
+  </si>
+  <si>
+    <t>TC15_Order_InvalidCity</t>
+  </si>
+  <si>
+    <t>Validate Invalid Order City</t>
+  </si>
+  <si>
+    <t>InvalidCity123</t>
+  </si>
+  <si>
+    <t>TC16_Order_InvalidOrderAmount</t>
+  </si>
+  <si>
+    <t>Validate Invalid Order Amount</t>
+  </si>
+  <si>
+    <t>999999|9999999</t>
+  </si>
+  <si>
+    <t>TC10_BulkPromotionTenantLogin</t>
+  </si>
+  <si>
+    <t>Bulk Promotion Tenant Login</t>
+  </si>
+  <si>
+    <t>nipigev2@gmail.com</t>
+  </si>
+  <si>
+    <t>8145031601|9787264649</t>
+  </si>
+  <si>
+    <t>Equal (eq)|Or</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -770,13 +880,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1115,14 +1234,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1133,7 +1252,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1144,7 +1263,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>233</v>
       </c>
@@ -1155,7 +1274,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>234</v>
       </c>
@@ -1166,7 +1285,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>231</v>
       </c>
@@ -1177,7 +1296,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>232</v>
       </c>
@@ -1188,7 +1307,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -1199,7 +1318,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -1210,7 +1329,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -1221,7 +1340,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -1232,7 +1351,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -1243,7 +1362,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -1254,7 +1373,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1276,9 +1395,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -1304,7 +1423,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>153</v>
       </c>
@@ -1327,7 +1446,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>158</v>
       </c>
@@ -1350,7 +1469,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>163</v>
       </c>
@@ -1376,7 +1495,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>168</v>
       </c>
@@ -1402,7 +1521,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>173</v>
       </c>
@@ -1428,7 +1547,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>179</v>
       </c>
@@ -1462,9 +1581,9 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -1490,7 +1609,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>184</v>
       </c>
@@ -1516,7 +1635,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>191</v>
       </c>
@@ -1542,7 +1661,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>196</v>
       </c>
@@ -1568,7 +1687,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>201</v>
       </c>
@@ -1611,9 +1730,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -1627,7 +1746,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>208</v>
       </c>
@@ -1641,7 +1760,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>211</v>
       </c>
@@ -1655,7 +1774,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>214</v>
       </c>
@@ -1669,7 +1788,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>216</v>
       </c>
@@ -1683,7 +1802,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>219</v>
       </c>
@@ -1697,7 +1816,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>221</v>
       </c>
@@ -1711,7 +1830,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>224</v>
       </c>
@@ -1736,7 +1855,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90FDD46F-321E-406B-BA60-13EEF3FF3405}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1745,7 +1864,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3361DFF-EE58-48FD-8CE6-2AFDE302B9DA}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1753,19 +1872,19 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="39.375" customWidth="1"/>
-    <col min="2" max="2" width="5.125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="39.33203125" customWidth="1"/>
+    <col min="2" max="2" width="5.08203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.08203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.625" customWidth="1"/>
+    <col min="7" max="7" width="17.58203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -1788,7 +1907,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>85</v>
       </c>
@@ -1808,7 +1927,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>90</v>
       </c>
@@ -1831,7 +1950,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>93</v>
       </c>
@@ -1851,7 +1970,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>95</v>
       </c>
@@ -1874,7 +1993,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>97</v>
       </c>
@@ -1891,7 +2010,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>226</v>
       </c>
@@ -1911,7 +2030,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>227</v>
       </c>
@@ -1934,7 +2053,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>228</v>
       </c>
@@ -1957,7 +2076,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>229</v>
       </c>
@@ -1978,6 +2097,26 @@
       </c>
       <c r="G10" t="s">
         <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>264</v>
+      </c>
+      <c r="B11">
+        <v>1251</v>
+      </c>
+      <c r="C11" t="s">
+        <v>265</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F11" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -1988,6 +2127,8 @@
     <hyperlink ref="D8" r:id="rId4" xr:uid="{33EA80E7-EC4F-41B9-9C67-2CEDFBF5C34A}"/>
     <hyperlink ref="D9" r:id="rId5" xr:uid="{FD23F8A3-A64F-4EDA-B8EA-97C2997BE764}"/>
     <hyperlink ref="D10" r:id="rId6" xr:uid="{E804A7F5-03A4-4223-84A7-C5315820A820}"/>
+    <hyperlink ref="D11" r:id="rId7" xr:uid="{346528A0-CA07-478D-B41D-0385E13B45A4}"/>
+    <hyperlink ref="E11" r:id="rId8" xr:uid="{390ACB72-9C8E-4726-B632-153FD8F494C7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -1999,13 +2140,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:L3"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="28.75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.08203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -2043,7 +2184,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>108</v>
       </c>
@@ -2078,7 +2219,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>117</v>
       </c>
@@ -2103,15 +2244,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:O3"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.58203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.75" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="14.625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -2158,7 +2299,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -2205,7 +2346,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>43</v>
       </c>
@@ -2267,7 +2408,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F107B412-2D3C-4F87-A9E1-F6E22431D809}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2276,12 +2417,12 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.08203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -2307,7 +2448,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>58</v>
       </c>
@@ -2333,7 +2474,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>65</v>
       </c>
@@ -2373,213 +2514,416 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.9140625" customWidth="1"/>
+    <col min="2" max="2" width="25.58203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.4140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>15</v>
       </c>
       <c r="B1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C1" t="s">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="D1" t="s">
-        <v>72</v>
+        <v>119</v>
       </c>
       <c r="E1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G1" t="s">
-        <v>121</v>
-      </c>
-      <c r="H1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>123</v>
       </c>
       <c r="B2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C2" t="s">
-        <v>124</v>
+        <v>89</v>
       </c>
       <c r="D2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E2" t="s">
+        <v>126</v>
+      </c>
+      <c r="F2" t="s">
+        <v>127</v>
+      </c>
+      <c r="G2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C3" t="s">
         <v>89</v>
       </c>
-      <c r="E2" t="s">
+      <c r="D3" t="s">
         <v>125</v>
       </c>
-      <c r="F2" t="s">
-        <v>126</v>
-      </c>
-      <c r="G2" t="s">
-        <v>127</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="E3" t="s">
+        <v>131</v>
+      </c>
+      <c r="F3" t="s">
+        <v>132</v>
+      </c>
+      <c r="G3" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
-        <v>129</v>
-      </c>
-      <c r="C3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D3" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B4" t="s">
+        <v>134</v>
+      </c>
+      <c r="C4" t="s">
         <v>89</v>
       </c>
-      <c r="E3" t="s">
+      <c r="D4" t="s">
         <v>125</v>
       </c>
-      <c r="F3" t="s">
-        <v>131</v>
-      </c>
-      <c r="G3" t="s">
-        <v>132</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
+        <v>135</v>
+      </c>
+      <c r="G4" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>133</v>
-      </c>
-      <c r="C4" t="s">
-        <v>134</v>
-      </c>
-      <c r="D4" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C5" t="s">
         <v>89</v>
       </c>
-      <c r="E4" t="s">
+      <c r="D5" t="s">
         <v>125</v>
       </c>
-      <c r="F4" t="s">
+      <c r="E5" t="s">
+        <v>138</v>
+      </c>
+      <c r="F5" t="s">
+        <v>267</v>
+      </c>
+      <c r="G5" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>139</v>
+      </c>
+      <c r="B6" t="s">
+        <v>140</v>
+      </c>
+      <c r="C6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D6" t="s">
+        <v>125</v>
+      </c>
+      <c r="E6" t="s">
+        <v>141</v>
+      </c>
+      <c r="F6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>143</v>
+      </c>
+      <c r="B7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" t="s">
+        <v>145</v>
+      </c>
+      <c r="G7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>146</v>
+      </c>
+      <c r="B8" t="s">
+        <v>147</v>
+      </c>
+      <c r="C8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D8" t="s">
+        <v>125</v>
+      </c>
+      <c r="E8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" t="s">
+        <v>148</v>
+      </c>
+      <c r="G8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G4" t="s">
-        <v>135</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="F10" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
-        <v>136</v>
-      </c>
-      <c r="C5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D5" t="s">
+    <row r="11" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E5" t="s">
+      <c r="D11" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="F5" t="s">
+      <c r="E11" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="G5">
-        <v>8145031601</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="F11" s="1">
+        <v>9999999999</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
-        <v>139</v>
-      </c>
-      <c r="C6" t="s">
-        <v>140</v>
-      </c>
-      <c r="D6" t="s">
+    <row r="12" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E6" t="s">
+      <c r="D12" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="F6" t="s">
+      <c r="E12" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="G6" t="s">
-        <v>142</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="F12" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="G12" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
-        <v>143</v>
-      </c>
-      <c r="C7" t="s">
-        <v>144</v>
-      </c>
-      <c r="D7" t="s">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E7" t="s">
-        <v>125</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="D13" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G7" t="s">
+      <c r="F13" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="H7" t="s">
+      <c r="G13" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
-        <v>146</v>
-      </c>
-      <c r="C8" t="s">
-        <v>147</v>
-      </c>
-      <c r="D8" t="s">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E8" t="s">
-        <v>125</v>
-      </c>
-      <c r="F8" t="s">
-        <v>27</v>
-      </c>
-      <c r="G8" t="s">
-        <v>148</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="D14" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="G16" s="1" t="s">
         <v>128</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>257</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G4" r:id="rId1" xr:uid="{00000000-0004-0000-0600-000000000000}"/>
+    <hyperlink ref="F4" r:id="rId1" xr:uid="{00000000-0004-0000-0600-000000000000}"/>
+    <hyperlink ref="F10" r:id="rId2" display="mailto:invalid@test.com" xr:uid="{2B0BCEEB-6DBA-4045-A62E-9E288076F940}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:H8" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:G4 A6:G8 A5:E5" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added Order Management automation test cases
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dbt\nipigeautomation\src\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10234118-E70A-4085-B825-86FFC29AC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29D97619-8B61-418D-B50F-F3F35555F58F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="734" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="734" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Regression" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="SOAPAccountServiceTest" sheetId="11" r:id="rId6"/>
     <sheet name="DatabaseTest" sheetId="10" r:id="rId7"/>
     <sheet name="DashboardTest" sheetId="12" r:id="rId8"/>
+    <sheet name="OrderManagementTest" sheetId="13" r:id="rId9"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="188">
   <si>
     <t>TestID</t>
   </si>
@@ -568,6 +569,36 @@
   </si>
   <si>
     <t>TC03_DashboardFilters</t>
+  </si>
+  <si>
+    <t>TC01_OrderManagementLoad</t>
+  </si>
+  <si>
+    <t>Verify Order Management Load</t>
+  </si>
+  <si>
+    <t>Verify Status Filter</t>
+  </si>
+  <si>
+    <t>Verify Date Filter</t>
+  </si>
+  <si>
+    <t>TC02_DateAndStatusFilter</t>
+  </si>
+  <si>
+    <t>TC03_DateAndSellerFilter</t>
+  </si>
+  <si>
+    <t>TC04_DateAndOrderIdFilter</t>
+  </si>
+  <si>
+    <t>Verify Date Filter and Order ID Search</t>
+  </si>
+  <si>
+    <t>TC05_DateStatusOrderViewInvoice</t>
+  </si>
+  <si>
+    <t>Verify Date Status Order View Invoice</t>
   </si>
 </sst>
 </file>
@@ -2046,4 +2077,158 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8E0A376-854F-457B-828F-0E5D4623CA7D}">
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.36328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="G1" s="6"/>
+    </row>
+    <row r="2" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="B2" s="7">
+        <v>3001</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="G2" s="7"/>
+    </row>
+    <row r="3" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="B3" s="7">
+        <v>3002</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="G3" s="7"/>
+    </row>
+    <row r="4" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="B4" s="7">
+        <v>3003</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="G4" s="7"/>
+    </row>
+    <row r="5" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="B5" s="7">
+        <v>3004</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="G5" s="7"/>
+    </row>
+    <row r="6" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="B6" s="7">
+        <v>3005</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="G6" s="7"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="7"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" display="mailto:freshcart@gmail.com" xr:uid="{39A8A2C6-51FA-4A8F-BBA2-C8F0A1866DDD}"/>
+    <hyperlink ref="D3" r:id="rId2" display="mailto:freshcart@gmail.com" xr:uid="{03EEE9D9-33A3-4E26-BD4A-9869753FCAA3}"/>
+    <hyperlink ref="D4" r:id="rId3" display="mailto:freshcart@gmail.com" xr:uid="{6AC17F8E-9110-4912-AAF9-6B89AE6B446B}"/>
+    <hyperlink ref="D5" r:id="rId4" display="mailto:freshcart@gmail.com" xr:uid="{BA4EE33D-B416-428D-A5C9-121DFB3CDC74}"/>
+    <hyperlink ref="D6" r:id="rId5" display="mailto:freshcart@gmail.com" xr:uid="{682055B1-D339-4015-AE73-93260B3C300B}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed service ticket errors
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sriro\Music\nipige_qa_automation\src\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C52E7691-6C80-4CA3-A594-10D1FC587B81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCCF6B2F-99CD-4DC3-A60D-93B68FA82991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Regression" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="260">
   <si>
     <t>TestName</t>
   </si>
@@ -231,55 +231,13 @@
     <t>TicketID</t>
   </si>
   <si>
-    <t>CustomerName</t>
-  </si>
-  <si>
     <t>Subject</t>
   </si>
   <si>
     <t>Status</t>
   </si>
   <si>
-    <t>NewStatus</t>
-  </si>
-  <si>
-    <t>NoteToCustomer</t>
-  </si>
-  <si>
-    <t>InternalNote</t>
-  </si>
-  <si>
-    <t>TC01_ViewAndCloseServiceTicket</t>
-  </si>
-  <si>
-    <t>Service Ticket View and Close</t>
-  </si>
-  <si>
-    <t>SR6351088432</t>
-  </si>
-  <si>
-    <t>Biswarup Roy</t>
-  </si>
-  <si>
-    <t>Test</t>
-  </si>
-  <si>
-    <t>OPEN</t>
-  </si>
-  <si>
-    <t>CLOSED</t>
-  </si>
-  <si>
-    <t>Ticket closed successfully</t>
-  </si>
-  <si>
-    <t>Closed by automation test</t>
-  </si>
-  <si>
     <t>TC02_InvalidTicketID</t>
-  </si>
-  <si>
-    <t>Service Ticket Invalid Ticket ID</t>
   </si>
   <si>
     <t>SR9999999999</t>
@@ -852,13 +810,16 @@
   </si>
   <si>
     <t>To execute a select query after delete</t>
+  </si>
+  <si>
+    <t>Service Ticket Invalid Ticket ID</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -870,6 +831,22 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -892,14 +869,26 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1455,166 +1444,166 @@
         <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>196</v>
+        <v>182</v>
       </c>
       <c r="E1" t="s">
-        <v>197</v>
+        <v>183</v>
       </c>
       <c r="F1" t="s">
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="G1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H1" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>200</v>
+        <v>186</v>
       </c>
       <c r="B2">
         <v>1137</v>
       </c>
       <c r="C2" t="s">
-        <v>201</v>
+        <v>187</v>
       </c>
       <c r="D2" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="E2" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="G2">
         <v>200</v>
       </c>
       <c r="H2" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>205</v>
+        <v>191</v>
       </c>
       <c r="B3">
         <v>1138</v>
       </c>
       <c r="C3" t="s">
-        <v>206</v>
+        <v>192</v>
       </c>
       <c r="D3" t="s">
-        <v>207</v>
+        <v>193</v>
       </c>
       <c r="E3" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="G3">
         <v>200</v>
       </c>
       <c r="H3" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="B4">
         <v>1139</v>
       </c>
       <c r="C4" t="s">
-        <v>211</v>
+        <v>197</v>
       </c>
       <c r="D4" t="s">
-        <v>212</v>
+        <v>198</v>
       </c>
       <c r="E4" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="F4" t="s">
-        <v>213</v>
+        <v>199</v>
       </c>
       <c r="G4">
         <v>201</v>
       </c>
       <c r="H4" t="s">
-        <v>214</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>215</v>
+        <v>201</v>
       </c>
       <c r="B5">
         <v>1140</v>
       </c>
       <c r="C5" t="s">
-        <v>216</v>
+        <v>202</v>
       </c>
       <c r="D5" t="s">
-        <v>217</v>
+        <v>203</v>
       </c>
       <c r="E5" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="F5" t="s">
-        <v>218</v>
+        <v>204</v>
       </c>
       <c r="G5">
         <v>200</v>
       </c>
       <c r="H5" t="s">
-        <v>219</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>220</v>
+        <v>206</v>
       </c>
       <c r="B6">
         <v>1141</v>
       </c>
       <c r="C6" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="D6" t="s">
-        <v>222</v>
+        <v>208</v>
       </c>
       <c r="E6" t="s">
-        <v>223</v>
+        <v>209</v>
       </c>
       <c r="F6" t="s">
-        <v>224</v>
+        <v>210</v>
       </c>
       <c r="G6">
         <v>201</v>
       </c>
       <c r="H6" t="s">
-        <v>225</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>226</v>
+        <v>212</v>
       </c>
       <c r="B7">
         <v>1142</v>
       </c>
       <c r="C7" t="s">
-        <v>227</v>
+        <v>213</v>
       </c>
       <c r="D7" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
       <c r="E7" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="G7">
         <v>200</v>
       </c>
       <c r="H7" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -1641,123 +1630,123 @@
         <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>196</v>
+        <v>182</v>
       </c>
       <c r="E1" t="s">
-        <v>197</v>
+        <v>183</v>
       </c>
       <c r="F1" t="s">
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="G1" t="s">
-        <v>229</v>
+        <v>215</v>
       </c>
       <c r="H1" t="s">
-        <v>230</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="B2">
         <v>1113</v>
       </c>
       <c r="C2" t="s">
-        <v>232</v>
+        <v>218</v>
       </c>
       <c r="D2" t="s">
-        <v>233</v>
+        <v>219</v>
       </c>
       <c r="E2" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="F2" t="s">
-        <v>235</v>
+        <v>221</v>
       </c>
       <c r="G2" t="s">
-        <v>236</v>
+        <v>222</v>
       </c>
       <c r="H2" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>238</v>
+        <v>224</v>
       </c>
       <c r="B3">
         <v>1114</v>
       </c>
       <c r="C3" t="s">
-        <v>239</v>
+        <v>225</v>
       </c>
       <c r="D3" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
       <c r="E3" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="F3" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="G3" t="s">
-        <v>236</v>
+        <v>222</v>
       </c>
       <c r="H3" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="B4">
         <v>1115</v>
       </c>
       <c r="C4" t="s">
-        <v>244</v>
+        <v>230</v>
       </c>
       <c r="D4" t="s">
-        <v>245</v>
+        <v>231</v>
       </c>
       <c r="E4" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="F4" t="s">
-        <v>246</v>
+        <v>232</v>
       </c>
       <c r="G4" t="s">
-        <v>236</v>
+        <v>222</v>
       </c>
       <c r="H4" t="s">
-        <v>247</v>
+        <v>233</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>248</v>
+        <v>234</v>
       </c>
       <c r="B5">
         <v>1116</v>
       </c>
       <c r="C5" t="s">
-        <v>249</v>
+        <v>235</v>
       </c>
       <c r="D5" t="s">
-        <v>250</v>
+        <v>236</v>
       </c>
       <c r="E5" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="F5" t="s">
-        <v>251</v>
+        <v>237</v>
       </c>
       <c r="G5" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
       <c r="H5" t="s">
-        <v>253</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>
@@ -1790,105 +1779,105 @@
         <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>254</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>255</v>
+        <v>241</v>
       </c>
       <c r="B2">
         <v>1467</v>
       </c>
       <c r="C2" t="s">
-        <v>256</v>
+        <v>242</v>
       </c>
       <c r="D2" t="s">
-        <v>257</v>
+        <v>243</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>258</v>
+        <v>244</v>
       </c>
       <c r="B3">
         <v>1468</v>
       </c>
       <c r="C3" t="s">
-        <v>259</v>
+        <v>245</v>
       </c>
       <c r="D3" t="s">
-        <v>260</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>261</v>
+        <v>247</v>
       </c>
       <c r="B4">
         <v>1469</v>
       </c>
       <c r="C4" t="s">
-        <v>262</v>
+        <v>248</v>
       </c>
       <c r="D4" t="s">
-        <v>257</v>
+        <v>243</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>263</v>
+        <v>249</v>
       </c>
       <c r="B5">
         <v>1470</v>
       </c>
       <c r="C5" t="s">
-        <v>264</v>
+        <v>250</v>
       </c>
       <c r="D5" t="s">
-        <v>265</v>
+        <v>251</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>266</v>
+        <v>252</v>
       </c>
       <c r="B6">
         <v>1471</v>
       </c>
       <c r="C6" t="s">
-        <v>267</v>
+        <v>253</v>
       </c>
       <c r="D6" t="s">
-        <v>257</v>
+        <v>243</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>268</v>
+        <v>254</v>
       </c>
       <c r="B7">
         <v>1472</v>
       </c>
       <c r="C7" t="s">
-        <v>269</v>
+        <v>255</v>
       </c>
       <c r="D7" t="s">
-        <v>270</v>
+        <v>256</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>271</v>
+        <v>257</v>
       </c>
       <c r="B8">
         <v>1473</v>
       </c>
       <c r="C8" t="s">
-        <v>272</v>
+        <v>258</v>
       </c>
       <c r="D8" t="s">
-        <v>257</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -1929,6 +1918,9 @@
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="36.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -2047,10 +2039,10 @@
       <c r="C6" t="s">
         <v>46</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="5" t="s">
         <v>48</v>
       </c>
       <c r="F6" t="s">
@@ -2176,120 +2168,80 @@
     <hyperlink ref="D10" r:id="rId6" xr:uid="{00000000-0004-0000-0300-000005000000}"/>
     <hyperlink ref="D11" r:id="rId7" xr:uid="{00000000-0004-0000-0300-000006000000}"/>
     <hyperlink ref="E11" r:id="rId8" xr:uid="{00000000-0004-0000-0300-000007000000}"/>
+    <hyperlink ref="D6" r:id="rId9" xr:uid="{FAF596BA-AF62-4C07-B70A-75B5EEAC08D8}"/>
+    <hyperlink ref="E6" r:id="rId10" xr:uid="{BC708EAE-BB71-4661-9C3E-175EF768F75A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:G11" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:G5 A7:G11 A6:C6 F6:G6" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:L3"/>
+  <dimension ref="C1:I5"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="28.75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.75" customWidth="1"/>
+    <col min="4" max="4" width="15.08203125" customWidth="1"/>
+    <col min="5" max="5" width="14.75" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.5" customWidth="1"/>
+    <col min="9" max="9" width="28" customWidth="1"/>
     <col min="10" max="10" width="9.58203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="21.58203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="22.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="D1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D1" t="s">
-        <v>24</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H1" t="s">
-        <v>67</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+    </row>
+    <row r="2" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C2" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="J1" t="s">
+      <c r="D2" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="K1" t="s">
-        <v>70</v>
-      </c>
-      <c r="L1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C2" t="s">
-        <v>73</v>
-      </c>
-      <c r="E2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F2" t="s">
-        <v>74</v>
-      </c>
-      <c r="G2" t="s">
-        <v>75</v>
-      </c>
-      <c r="H2" t="s">
-        <v>76</v>
-      </c>
-      <c r="I2" t="s">
-        <v>77</v>
-      </c>
-      <c r="J2" t="s">
-        <v>78</v>
-      </c>
-      <c r="K2" t="s">
-        <v>79</v>
-      </c>
-      <c r="L2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B3" t="s">
-        <v>81</v>
-      </c>
-      <c r="C3" t="s">
-        <v>82</v>
-      </c>
-      <c r="E3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F3" t="s">
-        <v>83</v>
-      </c>
-    </row>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" spans="3:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+    </row>
+    <row r="5" spans="3:9" ht="12" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:L3" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -2309,134 +2261,134 @@
         <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="E1" t="s">
         <v>27</v>
       </c>
       <c r="F1" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="G1" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="H1" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="I1" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="J1" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="K1" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="L1" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="M1" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="N1" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="O1" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="B2">
         <v>11235</v>
       </c>
       <c r="C2" t="s">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="D2" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="E2" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="F2" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="G2" t="s">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="H2" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="I2" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="J2" t="s">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="K2" t="s">
-        <v>103</v>
+        <v>89</v>
       </c>
       <c r="L2" t="s">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="M2" t="s">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="N2" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="O2" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="B3">
         <v>11645</v>
       </c>
       <c r="C3" t="s">
-        <v>109</v>
+        <v>95</v>
       </c>
       <c r="D3" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="E3" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="F3" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="G3" t="s">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="H3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I3" t="s">
+        <v>87</v>
+      </c>
+      <c r="J3" t="s">
+        <v>99</v>
+      </c>
+      <c r="K3" t="s">
         <v>100</v>
       </c>
-      <c r="I3" t="s">
+      <c r="L3" t="s">
         <v>101</v>
       </c>
-      <c r="J3" t="s">
-        <v>113</v>
-      </c>
-      <c r="K3" t="s">
-        <v>114</v>
-      </c>
-      <c r="L3" t="s">
-        <v>115</v>
-      </c>
       <c r="M3" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="N3" t="s">
-        <v>117</v>
+        <v>103</v>
       </c>
       <c r="O3" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -2479,71 +2431,71 @@
         <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>119</v>
+        <v>105</v>
       </c>
       <c r="E1" t="s">
-        <v>120</v>
+        <v>106</v>
       </c>
       <c r="F1" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="G1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H1" t="s">
-        <v>121</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="B2">
         <v>1337</v>
       </c>
       <c r="C2" t="s">
-        <v>123</v>
+        <v>109</v>
       </c>
       <c r="D2" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="E2" t="s">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="F2" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="G2" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="H2" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="B3">
         <v>1547</v>
       </c>
       <c r="C3" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="D3" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
       <c r="E3" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="F3" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="G3" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="H3" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -2581,384 +2533,384 @@
         <v>28</v>
       </c>
       <c r="D1" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="E1" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="F1" t="s">
-        <v>137</v>
+        <v>123</v>
       </c>
       <c r="G1" t="s">
-        <v>138</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="B2" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="C2" t="s">
         <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="E2" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="F2" t="s">
-        <v>143</v>
+        <v>129</v>
       </c>
       <c r="G2" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="B3" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
       <c r="C3" t="s">
         <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="E3" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="F3" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="G3" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="B4" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="C4" t="s">
         <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="E4" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="F4" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="G4" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="B5" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="C5" t="s">
         <v>34</v>
       </c>
       <c r="D5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E5" t="s">
+        <v>140</v>
+      </c>
+      <c r="F5" t="s">
         <v>141</v>
       </c>
-      <c r="E5" t="s">
-        <v>154</v>
-      </c>
-      <c r="F5" t="s">
-        <v>155</v>
-      </c>
       <c r="G5" t="s">
-        <v>156</v>
+        <v>142</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="B6" t="s">
-        <v>158</v>
+        <v>144</v>
       </c>
       <c r="C6" t="s">
         <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="E6" t="s">
-        <v>159</v>
+        <v>145</v>
       </c>
       <c r="F6" t="s">
-        <v>160</v>
+        <v>146</v>
       </c>
       <c r="G6" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>161</v>
+        <v>147</v>
       </c>
       <c r="B7" t="s">
-        <v>162</v>
+        <v>148</v>
       </c>
       <c r="C7" t="s">
         <v>34</v>
       </c>
       <c r="D7" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="E7" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="F7" t="s">
-        <v>163</v>
+        <v>149</v>
       </c>
       <c r="G7" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="B8" t="s">
-        <v>165</v>
+        <v>151</v>
       </c>
       <c r="C8" t="s">
         <v>34</v>
       </c>
       <c r="D8" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="E8" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="F8" t="s">
-        <v>166</v>
+        <v>152</v>
       </c>
       <c r="G8" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>167</v>
+        <v>153</v>
       </c>
       <c r="B9" t="s">
-        <v>168</v>
+        <v>154</v>
       </c>
       <c r="C9" t="s">
         <v>34</v>
       </c>
       <c r="D9" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="E9" t="s">
-        <v>169</v>
+        <v>155</v>
       </c>
       <c r="F9" t="s">
-        <v>170</v>
+        <v>156</v>
       </c>
       <c r="G9" t="s">
-        <v>169</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>171</v>
+        <v>157</v>
       </c>
       <c r="B10" t="s">
-        <v>172</v>
+        <v>158</v>
       </c>
       <c r="C10" t="s">
         <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="E10" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="F10" t="s">
-        <v>173</v>
+        <v>159</v>
       </c>
       <c r="G10" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>174</v>
+        <v>160</v>
       </c>
       <c r="B11" t="s">
-        <v>175</v>
+        <v>161</v>
       </c>
       <c r="C11" t="s">
         <v>34</v>
       </c>
       <c r="D11" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="E11" t="s">
-        <v>154</v>
+        <v>140</v>
       </c>
       <c r="F11">
         <v>9999999999</v>
       </c>
       <c r="G11" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>176</v>
+        <v>162</v>
       </c>
       <c r="B12" t="s">
-        <v>177</v>
+        <v>163</v>
       </c>
       <c r="C12" t="s">
         <v>34</v>
       </c>
       <c r="D12" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="E12" t="s">
-        <v>159</v>
+        <v>145</v>
       </c>
       <c r="F12" t="s">
-        <v>178</v>
+        <v>164</v>
       </c>
       <c r="G12" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="B13" t="s">
-        <v>180</v>
+        <v>166</v>
       </c>
       <c r="C13" t="s">
         <v>34</v>
       </c>
       <c r="D13" t="s">
-        <v>181</v>
+        <v>167</v>
       </c>
       <c r="E13" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="F13" t="s">
-        <v>163</v>
+        <v>149</v>
       </c>
       <c r="G13" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>182</v>
+        <v>168</v>
       </c>
       <c r="B14" t="s">
-        <v>183</v>
+        <v>169</v>
       </c>
       <c r="C14" t="s">
         <v>34</v>
       </c>
       <c r="D14" t="s">
-        <v>181</v>
+        <v>167</v>
       </c>
       <c r="E14" t="s">
-        <v>169</v>
+        <v>155</v>
       </c>
       <c r="F14" t="s">
-        <v>184</v>
+        <v>170</v>
       </c>
       <c r="G14" t="s">
-        <v>169</v>
+        <v>155</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>185</v>
+        <v>171</v>
       </c>
       <c r="B15" t="s">
-        <v>186</v>
+        <v>172</v>
       </c>
       <c r="C15" t="s">
         <v>34</v>
       </c>
       <c r="D15" t="s">
-        <v>181</v>
+        <v>167</v>
       </c>
       <c r="E15" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="F15" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="G15" t="s">
-        <v>189</v>
+        <v>175</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>190</v>
+        <v>176</v>
       </c>
       <c r="B16" t="s">
-        <v>191</v>
+        <v>177</v>
       </c>
       <c r="C16" t="s">
         <v>34</v>
       </c>
       <c r="D16" t="s">
-        <v>181</v>
+        <v>167</v>
       </c>
       <c r="E16" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="F16" t="s">
-        <v>192</v>
+        <v>178</v>
       </c>
       <c r="G16" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>193</v>
+        <v>179</v>
       </c>
       <c r="B17" t="s">
-        <v>194</v>
+        <v>180</v>
       </c>
       <c r="C17" t="s">
         <v>34</v>
       </c>
       <c r="D17" t="s">
+        <v>167</v>
+      </c>
+      <c r="E17" t="s">
+        <v>173</v>
+      </c>
+      <c r="F17" t="s">
         <v>181</v>
       </c>
-      <c r="E17" t="s">
-        <v>187</v>
-      </c>
-      <c r="F17" t="s">
-        <v>195</v>
-      </c>
       <c r="G17" t="s">
-        <v>189</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
payment report  automation test cases
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -8,28 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dbt\nipigeautomation\src\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CE17043-60E8-4B92-8336-DAE26C6504C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D745FB06-B87C-49EC-8D88-5B28D9182909}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Regression" sheetId="1" r:id="rId1"/>
     <sheet name="OrderManagementTest" sheetId="9" r:id="rId2"/>
-    <sheet name="DashboardTest" sheetId="10" r:id="rId3"/>
-    <sheet name="CreateAccountTest" sheetId="2" r:id="rId4"/>
-    <sheet name="ContactUsTest" sheetId="3" r:id="rId5"/>
-    <sheet name="LoginTest" sheetId="4" r:id="rId6"/>
-    <sheet name="CustomerManagement" sheetId="5" r:id="rId7"/>
-    <sheet name="RESTUserTest" sheetId="6" r:id="rId8"/>
-    <sheet name="SOAPAccountServiceTest" sheetId="7" r:id="rId9"/>
-    <sheet name="DatabaseTest" sheetId="8" r:id="rId10"/>
+    <sheet name="PaymentReportTest" sheetId="11" r:id="rId3"/>
+    <sheet name="DashboardTest" sheetId="10" r:id="rId4"/>
+    <sheet name="CreateAccountTest" sheetId="2" r:id="rId5"/>
+    <sheet name="ContactUsTest" sheetId="3" r:id="rId6"/>
+    <sheet name="LoginTest" sheetId="4" r:id="rId7"/>
+    <sheet name="CustomerManagement" sheetId="5" r:id="rId8"/>
+    <sheet name="RESTUserTest" sheetId="6" r:id="rId9"/>
+    <sheet name="SOAPAccountServiceTest" sheetId="7" r:id="rId10"/>
+    <sheet name="DatabaseTest" sheetId="8" r:id="rId11"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="264">
   <si>
     <t>TestName</t>
   </si>
@@ -778,6 +779,51 @@
   </si>
   <si>
     <t>DashboardTest</t>
+  </si>
+  <si>
+    <t>TC01_PaymentReportLoad</t>
+  </si>
+  <si>
+    <t>Verify Payment Report Page Load</t>
+  </si>
+  <si>
+    <t>TC02_DateFilterValidation</t>
+  </si>
+  <si>
+    <t>Verify Date Filters</t>
+  </si>
+  <si>
+    <t>TC03_RefreshValidation</t>
+  </si>
+  <si>
+    <t>Verify Refresh Button</t>
+  </si>
+  <si>
+    <t>TC04_ExportCSVValidation</t>
+  </si>
+  <si>
+    <t>Verify Export CSV</t>
+  </si>
+  <si>
+    <t>Verify PDF Download</t>
+  </si>
+  <si>
+    <t>PaymentReportTest</t>
+  </si>
+  <si>
+    <t>TC06_CollectionTrendFilters</t>
+  </si>
+  <si>
+    <t>Verify Collection Trend Filters</t>
+  </si>
+  <si>
+    <t>TC05_PDFValidation</t>
+  </si>
+  <si>
+    <t>FromDate</t>
+  </si>
+  <si>
+    <t>ToDate</t>
   </si>
 </sst>
 </file>
@@ -830,7 +876,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -839,6 +885,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1181,7 +1230,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24.58203125" customWidth="1"/>
@@ -1276,7 +1325,7 @@
         <v>10</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>5</v>
@@ -1300,7 +1349,7 @@
         <v>12</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>5</v>
@@ -1312,7 +1361,7 @@
         <v>13</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>9</v>
@@ -1324,7 +1373,7 @@
         <v>14</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>5</v>
@@ -1336,7 +1385,7 @@
         <v>3</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>5</v>
@@ -1348,7 +1397,7 @@
         <v>226</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>9</v>
@@ -1360,7 +1409,7 @@
         <v>227</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>5</v>
@@ -1372,7 +1421,7 @@
         <v>228</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>5</v>
@@ -1384,7 +1433,7 @@
         <v>229</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>9</v>
@@ -1398,6 +1447,17 @@
         <v>8</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>258</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1407,6 +1467,155 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E1" t="s">
+        <v>145</v>
+      </c>
+      <c r="F1" t="s">
+        <v>146</v>
+      </c>
+      <c r="G1" t="s">
+        <v>178</v>
+      </c>
+      <c r="H1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B2">
+        <v>1113</v>
+      </c>
+      <c r="C2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D2" t="s">
+        <v>182</v>
+      </c>
+      <c r="E2" t="s">
+        <v>183</v>
+      </c>
+      <c r="F2" t="s">
+        <v>184</v>
+      </c>
+      <c r="G2" t="s">
+        <v>185</v>
+      </c>
+      <c r="H2" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>187</v>
+      </c>
+      <c r="B3">
+        <v>1114</v>
+      </c>
+      <c r="C3" t="s">
+        <v>188</v>
+      </c>
+      <c r="D3" t="s">
+        <v>189</v>
+      </c>
+      <c r="E3" t="s">
+        <v>183</v>
+      </c>
+      <c r="F3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G3" t="s">
+        <v>185</v>
+      </c>
+      <c r="H3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>192</v>
+      </c>
+      <c r="B4">
+        <v>1115</v>
+      </c>
+      <c r="C4" t="s">
+        <v>193</v>
+      </c>
+      <c r="D4" t="s">
+        <v>194</v>
+      </c>
+      <c r="E4" t="s">
+        <v>183</v>
+      </c>
+      <c r="F4" t="s">
+        <v>195</v>
+      </c>
+      <c r="G4" t="s">
+        <v>185</v>
+      </c>
+      <c r="H4" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B5">
+        <v>1116</v>
+      </c>
+      <c r="C5" t="s">
+        <v>198</v>
+      </c>
+      <c r="D5" t="s">
+        <v>199</v>
+      </c>
+      <c r="E5" t="s">
+        <v>183</v>
+      </c>
+      <c r="F5" t="s">
+        <v>200</v>
+      </c>
+      <c r="G5" t="s">
+        <v>201</v>
+      </c>
+      <c r="H5" t="s">
+        <v>202</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0600-000000000000}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{00000000-0004-0000-0600-000001000000}"/>
+    <hyperlink ref="E4" r:id="rId3" xr:uid="{00000000-0004-0000-0600-000002000000}"/>
+    <hyperlink ref="E5" r:id="rId4" xr:uid="{00000000-0004-0000-0600-000003000000}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:H5" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -1672,6 +1881,191 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87D67471-D95E-4B77-BCF2-5FA11772A7DE}">
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="34.5" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="25.4140625" customWidth="1"/>
+    <col min="7" max="7" width="21.4140625" customWidth="1"/>
+    <col min="8" max="8" width="11.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="31" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="31" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="B2" s="1">
+        <v>4001</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="B3" s="1">
+        <v>4002</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="31" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="B4" s="1">
+        <v>4003</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="B5" s="1">
+        <v>4004</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="31" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="B6" s="1">
+        <v>4005</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="31" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B7" s="1">
+        <v>4006</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G7" s="4">
+        <v>45817</v>
+      </c>
+      <c r="H7" s="4">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" display="mailto:freshcart@gmail.com" xr:uid="{253F331E-AA9E-42D4-908D-2FB60DD250E3}"/>
+    <hyperlink ref="D3" r:id="rId2" display="mailto:freshcart@gmail.com" xr:uid="{50EC39AD-3F4C-4951-B154-470DC4F1C333}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{A046EAB4-AE42-4498-B8EC-604C7CF75EB9}"/>
+    <hyperlink ref="D5" r:id="rId4" display="mailto:freshcart@gmail.com" xr:uid="{86FEB3BA-AC9F-47BF-905C-08D79385B7B1}"/>
+    <hyperlink ref="D6" r:id="rId5" display="mailto:freshcart@gmail.com" xr:uid="{C860CAE3-AEBD-42EA-811A-3A578C48BA9E}"/>
+    <hyperlink ref="D7" r:id="rId6" display="mailto:freshcart@gmail.com" xr:uid="{E4E325B7-D92C-459B-A5EB-0C4EA8AE3137}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B8E7CFA-6FA1-4930-93E0-3BBDB2C8CA8B}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -1740,7 +2134,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:O3"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -1898,7 +2292,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -1993,7 +2387,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -2141,7 +2535,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -2476,7 +2870,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -2660,153 +3054,4 @@
     <ignoredError sqref="A1:H7" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" t="s">
-        <v>144</v>
-      </c>
-      <c r="E1" t="s">
-        <v>145</v>
-      </c>
-      <c r="F1" t="s">
-        <v>146</v>
-      </c>
-      <c r="G1" t="s">
-        <v>178</v>
-      </c>
-      <c r="H1" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>180</v>
-      </c>
-      <c r="B2">
-        <v>1113</v>
-      </c>
-      <c r="C2" t="s">
-        <v>181</v>
-      </c>
-      <c r="D2" t="s">
-        <v>182</v>
-      </c>
-      <c r="E2" t="s">
-        <v>183</v>
-      </c>
-      <c r="F2" t="s">
-        <v>184</v>
-      </c>
-      <c r="G2" t="s">
-        <v>185</v>
-      </c>
-      <c r="H2" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>187</v>
-      </c>
-      <c r="B3">
-        <v>1114</v>
-      </c>
-      <c r="C3" t="s">
-        <v>188</v>
-      </c>
-      <c r="D3" t="s">
-        <v>189</v>
-      </c>
-      <c r="E3" t="s">
-        <v>183</v>
-      </c>
-      <c r="F3" t="s">
-        <v>190</v>
-      </c>
-      <c r="G3" t="s">
-        <v>185</v>
-      </c>
-      <c r="H3" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>192</v>
-      </c>
-      <c r="B4">
-        <v>1115</v>
-      </c>
-      <c r="C4" t="s">
-        <v>193</v>
-      </c>
-      <c r="D4" t="s">
-        <v>194</v>
-      </c>
-      <c r="E4" t="s">
-        <v>183</v>
-      </c>
-      <c r="F4" t="s">
-        <v>195</v>
-      </c>
-      <c r="G4" t="s">
-        <v>185</v>
-      </c>
-      <c r="H4" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>197</v>
-      </c>
-      <c r="B5">
-        <v>1116</v>
-      </c>
-      <c r="C5" t="s">
-        <v>198</v>
-      </c>
-      <c r="D5" t="s">
-        <v>199</v>
-      </c>
-      <c r="E5" t="s">
-        <v>183</v>
-      </c>
-      <c r="F5" t="s">
-        <v>200</v>
-      </c>
-      <c r="G5" t="s">
-        <v>201</v>
-      </c>
-      <c r="H5" t="s">
-        <v>202</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0600-000000000000}"/>
-    <hyperlink ref="E3" r:id="rId2" xr:uid="{00000000-0004-0000-0600-000001000000}"/>
-    <hyperlink ref="E4" r:id="rId3" xr:uid="{00000000-0004-0000-0600-000002000000}"/>
-    <hyperlink ref="E5" r:id="rId4" xr:uid="{00000000-0004-0000-0600-000003000000}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:H5" numberStoredAsText="1"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add ZoneManagementTest to Regression sheet
Row was lost during binary merge conflict resolutions.
Added back with Run=YES, Mode=serial.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1037" uniqueCount="601">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="602">
   <si>
     <t>TestName</t>
   </si>
@@ -1845,6 +1845,9 @@
   </si>
   <si>
     <t>Verify Top Revenue Dropdown</t>
+  </si>
+  <si>
+    <t>ZoneManagementTest</t>
   </si>
 </sst>
 </file>
@@ -2631,6 +2634,17 @@
         <v>8</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>601</v>
+      </c>
+      <c r="B35" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
Add missing tests to Regression sheet
PaymentReportTest, DashboardTest, BulkPromotion and CustomerManagement
were missing from Regression sheet due to binary merge conflict overwrites.
All added with Run=YES, Mode=serial.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="602">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="606">
   <si>
     <t>TestName</t>
   </si>
@@ -1848,6 +1848,18 @@
   </si>
   <si>
     <t>ZoneManagementTest</t>
+  </si>
+  <si>
+    <t>PaymentReportTest</t>
+  </si>
+  <si>
+    <t>DashboardTest</t>
+  </si>
+  <si>
+    <t>BulkPromotion</t>
+  </si>
+  <si>
+    <t>CustomerManagement</t>
   </si>
 </sst>
 </file>
@@ -2645,6 +2657,50 @@
         <v>8</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>602</v>
+      </c>
+      <c r="B36" t="s">
+        <v>4</v>
+      </c>
+      <c r="C36" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>603</v>
+      </c>
+      <c r="B37" t="s">
+        <v>4</v>
+      </c>
+      <c r="C37" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>604</v>
+      </c>
+      <c r="B38" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>605</v>
+      </c>
+      <c r="B39" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
Implemented Subscription Plan automation
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -8,9 +8,11 @@
     <sheet name="ContactUsTest" sheetId="3" r:id="rId3"/>
     <sheet name="LoginTest" sheetId="4" r:id="rId4"/>
     <sheet name="CustomerManagement" sheetId="5" r:id="rId5"/>
-    <sheet name="RESTUserTest" sheetId="6" r:id="rId6"/>
-    <sheet name="SOAPAccountServiceTest" sheetId="7" r:id="rId7"/>
-    <sheet name="DatabaseTest" sheetId="8" r:id="rId8"/>
+    <sheet name="Subscription plan" sheetId="6" r:id="rId6"/>
+    <sheet name="RESTUserTest" sheetId="7" r:id="rId7"/>
+    <sheet name="SOAPAccountServiceTest" sheetId="8" r:id="rId8"/>
+    <sheet name="DatabaseTest" sheetId="9" r:id="rId9"/>
+    <sheet name="SubscriptionPlanTest" sheetId="10" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -488,6 +490,1939 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:T31"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>TC_ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Type</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Plan_Name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Scope</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Org_Access</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Payment_Type</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Tax_Code</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Charge_Code</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Currency</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Price</v>
+      </c>
+      <c r="K1" t="str">
+        <v>UOM</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Base_Qty</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Cadence</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Auto_Renewal</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Plan_Type</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Validity_Days</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Plan_Limit</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Feature1</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Feature2</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Expected_Result</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>TC01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C2" t="str">
+        <v>CreatePlan001</v>
+      </c>
+      <c r="D2" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E2" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F2" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G2" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H2" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I2" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J2" t="str">
+        <v>12</v>
+      </c>
+      <c r="K2" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L2" t="str">
+        <v>1</v>
+      </c>
+      <c r="M2" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O2" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P2" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S2" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Plan created successfully</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>TC02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C3" t="str">
+        <v>ScopeSelect001</v>
+      </c>
+      <c r="D3" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E3" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F3" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G3" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H3" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I3" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J3" t="str">
+        <v>12</v>
+      </c>
+      <c r="K3" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L3" t="str">
+        <v>1</v>
+      </c>
+      <c r="M3" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O3" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P3" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S3" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T3" t="str">
+        <v>Scope dropdown selection works</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TC03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C4" t="str">
+        <v>OrgAccess001</v>
+      </c>
+      <c r="D4" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E4" t="str">
+        <v>LIMITED</v>
+      </c>
+      <c r="F4" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G4" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H4" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I4" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J4" t="str">
+        <v>12</v>
+      </c>
+      <c r="K4" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L4" t="str">
+        <v>1</v>
+      </c>
+      <c r="M4" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O4" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P4" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S4" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T4" t="str">
+        <v>Org Access Level selection works</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TC04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C5" t="str">
+        <v>PaymentType001</v>
+      </c>
+      <c r="D5" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E5" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F5" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G5" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H5" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I5" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J5" t="str">
+        <v>12</v>
+      </c>
+      <c r="K5" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L5" t="str">
+        <v>1</v>
+      </c>
+      <c r="M5" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O5" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P5" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S5" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T5" t="str">
+        <v>Payment Type selection works</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TC05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C6" t="str">
+        <v>CadenceSel001</v>
+      </c>
+      <c r="D6" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E6" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F6" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G6" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H6" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I6" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J6" t="str">
+        <v>12</v>
+      </c>
+      <c r="K6" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L6" t="str">
+        <v>1</v>
+      </c>
+      <c r="M6" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O6" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P6" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S6" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T6" t="str">
+        <v>Cadence Type selection works</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TC06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Decimal001</v>
+      </c>
+      <c r="D7" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E7" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F7" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G7" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H7" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I7" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J7" t="str">
+        <v>12.50</v>
+      </c>
+      <c r="K7" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L7" t="str">
+        <v>1</v>
+      </c>
+      <c r="M7" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O7" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P7" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S7" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T7" t="str">
+        <v>Price accepts decimal values</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TC07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C8" t="str">
+        <v>AutoRenew001</v>
+      </c>
+      <c r="D8" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E8" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F8" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G8" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H8" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I8" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J8" t="str">
+        <v>12</v>
+      </c>
+      <c r="K8" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L8" t="str">
+        <v>1</v>
+      </c>
+      <c r="M8" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N8" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O8" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P8" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S8" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T8" t="str">
+        <v>Auto Renewal toggle works</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TC08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C9" t="str">
+        <v>SingleFeat001</v>
+      </c>
+      <c r="D9" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E9" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F9" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G9" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H9" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I9" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J9" t="str">
+        <v>12</v>
+      </c>
+      <c r="K9" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L9" t="str">
+        <v>1</v>
+      </c>
+      <c r="M9" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O9" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P9" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S9" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T9" t="str">
+        <v>Single feature creation works</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TC09</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C10" t="str">
+        <v>MultiFeat001</v>
+      </c>
+      <c r="D10" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E10" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F10" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G10" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H10" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I10" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J10" t="str">
+        <v>12</v>
+      </c>
+      <c r="K10" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L10" t="str">
+        <v>1</v>
+      </c>
+      <c r="M10" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O10" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P10" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S10" t="str">
+        <v>manager</v>
+      </c>
+      <c r="T10" t="str">
+        <v>Multiple feature creation works</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TC10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Preview001</v>
+      </c>
+      <c r="D11" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E11" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F11" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G11" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H11" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I11" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J11" t="str">
+        <v>12</v>
+      </c>
+      <c r="K11" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L11" t="str">
+        <v>1</v>
+      </c>
+      <c r="M11" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N11" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O11" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P11" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+      <c r="R11" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S11" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T11" t="str">
+        <v>Plan Preview updates dynamically</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TC11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Redirect001</v>
+      </c>
+      <c r="D12" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E12" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F12" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G12" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H12" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I12" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J12" t="str">
+        <v>12</v>
+      </c>
+      <c r="K12" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L12" t="str">
+        <v>1</v>
+      </c>
+      <c r="M12" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N12" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O12" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P12" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
+      <c r="R12" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S12" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T12" t="str">
+        <v>Create Plan redirects to listing</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TC12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Table001</v>
+      </c>
+      <c r="D13" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E13" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F13" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G13" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H13" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I13" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J13" t="str">
+        <v>12</v>
+      </c>
+      <c r="K13" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L13" t="str">
+        <v>1</v>
+      </c>
+      <c r="M13" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N13" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O13" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P13" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+      <c r="R13" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S13" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T13" t="str">
+        <v>Created plan appears in table</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TC13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Best Plan_95197</v>
+      </c>
+      <c r="D14" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E14" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F14" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G14" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H14" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I14" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J14" t="str">
+        <v>12</v>
+      </c>
+      <c r="K14" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L14" t="str">
+        <v>1</v>
+      </c>
+      <c r="M14" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N14" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O14" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P14" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q14" t="str">
+        <v/>
+      </c>
+      <c r="R14" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S14" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T14" t="str">
+        <v>Search returns matching plan</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TC14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Filter</v>
+      </c>
+      <c r="C15" t="str">
+        <v>CustomerFilter001</v>
+      </c>
+      <c r="D15" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E15" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F15" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G15" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H15" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I15" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J15" t="str">
+        <v>12</v>
+      </c>
+      <c r="K15" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L15" t="str">
+        <v>1</v>
+      </c>
+      <c r="M15" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N15" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O15" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P15" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+      <c r="R15" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S15" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T15" t="str">
+        <v>Customer scope filter — every row CUSTOMER</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TC15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Filter</v>
+      </c>
+      <c r="C16" t="str">
+        <v>PartnerFilter001</v>
+      </c>
+      <c r="D16" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E16" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F16" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G16" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H16" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I16" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J16" t="str">
+        <v>12</v>
+      </c>
+      <c r="K16" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L16" t="str">
+        <v>1</v>
+      </c>
+      <c r="M16" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N16" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O16" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P16" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
+      <c r="R16" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S16" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T16" t="str">
+        <v>Partner scope filter — every row PARTNER</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TC16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C17" t="str">
+        <v>BLANK</v>
+      </c>
+      <c r="D17" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E17" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F17" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G17" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H17" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I17" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J17" t="str">
+        <v>12</v>
+      </c>
+      <c r="K17" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L17" t="str">
+        <v>1</v>
+      </c>
+      <c r="M17" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N17" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O17" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P17" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q17" t="str">
+        <v/>
+      </c>
+      <c r="R17" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S17" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T17" t="str">
+        <v>Plan Name is required</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TC17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="D18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="E18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="F18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="G18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="H18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="I18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="J18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="K18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="L18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="M18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="N18" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="P18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="Q18" t="str">
+        <v/>
+      </c>
+      <c r="R18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="S18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T18" t="str">
+        <v>Mandatory fields are required</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TC18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C19" t="str">
+        <v>PriceAlpha001</v>
+      </c>
+      <c r="D19" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E19" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F19" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G19" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H19" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I19" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J19" t="str">
+        <v>ABC123</v>
+      </c>
+      <c r="K19" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L19" t="str">
+        <v>1</v>
+      </c>
+      <c r="M19" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N19" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O19" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P19" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
+      <c r="R19" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S19" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T19" t="str">
+        <v>Price rejects non-numeric input</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TC19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C20" t="str">
+        <v>NegQty001</v>
+      </c>
+      <c r="D20" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E20" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F20" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G20" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H20" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I20" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J20" t="str">
+        <v>12</v>
+      </c>
+      <c r="K20" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L20" t="str">
+        <v>-1</v>
+      </c>
+      <c r="M20" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N20" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O20" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P20" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q20" t="str">
+        <v/>
+      </c>
+      <c r="R20" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S20" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T20" t="str">
+        <v>Negative Base Quantity rejected</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TC20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C21" t="str">
+        <v>ZeroQty001</v>
+      </c>
+      <c r="D21" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E21" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F21" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G21" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H21" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I21" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J21" t="str">
+        <v>12</v>
+      </c>
+      <c r="K21" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L21" t="str">
+        <v>0</v>
+      </c>
+      <c r="M21" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N21" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O21" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P21" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q21" t="str">
+        <v/>
+      </c>
+      <c r="R21" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S21" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T21" t="str">
+        <v>Zero Base Quantity rejected</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>TC21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C22" t="str">
+        <v>ValidityAlpha001</v>
+      </c>
+      <c r="D22" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E22" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F22" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G22" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H22" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I22" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J22" t="str">
+        <v>12</v>
+      </c>
+      <c r="K22" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L22" t="str">
+        <v>1</v>
+      </c>
+      <c r="M22" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N22" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O22" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P22" t="str">
+        <v>ABC</v>
+      </c>
+      <c r="Q22" t="str">
+        <v/>
+      </c>
+      <c r="R22" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S22" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T22" t="str">
+        <v>Validity rejects non-numeric input</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>TC22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Best Plan_95197</v>
+      </c>
+      <c r="D23" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E23" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F23" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G23" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H23" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I23" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J23" t="str">
+        <v>12</v>
+      </c>
+      <c r="K23" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L23" t="str">
+        <v>1</v>
+      </c>
+      <c r="M23" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N23" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O23" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P23" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q23" t="str">
+        <v/>
+      </c>
+      <c r="R23" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S23" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T23" t="str">
+        <v>Duplicate name accepted (no uniqueness guard)</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TC23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C24" t="str">
+        <v>LongDesc001</v>
+      </c>
+      <c r="D24" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E24" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F24" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G24" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H24" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I24" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J24" t="str">
+        <v>12</v>
+      </c>
+      <c r="K24" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L24" t="str">
+        <v>1</v>
+      </c>
+      <c r="M24" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N24" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O24" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P24" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
+      <c r="R24" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S24" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T24" t="str">
+        <v>Long description accepted (no length limit)</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TC24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C25" t="str">
+        <v>BadTax001</v>
+      </c>
+      <c r="D25" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E25" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F25" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G25" t="str">
+        <v>INVALIDTAX999</v>
+      </c>
+      <c r="H25" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I25" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J25" t="str">
+        <v>12</v>
+      </c>
+      <c r="K25" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L25" t="str">
+        <v>1</v>
+      </c>
+      <c r="M25" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N25" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O25" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P25" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q25" t="str">
+        <v/>
+      </c>
+      <c r="R25" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S25" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T25" t="str">
+        <v>Invalid Tax Code not selectable</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TC25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C26" t="str">
+        <v>ScopeGuard001</v>
+      </c>
+      <c r="D26" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E26" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F26" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G26" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H26" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I26" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J26" t="str">
+        <v>12</v>
+      </c>
+      <c r="K26" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L26" t="str">
+        <v>1</v>
+      </c>
+      <c r="M26" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N26" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O26" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P26" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q26" t="str">
+        <v/>
+      </c>
+      <c r="R26" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S26" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T26" t="str">
+        <v>Scope is pre-filled (guarded by default)</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TC26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C27" t="str">
+        <v>BlankFeat001</v>
+      </c>
+      <c r="D27" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E27" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F27" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G27" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H27" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I27" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J27" t="str">
+        <v>12</v>
+      </c>
+      <c r="K27" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L27" t="str">
+        <v>1</v>
+      </c>
+      <c r="M27" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N27" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O27" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P27" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
+      <c r="R27" t="str">
+        <v>BLANK</v>
+      </c>
+      <c r="S27" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T27" t="str">
+        <v>Blank feature validation</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TC27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C28" t="str">
+        <v>CurrencyGuard001</v>
+      </c>
+      <c r="D28" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E28" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F28" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G28" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H28" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I28" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J28" t="str">
+        <v>12</v>
+      </c>
+      <c r="K28" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L28" t="str">
+        <v>1</v>
+      </c>
+      <c r="M28" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N28" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O28" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P28" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q28" t="str">
+        <v/>
+      </c>
+      <c r="R28" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S28" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T28" t="str">
+        <v>Currency is pre-filled (guarded by default)</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>TC28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C29" t="str">
+        <v>BadCadence001</v>
+      </c>
+      <c r="D29" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E29" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F29" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G29" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H29" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I29" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J29" t="str">
+        <v>12</v>
+      </c>
+      <c r="K29" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L29" t="str">
+        <v>1</v>
+      </c>
+      <c r="M29" t="str">
+        <v>INVALID</v>
+      </c>
+      <c r="N29" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O29" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P29" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q29" t="str">
+        <v/>
+      </c>
+      <c r="R29" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S29" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T29" t="str">
+        <v>Invalid Cadence Type not selectable</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TC29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C30" t="str">
+        <v>ApiFail001</v>
+      </c>
+      <c r="D30" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E30" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F30" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G30" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H30" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I30" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J30" t="str">
+        <v>12</v>
+      </c>
+      <c r="K30" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L30" t="str">
+        <v>1</v>
+      </c>
+      <c r="M30" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N30" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O30" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P30" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q30" t="str">
+        <v/>
+      </c>
+      <c r="R30" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S30" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T30" t="str">
+        <v>API/Network failure shows no false success</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TC30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C31" t="str">
+        <v>InvalidUrl001</v>
+      </c>
+      <c r="D31" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E31" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F31" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G31" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H31" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I31" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J31" t="str">
+        <v>12</v>
+      </c>
+      <c r="K31" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L31" t="str">
+        <v>1</v>
+      </c>
+      <c r="M31" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N31" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O31" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P31" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q31" t="str">
+        <v/>
+      </c>
+      <c r="R31" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S31" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T31" t="str">
+        <v>Invalid plan URL shows error/not-found</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:T31"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O3"/>
@@ -888,7 +2823,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -901,16 +2836,16 @@
         <v>SearchType</v>
       </c>
       <c r="D1" t="str">
+        <v>CustomerName</v>
+      </c>
+      <c r="E1" t="str">
         <v>SearchValue</v>
       </c>
-      <c r="E1" t="str">
-        <v>CustomerName</v>
-      </c>
       <c r="F1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="G1" t="str">
         <v>CustomerID</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Email</v>
       </c>
     </row>
     <row r="2">
@@ -920,20 +2855,20 @@
       <c r="B2" t="str">
         <v>Search customer using phone number</v>
       </c>
-      <c r="C2" t="str">
-        <v>Phone</v>
+      <c r="C2">
+        <v>7878787878</v>
       </c>
       <c r="D2" t="str">
-        <v>8145031601</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Biswarup Roy</v>
+        <v>Bapi Roy</v>
+      </c>
+      <c r="E2">
+        <v>7878787878</v>
       </c>
       <c r="F2" t="str">
-        <v>CGSO0007</v>
+        <v>ef0d1a26d81a020c@nipige.com</v>
       </c>
       <c r="G2" t="str">
-        <v>sdfghj@gmail.com</v>
+        <v>CRXC0020</v>
       </c>
     </row>
     <row r="3">
@@ -943,20 +2878,20 @@
       <c r="B3" t="str">
         <v>Search customer using wrong phone number</v>
       </c>
-      <c r="C3" t="str">
-        <v>Phone</v>
+      <c r="C3">
+        <v>9999999999</v>
       </c>
       <c r="D3" t="str">
+        <v>Bapi Roy</v>
+      </c>
+      <c r="E3">
         <v>9999999999</v>
       </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
       <c r="F3" t="str">
-        <v/>
+        <v>ef0d1a26d81a020c@nipige.com</v>
       </c>
       <c r="G3" t="str">
-        <v/>
+        <v>CRXC0020</v>
       </c>
     </row>
     <row r="4">
@@ -970,16 +2905,16 @@
         <v>CustomerID</v>
       </c>
       <c r="D4" t="str">
-        <v>CGSO0007</v>
+        <v>Bapi Roy</v>
       </c>
       <c r="E4" t="str">
-        <v>Biswarup Roy</v>
+        <v>CRXC0020</v>
       </c>
       <c r="F4" t="str">
-        <v>CGSO0007</v>
+        <v>ef0d1a26d81a020c@nipige.com</v>
       </c>
       <c r="G4" t="str">
-        <v>sdfghj@gmail.com</v>
+        <v>CRXC0020</v>
       </c>
     </row>
     <row r="5">
@@ -993,16 +2928,16 @@
         <v>CustomerID</v>
       </c>
       <c r="D5" t="str">
+        <v>Bapi Roy</v>
+      </c>
+      <c r="E5" t="str">
         <v>CRXC9999</v>
       </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
       <c r="F5" t="str">
-        <v/>
+        <v>ef0d1a26d81a020c@nipige.com</v>
       </c>
       <c r="G5" t="str">
-        <v/>
+        <v>CRXC0020</v>
       </c>
     </row>
     <row r="6">
@@ -1016,16 +2951,16 @@
         <v>Email</v>
       </c>
       <c r="D6" t="str">
-        <v>0f19d4e7f840d6a78e5221cb6eb463202e7f7321@example.com</v>
+        <v>Bapi Roy</v>
       </c>
       <c r="E6" t="str">
-        <v>New User1</v>
+        <v>ef0d1a26d81a020c@nipige.com</v>
       </c>
       <c r="F6" t="str">
-        <v>CGSO0065</v>
+        <v>ef0d1a26d81a020c@nipige.com</v>
       </c>
       <c r="G6" t="str">
-        <v>0f19d4e7f840d6a78e5221cb6eb463202e7f7321@example.com</v>
+        <v>CRXC0020</v>
       </c>
     </row>
     <row r="7">
@@ -1039,16 +2974,16 @@
         <v>Email</v>
       </c>
       <c r="D7" t="str">
+        <v>Bapi Roy</v>
+      </c>
+      <c r="E7" t="str">
         <v>invalidcustomer@test.com</v>
       </c>
-      <c r="E7" t="str">
-        <v/>
-      </c>
       <c r="F7" t="str">
-        <v/>
+        <v>ef0d1a26d81a020c@nipige.com</v>
       </c>
       <c r="G7" t="str">
-        <v/>
+        <v>CRXC0020</v>
       </c>
     </row>
     <row r="8">
@@ -1062,16 +2997,16 @@
         <v>OrderID</v>
       </c>
       <c r="D8" t="str">
-        <v>ORD-20260602-4B2E7A3B</v>
+        <v>Bapi Roy</v>
       </c>
       <c r="E8" t="str">
-        <v>Biswarup Roy</v>
+        <v>ORD-20260601-F0C2AACE</v>
       </c>
       <c r="F8" t="str">
-        <v>CGSO0007</v>
+        <v>ef0d1a26d81a020c@nipige.com</v>
       </c>
       <c r="G8" t="str">
-        <v>sdfghj@gmail.com</v>
+        <v>CRXC0020</v>
       </c>
     </row>
     <row r="9">
@@ -1085,16 +3020,16 @@
         <v>OrderID</v>
       </c>
       <c r="D9" t="str">
+        <v>Bapi Roy</v>
+      </c>
+      <c r="E9" t="str">
         <v>ORD-99999999-XXXXXX</v>
       </c>
-      <c r="E9" t="str">
-        <v/>
-      </c>
       <c r="F9" t="str">
-        <v/>
+        <v>ef0d1a26d81a020c@nipige.com</v>
       </c>
       <c r="G9" t="str">
-        <v/>
+        <v>CRXC0020</v>
       </c>
     </row>
     <row r="10">
@@ -1102,22 +3037,22 @@
         <v>TC09_SearchCustomerByTicketId</v>
       </c>
       <c r="B10" t="str">
-        <v>Search customer using ticket ID</v>
+        <v>Search customer using valid ticket ID</v>
       </c>
       <c r="C10" t="str">
         <v>Ticket ID</v>
       </c>
       <c r="D10" t="str">
+        <v>Bapi Roy</v>
+      </c>
+      <c r="E10" t="str">
         <v>SR2753520820</v>
       </c>
-      <c r="E10" t="str">
-        <v>New User</v>
-      </c>
       <c r="F10" t="str">
-        <v>CGSO0009</v>
+        <v>ef0d1a26d81a020c@nipige.com</v>
       </c>
       <c r="G10" t="str">
-        <v>sandi90saha@gmail.com</v>
+        <v>CRXC0020</v>
       </c>
     </row>
     <row r="11">
@@ -1131,95 +3066,1974 @@
         <v>Ticket ID</v>
       </c>
       <c r="D11" t="str">
+        <v>Bapi Roy</v>
+      </c>
+      <c r="E11" t="str">
         <v>SR9999999999</v>
       </c>
-      <c r="E11" t="str">
-        <v/>
-      </c>
       <c r="F11" t="str">
-        <v/>
+        <v>ef0d1a26d81a020c@nipige.com</v>
       </c>
       <c r="G11" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>TC11_VerifyOrdersTab</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Validate Orders tab for a customer with orders</v>
-      </c>
-      <c r="C12" t="str">
-        <v>CustomerID</v>
-      </c>
-      <c r="D12" t="str">
-        <v>CGSO0007</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Biswarup Roy</v>
-      </c>
-      <c r="F12" t="str">
-        <v>CGSO0007</v>
-      </c>
-      <c r="G12" t="str">
-        <v>sdfghj@gmail.com</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>TC12_VerifyAddressManagementTab</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Validate Address Management tab for a customer with addresses</v>
-      </c>
-      <c r="C13" t="str">
-        <v>CustomerID</v>
-      </c>
-      <c r="D13" t="str">
-        <v>CGSO0007</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Biswarup Roy</v>
-      </c>
-      <c r="F13" t="str">
-        <v>CGSO0007</v>
-      </c>
-      <c r="G13" t="str">
-        <v>sdfghj@gmail.com</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>TC13_VerifyServiceRequestsTab</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Validate Service Requests tab (records or empty state)</v>
-      </c>
-      <c r="C14" t="str">
-        <v>CustomerID</v>
-      </c>
-      <c r="D14" t="str">
-        <v>CGSO0007</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Biswarup Roy</v>
-      </c>
-      <c r="F14" t="str">
-        <v>CGSO0007</v>
-      </c>
-      <c r="G14" t="str">
-        <v>sdfghj@gmail.com</v>
+        <v>CRXC0020</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F2" r:id="rId1"/>
+    <hyperlink ref="F3" r:id="rId2"/>
+    <hyperlink ref="F4" r:id="rId3"/>
+    <hyperlink ref="F5" r:id="rId4"/>
+    <hyperlink ref="E6" r:id="rId5"/>
+    <hyperlink ref="F6" r:id="rId6"/>
+    <hyperlink ref="E7" r:id="rId7"/>
+    <hyperlink ref="F7" r:id="rId8"/>
+    <hyperlink ref="F8" r:id="rId9"/>
+    <hyperlink ref="F9" r:id="rId10"/>
+    <hyperlink ref="F10" r:id="rId11"/>
+    <hyperlink ref="F11" r:id="rId12"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:T31"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>TC_ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Type</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Plan_Name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Scope</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Org_Access</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Payment_Type</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Tax_Code</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Charge_Code</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Currency</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Price</v>
+      </c>
+      <c r="K1" t="str">
+        <v>UOM</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Base_Qty</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Cadence</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Auto_Renewal</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Plan_Type</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Validity_Days</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Plan_Limit</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Feature1</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Feature2</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Expected_Result</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>TC01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C2" t="str">
+        <v>AutoBestPlan001</v>
+      </c>
+      <c r="D2" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E2" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F2" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G2" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H2" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I2" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J2" t="str">
+        <v>12</v>
+      </c>
+      <c r="K2" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L2" t="str">
+        <v>1</v>
+      </c>
+      <c r="M2" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N2" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O2" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P2" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>100</v>
+      </c>
+      <c r="R2" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S2" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>TC02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C3" t="str">
+        <v>AutoPartner001</v>
+      </c>
+      <c r="D3" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E3" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F3" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G3" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H3" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I3" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J3" t="str">
+        <v>344</v>
+      </c>
+      <c r="K3" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L3" t="str">
+        <v>1</v>
+      </c>
+      <c r="M3" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N3" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O3" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P3" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>100</v>
+      </c>
+      <c r="R3" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S3" t="str">
+        <v>dashboard</v>
+      </c>
+      <c r="T3" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TC03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C4" t="str">
+        <v>AutoDecimal001</v>
+      </c>
+      <c r="D4" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E4" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F4" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G4" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H4" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I4" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J4" t="str">
+        <v>199.99</v>
+      </c>
+      <c r="K4" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L4" t="str">
+        <v>1</v>
+      </c>
+      <c r="M4" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N4" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O4" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P4" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>100</v>
+      </c>
+      <c r="R4" t="str">
+        <v>analytics</v>
+      </c>
+      <c r="S4" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T4" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TC04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C5" t="str">
+        <v>AutoRenewal001</v>
+      </c>
+      <c r="D5" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E5" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F5" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G5" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H5" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I5" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J5" t="str">
+        <v>49.99</v>
+      </c>
+      <c r="K5" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L5" t="str">
+        <v>1</v>
+      </c>
+      <c r="M5" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N5" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O5" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P5" t="str">
+        <v>10</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>50</v>
+      </c>
+      <c r="R5" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S5" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T5" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TC05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C6" t="str">
+        <v>SingleFeature001</v>
+      </c>
+      <c r="D6" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E6" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F6" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G6" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H6" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I6" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J6" t="str">
+        <v>99</v>
+      </c>
+      <c r="K6" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L6" t="str">
+        <v>1</v>
+      </c>
+      <c r="M6" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N6" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O6" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P6" t="str">
+        <v>15</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>25</v>
+      </c>
+      <c r="R6" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S6" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T6" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TC06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C7" t="str">
+        <v>MultiFeature001</v>
+      </c>
+      <c r="D7" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E7" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F7" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G7" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H7" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I7" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J7" t="str">
+        <v>149</v>
+      </c>
+      <c r="K7" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L7" t="str">
+        <v>1</v>
+      </c>
+      <c r="M7" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N7" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O7" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P7" t="str">
+        <v>20</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>50</v>
+      </c>
+      <c r="R7" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S7" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T7" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TC07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C8" t="str">
+        <v>PreviewPlan001</v>
+      </c>
+      <c r="D8" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E8" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F8" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G8" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H8" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I8" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J8" t="str">
+        <v>20</v>
+      </c>
+      <c r="K8" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L8" t="str">
+        <v>1</v>
+      </c>
+      <c r="M8" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N8" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O8" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P8" t="str">
+        <v>5</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>10</v>
+      </c>
+      <c r="R8" t="str">
+        <v>preview</v>
+      </c>
+      <c r="S8" t="str">
+        <v>dashboard</v>
+      </c>
+      <c r="T8" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TC08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C9" t="str">
+        <v>RedirectPlan001</v>
+      </c>
+      <c r="D9" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E9" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F9" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G9" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H9" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I9" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J9" t="str">
+        <v>75</v>
+      </c>
+      <c r="K9" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L9" t="str">
+        <v>1</v>
+      </c>
+      <c r="M9" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N9" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O9" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P9" t="str">
+        <v>12</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>30</v>
+      </c>
+      <c r="R9" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S9" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T9" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TC09</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C10" t="str">
+        <v>SearchPlan001</v>
+      </c>
+      <c r="D10" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E10" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F10" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G10" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H10" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I10" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J10" t="str">
+        <v>25</v>
+      </c>
+      <c r="K10" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L10" t="str">
+        <v>1</v>
+      </c>
+      <c r="M10" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N10" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O10" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P10" t="str">
+        <v>7</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>20</v>
+      </c>
+      <c r="R10" t="str">
+        <v>search</v>
+      </c>
+      <c r="S10" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T10" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TC10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C11" t="str">
+        <v>CustomerScope001</v>
+      </c>
+      <c r="D11" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E11" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F11" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G11" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H11" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I11" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J11" t="str">
+        <v>15</v>
+      </c>
+      <c r="K11" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L11" t="str">
+        <v>1</v>
+      </c>
+      <c r="M11" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N11" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O11" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P11" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>10</v>
+      </c>
+      <c r="R11" t="str">
+        <v>customer</v>
+      </c>
+      <c r="S11" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T11" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TC11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C12" t="str">
+        <v>PartnerScope001</v>
+      </c>
+      <c r="D12" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E12" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F12" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G12" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H12" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I12" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J12" t="str">
+        <v>150</v>
+      </c>
+      <c r="K12" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L12" t="str">
+        <v>1</v>
+      </c>
+      <c r="M12" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N12" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O12" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P12" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>100</v>
+      </c>
+      <c r="R12" t="str">
+        <v>partner</v>
+      </c>
+      <c r="S12" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T12" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TC12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C13" t="str">
+        <v>ViewPlan001</v>
+      </c>
+      <c r="D13" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E13" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F13" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G13" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H13" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I13" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J13" t="str">
+        <v>10</v>
+      </c>
+      <c r="K13" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L13" t="str">
+        <v>1</v>
+      </c>
+      <c r="M13" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N13" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O13" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P13" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>10</v>
+      </c>
+      <c r="R13" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S13" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T13" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TC13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C14" t="str">
+        <v>EditPlan001</v>
+      </c>
+      <c r="D14" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E14" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F14" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G14" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H14" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I14" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J14" t="str">
+        <v>199</v>
+      </c>
+      <c r="K14" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L14" t="str">
+        <v>1</v>
+      </c>
+      <c r="M14" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N14" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O14" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P14" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>50</v>
+      </c>
+      <c r="R14" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S14" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T14" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TC14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C15" t="str">
+        <v>UpdatedPlan001</v>
+      </c>
+      <c r="D15" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E15" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F15" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G15" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H15" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I15" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J15" t="str">
+        <v>249</v>
+      </c>
+      <c r="K15" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L15" t="str">
+        <v>1</v>
+      </c>
+      <c r="M15" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N15" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O15" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P15" t="str">
+        <v>45</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>75</v>
+      </c>
+      <c r="R15" t="str">
+        <v>analytics</v>
+      </c>
+      <c r="S15" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T15" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TC15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C16" t="str">
+        <v>PaginationPlan001</v>
+      </c>
+      <c r="D16" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E16" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F16" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G16" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H16" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I16" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J16" t="str">
+        <v>19</v>
+      </c>
+      <c r="K16" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L16" t="str">
+        <v>1</v>
+      </c>
+      <c r="M16" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N16" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O16" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P16" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>10</v>
+      </c>
+      <c r="R16" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S16" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T16" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TC16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C17" t="str">
+        <v>BLANK</v>
+      </c>
+      <c r="D17" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E17" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F17" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G17" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H17" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I17" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J17" t="str">
+        <v>12</v>
+      </c>
+      <c r="K17" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L17" t="str">
+        <v>1</v>
+      </c>
+      <c r="M17" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N17" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O17" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P17" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>10</v>
+      </c>
+      <c r="R17" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S17" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T17" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TC17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="D18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="E18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="F18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="G18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="H18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="I18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="J18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="K18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="L18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="M18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="N18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="O18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="P18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="R18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="S18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T18" t="str">
+        <v>Mandatory Validation</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TC18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C19" t="str">
+        <v>InvalidPrice001</v>
+      </c>
+      <c r="D19" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E19" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F19" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G19" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H19" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I19" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J19" t="str">
+        <v>ABC123</v>
+      </c>
+      <c r="K19" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L19" t="str">
+        <v>1</v>
+      </c>
+      <c r="M19" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N19" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O19" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P19" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>100</v>
+      </c>
+      <c r="R19" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S19" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T19" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TC19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C20" t="str">
+        <v>NegativeQty001</v>
+      </c>
+      <c r="D20" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E20" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F20" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G20" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H20" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I20" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J20" t="str">
+        <v>100</v>
+      </c>
+      <c r="K20" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L20" t="str">
+        <v>-1</v>
+      </c>
+      <c r="M20" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N20" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O20" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P20" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>100</v>
+      </c>
+      <c r="R20" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S20" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T20" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TC20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C21" t="str">
+        <v>ZeroQty001</v>
+      </c>
+      <c r="D21" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E21" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F21" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G21" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H21" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I21" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J21" t="str">
+        <v>100</v>
+      </c>
+      <c r="K21" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L21" t="str">
+        <v>0</v>
+      </c>
+      <c r="M21" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N21" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O21" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P21" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>100</v>
+      </c>
+      <c r="R21" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S21" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T21" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>TC21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C22" t="str">
+        <v>InvalidValidity001</v>
+      </c>
+      <c r="D22" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E22" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F22" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G22" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H22" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I22" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J22" t="str">
+        <v>12</v>
+      </c>
+      <c r="K22" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L22" t="str">
+        <v>1</v>
+      </c>
+      <c r="M22" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N22" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O22" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P22" t="str">
+        <v>ABC</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>10</v>
+      </c>
+      <c r="R22" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S22" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T22" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>TC22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Best Plan</v>
+      </c>
+      <c r="D23" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E23" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F23" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G23" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H23" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I23" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J23" t="str">
+        <v>12</v>
+      </c>
+      <c r="K23" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L23" t="str">
+        <v>1</v>
+      </c>
+      <c r="M23" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N23" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O23" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P23" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>10</v>
+      </c>
+      <c r="R23" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S23" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T23" t="str">
+        <v>Duplicate Validation</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TC23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C24" t="str">
+        <v>LongDescription001</v>
+      </c>
+      <c r="D24" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E24" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F24" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G24" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H24" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I24" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J24" t="str">
+        <v>100</v>
+      </c>
+      <c r="K24" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L24" t="str">
+        <v>1</v>
+      </c>
+      <c r="M24" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N24" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O24" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P24" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>100</v>
+      </c>
+      <c r="R24" t="str">
+        <v>DESCRIPTION_OVER_LIMIT</v>
+      </c>
+      <c r="S24" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T24" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TC24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C25" t="str">
+        <v>InvalidTax001</v>
+      </c>
+      <c r="D25" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E25" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F25" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G25" t="str">
+        <v>INVALIDTAX999</v>
+      </c>
+      <c r="H25" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I25" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J25" t="str">
+        <v>100</v>
+      </c>
+      <c r="K25" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L25" t="str">
+        <v>1</v>
+      </c>
+      <c r="M25" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N25" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O25" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P25" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q25" t="str">
+        <v>100</v>
+      </c>
+      <c r="R25" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S25" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T25" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TC25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C26" t="str">
+        <v>NoScope001</v>
+      </c>
+      <c r="D26" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="E26" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F26" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G26" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H26" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I26" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J26" t="str">
+        <v>100</v>
+      </c>
+      <c r="K26" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L26" t="str">
+        <v>1</v>
+      </c>
+      <c r="M26" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N26" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O26" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P26" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q26" t="str">
+        <v>100</v>
+      </c>
+      <c r="R26" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S26" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T26" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TC26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C27" t="str">
+        <v>BlankFeature001</v>
+      </c>
+      <c r="D27" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E27" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F27" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G27" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H27" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I27" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J27" t="str">
+        <v>12</v>
+      </c>
+      <c r="K27" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L27" t="str">
+        <v>1</v>
+      </c>
+      <c r="M27" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N27" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O27" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P27" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q27" t="str">
+        <v>10</v>
+      </c>
+      <c r="R27" t="str">
+        <v>BLANK</v>
+      </c>
+      <c r="S27" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T27" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TC27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C28" t="str">
+        <v>NoCurrency001</v>
+      </c>
+      <c r="D28" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E28" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F28" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G28" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H28" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I28" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="J28" t="str">
+        <v>12</v>
+      </c>
+      <c r="K28" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L28" t="str">
+        <v>1</v>
+      </c>
+      <c r="M28" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N28" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O28" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P28" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q28" t="str">
+        <v>10</v>
+      </c>
+      <c r="R28" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S28" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T28" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>TC28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C29" t="str">
+        <v>InvalidCadence001</v>
+      </c>
+      <c r="D29" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E29" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F29" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G29" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H29" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I29" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J29" t="str">
+        <v>100</v>
+      </c>
+      <c r="K29" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L29" t="str">
+        <v>1</v>
+      </c>
+      <c r="M29" t="str">
+        <v>INVALID</v>
+      </c>
+      <c r="N29" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O29" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P29" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q29" t="str">
+        <v>100</v>
+      </c>
+      <c r="R29" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S29" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T29" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TC29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C30" t="str">
+        <v>ApiFailure001</v>
+      </c>
+      <c r="D30" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E30" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F30" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G30" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H30" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I30" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J30" t="str">
+        <v>100</v>
+      </c>
+      <c r="K30" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L30" t="str">
+        <v>1</v>
+      </c>
+      <c r="M30" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N30" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O30" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P30" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q30" t="str">
+        <v>100</v>
+      </c>
+      <c r="R30" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S30" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T30" t="str">
+        <v>API Failure Message</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TC30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C31" t="str">
+        <v>InvalidURL001</v>
+      </c>
+      <c r="D31" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E31" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F31" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G31" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H31" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I31" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J31" t="str">
+        <v>12</v>
+      </c>
+      <c r="K31" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L31" t="str">
+        <v>1</v>
+      </c>
+      <c r="M31" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N31" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O31" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P31" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q31" t="str">
+        <v>10</v>
+      </c>
+      <c r="R31" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S31" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T31" t="str">
+        <v>Not Found/Error Page</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:T31"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H7"/>
   <sheetData>
@@ -1404,7 +5218,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H5"/>
   <sheetData>
@@ -1552,7 +5366,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D8"/>
   <sheetData>

</xml_diff>

<commit_message>
Merge Rohit's SubscriptionPlan and SubscriptionPlanTest sheets into testData.xlsx
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -34,6 +34,8 @@
     <sheet name="CustomerManagement" sheetId="17" r:id="rId19"/>
     <sheet name="DeliverySetupTest" sheetId="18" r:id="rId20"/>
     <sheet name="ZoneManagementTest" sheetId="21" r:id="rId24"/>
+    <sheet name="Subscription plan" sheetId="22" r:id="rId25"/>
+    <sheet name="SubscriptionPlanTest" sheetId="23" r:id="rId26"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -7391,6 +7393,3872 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:T31"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>TC_ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Type</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Plan_Name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Scope</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Org_Access</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Payment_Type</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Tax_Code</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Charge_Code</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Currency</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Price</v>
+      </c>
+      <c r="K1" t="str">
+        <v>UOM</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Base_Qty</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Cadence</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Auto_Renewal</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Plan_Type</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Validity_Days</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Plan_Limit</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Feature1</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Feature2</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Expected_Result</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>TC01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C2" t="str">
+        <v>AutoBestPlan001</v>
+      </c>
+      <c r="D2" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E2" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F2" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G2" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H2" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I2" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J2" t="str">
+        <v>12</v>
+      </c>
+      <c r="K2" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L2" t="str">
+        <v>1</v>
+      </c>
+      <c r="M2" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N2" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O2" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P2" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>100</v>
+      </c>
+      <c r="R2" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S2" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>TC02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C3" t="str">
+        <v>AutoPartner001</v>
+      </c>
+      <c r="D3" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E3" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F3" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G3" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H3" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I3" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J3" t="str">
+        <v>344</v>
+      </c>
+      <c r="K3" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L3" t="str">
+        <v>1</v>
+      </c>
+      <c r="M3" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N3" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O3" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P3" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>100</v>
+      </c>
+      <c r="R3" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S3" t="str">
+        <v>dashboard</v>
+      </c>
+      <c r="T3" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TC03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C4" t="str">
+        <v>AutoDecimal001</v>
+      </c>
+      <c r="D4" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E4" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F4" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G4" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H4" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I4" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J4" t="str">
+        <v>199.99</v>
+      </c>
+      <c r="K4" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L4" t="str">
+        <v>1</v>
+      </c>
+      <c r="M4" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N4" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O4" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P4" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>100</v>
+      </c>
+      <c r="R4" t="str">
+        <v>analytics</v>
+      </c>
+      <c r="S4" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T4" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TC04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C5" t="str">
+        <v>AutoRenewal001</v>
+      </c>
+      <c r="D5" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E5" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F5" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G5" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H5" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I5" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J5" t="str">
+        <v>49.99</v>
+      </c>
+      <c r="K5" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L5" t="str">
+        <v>1</v>
+      </c>
+      <c r="M5" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N5" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O5" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P5" t="str">
+        <v>10</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>50</v>
+      </c>
+      <c r="R5" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S5" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T5" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TC05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C6" t="str">
+        <v>SingleFeature001</v>
+      </c>
+      <c r="D6" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E6" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F6" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G6" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H6" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I6" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J6" t="str">
+        <v>99</v>
+      </c>
+      <c r="K6" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L6" t="str">
+        <v>1</v>
+      </c>
+      <c r="M6" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N6" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O6" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P6" t="str">
+        <v>15</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>25</v>
+      </c>
+      <c r="R6" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S6" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T6" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TC06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C7" t="str">
+        <v>MultiFeature001</v>
+      </c>
+      <c r="D7" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E7" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F7" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G7" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H7" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I7" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J7" t="str">
+        <v>149</v>
+      </c>
+      <c r="K7" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L7" t="str">
+        <v>1</v>
+      </c>
+      <c r="M7" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N7" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O7" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P7" t="str">
+        <v>20</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>50</v>
+      </c>
+      <c r="R7" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S7" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T7" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TC07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C8" t="str">
+        <v>PreviewPlan001</v>
+      </c>
+      <c r="D8" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E8" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F8" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G8" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H8" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I8" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J8" t="str">
+        <v>20</v>
+      </c>
+      <c r="K8" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L8" t="str">
+        <v>1</v>
+      </c>
+      <c r="M8" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N8" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O8" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P8" t="str">
+        <v>5</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>10</v>
+      </c>
+      <c r="R8" t="str">
+        <v>preview</v>
+      </c>
+      <c r="S8" t="str">
+        <v>dashboard</v>
+      </c>
+      <c r="T8" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TC08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C9" t="str">
+        <v>RedirectPlan001</v>
+      </c>
+      <c r="D9" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E9" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F9" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G9" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H9" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I9" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J9" t="str">
+        <v>75</v>
+      </c>
+      <c r="K9" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L9" t="str">
+        <v>1</v>
+      </c>
+      <c r="M9" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N9" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O9" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P9" t="str">
+        <v>12</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>30</v>
+      </c>
+      <c r="R9" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S9" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T9" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TC09</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C10" t="str">
+        <v>SearchPlan001</v>
+      </c>
+      <c r="D10" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E10" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F10" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G10" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H10" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I10" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J10" t="str">
+        <v>25</v>
+      </c>
+      <c r="K10" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L10" t="str">
+        <v>1</v>
+      </c>
+      <c r="M10" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N10" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O10" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P10" t="str">
+        <v>7</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>20</v>
+      </c>
+      <c r="R10" t="str">
+        <v>search</v>
+      </c>
+      <c r="S10" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T10" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TC10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C11" t="str">
+        <v>CustomerScope001</v>
+      </c>
+      <c r="D11" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E11" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F11" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G11" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H11" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I11" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J11" t="str">
+        <v>15</v>
+      </c>
+      <c r="K11" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L11" t="str">
+        <v>1</v>
+      </c>
+      <c r="M11" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N11" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O11" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P11" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>10</v>
+      </c>
+      <c r="R11" t="str">
+        <v>customer</v>
+      </c>
+      <c r="S11" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T11" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TC11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C12" t="str">
+        <v>PartnerScope001</v>
+      </c>
+      <c r="D12" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E12" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F12" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G12" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H12" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I12" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J12" t="str">
+        <v>150</v>
+      </c>
+      <c r="K12" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L12" t="str">
+        <v>1</v>
+      </c>
+      <c r="M12" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N12" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O12" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P12" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>100</v>
+      </c>
+      <c r="R12" t="str">
+        <v>partner</v>
+      </c>
+      <c r="S12" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T12" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TC12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C13" t="str">
+        <v>ViewPlan001</v>
+      </c>
+      <c r="D13" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E13" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F13" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G13" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H13" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I13" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J13" t="str">
+        <v>10</v>
+      </c>
+      <c r="K13" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L13" t="str">
+        <v>1</v>
+      </c>
+      <c r="M13" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N13" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O13" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P13" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>10</v>
+      </c>
+      <c r="R13" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S13" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T13" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TC13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C14" t="str">
+        <v>EditPlan001</v>
+      </c>
+      <c r="D14" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E14" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F14" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G14" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H14" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I14" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J14" t="str">
+        <v>199</v>
+      </c>
+      <c r="K14" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L14" t="str">
+        <v>1</v>
+      </c>
+      <c r="M14" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N14" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O14" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P14" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>50</v>
+      </c>
+      <c r="R14" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S14" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T14" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TC14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C15" t="str">
+        <v>UpdatedPlan001</v>
+      </c>
+      <c r="D15" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E15" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F15" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G15" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H15" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I15" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J15" t="str">
+        <v>249</v>
+      </c>
+      <c r="K15" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L15" t="str">
+        <v>1</v>
+      </c>
+      <c r="M15" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N15" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O15" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P15" t="str">
+        <v>45</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>75</v>
+      </c>
+      <c r="R15" t="str">
+        <v>analytics</v>
+      </c>
+      <c r="S15" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T15" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TC15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C16" t="str">
+        <v>PaginationPlan001</v>
+      </c>
+      <c r="D16" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E16" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F16" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G16" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H16" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I16" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J16" t="str">
+        <v>19</v>
+      </c>
+      <c r="K16" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L16" t="str">
+        <v>1</v>
+      </c>
+      <c r="M16" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N16" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O16" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P16" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>10</v>
+      </c>
+      <c r="R16" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S16" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T16" t="str">
+        <v>Success</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TC16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C17" t="str">
+        <v>BLANK</v>
+      </c>
+      <c r="D17" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E17" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F17" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G17" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H17" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I17" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J17" t="str">
+        <v>12</v>
+      </c>
+      <c r="K17" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L17" t="str">
+        <v>1</v>
+      </c>
+      <c r="M17" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N17" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O17" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P17" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>10</v>
+      </c>
+      <c r="R17" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S17" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T17" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TC17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="D18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="E18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="F18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="G18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="H18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="I18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="J18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="K18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="L18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="M18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="N18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="O18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="P18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="R18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="S18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T18" t="str">
+        <v>Mandatory Validation</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TC18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C19" t="str">
+        <v>InvalidPrice001</v>
+      </c>
+      <c r="D19" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E19" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F19" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G19" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H19" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I19" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J19" t="str">
+        <v>ABC123</v>
+      </c>
+      <c r="K19" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L19" t="str">
+        <v>1</v>
+      </c>
+      <c r="M19" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N19" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O19" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P19" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>100</v>
+      </c>
+      <c r="R19" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S19" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T19" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TC19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C20" t="str">
+        <v>NegativeQty001</v>
+      </c>
+      <c r="D20" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E20" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F20" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G20" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H20" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I20" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J20" t="str">
+        <v>100</v>
+      </c>
+      <c r="K20" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L20" t="str">
+        <v>-1</v>
+      </c>
+      <c r="M20" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N20" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O20" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P20" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>100</v>
+      </c>
+      <c r="R20" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S20" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T20" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TC20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C21" t="str">
+        <v>ZeroQty001</v>
+      </c>
+      <c r="D21" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E21" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F21" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G21" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H21" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I21" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J21" t="str">
+        <v>100</v>
+      </c>
+      <c r="K21" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L21" t="str">
+        <v>0</v>
+      </c>
+      <c r="M21" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N21" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O21" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P21" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>100</v>
+      </c>
+      <c r="R21" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S21" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T21" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>TC21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C22" t="str">
+        <v>InvalidValidity001</v>
+      </c>
+      <c r="D22" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E22" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F22" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G22" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H22" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I22" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J22" t="str">
+        <v>12</v>
+      </c>
+      <c r="K22" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L22" t="str">
+        <v>1</v>
+      </c>
+      <c r="M22" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N22" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O22" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P22" t="str">
+        <v>ABC</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>10</v>
+      </c>
+      <c r="R22" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S22" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T22" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>TC22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Best Plan</v>
+      </c>
+      <c r="D23" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E23" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F23" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G23" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H23" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I23" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J23" t="str">
+        <v>12</v>
+      </c>
+      <c r="K23" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L23" t="str">
+        <v>1</v>
+      </c>
+      <c r="M23" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N23" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O23" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P23" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>10</v>
+      </c>
+      <c r="R23" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S23" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T23" t="str">
+        <v>Duplicate Validation</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TC23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C24" t="str">
+        <v>LongDescription001</v>
+      </c>
+      <c r="D24" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E24" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F24" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G24" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H24" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I24" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J24" t="str">
+        <v>100</v>
+      </c>
+      <c r="K24" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L24" t="str">
+        <v>1</v>
+      </c>
+      <c r="M24" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N24" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O24" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P24" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>100</v>
+      </c>
+      <c r="R24" t="str">
+        <v>DESCRIPTION_OVER_LIMIT</v>
+      </c>
+      <c r="S24" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T24" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TC24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C25" t="str">
+        <v>InvalidTax001</v>
+      </c>
+      <c r="D25" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E25" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F25" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G25" t="str">
+        <v>INVALIDTAX999</v>
+      </c>
+      <c r="H25" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I25" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J25" t="str">
+        <v>100</v>
+      </c>
+      <c r="K25" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L25" t="str">
+        <v>1</v>
+      </c>
+      <c r="M25" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N25" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O25" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P25" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q25" t="str">
+        <v>100</v>
+      </c>
+      <c r="R25" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S25" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T25" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TC25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C26" t="str">
+        <v>NoScope001</v>
+      </c>
+      <c r="D26" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="E26" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F26" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G26" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H26" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I26" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J26" t="str">
+        <v>100</v>
+      </c>
+      <c r="K26" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L26" t="str">
+        <v>1</v>
+      </c>
+      <c r="M26" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N26" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O26" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P26" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q26" t="str">
+        <v>100</v>
+      </c>
+      <c r="R26" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S26" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T26" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TC26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C27" t="str">
+        <v>BlankFeature001</v>
+      </c>
+      <c r="D27" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E27" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F27" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G27" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H27" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I27" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J27" t="str">
+        <v>12</v>
+      </c>
+      <c r="K27" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L27" t="str">
+        <v>1</v>
+      </c>
+      <c r="M27" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N27" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O27" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P27" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q27" t="str">
+        <v>10</v>
+      </c>
+      <c r="R27" t="str">
+        <v>BLANK</v>
+      </c>
+      <c r="S27" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T27" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TC27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C28" t="str">
+        <v>NoCurrency001</v>
+      </c>
+      <c r="D28" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E28" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F28" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G28" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H28" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I28" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="J28" t="str">
+        <v>12</v>
+      </c>
+      <c r="K28" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L28" t="str">
+        <v>1</v>
+      </c>
+      <c r="M28" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N28" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O28" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P28" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q28" t="str">
+        <v>10</v>
+      </c>
+      <c r="R28" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S28" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T28" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>TC28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C29" t="str">
+        <v>InvalidCadence001</v>
+      </c>
+      <c r="D29" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E29" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F29" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G29" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H29" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I29" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J29" t="str">
+        <v>100</v>
+      </c>
+      <c r="K29" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L29" t="str">
+        <v>1</v>
+      </c>
+      <c r="M29" t="str">
+        <v>INVALID</v>
+      </c>
+      <c r="N29" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O29" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P29" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q29" t="str">
+        <v>100</v>
+      </c>
+      <c r="R29" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S29" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T29" t="str">
+        <v>Validation Error</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TC29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C30" t="str">
+        <v>ApiFailure001</v>
+      </c>
+      <c r="D30" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E30" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F30" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G30" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H30" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I30" t="str">
+        <v>INR</v>
+      </c>
+      <c r="J30" t="str">
+        <v>100</v>
+      </c>
+      <c r="K30" t="str">
+        <v>OCCURRENCE</v>
+      </c>
+      <c r="L30" t="str">
+        <v>1</v>
+      </c>
+      <c r="M30" t="str">
+        <v>MONTHLY</v>
+      </c>
+      <c r="N30" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O30" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P30" t="str">
+        <v>30</v>
+      </c>
+      <c r="Q30" t="str">
+        <v>100</v>
+      </c>
+      <c r="R30" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S30" t="str">
+        <v>reports</v>
+      </c>
+      <c r="T30" t="str">
+        <v>API Failure Message</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TC30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C31" t="str">
+        <v>InvalidURL001</v>
+      </c>
+      <c r="D31" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E31" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F31" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G31" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H31" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I31" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J31" t="str">
+        <v>12</v>
+      </c>
+      <c r="K31" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L31" t="str">
+        <v>1</v>
+      </c>
+      <c r="M31" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N31" t="str">
+        <v>YES</v>
+      </c>
+      <c r="O31" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P31" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q31" t="str">
+        <v>10</v>
+      </c>
+      <c r="R31" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S31" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T31" t="str">
+        <v>Not Found/Error Page</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:T31"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:T31"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>TC_ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Type</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Plan_Name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Scope</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Org_Access</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Payment_Type</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Tax_Code</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Charge_Code</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Currency</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Price</v>
+      </c>
+      <c r="K1" t="str">
+        <v>UOM</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Base_Qty</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Cadence</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Auto_Renewal</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Plan_Type</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Validity_Days</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Plan_Limit</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Feature1</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Feature2</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Expected_Result</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>TC01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C2" t="str">
+        <v>CreatePlan001</v>
+      </c>
+      <c r="D2" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E2" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F2" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G2" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H2" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I2" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J2" t="str">
+        <v>12</v>
+      </c>
+      <c r="K2" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L2" t="str">
+        <v>1</v>
+      </c>
+      <c r="M2" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O2" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P2" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S2" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Plan created successfully</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>TC02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C3" t="str">
+        <v>ScopeSelect001</v>
+      </c>
+      <c r="D3" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E3" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F3" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G3" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H3" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I3" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J3" t="str">
+        <v>12</v>
+      </c>
+      <c r="K3" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L3" t="str">
+        <v>1</v>
+      </c>
+      <c r="M3" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O3" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P3" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S3" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T3" t="str">
+        <v>Scope dropdown selection works</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TC03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C4" t="str">
+        <v>OrgAccess001</v>
+      </c>
+      <c r="D4" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E4" t="str">
+        <v>LIMITED</v>
+      </c>
+      <c r="F4" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G4" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H4" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I4" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J4" t="str">
+        <v>12</v>
+      </c>
+      <c r="K4" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L4" t="str">
+        <v>1</v>
+      </c>
+      <c r="M4" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O4" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P4" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S4" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T4" t="str">
+        <v>Org Access Level selection works</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TC04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C5" t="str">
+        <v>PaymentType001</v>
+      </c>
+      <c r="D5" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E5" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F5" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G5" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H5" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I5" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J5" t="str">
+        <v>12</v>
+      </c>
+      <c r="K5" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L5" t="str">
+        <v>1</v>
+      </c>
+      <c r="M5" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O5" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P5" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S5" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T5" t="str">
+        <v>Payment Type selection works</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TC05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C6" t="str">
+        <v>CadenceSel001</v>
+      </c>
+      <c r="D6" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E6" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F6" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G6" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H6" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I6" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J6" t="str">
+        <v>12</v>
+      </c>
+      <c r="K6" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L6" t="str">
+        <v>1</v>
+      </c>
+      <c r="M6" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O6" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P6" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S6" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T6" t="str">
+        <v>Cadence Type selection works</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TC06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Decimal001</v>
+      </c>
+      <c r="D7" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E7" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F7" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G7" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H7" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I7" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J7" t="str">
+        <v>12.50</v>
+      </c>
+      <c r="K7" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L7" t="str">
+        <v>1</v>
+      </c>
+      <c r="M7" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O7" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P7" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S7" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T7" t="str">
+        <v>Price accepts decimal values</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TC07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C8" t="str">
+        <v>AutoRenew001</v>
+      </c>
+      <c r="D8" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E8" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F8" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G8" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H8" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I8" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J8" t="str">
+        <v>12</v>
+      </c>
+      <c r="K8" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L8" t="str">
+        <v>1</v>
+      </c>
+      <c r="M8" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N8" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O8" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P8" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S8" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T8" t="str">
+        <v>Auto Renewal toggle works</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TC08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C9" t="str">
+        <v>SingleFeat001</v>
+      </c>
+      <c r="D9" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E9" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F9" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G9" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H9" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I9" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J9" t="str">
+        <v>12</v>
+      </c>
+      <c r="K9" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L9" t="str">
+        <v>1</v>
+      </c>
+      <c r="M9" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O9" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P9" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S9" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T9" t="str">
+        <v>Single feature creation works</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TC09</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C10" t="str">
+        <v>MultiFeat001</v>
+      </c>
+      <c r="D10" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E10" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F10" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G10" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H10" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I10" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J10" t="str">
+        <v>12</v>
+      </c>
+      <c r="K10" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L10" t="str">
+        <v>1</v>
+      </c>
+      <c r="M10" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O10" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P10" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S10" t="str">
+        <v>manager</v>
+      </c>
+      <c r="T10" t="str">
+        <v>Multiple feature creation works</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TC10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Preview001</v>
+      </c>
+      <c r="D11" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E11" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F11" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G11" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H11" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I11" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J11" t="str">
+        <v>12</v>
+      </c>
+      <c r="K11" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L11" t="str">
+        <v>1</v>
+      </c>
+      <c r="M11" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N11" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O11" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P11" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+      <c r="R11" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S11" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T11" t="str">
+        <v>Plan Preview updates dynamically</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TC11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Redirect001</v>
+      </c>
+      <c r="D12" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E12" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F12" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G12" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H12" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I12" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J12" t="str">
+        <v>12</v>
+      </c>
+      <c r="K12" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L12" t="str">
+        <v>1</v>
+      </c>
+      <c r="M12" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N12" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O12" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P12" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
+      <c r="R12" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S12" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T12" t="str">
+        <v>Create Plan redirects to listing</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TC12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Table001</v>
+      </c>
+      <c r="D13" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E13" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F13" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G13" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H13" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I13" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J13" t="str">
+        <v>12</v>
+      </c>
+      <c r="K13" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L13" t="str">
+        <v>1</v>
+      </c>
+      <c r="M13" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N13" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O13" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P13" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+      <c r="R13" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S13" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T13" t="str">
+        <v>Created plan appears in table</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TC13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Best Plan_95197</v>
+      </c>
+      <c r="D14" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E14" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F14" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G14" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H14" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I14" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J14" t="str">
+        <v>12</v>
+      </c>
+      <c r="K14" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L14" t="str">
+        <v>1</v>
+      </c>
+      <c r="M14" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N14" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O14" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P14" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q14" t="str">
+        <v/>
+      </c>
+      <c r="R14" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S14" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T14" t="str">
+        <v>Search returns matching plan</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TC14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Filter</v>
+      </c>
+      <c r="C15" t="str">
+        <v>CustomerFilter001</v>
+      </c>
+      <c r="D15" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E15" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F15" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G15" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H15" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I15" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J15" t="str">
+        <v>12</v>
+      </c>
+      <c r="K15" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L15" t="str">
+        <v>1</v>
+      </c>
+      <c r="M15" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N15" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O15" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P15" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+      <c r="R15" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S15" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T15" t="str">
+        <v>Customer scope filter — every row CUSTOMER</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TC15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Filter</v>
+      </c>
+      <c r="C16" t="str">
+        <v>PartnerFilter001</v>
+      </c>
+      <c r="D16" t="str">
+        <v>PARTNER</v>
+      </c>
+      <c r="E16" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F16" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G16" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H16" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I16" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J16" t="str">
+        <v>12</v>
+      </c>
+      <c r="K16" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L16" t="str">
+        <v>1</v>
+      </c>
+      <c r="M16" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N16" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O16" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P16" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
+      <c r="R16" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S16" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T16" t="str">
+        <v>Partner scope filter — every row PARTNER</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TC16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C17" t="str">
+        <v>BLANK</v>
+      </c>
+      <c r="D17" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E17" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F17" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G17" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H17" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I17" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J17" t="str">
+        <v>12</v>
+      </c>
+      <c r="K17" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L17" t="str">
+        <v>1</v>
+      </c>
+      <c r="M17" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N17" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O17" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P17" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q17" t="str">
+        <v/>
+      </c>
+      <c r="R17" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S17" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T17" t="str">
+        <v>Plan Name is required</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TC17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="D18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="E18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="F18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="G18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="H18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="I18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="J18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="K18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="L18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="M18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="N18" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="P18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="Q18" t="str">
+        <v/>
+      </c>
+      <c r="R18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="S18" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T18" t="str">
+        <v>Mandatory fields are required</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TC18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C19" t="str">
+        <v>PriceAlpha001</v>
+      </c>
+      <c r="D19" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E19" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F19" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G19" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H19" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I19" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J19" t="str">
+        <v>ABC123</v>
+      </c>
+      <c r="K19" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L19" t="str">
+        <v>1</v>
+      </c>
+      <c r="M19" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N19" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O19" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P19" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
+      <c r="R19" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S19" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T19" t="str">
+        <v>Price rejects non-numeric input</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TC19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C20" t="str">
+        <v>NegQty001</v>
+      </c>
+      <c r="D20" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E20" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F20" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G20" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H20" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I20" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J20" t="str">
+        <v>12</v>
+      </c>
+      <c r="K20" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L20" t="str">
+        <v>-1</v>
+      </c>
+      <c r="M20" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N20" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O20" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P20" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q20" t="str">
+        <v/>
+      </c>
+      <c r="R20" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S20" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T20" t="str">
+        <v>Negative Base Quantity rejected</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TC20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C21" t="str">
+        <v>ZeroQty001</v>
+      </c>
+      <c r="D21" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E21" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F21" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G21" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H21" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I21" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J21" t="str">
+        <v>12</v>
+      </c>
+      <c r="K21" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L21" t="str">
+        <v>0</v>
+      </c>
+      <c r="M21" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N21" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O21" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P21" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q21" t="str">
+        <v/>
+      </c>
+      <c r="R21" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S21" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T21" t="str">
+        <v>Zero Base Quantity rejected</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>TC21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C22" t="str">
+        <v>ValidityAlpha001</v>
+      </c>
+      <c r="D22" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E22" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F22" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G22" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H22" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I22" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J22" t="str">
+        <v>12</v>
+      </c>
+      <c r="K22" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L22" t="str">
+        <v>1</v>
+      </c>
+      <c r="M22" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N22" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O22" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P22" t="str">
+        <v>ABC</v>
+      </c>
+      <c r="Q22" t="str">
+        <v/>
+      </c>
+      <c r="R22" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S22" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T22" t="str">
+        <v>Validity rejects non-numeric input</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>TC22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Best Plan_95197</v>
+      </c>
+      <c r="D23" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E23" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F23" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G23" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H23" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I23" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J23" t="str">
+        <v>12</v>
+      </c>
+      <c r="K23" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L23" t="str">
+        <v>1</v>
+      </c>
+      <c r="M23" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N23" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O23" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P23" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q23" t="str">
+        <v/>
+      </c>
+      <c r="R23" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S23" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T23" t="str">
+        <v>Duplicate name accepted (no uniqueness guard)</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TC23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C24" t="str">
+        <v>LongDesc001</v>
+      </c>
+      <c r="D24" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E24" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F24" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G24" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H24" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I24" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J24" t="str">
+        <v>12</v>
+      </c>
+      <c r="K24" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L24" t="str">
+        <v>1</v>
+      </c>
+      <c r="M24" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N24" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O24" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P24" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
+      <c r="R24" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S24" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T24" t="str">
+        <v>Long description accepted (no length limit)</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TC24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C25" t="str">
+        <v>BadTax001</v>
+      </c>
+      <c r="D25" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E25" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F25" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G25" t="str">
+        <v>INVALIDTAX999</v>
+      </c>
+      <c r="H25" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I25" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J25" t="str">
+        <v>12</v>
+      </c>
+      <c r="K25" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L25" t="str">
+        <v>1</v>
+      </c>
+      <c r="M25" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N25" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O25" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P25" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q25" t="str">
+        <v/>
+      </c>
+      <c r="R25" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S25" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T25" t="str">
+        <v>Invalid Tax Code not selectable</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TC25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C26" t="str">
+        <v>ScopeGuard001</v>
+      </c>
+      <c r="D26" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E26" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F26" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G26" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H26" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I26" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J26" t="str">
+        <v>12</v>
+      </c>
+      <c r="K26" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L26" t="str">
+        <v>1</v>
+      </c>
+      <c r="M26" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N26" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O26" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P26" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q26" t="str">
+        <v/>
+      </c>
+      <c r="R26" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S26" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T26" t="str">
+        <v>Scope is pre-filled (guarded by default)</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TC26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C27" t="str">
+        <v>BlankFeat001</v>
+      </c>
+      <c r="D27" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E27" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F27" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G27" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H27" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I27" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J27" t="str">
+        <v>12</v>
+      </c>
+      <c r="K27" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L27" t="str">
+        <v>1</v>
+      </c>
+      <c r="M27" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N27" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O27" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P27" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
+      <c r="R27" t="str">
+        <v>BLANK</v>
+      </c>
+      <c r="S27" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T27" t="str">
+        <v>Blank feature validation</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TC27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C28" t="str">
+        <v>CurrencyGuard001</v>
+      </c>
+      <c r="D28" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E28" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F28" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G28" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H28" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I28" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J28" t="str">
+        <v>12</v>
+      </c>
+      <c r="K28" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L28" t="str">
+        <v>1</v>
+      </c>
+      <c r="M28" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N28" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O28" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P28" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q28" t="str">
+        <v/>
+      </c>
+      <c r="R28" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S28" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T28" t="str">
+        <v>Currency is pre-filled (guarded by default)</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>TC28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C29" t="str">
+        <v>BadCadence001</v>
+      </c>
+      <c r="D29" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E29" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F29" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G29" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H29" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I29" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J29" t="str">
+        <v>12</v>
+      </c>
+      <c r="K29" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L29" t="str">
+        <v>1</v>
+      </c>
+      <c r="M29" t="str">
+        <v>INVALID</v>
+      </c>
+      <c r="N29" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O29" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P29" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q29" t="str">
+        <v/>
+      </c>
+      <c r="R29" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S29" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T29" t="str">
+        <v>Invalid Cadence Type not selectable</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TC29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C30" t="str">
+        <v>ApiFail001</v>
+      </c>
+      <c r="D30" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E30" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F30" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G30" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H30" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I30" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J30" t="str">
+        <v>12</v>
+      </c>
+      <c r="K30" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L30" t="str">
+        <v>1</v>
+      </c>
+      <c r="M30" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N30" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O30" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P30" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q30" t="str">
+        <v/>
+      </c>
+      <c r="R30" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S30" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T30" t="str">
+        <v>API/Network failure shows no false success</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TC30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="C31" t="str">
+        <v>InvalidUrl001</v>
+      </c>
+      <c r="D31" t="str">
+        <v>CUSTOMER</v>
+      </c>
+      <c r="E31" t="str">
+        <v>GLOBAL</v>
+      </c>
+      <c r="F31" t="str">
+        <v>PRE-PAID</v>
+      </c>
+      <c r="G31" t="str">
+        <v>TAX_VALIDATION_806531</v>
+      </c>
+      <c r="H31" t="str">
+        <v>73301</v>
+      </c>
+      <c r="I31" t="str">
+        <v>USD</v>
+      </c>
+      <c r="J31" t="str">
+        <v>12</v>
+      </c>
+      <c r="K31" t="str">
+        <v>AMOUNT</v>
+      </c>
+      <c r="L31" t="str">
+        <v>1</v>
+      </c>
+      <c r="M31" t="str">
+        <v>QUARTERLY</v>
+      </c>
+      <c r="N31" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="O31" t="str">
+        <v>DURATION</v>
+      </c>
+      <c r="P31" t="str">
+        <v>3</v>
+      </c>
+      <c r="Q31" t="str">
+        <v/>
+      </c>
+      <c r="R31" t="str">
+        <v>admin</v>
+      </c>
+      <c r="S31" t="str">
+        <v>NULL</v>
+      </c>
+      <c r="T31" t="str">
+        <v>Invalid plan URL shows error/not-found</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:T31"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B1"/>

</xml_diff>

<commit_message>
Merge RoleManagementTest sheet into testData.xlsx
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -36,6 +36,7 @@
     <sheet name="ZoneManagementTest" sheetId="21" r:id="rId24"/>
     <sheet name="Subscription plan" sheetId="22" r:id="rId25"/>
     <sheet name="SubscriptionPlanTest" sheetId="23" r:id="rId26"/>
+    <sheet name="RoleManagementTest" sheetId="24" r:id="rId27"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -11259,6 +11260,925 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
+  <dimension ref="A1:G39"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="42.83203125" customWidth="1"/>
+    <col min="2" max="2" width="80.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+    <col min="5" max="5" width="25.83203125" customWidth="1"/>
+    <col min="6" max="6" width="70.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" t="s">
+        <v>753</v>
+      </c>
+      <c r="D1" t="s">
+        <v>754</v>
+      </c>
+      <c r="E1" t="s">
+        <v>755</v>
+      </c>
+      <c r="F1" t="s">
+        <v>611</v>
+      </c>
+      <c r="G1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>756</v>
+      </c>
+      <c r="B2" t="s">
+        <v>757</v>
+      </c>
+      <c r="C2" t="s">
+        <v>615</v>
+      </c>
+      <c r="D2" t="s">
+        <v>615</v>
+      </c>
+      <c r="E2" t="s">
+        <v>615</v>
+      </c>
+      <c r="F2" t="s">
+        <v>758</v>
+      </c>
+      <c r="G2" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>759</v>
+      </c>
+      <c r="B3" t="s">
+        <v>760</v>
+      </c>
+      <c r="C3" t="s">
+        <v>615</v>
+      </c>
+      <c r="D3" t="s">
+        <v>615</v>
+      </c>
+      <c r="E3" t="s">
+        <v>615</v>
+      </c>
+      <c r="F3" t="s">
+        <v>761</v>
+      </c>
+      <c r="G3" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>762</v>
+      </c>
+      <c r="B4" t="s">
+        <v>763</v>
+      </c>
+      <c r="C4" t="s">
+        <v>615</v>
+      </c>
+      <c r="D4" t="s">
+        <v>615</v>
+      </c>
+      <c r="E4" t="s">
+        <v>764</v>
+      </c>
+      <c r="F4" t="s">
+        <v>765</v>
+      </c>
+      <c r="G4" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>766</v>
+      </c>
+      <c r="B5" t="s">
+        <v>767</v>
+      </c>
+      <c r="C5" t="s">
+        <v>615</v>
+      </c>
+      <c r="D5" t="s">
+        <v>615</v>
+      </c>
+      <c r="E5" t="s">
+        <v>768</v>
+      </c>
+      <c r="F5" t="s">
+        <v>769</v>
+      </c>
+      <c r="G5" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>770</v>
+      </c>
+      <c r="B6" t="s">
+        <v>771</v>
+      </c>
+      <c r="C6" t="s">
+        <v>615</v>
+      </c>
+      <c r="D6" t="s">
+        <v>615</v>
+      </c>
+      <c r="E6" t="s">
+        <v>615</v>
+      </c>
+      <c r="F6" t="s">
+        <v>772</v>
+      </c>
+      <c r="G6" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>773</v>
+      </c>
+      <c r="B7" t="s">
+        <v>774</v>
+      </c>
+      <c r="C7" t="s">
+        <v>615</v>
+      </c>
+      <c r="D7" t="s">
+        <v>615</v>
+      </c>
+      <c r="E7" t="s">
+        <v>615</v>
+      </c>
+      <c r="F7" t="s">
+        <v>775</v>
+      </c>
+      <c r="G7" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>776</v>
+      </c>
+      <c r="B8" t="s">
+        <v>777</v>
+      </c>
+      <c r="C8" t="s">
+        <v>615</v>
+      </c>
+      <c r="D8" t="s">
+        <v>615</v>
+      </c>
+      <c r="E8" t="s">
+        <v>615</v>
+      </c>
+      <c r="F8" t="s">
+        <v>778</v>
+      </c>
+      <c r="G8" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>779</v>
+      </c>
+      <c r="B9" t="s">
+        <v>780</v>
+      </c>
+      <c r="C9" t="s">
+        <v>615</v>
+      </c>
+      <c r="D9" t="s">
+        <v>615</v>
+      </c>
+      <c r="E9" t="s">
+        <v>615</v>
+      </c>
+      <c r="F9" t="s">
+        <v>781</v>
+      </c>
+      <c r="G9" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>782</v>
+      </c>
+      <c r="B10" t="s">
+        <v>783</v>
+      </c>
+      <c r="C10" t="s">
+        <v>615</v>
+      </c>
+      <c r="D10" t="s">
+        <v>615</v>
+      </c>
+      <c r="E10" t="s">
+        <v>615</v>
+      </c>
+      <c r="F10" t="s">
+        <v>784</v>
+      </c>
+      <c r="G10" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>785</v>
+      </c>
+      <c r="B11" t="s">
+        <v>786</v>
+      </c>
+      <c r="C11" t="s">
+        <v>615</v>
+      </c>
+      <c r="D11" t="s">
+        <v>615</v>
+      </c>
+      <c r="E11" t="s">
+        <v>615</v>
+      </c>
+      <c r="F11" t="s">
+        <v>787</v>
+      </c>
+      <c r="G11" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>788</v>
+      </c>
+      <c r="B12" t="s">
+        <v>789</v>
+      </c>
+      <c r="C12" t="s">
+        <v>790</v>
+      </c>
+      <c r="D12" t="s">
+        <v>791</v>
+      </c>
+      <c r="E12" t="s">
+        <v>615</v>
+      </c>
+      <c r="F12" t="s">
+        <v>792</v>
+      </c>
+      <c r="G12" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>793</v>
+      </c>
+      <c r="B13" t="s">
+        <v>794</v>
+      </c>
+      <c r="C13" t="s">
+        <v>790</v>
+      </c>
+      <c r="D13" t="s">
+        <v>791</v>
+      </c>
+      <c r="E13" t="s">
+        <v>615</v>
+      </c>
+      <c r="F13" t="s">
+        <v>795</v>
+      </c>
+      <c r="G13" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>796</v>
+      </c>
+      <c r="B14" t="s">
+        <v>797</v>
+      </c>
+      <c r="C14" t="s">
+        <v>615</v>
+      </c>
+      <c r="D14" t="s">
+        <v>615</v>
+      </c>
+      <c r="E14" t="s">
+        <v>615</v>
+      </c>
+      <c r="F14" t="s">
+        <v>798</v>
+      </c>
+      <c r="G14" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>799</v>
+      </c>
+      <c r="B15" t="s">
+        <v>800</v>
+      </c>
+      <c r="C15" t="s">
+        <v>615</v>
+      </c>
+      <c r="D15" t="s">
+        <v>615</v>
+      </c>
+      <c r="E15" t="s">
+        <v>615</v>
+      </c>
+      <c r="F15" t="s">
+        <v>801</v>
+      </c>
+      <c r="G15" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>802</v>
+      </c>
+      <c r="B16" t="s">
+        <v>803</v>
+      </c>
+      <c r="C16" t="s">
+        <v>615</v>
+      </c>
+      <c r="D16" t="s">
+        <v>791</v>
+      </c>
+      <c r="E16" t="s">
+        <v>615</v>
+      </c>
+      <c r="F16" t="s">
+        <v>804</v>
+      </c>
+      <c r="G16" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>805</v>
+      </c>
+      <c r="B17" t="s">
+        <v>806</v>
+      </c>
+      <c r="C17" t="s">
+        <v>807</v>
+      </c>
+      <c r="D17" t="s">
+        <v>791</v>
+      </c>
+      <c r="E17" t="s">
+        <v>615</v>
+      </c>
+      <c r="F17" t="s">
+        <v>808</v>
+      </c>
+      <c r="G17" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>809</v>
+      </c>
+      <c r="B18" t="s">
+        <v>810</v>
+      </c>
+      <c r="C18" t="s">
+        <v>790</v>
+      </c>
+      <c r="D18" t="s">
+        <v>791</v>
+      </c>
+      <c r="E18" t="s">
+        <v>615</v>
+      </c>
+      <c r="F18" t="s">
+        <v>811</v>
+      </c>
+      <c r="G18" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>812</v>
+      </c>
+      <c r="B19" t="s">
+        <v>813</v>
+      </c>
+      <c r="C19" t="s">
+        <v>615</v>
+      </c>
+      <c r="D19" t="s">
+        <v>615</v>
+      </c>
+      <c r="E19" t="s">
+        <v>615</v>
+      </c>
+      <c r="F19" t="s">
+        <v>814</v>
+      </c>
+      <c r="G19" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>815</v>
+      </c>
+      <c r="B20" t="s">
+        <v>816</v>
+      </c>
+      <c r="C20" t="s">
+        <v>615</v>
+      </c>
+      <c r="D20" t="s">
+        <v>615</v>
+      </c>
+      <c r="E20" t="s">
+        <v>615</v>
+      </c>
+      <c r="F20" t="s">
+        <v>817</v>
+      </c>
+      <c r="G20" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>818</v>
+      </c>
+      <c r="B21" t="s">
+        <v>819</v>
+      </c>
+      <c r="C21" t="s">
+        <v>615</v>
+      </c>
+      <c r="D21" t="s">
+        <v>615</v>
+      </c>
+      <c r="E21" t="s">
+        <v>615</v>
+      </c>
+      <c r="F21" t="s">
+        <v>820</v>
+      </c>
+      <c r="G21" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>821</v>
+      </c>
+      <c r="B22" t="s">
+        <v>822</v>
+      </c>
+      <c r="C22" t="s">
+        <v>615</v>
+      </c>
+      <c r="D22" t="s">
+        <v>615</v>
+      </c>
+      <c r="E22" t="s">
+        <v>615</v>
+      </c>
+      <c r="F22" t="s">
+        <v>823</v>
+      </c>
+      <c r="G22" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>824</v>
+      </c>
+      <c r="B23" t="s">
+        <v>825</v>
+      </c>
+      <c r="C23" t="s">
+        <v>615</v>
+      </c>
+      <c r="D23" t="s">
+        <v>615</v>
+      </c>
+      <c r="E23" t="s">
+        <v>826</v>
+      </c>
+      <c r="F23" t="s">
+        <v>827</v>
+      </c>
+      <c r="G23" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>828</v>
+      </c>
+      <c r="B24" t="s">
+        <v>829</v>
+      </c>
+      <c r="C24" t="s">
+        <v>615</v>
+      </c>
+      <c r="D24" t="s">
+        <v>615</v>
+      </c>
+      <c r="E24" t="s">
+        <v>615</v>
+      </c>
+      <c r="F24" t="s">
+        <v>830</v>
+      </c>
+      <c r="G24" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>831</v>
+      </c>
+      <c r="B25" t="s">
+        <v>832</v>
+      </c>
+      <c r="C25" t="s">
+        <v>615</v>
+      </c>
+      <c r="D25" t="s">
+        <v>615</v>
+      </c>
+      <c r="E25" t="s">
+        <v>615</v>
+      </c>
+      <c r="F25" t="s">
+        <v>833</v>
+      </c>
+      <c r="G25" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>834</v>
+      </c>
+      <c r="B26" t="s">
+        <v>835</v>
+      </c>
+      <c r="C26" t="s">
+        <v>615</v>
+      </c>
+      <c r="D26" t="s">
+        <v>615</v>
+      </c>
+      <c r="E26" t="s">
+        <v>615</v>
+      </c>
+      <c r="F26" t="s">
+        <v>836</v>
+      </c>
+      <c r="G26" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>837</v>
+      </c>
+      <c r="B27" t="s">
+        <v>838</v>
+      </c>
+      <c r="C27" t="s">
+        <v>615</v>
+      </c>
+      <c r="D27" t="s">
+        <v>615</v>
+      </c>
+      <c r="E27" t="s">
+        <v>615</v>
+      </c>
+      <c r="F27" t="s">
+        <v>839</v>
+      </c>
+      <c r="G27" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>840</v>
+      </c>
+      <c r="B28" t="s">
+        <v>841</v>
+      </c>
+      <c r="C28" t="s">
+        <v>615</v>
+      </c>
+      <c r="D28" t="s">
+        <v>615</v>
+      </c>
+      <c r="E28" t="s">
+        <v>615</v>
+      </c>
+      <c r="F28" t="s">
+        <v>842</v>
+      </c>
+      <c r="G28" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>843</v>
+      </c>
+      <c r="B29" t="s">
+        <v>844</v>
+      </c>
+      <c r="C29" t="s">
+        <v>845</v>
+      </c>
+      <c r="D29" t="s">
+        <v>846</v>
+      </c>
+      <c r="E29" t="s">
+        <v>615</v>
+      </c>
+      <c r="F29" t="s">
+        <v>847</v>
+      </c>
+      <c r="G29" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>848</v>
+      </c>
+      <c r="B30" t="s">
+        <v>849</v>
+      </c>
+      <c r="C30" t="s">
+        <v>845</v>
+      </c>
+      <c r="D30" t="s">
+        <v>850</v>
+      </c>
+      <c r="E30" t="s">
+        <v>615</v>
+      </c>
+      <c r="F30" t="s">
+        <v>851</v>
+      </c>
+      <c r="G30" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>852</v>
+      </c>
+      <c r="B31" t="s">
+        <v>853</v>
+      </c>
+      <c r="C31" t="s">
+        <v>615</v>
+      </c>
+      <c r="D31" t="s">
+        <v>615</v>
+      </c>
+      <c r="E31" t="s">
+        <v>615</v>
+      </c>
+      <c r="F31" t="s">
+        <v>854</v>
+      </c>
+      <c r="G31" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>855</v>
+      </c>
+      <c r="B32" t="s">
+        <v>856</v>
+      </c>
+      <c r="C32" t="s">
+        <v>615</v>
+      </c>
+      <c r="D32" t="s">
+        <v>615</v>
+      </c>
+      <c r="E32" t="s">
+        <v>615</v>
+      </c>
+      <c r="F32" t="s">
+        <v>857</v>
+      </c>
+      <c r="G32" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>858</v>
+      </c>
+      <c r="B33" t="s">
+        <v>859</v>
+      </c>
+      <c r="C33" t="s">
+        <v>615</v>
+      </c>
+      <c r="D33" t="s">
+        <v>615</v>
+      </c>
+      <c r="E33" t="s">
+        <v>615</v>
+      </c>
+      <c r="F33" t="s">
+        <v>860</v>
+      </c>
+      <c r="G33" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>861</v>
+      </c>
+      <c r="B34" t="s">
+        <v>862</v>
+      </c>
+      <c r="C34" t="s">
+        <v>615</v>
+      </c>
+      <c r="D34" t="s">
+        <v>863</v>
+      </c>
+      <c r="E34" t="s">
+        <v>615</v>
+      </c>
+      <c r="F34" t="s">
+        <v>864</v>
+      </c>
+      <c r="G34" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>865</v>
+      </c>
+      <c r="B35" t="s">
+        <v>866</v>
+      </c>
+      <c r="C35" t="s">
+        <v>615</v>
+      </c>
+      <c r="D35" t="s">
+        <v>615</v>
+      </c>
+      <c r="E35" t="s">
+        <v>615</v>
+      </c>
+      <c r="F35" t="s">
+        <v>867</v>
+      </c>
+      <c r="G35" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>868</v>
+      </c>
+      <c r="B36" t="s">
+        <v>869</v>
+      </c>
+      <c r="C36" t="s">
+        <v>870</v>
+      </c>
+      <c r="D36" t="s">
+        <v>791</v>
+      </c>
+      <c r="E36" t="s">
+        <v>615</v>
+      </c>
+      <c r="F36" t="s">
+        <v>871</v>
+      </c>
+      <c r="G36" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>872</v>
+      </c>
+      <c r="B37" t="s">
+        <v>873</v>
+      </c>
+      <c r="C37" t="s">
+        <v>870</v>
+      </c>
+      <c r="D37" t="s">
+        <v>791</v>
+      </c>
+      <c r="E37" t="s">
+        <v>615</v>
+      </c>
+      <c r="F37" t="s">
+        <v>874</v>
+      </c>
+      <c r="G37" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>875</v>
+      </c>
+      <c r="B38" t="s">
+        <v>876</v>
+      </c>
+      <c r="C38" t="s">
+        <v>870</v>
+      </c>
+      <c r="D38" t="s">
+        <v>791</v>
+      </c>
+      <c r="E38" t="s">
+        <v>615</v>
+      </c>
+      <c r="F38" t="s">
+        <v>877</v>
+      </c>
+      <c r="G38" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>878</v>
+      </c>
+      <c r="B39" t="s">
+        <v>879</v>
+      </c>
+      <c r="C39" t="s">
+        <v>870</v>
+      </c>
+      <c r="D39" t="s">
+        <v>791</v>
+      </c>
+      <c r="E39" t="s">
+        <v>615</v>
+      </c>
+      <c r="F39" t="s">
+        <v>880</v>
+      </c>
+      <c r="G39" t="s">
+        <v>615</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:G39" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B1"/>

</xml_diff>

<commit_message>
Restore RoleManagementTest sheet and add to Regression suite
- Restored 38-row RoleManagementTest sheet from original commit 088be38
- Added RoleManagementTest (serial) to Regression sheet as row 40
- Retained all 24 sheets with no data loss
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -36,14 +36,14 @@
     <sheet name="ZoneManagementTest" sheetId="21" r:id="rId24"/>
     <sheet name="Subscription plan" sheetId="22" r:id="rId25"/>
     <sheet name="SubscriptionPlanTest" sheetId="23" r:id="rId26"/>
-    <sheet name="RoleManagementTest" sheetId="24" r:id="rId27"/>
+    <sheet name="RoleManagementTest" sheetId="24" r:id="rId28"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="606">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="736">
   <si>
     <t>TestName</t>
   </si>
@@ -1863,6 +1863,396 @@
   </si>
   <si>
     <t>CustomerManagement</t>
+  </si>
+  <si>
+    <t>Description_Input</t>
+  </si>
+  <si>
+    <t>SearchTerm</t>
+  </si>
+  <si>
+    <t>TC01_RolePageLoad</t>
+  </si>
+  <si>
+    <t>ExpectedMessage</t>
+  </si>
+  <si>
+    <t>Verify Role page loads successfully</t>
+  </si>
+  <si>
+    <t>Role listing page with Create Role button should be visible</t>
+  </si>
+  <si>
+    <t>Zone list visible</t>
+  </si>
+  <si>
+    <t>TC02_RoleGridDisplay</t>
+  </si>
+  <si>
+    <t>Verify role grid displays with Name, Description and Action icons</t>
+  </si>
+  <si>
+    <t>Name column, Description column and Action icons should be visible</t>
+  </si>
+  <si>
+    <t>TC03_SearchValidRole</t>
+  </si>
+  <si>
+    <t>Verify search with valid role name returns matching results</t>
+  </si>
+  <si>
+    <t>Agent</t>
+  </si>
+  <si>
+    <t>Matching role should be displayed</t>
+  </si>
+  <si>
+    <t>TC04_SearchInvalidRole</t>
+  </si>
+  <si>
+    <t>Verify search with invalid role name shows no matching records</t>
+  </si>
+  <si>
+    <t>INVALID_ROLE_123</t>
+  </si>
+  <si>
+    <t>No data / no matching records message should be displayed</t>
+  </si>
+  <si>
+    <t>TC05_CreateRoleButtonPopup</t>
+  </si>
+  <si>
+    <t>Verify Create Role button opens the Create Role popup</t>
+  </si>
+  <si>
+    <t>Create Role popup should be displayed</t>
+  </si>
+  <si>
+    <t>TC06_LockIconPermPage</t>
+  </si>
+  <si>
+    <t>Verify Lock icon opens the Role Permission page</t>
+  </si>
+  <si>
+    <t>Role Permission page should be displayed</t>
+  </si>
+  <si>
+    <t>TC07_EditIconPopup</t>
+  </si>
+  <si>
+    <t>Verify Edit icon opens the Edit Role popup</t>
+  </si>
+  <si>
+    <t>Edit Role popup should be displayed</t>
+  </si>
+  <si>
+    <t>TC08_DeleteIconPopup</t>
+  </si>
+  <si>
+    <t>Verify Delete icon opens the delete confirmation popup</t>
+  </si>
+  <si>
+    <t>Delete confirmation popup should be displayed</t>
+  </si>
+  <si>
+    <t>TC09_RefreshReloads</t>
+  </si>
+  <si>
+    <t>Verify Refresh button reloads the role listing</t>
+  </si>
+  <si>
+    <t>Role listing should reload successfully</t>
+  </si>
+  <si>
+    <t>TC10_PaginationVisible</t>
+  </si>
+  <si>
+    <t>Verify pagination controls are displayed when available</t>
+  </si>
+  <si>
+    <t>Pagination controls should be visible when multiple pages exist</t>
+  </si>
+  <si>
+    <t>TC11_CreateRoleSuccess</t>
+  </si>
+  <si>
+    <t>Verify role is created successfully with valid name and description</t>
+  </si>
+  <si>
+    <t>AutoRole_</t>
+  </si>
+  <si>
+    <t>Automation Role Description</t>
+  </si>
+  <si>
+    <t>Role should be created successfully</t>
+  </si>
+  <si>
+    <t>TC12_CreatedRoleInListing</t>
+  </si>
+  <si>
+    <t>Verify newly created role appears in the role listing</t>
+  </si>
+  <si>
+    <t>Created role should appear in the listing after search</t>
+  </si>
+  <si>
+    <t>TC13_CancelClosesCreatePopup</t>
+  </si>
+  <si>
+    <t>Verify Cancel button closes the Create Role popup without creating a role</t>
+  </si>
+  <si>
+    <t>Popup should be closed after clicking Cancel</t>
+  </si>
+  <si>
+    <t>TC14_CloseXClosesCreatePopup</t>
+  </si>
+  <si>
+    <t>Verify Close (X) icon closes the Create Role popup</t>
+  </si>
+  <si>
+    <t>Popup should be closed after clicking Close (X)</t>
+  </si>
+  <si>
+    <t>TC15_RoleNameRequiredValidation</t>
+  </si>
+  <si>
+    <t>Verify Role Name required validation when Role Name is blank</t>
+  </si>
+  <si>
+    <t>Validation message should be displayed for blank Role Name</t>
+  </si>
+  <si>
+    <t>TC16_SpacesOnlyRoleName</t>
+  </si>
+  <si>
+    <t>Verify spaces-only Role Name input shows validation message</t>
+  </si>
+  <si>
+    <t>     </t>
+  </si>
+  <si>
+    <t>Validation message should be displayed for spaces-only Role Name</t>
+  </si>
+  <si>
+    <t>TC17_DuplicateRoleValidation</t>
+  </si>
+  <si>
+    <t>Verify duplicate role creation shows validation message</t>
+  </si>
+  <si>
+    <t>Duplicate role validation message should be displayed</t>
+  </si>
+  <si>
+    <t>TC18_PermissionPageOpens</t>
+  </si>
+  <si>
+    <t>Verify Role Permission page opens when Lock icon is clicked</t>
+  </si>
+  <si>
+    <t>Role Permission page should be visible</t>
+  </si>
+  <si>
+    <t>TC19_AssignPermissionToast</t>
+  </si>
+  <si>
+    <t>Assign permission successfully and verify success toast</t>
+  </si>
+  <si>
+    <t>Permission added to role!</t>
+  </si>
+  <si>
+    <t>TC20_PermissionCountIncrements</t>
+  </si>
+  <si>
+    <t>Verify permission count increments by 1 after assigning a permission</t>
+  </si>
+  <si>
+    <t>afterCount should equal beforeCount + 1</t>
+  </si>
+  <si>
+    <t>TC21_PermissionSearchValid</t>
+  </si>
+  <si>
+    <t>Verify permission search returns matching results</t>
+  </si>
+  <si>
+    <t>Matching permissions should be displayed</t>
+  </si>
+  <si>
+    <t>TC22_PermissionSearchInvalid</t>
+  </si>
+  <si>
+    <t>Verify invalid permission search shows no matching results</t>
+  </si>
+  <si>
+    <t>INVALID_PERMISSION_123</t>
+  </si>
+  <si>
+    <t>No results message should be displayed</t>
+  </si>
+  <si>
+    <t>TC23_DeletePermission</t>
+  </si>
+  <si>
+    <t>Verify permission is removed after clicking Delete icon</t>
+  </si>
+  <si>
+    <t>Permission should be removed from the assigned list</t>
+  </si>
+  <si>
+    <t>TC24_PermissionCountDecrements</t>
+  </si>
+  <si>
+    <t>Verify permission count decrements by 1 after deleting a permission</t>
+  </si>
+  <si>
+    <t>afterCount should equal beforeCount - 1</t>
+  </si>
+  <si>
+    <t>TC25_BackButtonReturnsListing</t>
+  </si>
+  <si>
+    <t>Verify Back button on Permission page returns to Role listing</t>
+  </si>
+  <si>
+    <t>Role listing page should be displayed after clicking Back</t>
+  </si>
+  <si>
+    <t>TC26_AssignWithoutSelectValidation</t>
+  </si>
+  <si>
+    <t>Verify clicking Assign Permission without selecting shows validation</t>
+  </si>
+  <si>
+    <t>Validation or error message should be displayed</t>
+  </si>
+  <si>
+    <t>TC27_EditPopupPrePopulated</t>
+  </si>
+  <si>
+    <t>Verify Edit popup is pre-populated with existing Role Name and Description</t>
+  </si>
+  <si>
+    <t>Role Name and Description should be pre-populated in Edit popup</t>
+  </si>
+  <si>
+    <t>TC28_UpdateDescription</t>
+  </si>
+  <si>
+    <t>Verify role description can be updated successfully</t>
+  </si>
+  <si>
+    <t>AutoEdit_</t>
+  </si>
+  <si>
+    <t>Updated_Desc_</t>
+  </si>
+  <si>
+    <t>Update should be successful and popup should close</t>
+  </si>
+  <si>
+    <t>TC29_UpdatedDescriptionSaved</t>
+  </si>
+  <si>
+    <t>Verify updated description is saved and visible in the listing</t>
+  </si>
+  <si>
+    <t>SavedDesc_</t>
+  </si>
+  <si>
+    <t>Updated description should be visible in the listing row</t>
+  </si>
+  <si>
+    <t>TC30_CancelClosesEditPopup</t>
+  </si>
+  <si>
+    <t>Verify Cancel button closes Edit popup without saving changes</t>
+  </si>
+  <si>
+    <t>Edit popup should be closed after clicking Cancel</t>
+  </si>
+  <si>
+    <t>TC31_CloseXClosesEditPopup</t>
+  </si>
+  <si>
+    <t>Verify Close (X) icon closes the Edit popup</t>
+  </si>
+  <si>
+    <t>Edit popup should be closed after clicking Close (X)</t>
+  </si>
+  <si>
+    <t>TC32_EmptyDescriptionValidation</t>
+  </si>
+  <si>
+    <t>Verify empty Description field shows validation message on Update</t>
+  </si>
+  <si>
+    <t>Validation message should be displayed for empty Description</t>
+  </si>
+  <si>
+    <t>TC33_SpacesDescriptionValidation</t>
+  </si>
+  <si>
+    <t>Verify spaces-only Description shows validation message on Update</t>
+  </si>
+  <si>
+    <t>      </t>
+  </si>
+  <si>
+    <t>Validation message should be displayed for spaces-only Description</t>
+  </si>
+  <si>
+    <t>TC34_DeletePopupVisible</t>
+  </si>
+  <si>
+    <t>Verify delete confirmation popup is displayed when Delete icon is clicked</t>
+  </si>
+  <si>
+    <t>Delete confirmation popup should be visible</t>
+  </si>
+  <si>
+    <t>TC35_CancelDeletePreservesRole</t>
+  </si>
+  <si>
+    <t>Verify clicking Cancel on delete popup does not delete the role</t>
+  </si>
+  <si>
+    <t>AutoDelete_</t>
+  </si>
+  <si>
+    <t>Role should still exist in the listing after cancelling delete</t>
+  </si>
+  <si>
+    <t>TC36_ConfirmDeleteSuccess</t>
+  </si>
+  <si>
+    <t>Verify role is deleted successfully after confirming deletion</t>
+  </si>
+  <si>
+    <t>Role should be deleted successfully</t>
+  </si>
+  <si>
+    <t>TC37_DeletedRoleNotInListing</t>
+  </si>
+  <si>
+    <t>Verify deleted role is no longer visible in the listing</t>
+  </si>
+  <si>
+    <t>Deleted role should not be found in search results</t>
+  </si>
+  <si>
+    <t>TC38_DeleteSuccessMessage</t>
+  </si>
+  <si>
+    <t>Verify success message is displayed after successful role deletion</t>
+  </si>
+  <si>
+    <t>Success message should be displayed after deletion</t>
+  </si>
+  <si>
+    <t>RoleManagementTest</t>
   </si>
 </sst>
 </file>
@@ -2269,7 +2659,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
@@ -2701,6 +3091,17 @@
         <v>4</v>
       </c>
       <c r="C39" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>735</v>
+      </c>
+      <c r="B40" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" t="s">
         <v>8</v>
       </c>
     </row>
@@ -11260,7 +11661,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
   <dimension ref="A1:G39"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -11276,899 +11677,899 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C1" t="s">
-        <v>753</v>
+        <v>606</v>
       </c>
       <c r="D1" t="s">
-        <v>754</v>
+        <v>607</v>
       </c>
       <c r="E1" t="s">
-        <v>755</v>
+        <v>608</v>
       </c>
       <c r="F1" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="G1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>756</v>
+        <v>610</v>
       </c>
       <c r="B2" t="s">
-        <v>757</v>
+        <v>611</v>
       </c>
       <c r="C2" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D2" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E2" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F2" t="s">
-        <v>758</v>
+        <v>613</v>
       </c>
       <c r="G2" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>759</v>
+        <v>614</v>
       </c>
       <c r="B3" t="s">
-        <v>760</v>
+        <v>615</v>
       </c>
       <c r="C3" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D3" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E3" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F3" t="s">
-        <v>761</v>
+        <v>616</v>
       </c>
       <c r="G3" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>762</v>
+        <v>617</v>
       </c>
       <c r="B4" t="s">
-        <v>763</v>
+        <v>618</v>
       </c>
       <c r="C4" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D4" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E4" t="s">
-        <v>764</v>
+        <v>619</v>
       </c>
       <c r="F4" t="s">
-        <v>765</v>
+        <v>620</v>
       </c>
       <c r="G4" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>766</v>
+        <v>621</v>
       </c>
       <c r="B5" t="s">
-        <v>767</v>
+        <v>622</v>
       </c>
       <c r="C5" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D5" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E5" t="s">
-        <v>768</v>
+        <v>623</v>
       </c>
       <c r="F5" t="s">
-        <v>769</v>
+        <v>624</v>
       </c>
       <c r="G5" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>770</v>
+        <v>625</v>
       </c>
       <c r="B6" t="s">
-        <v>771</v>
+        <v>626</v>
       </c>
       <c r="C6" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D6" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E6" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F6" t="s">
-        <v>772</v>
+        <v>627</v>
       </c>
       <c r="G6" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>773</v>
+        <v>628</v>
       </c>
       <c r="B7" t="s">
-        <v>774</v>
+        <v>629</v>
       </c>
       <c r="C7" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D7" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E7" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F7" t="s">
-        <v>775</v>
+        <v>630</v>
       </c>
       <c r="G7" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>776</v>
+        <v>631</v>
       </c>
       <c r="B8" t="s">
-        <v>777</v>
+        <v>632</v>
       </c>
       <c r="C8" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D8" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E8" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F8" t="s">
-        <v>778</v>
+        <v>633</v>
       </c>
       <c r="G8" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>779</v>
+        <v>634</v>
       </c>
       <c r="B9" t="s">
-        <v>780</v>
+        <v>635</v>
       </c>
       <c r="C9" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D9" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E9" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F9" t="s">
-        <v>781</v>
+        <v>636</v>
       </c>
       <c r="G9" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>782</v>
+        <v>637</v>
       </c>
       <c r="B10" t="s">
-        <v>783</v>
+        <v>638</v>
       </c>
       <c r="C10" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D10" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E10" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F10" t="s">
-        <v>784</v>
+        <v>639</v>
       </c>
       <c r="G10" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>785</v>
+        <v>640</v>
       </c>
       <c r="B11" t="s">
-        <v>786</v>
+        <v>641</v>
       </c>
       <c r="C11" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D11" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E11" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F11" t="s">
-        <v>787</v>
+        <v>642</v>
       </c>
       <c r="G11" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>788</v>
+        <v>643</v>
       </c>
       <c r="B12" t="s">
-        <v>789</v>
+        <v>644</v>
       </c>
       <c r="C12" t="s">
-        <v>790</v>
+        <v>645</v>
       </c>
       <c r="D12" t="s">
-        <v>791</v>
+        <v>646</v>
       </c>
       <c r="E12" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F12" t="s">
-        <v>792</v>
+        <v>647</v>
       </c>
       <c r="G12" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>793</v>
+        <v>648</v>
       </c>
       <c r="B13" t="s">
-        <v>794</v>
+        <v>649</v>
       </c>
       <c r="C13" t="s">
-        <v>790</v>
+        <v>645</v>
       </c>
       <c r="D13" t="s">
-        <v>791</v>
+        <v>646</v>
       </c>
       <c r="E13" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F13" t="s">
-        <v>795</v>
+        <v>650</v>
       </c>
       <c r="G13" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>796</v>
+        <v>651</v>
       </c>
       <c r="B14" t="s">
-        <v>797</v>
+        <v>652</v>
       </c>
       <c r="C14" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D14" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E14" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F14" t="s">
-        <v>798</v>
+        <v>653</v>
       </c>
       <c r="G14" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>799</v>
+        <v>654</v>
       </c>
       <c r="B15" t="s">
-        <v>800</v>
+        <v>655</v>
       </c>
       <c r="C15" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D15" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E15" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F15" t="s">
-        <v>801</v>
+        <v>656</v>
       </c>
       <c r="G15" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>802</v>
+        <v>657</v>
       </c>
       <c r="B16" t="s">
-        <v>803</v>
+        <v>658</v>
       </c>
       <c r="C16" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D16" t="s">
-        <v>791</v>
+        <v>646</v>
       </c>
       <c r="E16" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F16" t="s">
-        <v>804</v>
+        <v>659</v>
       </c>
       <c r="G16" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>805</v>
+        <v>660</v>
       </c>
       <c r="B17" t="s">
-        <v>806</v>
+        <v>661</v>
       </c>
       <c r="C17" t="s">
-        <v>807</v>
+        <v>662</v>
       </c>
       <c r="D17" t="s">
-        <v>791</v>
+        <v>646</v>
       </c>
       <c r="E17" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F17" t="s">
-        <v>808</v>
+        <v>663</v>
       </c>
       <c r="G17" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>809</v>
+        <v>664</v>
       </c>
       <c r="B18" t="s">
-        <v>810</v>
+        <v>665</v>
       </c>
       <c r="C18" t="s">
-        <v>790</v>
+        <v>645</v>
       </c>
       <c r="D18" t="s">
-        <v>791</v>
+        <v>646</v>
       </c>
       <c r="E18" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F18" t="s">
-        <v>811</v>
+        <v>666</v>
       </c>
       <c r="G18" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>812</v>
+        <v>667</v>
       </c>
       <c r="B19" t="s">
-        <v>813</v>
+        <v>668</v>
       </c>
       <c r="C19" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D19" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E19" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F19" t="s">
-        <v>814</v>
+        <v>669</v>
       </c>
       <c r="G19" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>815</v>
+        <v>670</v>
       </c>
       <c r="B20" t="s">
-        <v>816</v>
+        <v>671</v>
       </c>
       <c r="C20" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D20" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E20" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F20" t="s">
-        <v>817</v>
+        <v>672</v>
       </c>
       <c r="G20" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>818</v>
+        <v>673</v>
       </c>
       <c r="B21" t="s">
-        <v>819</v>
+        <v>674</v>
       </c>
       <c r="C21" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D21" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E21" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F21" t="s">
-        <v>820</v>
+        <v>675</v>
       </c>
       <c r="G21" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>821</v>
+        <v>676</v>
       </c>
       <c r="B22" t="s">
-        <v>822</v>
+        <v>677</v>
       </c>
       <c r="C22" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D22" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E22" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F22" t="s">
-        <v>823</v>
+        <v>678</v>
       </c>
       <c r="G22" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>824</v>
+        <v>679</v>
       </c>
       <c r="B23" t="s">
-        <v>825</v>
+        <v>680</v>
       </c>
       <c r="C23" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D23" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E23" t="s">
-        <v>826</v>
+        <v>681</v>
       </c>
       <c r="F23" t="s">
-        <v>827</v>
+        <v>682</v>
       </c>
       <c r="G23" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>828</v>
+        <v>683</v>
       </c>
       <c r="B24" t="s">
-        <v>829</v>
+        <v>684</v>
       </c>
       <c r="C24" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D24" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E24" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F24" t="s">
-        <v>830</v>
+        <v>685</v>
       </c>
       <c r="G24" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>831</v>
+        <v>686</v>
       </c>
       <c r="B25" t="s">
-        <v>832</v>
+        <v>687</v>
       </c>
       <c r="C25" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D25" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E25" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F25" t="s">
-        <v>833</v>
+        <v>688</v>
       </c>
       <c r="G25" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>834</v>
+        <v>689</v>
       </c>
       <c r="B26" t="s">
-        <v>835</v>
+        <v>690</v>
       </c>
       <c r="C26" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D26" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E26" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F26" t="s">
-        <v>836</v>
+        <v>691</v>
       </c>
       <c r="G26" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>837</v>
+        <v>692</v>
       </c>
       <c r="B27" t="s">
-        <v>838</v>
+        <v>693</v>
       </c>
       <c r="C27" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D27" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E27" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F27" t="s">
-        <v>839</v>
+        <v>694</v>
       </c>
       <c r="G27" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>840</v>
+        <v>695</v>
       </c>
       <c r="B28" t="s">
-        <v>841</v>
+        <v>696</v>
       </c>
       <c r="C28" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D28" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E28" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F28" t="s">
-        <v>842</v>
+        <v>697</v>
       </c>
       <c r="G28" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>843</v>
+        <v>698</v>
       </c>
       <c r="B29" t="s">
-        <v>844</v>
+        <v>699</v>
       </c>
       <c r="C29" t="s">
-        <v>845</v>
+        <v>700</v>
       </c>
       <c r="D29" t="s">
-        <v>846</v>
+        <v>701</v>
       </c>
       <c r="E29" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F29" t="s">
-        <v>847</v>
+        <v>702</v>
       </c>
       <c r="G29" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>848</v>
+        <v>703</v>
       </c>
       <c r="B30" t="s">
-        <v>849</v>
+        <v>704</v>
       </c>
       <c r="C30" t="s">
-        <v>845</v>
+        <v>700</v>
       </c>
       <c r="D30" t="s">
-        <v>850</v>
+        <v>705</v>
       </c>
       <c r="E30" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F30" t="s">
-        <v>851</v>
+        <v>706</v>
       </c>
       <c r="G30" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>852</v>
+        <v>707</v>
       </c>
       <c r="B31" t="s">
-        <v>853</v>
+        <v>708</v>
       </c>
       <c r="C31" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D31" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E31" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F31" t="s">
-        <v>854</v>
+        <v>709</v>
       </c>
       <c r="G31" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>855</v>
+        <v>710</v>
       </c>
       <c r="B32" t="s">
-        <v>856</v>
+        <v>711</v>
       </c>
       <c r="C32" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D32" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E32" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F32" t="s">
-        <v>857</v>
+        <v>712</v>
       </c>
       <c r="G32" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>858</v>
+        <v>713</v>
       </c>
       <c r="B33" t="s">
-        <v>859</v>
+        <v>714</v>
       </c>
       <c r="C33" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D33" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E33" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F33" t="s">
-        <v>860</v>
+        <v>715</v>
       </c>
       <c r="G33" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>861</v>
+        <v>716</v>
       </c>
       <c r="B34" t="s">
-        <v>862</v>
+        <v>717</v>
       </c>
       <c r="C34" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D34" t="s">
-        <v>863</v>
+        <v>718</v>
       </c>
       <c r="E34" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F34" t="s">
-        <v>864</v>
+        <v>719</v>
       </c>
       <c r="G34" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>865</v>
+        <v>720</v>
       </c>
       <c r="B35" t="s">
-        <v>866</v>
+        <v>721</v>
       </c>
       <c r="C35" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D35" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E35" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F35" t="s">
-        <v>867</v>
+        <v>722</v>
       </c>
       <c r="G35" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>868</v>
+        <v>723</v>
       </c>
       <c r="B36" t="s">
-        <v>869</v>
+        <v>724</v>
       </c>
       <c r="C36" t="s">
-        <v>870</v>
+        <v>725</v>
       </c>
       <c r="D36" t="s">
-        <v>791</v>
+        <v>646</v>
       </c>
       <c r="E36" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F36" t="s">
-        <v>871</v>
+        <v>726</v>
       </c>
       <c r="G36" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>872</v>
+        <v>727</v>
       </c>
       <c r="B37" t="s">
-        <v>873</v>
+        <v>728</v>
       </c>
       <c r="C37" t="s">
-        <v>870</v>
+        <v>725</v>
       </c>
       <c r="D37" t="s">
-        <v>791</v>
+        <v>646</v>
       </c>
       <c r="E37" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F37" t="s">
-        <v>874</v>
+        <v>729</v>
       </c>
       <c r="G37" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>875</v>
+        <v>730</v>
       </c>
       <c r="B38" t="s">
-        <v>876</v>
+        <v>731</v>
       </c>
       <c r="C38" t="s">
-        <v>870</v>
+        <v>725</v>
       </c>
       <c r="D38" t="s">
-        <v>791</v>
+        <v>646</v>
       </c>
       <c r="E38" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F38" t="s">
-        <v>877</v>
+        <v>732</v>
       </c>
       <c r="G38" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>878</v>
+        <v>733</v>
       </c>
       <c r="B39" t="s">
-        <v>879</v>
+        <v>734</v>
       </c>
       <c r="C39" t="s">
-        <v>870</v>
+        <v>725</v>
       </c>
       <c r="D39" t="s">
-        <v>791</v>
+        <v>646</v>
       </c>
       <c r="E39" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="F39" t="s">
-        <v>880</v>
+        <v>735</v>
       </c>
       <c r="G39" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Save local Commission Rule automation and testData.xlsx changes before pull
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -13,8 +13,31 @@
     <sheet name="RESTUserTest" sheetId="8" r:id="rId8"/>
     <sheet name="SOAPAccountServiceTest" sheetId="9" r:id="rId9"/>
     <sheet name="DatabaseTest" sheetId="10" r:id="rId10"/>
+    <sheet name="Commission Rules" sheetId="11" r:id="rId11"/>
   </sheets>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -616,6 +639,815 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D57"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Test Case ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Module</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Test Case Name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Scenario Type</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>TC_COM_01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Verify Commission Rules page loads successfully with all summary cards, filters, search bar, and rules list.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>TC_COM_02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Verify user can search for an existing Rule Name and the correct rule is displayed.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TC_COM_03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Verify user can filter rules using tabs (All Types, Basement, Ground, Develop) and matching records are displayed.</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TC_COM_04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Verify user can filter rules using the 'Applicable To' dropdown and only relevant rules are shown.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TC_COM_05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Verify clicking the View icon opens the selected Commission Rule details page.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TC_COM_06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Verify clicking the Edit icon opens the selected Commission Rule in edit mode.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TC_COM_07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Verify clicking the '+ Create Commission Rule' button navigates to the Create Commission Rule page.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TC_COM_08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Verify Export button successfully downloads the Commission Rules data.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TC_COM_09</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Verify searching with an invalid Rule Name displays 'No Records Found' or an empty result.</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TC_COM_10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Verify system handles special characters entered in the search field without crashing.</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TC_COM_11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Verify unauthorized users cannot access the Create Commission Rule page.</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TC_COM_12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Verify unauthorized users cannot edit an existing Commission Rule.</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TC_COM_13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Verify Export functionality displays an appropriate error message when the export service is unavailable.</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TC_COM_14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Verify clicking View for a deleted/non-existing Commission Rule displays an appropriate error message.</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TC_COM_15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Verify pagination controls are disabled or handled correctly when there is only one page of records.</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TC_COM_16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Verify expired user session redirects the user to the Login page when attempting any action (Search, View, Edit, Export, Create).</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TC_COM_17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Verify user can create a Commission Rule by entering all valid mandatory fields and clicking Save.</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TC_COM_18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Verify Rule Name field accepts valid alphanumeric values and saves successfully.</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TC_COM_19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Verify user can select Rule Type, Event Type, Applicable To, and Applied On from the dropdown lists.</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TC_COM_20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Verify Charge Code field accepts a valid charge code value.</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>TC_COM_21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Verify Commission Value (%) can be entered manually and reflected correctly in Live Preview.</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>TC_COM_22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Verify Commission Value (%) can be adjusted using the slider control.</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TC_COM_23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Verify Live Preview section updates dynamically when Rule Name is changed.</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TC_COM_24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Verify Live Preview displays correct Rule Type, Event Type, Applicable To, and Applied On values based on user selections.</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TC_COM_25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Verify clicking Cancel returns the user to the Commission Rules listing page without saving data.</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TC_COM_26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Verify newly created Commission Rule appears in the Commission Rules list after successful save.</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TC_COM_27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Verify validation message appears when Rule Name is left blank.</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>TC_COM_28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Verify validation message appears when Event Type is not selected.</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TC_COM_29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Verify validation message appears when Applicable To is not selected.</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TC_COM_30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Verify validation message appears when Applied On is not selected.</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>TC_COM_31</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Verify validation message appears when Charge Code is left blank.</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>TC_COM_32</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Verify system does not allow Commission Value below the minimum allowed percentage.</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TC_COM_33</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Verify system does not allow Commission Value above the maximum allowed percentage.</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>TC_COM_34</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Verify Rule Name field rejects special characters if they are not permitted by business rules.</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TC_COM_35</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Verify duplicate Rule Name cannot be created if uniqueness is required.</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TC_COM_36</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Verify user cannot save the Commission Rule when one or more mandatory fields are empty.</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>TC_COM_37</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Verify View Commission Rule page loads successfully with all commission rule details displayed correctly.</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>TC_COM_38</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Verify Rule Name, Rule Type, Event Type, Applicable To, Applied On, Charge Code, and Commission Percentage are displayed correctly.</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>TC_COM_39</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Verify MTD Revenue, Applied Orders, and Rate summary cards display correct values.</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>TC_COM_40</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Verify Recent Applications section displays the latest commission transactions with correct order numbers and amounts.</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>TC_COM_41</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Verify clicking the Edit Rule button navigates the user to the Edit Commission Rule screen.</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>TC_COM_42</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Verify appropriate error message is displayed when an invalid Commission Rule ID is accessed.</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>TC_COM_43</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Verify deleted or inactive Commission Rules cannot be viewed and display an appropriate error message.</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>TC_COM_44</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Verify unauthorized users cannot access the View Commission Rule page.</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>TC_COM_45</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Verify the system handles missing or null Commission Rule data without page crashes.</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>TC_COM_46</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Verify expired user sessions redirect the user to the Login page when accessing the View Commission Rule page.</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>TC_COM_47</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Verify user can successfully update the Commission Rule by modifying valid field values and clicking Update Rule.</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>TC_COM_48</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Verify changes made to Rule Name, Rule Type, Event Type, Applicable To, Applied On, Charge Code, and Commission Value are saved successfully.</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>TC_COM_49</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Verify Live Preview updates automatically when Commission Value (%) is changed.</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>TC_COM_50</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Verify user can update Commission Value using both the input field and slider control.</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>TC_COM_51</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Verify clicking Delete successfully removes the Commission Rule and redirects to the Commission Rules listing page.</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>TC_COM_52</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Verify validation message appears when Rule Name is cleared and user clicks Update Rule.</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>TC_COM_53</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Verify validation message appears when Charge Code is removed and user attempts to save.</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>TC_COM_54</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Verify system does not allow Commission Value below the minimum allowed percentage.</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>TC_COM_55</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Verify system does not allow Commission Value above the maximum allowed percentage.</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>TC_COM_56</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Commission Rules</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Verify user cannot update the Commission Rule when one or more mandatory fields are empty.</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D57"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O3"/>

</xml_diff>

<commit_message>
Add AdvertisementTest, CommissionRuleTest, and SubscriptionPlanTest to Regression sheet
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -423,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C30"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -722,9 +722,42 @@
         <v>serial</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>AdvertisementTest</v>
+      </c>
+      <c r="B28" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C28" t="str">
+        <v>serial</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>CommissionRuleTest</v>
+      </c>
+      <c r="B29" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C29" t="str">
+        <v>serial</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>SubscriptionPlanTest</v>
+      </c>
+      <c r="B30" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C30" t="str">
+        <v>serial</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C30"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update Regression sheet: add missing tests and remove duplicate BulkPromotionTest
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C45"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -811,7 +811,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>BulkPromotionTest</v>
+        <v>CustomerManagement</v>
       </c>
       <c r="B38" t="str">
         <v>YES</v>
@@ -822,7 +822,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>CustomerManagement</v>
+        <v>RoleManagementTest</v>
       </c>
       <c r="B39" t="str">
         <v>YES</v>
@@ -833,7 +833,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>RoleManagementTest</v>
+        <v>AttributeTest</v>
       </c>
       <c r="B40" t="str">
         <v>YES</v>
@@ -844,7 +844,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>AttributeTest</v>
+        <v>OrderReportTest</v>
       </c>
       <c r="B41" t="str">
         <v>YES</v>
@@ -855,7 +855,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>OrderReportTest</v>
+        <v>NotificationTemplateTest</v>
       </c>
       <c r="B42" t="str">
         <v>YES</v>
@@ -864,9 +864,42 @@
         <v>serial</v>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>AdvertisementTest</v>
+      </c>
+      <c r="B43" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C43" t="str">
+        <v>serial</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>CommissionRuleTest</v>
+      </c>
+      <c r="B44" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C44" t="str">
+        <v>serial</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>SubscriptionPlanTest</v>
+      </c>
+      <c r="B45" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C45" t="str">
+        <v>serial</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C45"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix BulkPromotion name in Regression and add missing sheets
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C49"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -737,7 +737,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>BulkPromotionTest</v>
+        <v>BulkPromotion</v>
       </c>
       <c r="B31" t="str">
         <v>YES</v>
@@ -900,9 +900,53 @@
         <v>serial</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Subscription plan</v>
+      </c>
+      <c r="B46" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C46" t="str">
+        <v>serial</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Permission</v>
+      </c>
+      <c r="B47" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C47" t="str">
+        <v>serial</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>NotificationTemplate</v>
+      </c>
+      <c r="B48" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C48" t="str">
+        <v>serial</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Subscription Plan(Super admin)</v>
+      </c>
+      <c r="B49" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C49" t="str">
+        <v>serial</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C49"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Implemented Tenants Super Admin automation
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -40,6 +40,7 @@
     <sheet name="BulkNotification" sheetId="35" r:id="rId35"/>
     <sheet name="Features(Admin)" sheetId="36" r:id="rId36"/>
     <sheet name="FeaturesSuperAdminTest" sheetId="37" r:id="rId37"/>
+    <sheet name="Tenant super admin" sheetId="38" r:id="rId38"/>
   </sheets>
 </workbook>
 </file>
@@ -18941,7 +18942,7 @@
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -19361,9 +19362,20 @@
         <v>serial</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>TenantsSuperAdminTest</v>
+      </c>
+      <c r="B39" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C39" t="str">
+        <v>serial</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C39"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -22015,6 +22027,2789 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D198"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>TC_ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Module</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Scenario</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Type</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>TC_LIST_01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Verify Tenant List page loads successfully with all tenant records displayed.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>TC_LIST_02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Verify search by ID returns the correct tenant record.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TC_LIST_03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Verify search by User Name returns matching tenant records.</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TC_LIST_04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Verify search by Email returns the correct tenant record.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TC_LIST_05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Verify clicking the View icon opens Tenant Details successfully.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TC_LIST_06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Verify clicking the Edit icon opens the Edit Tenant page with pre-filled data.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TC_LIST_07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Verify Active tenants display the Active status badge correctly.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TC_LIST_08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Verify Draft tenants display the Draft status badge correctly.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TC_LIST_09</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Verify clicking Create Tenant navigates to the Tenant Creation page.</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TC_LIST_10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Verify pagination Next button loads the next page of tenant records successfully.</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TC_LIST_NEG_01</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Verify searching with a non-existing ID displays 'No Records Found' message.</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TC_LIST_NEG_02</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Verify searching with an invalid email format does not return unrelated records.</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TC_LIST_NEG_03</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Verify search field does not accept only blank spaces as valid input.</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TC_LIST_NEG_04</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Verify special characters entered in the search field do not crash the application.</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TC_LIST_NEG_05</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Verify SQL injection strings entered in the search field are handled securely.</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TC_LIST_NEG_06</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Verify clicking Next on the last page does not navigate beyond available pages.</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TC_LIST_NEG_07</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Verify clicking Previous on the first page does not navigate to an invalid page.</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TC_LIST_NEG_08</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Verify Tenant List page handles empty tenant data without UI breakage.</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TC_LIST_NEG_09</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Verify clicking View/Edit for a deleted tenant displays an appropriate error message.</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TC_LIST_NEG_10</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Verify refresh action during network interruption does not display duplicate or corrupted tenant data.</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>TC_VIEW_01</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Verify Tenant View page loads successfully with all tenant details displayed.</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>TC_VIEW_02</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Verify tenant logo/image is displayed correctly.</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TC_VIEW_03</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Verify tenant name is displayed accurately.</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TC_VIEW_04</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Verify tenant email is displayed correctly.</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TC_VIEW_05</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Verify tenant phone number is displayed correctly.</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TC_VIEW_06</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Verify Country field displays the correct country value.</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TC_VIEW_07</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Verify State field displays the correct state value.</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>TC_VIEW_08</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Verify City field displays the correct city value.</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TC_VIEW_09</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Verify Zipcode field displays the correct postal code.</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TC_VIEW_10</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Verify User Name field displays the correct tenant username.</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>TC_VIEW_11</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Verify Category field displays the correct tenant category.</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>TC_VIEW_12</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Verify clicking the Back button navigates to the Tenant List page successfully.</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TC_VIEW_NEG_01</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Verify page displays a proper message when tenant details are unavailable.</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>TC_VIEW_NEG_02</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Verify missing tenant logo displays a default placeholder image.</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TC_VIEW_NEG_03</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Verify invalid or deleted tenant ID does not load the View Tenant page.</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TC_VIEW_NEG_04</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Verify page handles null email values without UI breakage.</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>TC_VIEW_NEG_05</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Verify page handles null phone number values without UI breakage.</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>TC_VIEW_NEG_06</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Verify page handles missing address information gracefully.</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>TC_VIEW_NEG_07</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Verify invalid zipcode data is displayed correctly without application failure.</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>TC_VIEW_NEG_08</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Verify excessively long tenant names do not break the page layout.</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>TC_VIEW_NEG_09</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Verify special characters in address fields are displayed correctly.</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>TC_VIEW_NEG_10</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Verify KYC Details button is disabled or shows an error when KYC data is unavailable.</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>TC_VIEW_NEG_11</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Verify unauthorized users cannot access the Tenant View page directly via URL.</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>TC_VIEW_NEG_12</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Verify page handles network/API failure during data loading without crashing.</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>TC_EDIT_01</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Verify user can successfully update tenant details with valid data in all fields.</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>TC_EDIT_02</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Verify Company Name field accepts valid alphanumeric values and updates successfully.</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>TC_EDIT_03</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Verify user can upload a valid company logo image (JPG/PNG) and save changes.</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>TC_EDIT_04</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Verify Google Address search populates Country, State, City, and Zipcode correctly.</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>TC_EDIT_05</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Verify Country field updates successfully with a valid country value.</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>TC_EDIT_06</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Verify State field updates successfully with a valid state value.</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>TC_EDIT_07</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Verify City field updates successfully with a valid city value.</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>TC_EDIT_08</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Verify Zipcode field accepts a valid postal code and saves successfully.</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>TC_EDIT_09</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Verify Street 1 and Street 2 fields accept valid address information.</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>TC_EDIT_10</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Verify Email field accepts a valid email address and updates successfully.</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>TC_EDIT_11</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Verify Phone Number field accepts a valid international phone number and updates successfully.</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>TC_EDIT_12</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Verify User Name field accepts valid input and updates successfully.</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>TC_EDIT_13</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Verify Password field accepts a valid password meeting system requirements.</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>TC_EDIT_14</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Verify KYC Details button opens the tenant KYC information page successfully.</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>TC_EDIT_15</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Verify clicking Update saves all modified tenant details and displays a success message.</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>TC_EDIT_NEG_01</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Verify update fails when Company Name is left blank.</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>TC_EDIT_NEG_02</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Verify Company Name field does not accept only spaces.</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>TC_EDIT_NEG_03</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Verify upload of unsupported logo file formats (.exe, .txt, .zip) is rejected.</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>TC_EDIT_NEG_04</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Verify oversized logo files are not uploaded and an error message is displayed.</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>TC_EDIT_NEG_05</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Verify update fails when Email field contains an invalid email format.</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>TC_EDIT_NEG_06</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Verify duplicate email address cannot be used if uniqueness is enforced.</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>TC_EDIT_NEG_07</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Verify Phone Number field rejects alphabetic characters.</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>TC_EDIT_NEG_08</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Verify Phone Number field rejects special characters other than allowed symbols.</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>TC_EDIT_NEG_09</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Verify update fails when Phone Number exceeds the maximum allowed length.</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>TC_EDIT_NEG_10</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Verify Zipcode field rejects invalid formats or non-numeric values if numeric-only.</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>TC_EDIT_NEG_11</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Verify Password field rejects values that do not meet password policy requirements.</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>TC_EDIT_NEG_12</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Verify SQL Injection strings entered in text fields are handled securely.</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>TC_EDIT_NEG_13</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Verify Cross-Site Scripting (XSS) scripts entered in input fields are sanitized.</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>TC_EDIT_NEG_14</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Verify clicking Update with mandatory fields missing displays validation messages.</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>TC_EDIT_NEG_15</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Verify application handles network/API failure during update without data corruption.</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>TC_CREATE_BASIC_01</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Verify user can enter a valid Company Name and proceed to the Authentication step.</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>TC_CREATE_BASIC_02</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Verify user can enter valid First Name and Last Name values successfully.</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>TC_CREATE_BASIC_03</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Verify user can upload a valid company logo image (JPG/PNG) successfully.</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>TC_CREATE_BASIC_04</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Verify uploaded logo preview is displayed correctly in the Company Logo section.</v>
+      </c>
+      <c r="D79" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>TC_CREATE_BASIC_05</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Verify Google Address search populates Country, State, City, Zipcode, and Coordinates correctly.</v>
+      </c>
+      <c r="D80" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>TC_CREATE_BASIC_06</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Verify Country field accepts and displays a valid country value.</v>
+      </c>
+      <c r="D81" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>TC_CREATE_BASIC_07</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Verify State field accepts and displays a valid state value.</v>
+      </c>
+      <c r="D82" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>TC_CREATE_BASIC_08</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Verify City field accepts and displays a valid city value.</v>
+      </c>
+      <c r="D83" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>TC_CREATE_BASIC_09</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Verify Zipcode field accepts a valid postal code.</v>
+      </c>
+      <c r="D84" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>TC_CREATE_BASIC_10</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Verify Street 1 field accepts a valid address value.</v>
+      </c>
+      <c r="D85" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>TC_CREATE_BASIC_11</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Verify Street 2 field accepts an optional address value.</v>
+      </c>
+      <c r="D86" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>TC_CREATE_BASIC_12</v>
+      </c>
+      <c r="B87" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C87" t="str">
+        <v>Verify Resolved Coordinates are populated correctly after selecting an address.</v>
+      </c>
+      <c r="D87" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>TC_CREATE_BASIC_13</v>
+      </c>
+      <c r="B88" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Verify clicking Continue to Authentication navigates to the Authentication step when all required fields are valid.</v>
+      </c>
+      <c r="D88" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>TC_CREATE_BASIC_14</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C89" t="str">
+        <v>Verify clicking Cancel navigates back without application errors.</v>
+      </c>
+      <c r="D89" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>TC_CREATE_BASIC_15</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Verify all entered data is retained when moving from Basic Info to Authentication step.</v>
+      </c>
+      <c r="D90" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>TC_CREATE_BASIC_NEG_01</v>
+      </c>
+      <c r="B91" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C91" t="str">
+        <v>Verify user cannot proceed when Company Name is left blank.</v>
+      </c>
+      <c r="D91" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>TC_CREATE_BASIC_NEG_02</v>
+      </c>
+      <c r="B92" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C92" t="str">
+        <v>Verify user cannot proceed when First Name is left blank.</v>
+      </c>
+      <c r="D92" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>TC_CREATE_BASIC_NEG_03</v>
+      </c>
+      <c r="B93" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C93" t="str">
+        <v>Verify user cannot proceed when Last Name is left blank.</v>
+      </c>
+      <c r="D93" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>TC_CREATE_BASIC_NEG_04</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C94" t="str">
+        <v>Verify Company Name field does not accept only blank spaces.</v>
+      </c>
+      <c r="D94" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>TC_CREATE_BASIC_NEG_05</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C95" t="str">
+        <v>Verify First Name field rejects numeric-only values.</v>
+      </c>
+      <c r="D95" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>TC_CREATE_BASIC_NEG_06</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C96" t="str">
+        <v>Verify Last Name field rejects special characters if validation is enforced.</v>
+      </c>
+      <c r="D96" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>TC_CREATE_BASIC_NEG_07</v>
+      </c>
+      <c r="B97" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Verify upload of unsupported file types (.exe, .txt, .zip) is rejected.</v>
+      </c>
+      <c r="D97" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>TC_CREATE_BASIC_NEG_08</v>
+      </c>
+      <c r="B98" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Verify oversized logo files are not uploaded and an error message is displayed.</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>TC_CREATE_BASIC_NEG_09</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C99" t="str">
+        <v>Verify corrupted image files cannot be uploaded.</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>TC_CREATE_BASIC_NEG_10</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Verify invalid or non-existent address entered in Google Search does not populate address fields incorrectly.</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>TC_CREATE_BASIC_NEG_11</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Verify Zipcode field rejects alphabetic characters if numeric-only validation exists.</v>
+      </c>
+      <c r="D101" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>TC_CREATE_BASIC_NEG_12</v>
+      </c>
+      <c r="B102" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Verify SQL Injection strings entered in text fields are handled securely.</v>
+      </c>
+      <c r="D102" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>TC_CREATE_BASIC_NEG_13</v>
+      </c>
+      <c r="B103" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Verify XSS scripts entered in input fields are sanitized and not executed.</v>
+      </c>
+      <c r="D103" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>TC_CREATE_BASIC_NEG_14</v>
+      </c>
+      <c r="B104" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Verify clicking Continue to Authentication with mandatory fields missing displays validation messages.</v>
+      </c>
+      <c r="D104" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>TC_CREATE_BASIC_NEG_15</v>
+      </c>
+      <c r="B105" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Verify application handles network/API failure during address lookup without crashing.</v>
+      </c>
+      <c r="D105" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>TC_CREATE_AUTH_01</v>
+      </c>
+      <c r="B106" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Verify user can enter a valid Email, Phone Number, and Username and proceed to the Business Plan step.</v>
+      </c>
+      <c r="D106" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>TC_CREATE_AUTH_02</v>
+      </c>
+      <c r="B107" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C107" t="str">
+        <v>Verify a valid email address format is accepted successfully.</v>
+      </c>
+      <c r="D107" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>TC_CREATE_AUTH_03</v>
+      </c>
+      <c r="B108" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C108" t="str">
+        <v>Verify a valid phone number with the selected country code is accepted.</v>
+      </c>
+      <c r="D108" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>TC_CREATE_AUTH_04</v>
+      </c>
+      <c r="B109" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C109" t="str">
+        <v>Verify a unique username is accepted and saved successfully.</v>
+      </c>
+      <c r="D109" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>TC_CREATE_AUTH_05</v>
+      </c>
+      <c r="B110" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C110" t="str">
+        <v>Verify clicking Continue to Business Plan navigates to the next step when all required fields are valid.</v>
+      </c>
+      <c r="D110" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>TC_CREATE_AUTH_06</v>
+      </c>
+      <c r="B111" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C111" t="str">
+        <v>Verify clicking Go back to Basic Info navigates to the Basic Info step while retaining entered Authentication data.</v>
+      </c>
+      <c r="D111" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>TC_CREATE_AUTH_NEG_01</v>
+      </c>
+      <c r="B112" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C112" t="str">
+        <v>Verify user cannot proceed when the Email field is left blank.</v>
+      </c>
+      <c r="D112" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>TC_CREATE_AUTH_NEG_02</v>
+      </c>
+      <c r="B113" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C113" t="str">
+        <v>Verify user cannot proceed when the Phone Number field is left blank.</v>
+      </c>
+      <c r="D113" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>TC_CREATE_AUTH_NEG_03</v>
+      </c>
+      <c r="B114" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C114" t="str">
+        <v>Verify user cannot proceed when the Username field is left blank.</v>
+      </c>
+      <c r="D114" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>TC_CREATE_AUTH_NEG_04</v>
+      </c>
+      <c r="B115" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C115" t="str">
+        <v>Verify invalid email formats (e.g., user@, test.com) are rejected with a validation message.</v>
+      </c>
+      <c r="D115" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>TC_CREATE_AUTH_NEG_05</v>
+      </c>
+      <c r="B116" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C116" t="str">
+        <v>Verify phone number field rejects alphabetic and special characters.</v>
+      </c>
+      <c r="D116" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>TC_CREATE_AUTH_NEG_06</v>
+      </c>
+      <c r="B117" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C117" t="str">
+        <v>Verify duplicate/existing username is not accepted and displays an appropriate error message.</v>
+      </c>
+      <c r="D117" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>TC_CREATE_PLAN_01</v>
+      </c>
+      <c r="B118" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C118" t="str">
+        <v>Verify user can select a valid Business Plan and the selection is displayed correctly.</v>
+      </c>
+      <c r="D118" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>TC_CREATE_PLAN_02</v>
+      </c>
+      <c r="B119" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C119" t="str">
+        <v>Verify user can upload a valid Agreement file (PDF/DOC) successfully.</v>
+      </c>
+      <c r="D119" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>TC_CREATE_PLAN_03</v>
+      </c>
+      <c r="B120" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C120" t="str">
+        <v>Verify user can select a valid From Date using the date picker.</v>
+      </c>
+      <c r="D120" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>TC_CREATE_PLAN_04</v>
+      </c>
+      <c r="B121" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C121" t="str">
+        <v>Verify user can select a valid To Date greater than the From Date.</v>
+      </c>
+      <c r="D121" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>TC_CREATE_PLAN_05</v>
+      </c>
+      <c r="B122" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C122" t="str">
+        <v>Verify user can select one or more Domains from the Domain dropdown.</v>
+      </c>
+      <c r="D122" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>TC_CREATE_PLAN_06</v>
+      </c>
+      <c r="B123" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C123" t="str">
+        <v>Verify user can enable the Select Market checkbox and save successfully.</v>
+      </c>
+      <c r="D123" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>TC_CREATE_PLAN_07</v>
+      </c>
+      <c r="B124" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C124" t="str">
+        <v>Verify user can enable the Enable Manufacturer checkbox and save successfully.</v>
+      </c>
+      <c r="D124" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>TC_CREATE_PLAN_08</v>
+      </c>
+      <c r="B125" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C125" t="str">
+        <v>Verify user can select a valid Payment Gateway (COD/CASHFREE/PAYTM).</v>
+      </c>
+      <c r="D125" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>TC_CREATE_PLAN_09</v>
+      </c>
+      <c r="B126" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C126" t="str">
+        <v>Verify user can select multiple required fields and successfully create a tenant.</v>
+      </c>
+      <c r="D126" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>TC_CREATE_PLAN_10</v>
+      </c>
+      <c r="B127" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C127" t="str">
+        <v>Verify clicking Create Tenant with all mandatory fields completed creates the tenant successfully.</v>
+      </c>
+      <c r="D127" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>TC_CREATE_PLAN_NEG_01</v>
+      </c>
+      <c r="B128" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C128" t="str">
+        <v>Verify tenant creation is blocked when no Business Plan is selected.</v>
+      </c>
+      <c r="D128" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>TC_CREATE_PLAN_NEG_02</v>
+      </c>
+      <c r="B129" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C129" t="str">
+        <v>Verify tenant creation is blocked when the Agreement file is not uploaded.</v>
+      </c>
+      <c r="D129" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>TC_CREATE_PLAN_NEG_03</v>
+      </c>
+      <c r="B130" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C130" t="str">
+        <v>Verify tenant creation is blocked when the From Date field is left empty.</v>
+      </c>
+      <c r="D130" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>TC_CREATE_PLAN_NEG_04</v>
+      </c>
+      <c r="B131" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C131" t="str">
+        <v>Verify tenant creation is blocked when the To Date field is left empty.</v>
+      </c>
+      <c r="D131" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>TC_CREATE_PLAN_NEG_05</v>
+      </c>
+      <c r="B132" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C132" t="str">
+        <v>Verify validation is displayed when To Date is earlier than From Date.</v>
+      </c>
+      <c r="D132" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>TC_CREATE_PLAN_NEG_06</v>
+      </c>
+      <c r="B133" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C133" t="str">
+        <v>Verify tenant creation is blocked when no Domain is selected.</v>
+      </c>
+      <c r="D133" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>TC_CREATE_PLAN_NEG_07</v>
+      </c>
+      <c r="B134" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C134" t="str">
+        <v>Verify tenant creation is blocked when no Payment Gateway is selected.</v>
+      </c>
+      <c r="D134" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>TC_CREATE_PLAN_NEG_08</v>
+      </c>
+      <c r="B135" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C135" t="str">
+        <v>Verify invalid file formats (.exe, .bat, .zip) are rejected during Agreement file upload.</v>
+      </c>
+      <c r="D135" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>TC_CREATE_PLAN_NEG_09</v>
+      </c>
+      <c r="B136" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C136" t="str">
+        <v>Verify oversized Agreement files exceeding the allowed limit are rejected.</v>
+      </c>
+      <c r="D136" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>TC_CREATE_PLAN_NEG_10</v>
+      </c>
+      <c r="B137" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C137" t="str">
+        <v>Verify clicking Create Tenant with multiple mandatory fields empty displays all required validation messages.</v>
+      </c>
+      <c r="D137" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>TC_CONFIRM_01</v>
+      </c>
+      <c r="B138" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C138" t="str">
+        <v>Verify clicking CREATE on the confirmation popup successfully creates the tenant and redirects to the success page/list.</v>
+      </c>
+      <c r="D138" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>TC_CONFIRM_02</v>
+      </c>
+      <c r="B139" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C139" t="str">
+        <v>Verify the confirmation popup is displayed after clicking Create Tenant with all mandatory fields completed.</v>
+      </c>
+      <c r="D139" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>TC_CONFIRM_03</v>
+      </c>
+      <c r="B140" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C140" t="str">
+        <v>Verify the selected Business Plan, Domain, Market, and Payment Gateway are retained correctly in the creation request.</v>
+      </c>
+      <c r="D140" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>TC_CONFIRM_04</v>
+      </c>
+      <c r="B141" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C141" t="str">
+        <v>Verify clicking DISCARD closes the confirmation popup and no tenant record is created.</v>
+      </c>
+      <c r="D141" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>TC_CONFIRM_NEG_01</v>
+      </c>
+      <c r="B142" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C142" t="str">
+        <v>Verify tenant creation is not performed when the user clicks DISCARD on the confirmation popup.</v>
+      </c>
+      <c r="D142" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>TC_CONFIRM_NEG_02</v>
+      </c>
+      <c r="B143" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C143" t="str">
+        <v>Verify clicking CREATE fails with an appropriate error message if the backend API returns an error response.</v>
+      </c>
+      <c r="D143" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>TC_CONFIRM_NEG_03</v>
+      </c>
+      <c r="B144" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C144" t="str">
+        <v>Verify duplicate tenant creation is prevented when the CREATE button is clicked multiple times rapidly.</v>
+      </c>
+      <c r="D144" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>TC_CONFIRM_NEG_04</v>
+      </c>
+      <c r="B145" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C145" t="str">
+        <v>Verify the confirmation popup is not displayed if any mandatory Business Plan fields are missing before submission.</v>
+      </c>
+      <c r="D145" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>TC_SUCCESS_01</v>
+      </c>
+      <c r="B146" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C146" t="str">
+        <v>Verify the success popup is displayed with the message 'Tenant created successfully' after successful tenant creation.</v>
+      </c>
+      <c r="D146" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>TC_SUCCESS_02</v>
+      </c>
+      <c r="B147" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C147" t="str">
+        <v>Verify clicking the OK button on the success popup closes the popup and redirects to the Tenant List page.</v>
+      </c>
+      <c r="D147" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>TC_SUCCESS_03</v>
+      </c>
+      <c r="B148" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C148" t="str">
+        <v>Verify the newly created tenant appears in the Tenant List with the correct details after clicking OK.</v>
+      </c>
+      <c r="D148" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>TC_SUCCESS_04</v>
+      </c>
+      <c r="B149" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C149" t="str">
+        <v>Verify only one success popup is displayed even if the Create Tenant button was clicked multiple times before completion.</v>
+      </c>
+      <c r="D149" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>TC_SUCCESS_NEG_01</v>
+      </c>
+      <c r="B150" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C150" t="str">
+        <v>Verify the success popup is not displayed when tenant creation fails due to a backend/API error.</v>
+      </c>
+      <c r="D150" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>TC_SUCCESS_NEG_02</v>
+      </c>
+      <c r="B151" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C151" t="str">
+        <v>Verify the success popup is not displayed if mandatory fields were bypassed and invalid data is submitted.</v>
+      </c>
+      <c r="D151" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>TC_SUCCESS_NEG_03</v>
+      </c>
+      <c r="B152" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C152" t="str">
+        <v>Verify clicking outside the success popup does not close it if the popup is configured as a mandatory acknowledgment dialog.</v>
+      </c>
+      <c r="D152" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>TC_SUCCESS_NEG_04</v>
+      </c>
+      <c r="B153" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C153" t="str">
+        <v>Verify duplicate tenant records are not created when the user refreshes the page immediately after the success popup appears.</v>
+      </c>
+      <c r="D153" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>TC_THEME_01</v>
+      </c>
+      <c r="B154" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C154" t="str">
+        <v>Verify user can enter a valid unique Sub-domain and proceed to the KYC step successfully.</v>
+      </c>
+      <c r="D154" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>TC_THEME_02</v>
+      </c>
+      <c r="B155" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C155" t="str">
+        <v>Verify user can select a valid Brand Color using the color picker and the selected color is saved.</v>
+      </c>
+      <c r="D155" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>TC_THEME_03</v>
+      </c>
+      <c r="B156" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C156" t="str">
+        <v>Verify user can select a valid Primary Dark color and the value is stored correctly.</v>
+      </c>
+      <c r="D156" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>TC_THEME_04</v>
+      </c>
+      <c r="B157" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C157" t="str">
+        <v>Verify user can select a valid Primary Light color and the value is stored correctly.</v>
+      </c>
+      <c r="D157" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>TC_THEME_05</v>
+      </c>
+      <c r="B158" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C158" t="str">
+        <v>Verify user can enter a valid Font Color (Hex Code) and proceed successfully.</v>
+      </c>
+      <c r="D158" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>TC_THEME_06</v>
+      </c>
+      <c r="B159" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C159" t="str">
+        <v>Verify user can select a font family (e.g., Verdana, Arial, Helvetica) from the dropdown.</v>
+      </c>
+      <c r="D159" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>TC_THEME_07</v>
+      </c>
+      <c r="B160" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C160" t="str">
+        <v>Verify clicking Continue to KYC with all mandatory Theme fields completed navigates to the KYC screen.</v>
+      </c>
+      <c r="D160" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="str">
+        <v>TC_THEME_08</v>
+      </c>
+      <c r="B161" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C161" t="str">
+        <v>Verify clicking Draft &amp; Quit saves the tenant as a draft and exits the wizard.</v>
+      </c>
+      <c r="D161" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>TC_THEME_09</v>
+      </c>
+      <c r="B162" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C162" t="str">
+        <v>Verify previously entered Theme data is retained when navigating back and returning to the Theme screen.</v>
+      </c>
+      <c r="D162" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>TC_THEME_NEG_01</v>
+      </c>
+      <c r="B163" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C163" t="str">
+        <v>Verify validation is displayed when the Sub-domain field is left blank.</v>
+      </c>
+      <c r="D163" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>TC_THEME_NEG_02</v>
+      </c>
+      <c r="B164" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C164" t="str">
+        <v>Verify user cannot proceed when an already existing Sub-domain is entered.</v>
+      </c>
+      <c r="D164" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>TC_THEME_NEG_03</v>
+      </c>
+      <c r="B165" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C165" t="str">
+        <v>Verify validation is displayed when an invalid Sub-domain format is entered (special characters/spaces).</v>
+      </c>
+      <c r="D165" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>TC_THEME_NEG_04</v>
+      </c>
+      <c r="B166" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C166" t="str">
+        <v>Verify user cannot proceed when the Brand Color field is empty.</v>
+      </c>
+      <c r="D166" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>TC_THEME_NEG_05</v>
+      </c>
+      <c r="B167" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C167" t="str">
+        <v>Verify user cannot proceed when the Primary Dark color field is empty.</v>
+      </c>
+      <c r="D167" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="str">
+        <v>TC_THEME_NEG_06</v>
+      </c>
+      <c r="B168" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C168" t="str">
+        <v>Verify user cannot proceed when the Font Family is not selected.</v>
+      </c>
+      <c r="D168" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="str">
+        <v>TC_THEME_NEG_07</v>
+      </c>
+      <c r="B169" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C169" t="str">
+        <v>Verify validation is displayed when an invalid Font Color value (e.g., #ZZZZZZ) is entered.</v>
+      </c>
+      <c r="D169" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="str">
+        <v>TC_THEME_NEG_08</v>
+      </c>
+      <c r="B170" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C170" t="str">
+        <v>Verify clicking Continue to KYC with one or more mandatory Theme fields missing prevents navigation and displays error messages.</v>
+      </c>
+      <c r="D170" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="str">
+        <v>TC_KYC_01</v>
+      </c>
+      <c r="B171" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C171" t="str">
+        <v>Verify user can select a valid ID Proof document type and proceed successfully.</v>
+      </c>
+      <c r="D171" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="str">
+        <v>TC_KYC_02</v>
+      </c>
+      <c r="B172" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C172" t="str">
+        <v>Verify user can enter a valid ID Number and the value is accepted.</v>
+      </c>
+      <c r="D172" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>TC_KYC_03</v>
+      </c>
+      <c r="B173" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C173" t="str">
+        <v>Verify user can upload a valid Front Side image for ID Proof successfully.</v>
+      </c>
+      <c r="D173" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>TC_KYC_04</v>
+      </c>
+      <c r="B174" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C174" t="str">
+        <v>Verify user can upload a valid Back Side image for ID Proof successfully.</v>
+      </c>
+      <c r="D174" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>TC_KYC_05</v>
+      </c>
+      <c r="B175" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C175" t="str">
+        <v>Verify user can select a valid Address Proof document type successfully.</v>
+      </c>
+      <c r="D175" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>TC_KYC_06</v>
+      </c>
+      <c r="B176" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C176" t="str">
+        <v>Verify user can enter a valid Address Number and the value is accepted.</v>
+      </c>
+      <c r="D176" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>TC_KYC_07</v>
+      </c>
+      <c r="B177" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C177" t="str">
+        <v>Verify user can upload valid Front Side and Back Side images for Address Proof successfully.</v>
+      </c>
+      <c r="D177" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>TC_KYC_08</v>
+      </c>
+      <c r="B178" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C178" t="str">
+        <v>Verify clicking Draft &amp; Approve Later saves the KYC details in draft status successfully.</v>
+      </c>
+      <c r="D178" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>TC_KYC_09</v>
+      </c>
+      <c r="B179" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C179" t="str">
+        <v>Verify clicking Approve &amp; Send Verification Mail with all mandatory fields completed submits KYC successfully.</v>
+      </c>
+      <c r="D179" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>TC_KYC_10</v>
+      </c>
+      <c r="B180" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C180" t="str">
+        <v>Verify a verification email is sent successfully after clicking Approve &amp; Send Verification Mail.</v>
+      </c>
+      <c r="D180" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>TC_KYC_NEG_01</v>
+      </c>
+      <c r="B181" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C181" t="str">
+        <v>Verify validation is displayed when ID Proof Document Type is not selected.</v>
+      </c>
+      <c r="D181" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>TC_KYC_NEG_02</v>
+      </c>
+      <c r="B182" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C182" t="str">
+        <v>Verify validation is displayed when ID Number is left blank.</v>
+      </c>
+      <c r="D182" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>TC_KYC_NEG_03</v>
+      </c>
+      <c r="B183" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C183" t="str">
+        <v>Verify validation is displayed when ID Proof Front Side document is not uploaded.</v>
+      </c>
+      <c r="D183" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>TC_KYC_NEG_04</v>
+      </c>
+      <c r="B184" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C184" t="str">
+        <v>Verify validation is displayed when ID Proof Back Side document is not uploaded.</v>
+      </c>
+      <c r="D184" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>TC_KYC_NEG_05</v>
+      </c>
+      <c r="B185" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C185" t="str">
+        <v>Verify validation is displayed when Address Proof Document Type is not selected.</v>
+      </c>
+      <c r="D185" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>TC_KYC_NEG_06</v>
+      </c>
+      <c r="B186" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C186" t="str">
+        <v>Verify validation is displayed when Address Number is left blank.</v>
+      </c>
+      <c r="D186" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>TC_KYC_NEG_07</v>
+      </c>
+      <c r="B187" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C187" t="str">
+        <v>Verify validation is displayed when Address Proof Front Side document is not uploaded.</v>
+      </c>
+      <c r="D187" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>TC_KYC_NEG_08</v>
+      </c>
+      <c r="B188" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C188" t="str">
+        <v>Verify validation is displayed when Address Proof Back Side document is not uploaded.</v>
+      </c>
+      <c r="D188" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v>TC_KYC_NEG_09</v>
+      </c>
+      <c r="B189" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C189" t="str">
+        <v>Verify unsupported file formats (e.g., .exe, .bat, .zip) are rejected during document upload.</v>
+      </c>
+      <c r="D189" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="str">
+        <v>TC_KYC_NEG_10</v>
+      </c>
+      <c r="B190" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C190" t="str">
+        <v>Verify oversized document files exceeding the allowed limit are rejected with an appropriate error message.</v>
+      </c>
+      <c r="D190" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>TC_KYC_APP_01</v>
+      </c>
+      <c r="B191" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C191" t="str">
+        <v>Verify clicking APPROVE successfully approves the tenant KYC and displays a success message.</v>
+      </c>
+      <c r="D191" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>TC_KYC_APP_02</v>
+      </c>
+      <c r="B192" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C192" t="str">
+        <v>Verify clicking CANCEL closes the KYC approval popup without approving the KYC.</v>
+      </c>
+      <c r="D192" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>TC_KYC_APP_03</v>
+      </c>
+      <c r="B193" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C193" t="str">
+        <v>Verify the Approve KYC confirmation popup appears when the user clicks Approve &amp; Send Verification Mail.</v>
+      </c>
+      <c r="D193" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>TC_KYC_APP_04</v>
+      </c>
+      <c r="B194" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C194" t="str">
+        <v>Verify KYC status is updated to Approved after successful approval.</v>
+      </c>
+      <c r="D194" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>TC_KYC_APP_NEG_01</v>
+      </c>
+      <c r="B195" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C195" t="str">
+        <v>Verify KYC approval is blocked when mandatory KYC details are missing.</v>
+      </c>
+      <c r="D195" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>TC_KYC_APP_NEG_02</v>
+      </c>
+      <c r="B196" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C196" t="str">
+        <v>Verify KYC approval fails when invalid or corrupted documents are uploaded.</v>
+      </c>
+      <c r="D196" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>TC_KYC_APP_NEG_03</v>
+      </c>
+      <c r="B197" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C197" t="str">
+        <v>Verify an error message is displayed when the KYC approval API returns a failure response.</v>
+      </c>
+      <c r="D197" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>TC_KYC_APP_NEG_04</v>
+      </c>
+      <c r="B198" t="str">
+        <v>Tenant super admin</v>
+      </c>
+      <c r="C198" t="str">
+        <v>Verify multiple rapid clicks on APPROVE do not create duplicate KYC approvals.</v>
+      </c>
+      <c r="D198" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D198"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K4"/>

</xml_diff>

<commit_message>
Added Partner Tenant automation test cases
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -41,6 +41,7 @@
     <sheet name="Features(Admin)" sheetId="36" r:id="rId36"/>
     <sheet name="FeaturesSuperAdminTest" sheetId="37" r:id="rId37"/>
     <sheet name="Tenant super admin" sheetId="38" r:id="rId38"/>
+    <sheet name="Partner (Tenant)" sheetId="39" r:id="rId39"/>
   </sheets>
 </workbook>
 </file>
@@ -18942,7 +18943,7 @@
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -19373,9 +19374,20 @@
         <v>serial</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>PartnerTest</v>
+      </c>
+      <c r="B40" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C40" t="str">
+        <v>serial</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C40"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -24810,6 +24822,1263 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D89"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>TC_ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Module</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Scenario</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Type</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>TC_LIST_01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Verify the Partners page loads successfully with dashboard metrics, partner filters, search box, and partner list.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>TC_LIST_02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Verify user can filter partners by Seller and only Seller-type partners are displayed.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TC_LIST_03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Verify user can search a partner using a valid Name, Email, or Phone Number and view matching results.</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TC_LIST_04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Verify clicking the View icon opens the selected partner's details page successfully.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TC_LIST_05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Verify clicking the Create Partner button navigates the user to the partner creation screen.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TC_LIST_06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Verify dashboard counts (Total Partners, Sellers, New This Month, Total Orders) are displayed correctly.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TC_LIST_NEG_01</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Verify searching with a non-existing partner name/email/phone displays a "No Records Found" message.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TC_LIST_NEG_02</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Verify search field handles special characters and invalid inputs without application failure.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TC_LIST_NEG_03</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Verify the page displays an appropriate error message when partner data fails to load due to API/network issues.</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TC_LIST_NEG_04</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Verify clicking the View icon for a deleted or inaccessible partner displays an appropriate error message.</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TC_LIST_NEG_05</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Verify partner type filters display an empty state message when no records exist for the selected type.</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TC_LIST_NEG_06</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Verify rapid multiple clicks on filter tabs or action buttons do not cause duplicate requests or UI issues.</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TC_VIEW_01</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Verify the Partner Details page loads successfully with all partner information displayed correctly.</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TC_VIEW_02</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Verify clicking the Back button navigates the user back to the Partners listing page.</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TC_VIEW_03</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Verify partner profile information (Logo, Name, Email, Phone) is displayed correctly in the left panel.</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TC_VIEW_04</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Verify clicking the Edit button in the Organization Info section opens the edit form with pre-populated data.</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TC_VIEW_05</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Verify clicking the Manage Account button opens the partner account management screen successfully.</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TC_VIEW_06</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Verify user can navigate between all left-menu sections (Subscription, Payments, Orders, Invoices, Users, etc.) successfully.</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TC_VIEW_07</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Verify all information sections (Organization Info, Office, Billing Info, Agreement, Credentials, Additional Info) display correct data.</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TC_VIEW_08</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Verify individual Edit buttons open the corresponding section for modification without affecting other sections.</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>TC_VIEW_NEG_01</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Verify an appropriate error message is displayed when partner details fail to load due to API/network failure.</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>TC_VIEW_NEG_02</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Verify the page handles missing partner profile image by displaying a default placeholder image.</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TC_VIEW_NEG_03</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Verify clicking Edit without sufficient permissions displays an authorization error.</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TC_VIEW_NEG_04</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Verify navigation to a non-existent partner record displays a "Partner Not Found" message.</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TC_VIEW_NEG_05</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Verify sections with missing data (e.g., Agreement, Additional Info) display appropriate empty-state messages instead of blank screens.</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TC_VIEW_NEG_06</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Verify clicking Manage Account for an inactive or disabled partner displays an appropriate validation message.</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TC_VIEW_NEG_07</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Verify rapid multiple clicks on Edit buttons do not open duplicate forms or create UI inconsistencies.</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>TC_VIEW_NEG_08</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Verify the page handles invalid or corrupted partner data without breaking the layout or displaying incorrect information.</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TC_DEL_01</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Verify clicking Delete successfully removes the selected partner and updates the partner list.</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TC_DEL_02</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Verify clicking Cancel closes the delete confirmation popup without deleting the partner.</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>TC_DEL_03</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Verify clicking the X (Close) icon dismisses the popup and retains the partner record.</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>TC_DEL_04</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Verify the delete confirmation popup displays correctly with warning message, Cancel button, and Delete button.</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TC_DEL_NEG_01</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Verify an appropriate error message is displayed when partner deletion fails due to API/network failure.</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>TC_DEL_NEG_02</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Verify a user without delete permissions cannot delete a partner and receives an authorization error.</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TC_DEL_NEG_03</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Verify multiple rapid clicks on the Delete button do not trigger duplicate delete requests.</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TC_DEL_NEG_04</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Verify attempting to delete a partner associated with active orders, subscriptions, or transactions displays a validation error and prevents deletion.</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>TC_CR_OFF_01</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Verify user can enter valid Office details and successfully proceed to the next step by clicking Next.</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>TC_CR_OFF_02</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Verify user can add a valid email address and it is saved successfully.</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>TC_CR_OFF_03</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Verify user can enter a valid phone number with country code and proceed successfully.</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>TC_CR_OFF_04</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Verify selecting a valid partner type (e.g., Seller) saves the selection correctly.</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>TC_CR_OFF_05</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Verify address fields (Address, City, State, Country, Zipcode) accept valid inputs and are saved successfully.</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>TC_CR_OFF_06</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Verify the map location updates correctly based on the entered address/location details.</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>TC_CR_OFF_NEG_01</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Verify system displays validation errors when mandatory fields are left blank and Next is clicked.</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>TC_CR_OFF_NEG_02</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Verify system rejects invalid email formats and prevents navigation to the next step.</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>TC_CR_OFF_NEG_03</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Verify system rejects invalid phone numbers containing alphabets, special characters, or incorrect length.</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>TC_CR_OFF_NEG_04</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Verify system prevents proceeding when an unsupported or invalid partner type is selected.</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>TC_CR_OFF_NEG_05</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Verify system displays an error when an invalid or non-existent address/location is entered.</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>TC_CR_OFF_NEG_06</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Verify system prevents proceeding when Zipcode contains invalid characters or exceeds the allowed length.</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>TC_CR_ORG_01</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Verify user can enter valid Organization details and successfully proceed to the next step by clicking Next.</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>TC_CR_ORG_02</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Verify user can upload a valid company logo image and the logo preview is displayed correctly.</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>TC_CR_ORG_03</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Verify user can enter a unique Organization Name and save it successfully.</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>TC_CR_ORG_04</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Verify user can enter valid Registration Number, GST/License Number, and FSSAI Number and proceed successfully.</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>TC_CR_ORG_05</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Verify user can enable the Own Company checkbox and save the organization details successfully.</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>TC_CR_ORG_06</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Verify clicking the Back button navigates to the previous step while retaining entered data.</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>TC_CR_ORG_NEG_01</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Verify validation errors are displayed when mandatory fields (Organization Name, Logo, Registration No, GST/License No, FSSAI No) are left blank and Next is clicked.</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>TC_CR_ORG_NEG_02</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Verify system prevents proceeding when a duplicate Organization Name is entered.</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>TC_CR_ORG_NEG_03</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Verify system rejects unsupported logo file formats or files exceeding the allowed size limit.</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>TC_CR_ORG_NEG_04</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Verify system displays a validation error when invalid GST/License Number format is entered.</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>TC_CR_ORG_NEG_05</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Verify system displays a validation error when FSSAI Number contains alphabetic or special characters instead of valid numeric input.</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>TC_CR_ORG_NEG_06</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Verify an appropriate error message is displayed when organization details fail to save due to API/network issues.</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>TC_CR_AUTH_01</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Verify user can enter valid Username, Email, Phone Number, and Password and proceed to the next step by clicking Next.</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>TC_CR_AUTH_02</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Verify system accepts a valid email address format and saves it successfully.</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>TC_CR_AUTH_03</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Verify user can enter a valid phone number with country code and proceed successfully.</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>TC_CR_AUTH_04</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Verify clicking the Show/Hide Password icon correctly toggles password visibility.</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>TC_CR_AUTH_05</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Verify clicking the Back button navigates to the previous step while retaining entered authentication details.</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>TC_CR_AUTH_NEG_01</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Verify validation errors are displayed when mandatory fields (Username, Email, Phone Number, Password) are left blank and Next is clicked.</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>TC_CR_AUTH_NEG_02</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Verify system rejects invalid email formats and prevents proceeding to the next step.</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>TC_CR_AUTH_NEG_03</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Verify system prevents proceeding when an already existing Username is entered.</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>TC_CR_AUTH_NEG_04</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Verify system rejects weak passwords that do not meet the password policy requirements.</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>TC_CR_AUTH_NEG_05</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Verify system rejects invalid phone numbers containing alphabets, special characters, or incorrect length.</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>TC_CR_AGR_01</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Verify user can upload a valid agreement document and proceed to the next step successfully.</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>TC_CR_AGR_02</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Verify user can select a valid Catalog Option and Market and save the selections correctly.</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>TC_CR_AGR_03</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Verify user can select one or more markets and the selected markets are displayed in the Selected Markets section.</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>TC_CR_AGR_04</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Verify user can enter valid Agreement Start Date and Agreement End Date and proceed successfully.</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>TC_CR_AGR_05</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Verify user can select one or more Payment Methods (COD/Online) and save the agreement details successfully.</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>TC_CR_AGR_NEG_01</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Verify validation errors are displayed when mandatory fields (Agreement Document, Catalog Option, Market, Start Date, End Date) are left blank and Next is clicked.</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>TC_CR_AGR_NEG_02</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Verify system rejects unsupported agreement document file formats or files exceeding the allowed size limit.</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>TC_CR_AGR_NEG_03</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Verify system prevents proceeding when Agreement End Date is earlier than Agreement Start Date.</v>
+      </c>
+      <c r="D79" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>TC_CR_AGR_NEG_04</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Verify system displays a validation error when no market is selected after choosing a catalog option.</v>
+      </c>
+      <c r="D80" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>TC_CR_AGR_NEG_05</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Verify system prevents proceeding when no payment method is selected if at least one payment method is mandatory.</v>
+      </c>
+      <c r="D81" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>TC_CR_DN_01</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Verify the success page is displayed after completing all partner creation steps successfully.</v>
+      </c>
+      <c r="D82" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>TC_CR_DN_02</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Verify the success message "Partner details submitted successfully!" is displayed correctly.</v>
+      </c>
+      <c r="D83" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>TC_CR_DN_03</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Verify clicking the Done button redirects the user to the Partners list or Partner Details page as per business requirement.</v>
+      </c>
+      <c r="D84" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>TC_CR_DN_04</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Verify the newly created partner record is available in the Partners listing after clicking Done.</v>
+      </c>
+      <c r="D85" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>TC_CR_DN_NEG_01</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Verify the success page is not displayed if partner creation fails due to API/server error.</v>
+      </c>
+      <c r="D86" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>TC_CR_DN_NEG_02</v>
+      </c>
+      <c r="B87" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C87" t="str">
+        <v>Verify clicking the Done button during a network interruption displays an appropriate error message.</v>
+      </c>
+      <c r="D87" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>TC_CR_DN_NEG_03</v>
+      </c>
+      <c r="B88" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Verify refreshing the success page does not create a duplicate partner record.</v>
+      </c>
+      <c r="D88" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>TC_CR_DN_NEG_04</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C89" t="str">
+        <v>Verify using the browser Back button after successful submission does not resubmit or duplicate the partner creation request.</v>
+      </c>
+      <c r="D89" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D89"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K4"/>

</xml_diff>

<commit_message>
Merge testData.xlsx: add Partner (Tenant) sheet from develop, keep BusinessPlanTest + NotificationApproval + CatalogTest, add PartnerTest row to Regression
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -54,13 +54,14 @@
     <sheet name="BusinessPlanTest" sheetId="39" r:id="rId39"/>
     <sheet name="NotificationApproval" sheetId="240" r:id="rId40"/>
     <sheet name="CatalogTest" sheetId="241" r:id="rId41"/>
+    <sheet name="Partner (Tenant)" sheetId="242" r:id="rId42"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3314" uniqueCount="3314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3315" uniqueCount="3315">
   <si>
     <t>Test</t>
   </si>
@@ -10004,6 +10005,9 @@
   </si>
   <si>
     <t>AutoCat Display 140</t>
+  </si>
+  <si>
+    <t>PartnerTest</t>
   </si>
 </sst>
 </file>
@@ -28692,7 +28696,7 @@
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93DE4F72-EBB9-4825-A620-D1DF4D936AA5}">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="29.33203125" bestFit="1" customWidth="1"/>
@@ -29157,6 +29161,17 @@
         <v>573</v>
       </c>
       <c r="C42" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>3314</v>
+      </c>
+      <c r="B43" t="s">
+        <v>573</v>
+      </c>
+      <c r="C43" t="s">
         <v>574</v>
       </c>
     </row>
@@ -40145,6 +40160,1263 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D89"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>TC_ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Module</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Scenario</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Type</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>TC_LIST_01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Verify the Partners page loads successfully with dashboard metrics, partner filters, search box, and partner list.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>TC_LIST_02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Verify user can filter partners by Seller and only Seller-type partners are displayed.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TC_LIST_03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Verify user can search a partner using a valid Name, Email, or Phone Number and view matching results.</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TC_LIST_04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Verify clicking the View icon opens the selected partner's details page successfully.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TC_LIST_05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Verify clicking the Create Partner button navigates the user to the partner creation screen.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TC_LIST_06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Verify dashboard counts (Total Partners, Sellers, New This Month, Total Orders) are displayed correctly.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TC_LIST_NEG_01</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Verify searching with a non-existing partner name/email/phone displays a "No Records Found" message.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TC_LIST_NEG_02</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Verify search field handles special characters and invalid inputs without application failure.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TC_LIST_NEG_03</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Verify the page displays an appropriate error message when partner data fails to load due to API/network issues.</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TC_LIST_NEG_04</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Verify clicking the View icon for a deleted or inaccessible partner displays an appropriate error message.</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TC_LIST_NEG_05</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Verify partner type filters display an empty state message when no records exist for the selected type.</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TC_LIST_NEG_06</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Verify rapid multiple clicks on filter tabs or action buttons do not cause duplicate requests or UI issues.</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TC_VIEW_01</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Verify the Partner Details page loads successfully with all partner information displayed correctly.</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TC_VIEW_02</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Verify clicking the Back button navigates the user back to the Partners listing page.</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TC_VIEW_03</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Verify partner profile information (Logo, Name, Email, Phone) is displayed correctly in the left panel.</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TC_VIEW_04</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Verify clicking the Edit button in the Organization Info section opens the edit form with pre-populated data.</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TC_VIEW_05</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Verify clicking the Manage Account button opens the partner account management screen successfully.</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TC_VIEW_06</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Verify user can navigate between all left-menu sections (Subscription, Payments, Orders, Invoices, Users, etc.) successfully.</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TC_VIEW_07</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Verify all information sections (Organization Info, Office, Billing Info, Agreement, Credentials, Additional Info) display correct data.</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TC_VIEW_08</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Verify individual Edit buttons open the corresponding section for modification without affecting other sections.</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>TC_VIEW_NEG_01</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Verify an appropriate error message is displayed when partner details fail to load due to API/network failure.</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>TC_VIEW_NEG_02</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Verify the page handles missing partner profile image by displaying a default placeholder image.</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TC_VIEW_NEG_03</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Verify clicking Edit without sufficient permissions displays an authorization error.</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TC_VIEW_NEG_04</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Verify navigation to a non-existent partner record displays a "Partner Not Found" message.</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TC_VIEW_NEG_05</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Verify sections with missing data (e.g., Agreement, Additional Info) display appropriate empty-state messages instead of blank screens.</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TC_VIEW_NEG_06</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Verify clicking Manage Account for an inactive or disabled partner displays an appropriate validation message.</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TC_VIEW_NEG_07</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Verify rapid multiple clicks on Edit buttons do not open duplicate forms or create UI inconsistencies.</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>TC_VIEW_NEG_08</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Verify the page handles invalid or corrupted partner data without breaking the layout or displaying incorrect information.</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TC_DEL_01</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Verify clicking Delete successfully removes the selected partner and updates the partner list.</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TC_DEL_02</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Verify clicking Cancel closes the delete confirmation popup without deleting the partner.</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>TC_DEL_03</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Verify clicking the X (Close) icon dismisses the popup and retains the partner record.</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>TC_DEL_04</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Verify the delete confirmation popup displays correctly with warning message, Cancel button, and Delete button.</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TC_DEL_NEG_01</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Verify an appropriate error message is displayed when partner deletion fails due to API/network failure.</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>TC_DEL_NEG_02</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Verify a user without delete permissions cannot delete a partner and receives an authorization error.</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TC_DEL_NEG_03</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Verify multiple rapid clicks on the Delete button do not trigger duplicate delete requests.</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TC_DEL_NEG_04</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Verify attempting to delete a partner associated with active orders, subscriptions, or transactions displays a validation error and prevents deletion.</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>TC_CR_OFF_01</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Verify user can enter valid Office details and successfully proceed to the next step by clicking Next.</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>TC_CR_OFF_02</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Verify user can add a valid email address and it is saved successfully.</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>TC_CR_OFF_03</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Verify user can enter a valid phone number with country code and proceed successfully.</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>TC_CR_OFF_04</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Verify selecting a valid partner type (e.g., Seller) saves the selection correctly.</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>TC_CR_OFF_05</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Verify address fields (Address, City, State, Country, Zipcode) accept valid inputs and are saved successfully.</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>TC_CR_OFF_06</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Verify the map location updates correctly based on the entered address/location details.</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>TC_CR_OFF_NEG_01</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Verify system displays validation errors when mandatory fields are left blank and Next is clicked.</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>TC_CR_OFF_NEG_02</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Verify system rejects invalid email formats and prevents navigation to the next step.</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>TC_CR_OFF_NEG_03</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Verify system rejects invalid phone numbers containing alphabets, special characters, or incorrect length.</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>TC_CR_OFF_NEG_04</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Verify system prevents proceeding when an unsupported or invalid partner type is selected.</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>TC_CR_OFF_NEG_05</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Verify system displays an error when an invalid or non-existent address/location is entered.</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>TC_CR_OFF_NEG_06</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Verify system prevents proceeding when Zipcode contains invalid characters or exceeds the allowed length.</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>TC_CR_ORG_01</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Verify user can enter valid Organization details and successfully proceed to the next step by clicking Next.</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>TC_CR_ORG_02</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Verify user can upload a valid company logo image and the logo preview is displayed correctly.</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>TC_CR_ORG_03</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Verify user can enter a unique Organization Name and save it successfully.</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>TC_CR_ORG_04</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Verify user can enter valid Registration Number, GST/License Number, and FSSAI Number and proceed successfully.</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>TC_CR_ORG_05</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Verify user can enable the Own Company checkbox and save the organization details successfully.</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>TC_CR_ORG_06</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Verify clicking the Back button navigates to the previous step while retaining entered data.</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>TC_CR_ORG_NEG_01</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Verify validation errors are displayed when mandatory fields (Organization Name, Logo, Registration No, GST/License No, FSSAI No) are left blank and Next is clicked.</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>TC_CR_ORG_NEG_02</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Verify system prevents proceeding when a duplicate Organization Name is entered.</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>TC_CR_ORG_NEG_03</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Verify system rejects unsupported logo file formats or files exceeding the allowed size limit.</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>TC_CR_ORG_NEG_04</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Verify system displays a validation error when invalid GST/License Number format is entered.</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>TC_CR_ORG_NEG_05</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Verify system displays a validation error when FSSAI Number contains alphabetic or special characters instead of valid numeric input.</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>TC_CR_ORG_NEG_06</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Verify an appropriate error message is displayed when organization details fail to save due to API/network issues.</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>TC_CR_AUTH_01</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Verify user can enter valid Username, Email, Phone Number, and Password and proceed to the next step by clicking Next.</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>TC_CR_AUTH_02</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Verify system accepts a valid email address format and saves it successfully.</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>TC_CR_AUTH_03</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Verify user can enter a valid phone number with country code and proceed successfully.</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>TC_CR_AUTH_04</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Verify clicking the Show/Hide Password icon correctly toggles password visibility.</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>TC_CR_AUTH_05</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Verify clicking the Back button navigates to the previous step while retaining entered authentication details.</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>TC_CR_AUTH_NEG_01</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Verify validation errors are displayed when mandatory fields (Username, Email, Phone Number, Password) are left blank and Next is clicked.</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>TC_CR_AUTH_NEG_02</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Verify system rejects invalid email formats and prevents proceeding to the next step.</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>TC_CR_AUTH_NEG_03</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Verify system prevents proceeding when an already existing Username is entered.</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>TC_CR_AUTH_NEG_04</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Verify system rejects weak passwords that do not meet the password policy requirements.</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>TC_CR_AUTH_NEG_05</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Verify system rejects invalid phone numbers containing alphabets, special characters, or incorrect length.</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>TC_CR_AGR_01</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Verify user can upload a valid agreement document and proceed to the next step successfully.</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>TC_CR_AGR_02</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Verify user can select a valid Catalog Option and Market and save the selections correctly.</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>TC_CR_AGR_03</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Verify user can select one or more markets and the selected markets are displayed in the Selected Markets section.</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>TC_CR_AGR_04</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Verify user can enter valid Agreement Start Date and Agreement End Date and proceed successfully.</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>TC_CR_AGR_05</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Verify user can select one or more Payment Methods (COD/Online) and save the agreement details successfully.</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>TC_CR_AGR_NEG_01</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Verify validation errors are displayed when mandatory fields (Agreement Document, Catalog Option, Market, Start Date, End Date) are left blank and Next is clicked.</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>TC_CR_AGR_NEG_02</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Verify system rejects unsupported agreement document file formats or files exceeding the allowed size limit.</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>TC_CR_AGR_NEG_03</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Verify system prevents proceeding when Agreement End Date is earlier than Agreement Start Date.</v>
+      </c>
+      <c r="D79" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>TC_CR_AGR_NEG_04</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Verify system displays a validation error when no market is selected after choosing a catalog option.</v>
+      </c>
+      <c r="D80" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>TC_CR_AGR_NEG_05</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Verify system prevents proceeding when no payment method is selected if at least one payment method is mandatory.</v>
+      </c>
+      <c r="D81" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>TC_CR_DN_01</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Verify the success page is displayed after completing all partner creation steps successfully.</v>
+      </c>
+      <c r="D82" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>TC_CR_DN_02</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Verify the success message "Partner details submitted successfully!" is displayed correctly.</v>
+      </c>
+      <c r="D83" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>TC_CR_DN_03</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Verify clicking the Done button redirects the user to the Partners list or Partner Details page as per business requirement.</v>
+      </c>
+      <c r="D84" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>TC_CR_DN_04</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Verify the newly created partner record is available in the Partners listing after clicking Done.</v>
+      </c>
+      <c r="D85" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>TC_CR_DN_NEG_01</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Verify the success page is not displayed if partner creation fails due to API/server error.</v>
+      </c>
+      <c r="D86" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>TC_CR_DN_NEG_02</v>
+      </c>
+      <c r="B87" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C87" t="str">
+        <v>Verify clicking the Done button during a network interruption displays an appropriate error message.</v>
+      </c>
+      <c r="D87" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>TC_CR_DN_NEG_03</v>
+      </c>
+      <c r="B88" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Verify refreshing the success page does not create a duplicate partner record.</v>
+      </c>
+      <c r="D88" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>TC_CR_DN_NEG_04</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Partner (Tenant)</v>
+      </c>
+      <c r="C89" t="str">
+        <v>Verify using the browser Back button after successful submission does not resubmit or duplicate the partner creation request.</v>
+      </c>
+      <c r="D89" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D89"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9F7E00C-F1FE-4050-B47A-3E8ACFECFE43}">
   <dimension ref="A1:O3"/>

</xml_diff>

<commit_message>
feat(daily-reg): implement daily registration report and download history regression test suite
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -46,6 +46,7 @@
     <sheet name="CatalogTest" sheetId="41" r:id="rId41"/>
     <sheet name="Partner (Tenant)" sheetId="42" r:id="rId42"/>
     <sheet name="OfficeManagement" sheetId="43" r:id="rId43"/>
+    <sheet name="Daily Registration Regression" sheetId="44" r:id="rId44"/>
   </sheets>
 </workbook>
 </file>
@@ -33694,6 +33695,1924 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N42"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Test Case ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Module</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Screen Name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Test Scenario</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Test Case Type</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Preconditions</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Test Steps</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Test Data</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Expected Result</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Priority</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Actual Result</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Screenshot Path</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Execution Time</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>DRR-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Verify Daily Registration Report page loads successfully with all KPI cards, charts and tables displayed.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F2" t="str">
+        <v>User is logged in as Tenant admin</v>
+      </c>
+      <c r="G2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to BI &amp; Analytics &gt; Daily Registration Report
+2. Verify page heading visible
+3. Verify KPI cards (Total, Customers, Partners, Staff, Verified Rate) visible
+4. Verify trend chart and Registration Detail table visible</v>
+      </c>
+      <c r="H2" t="str">
+        <v>URL: /analytics/dailyRegistration</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Page loads with heading, 5 KPI cards, trend chart, and detail table</v>
+      </c>
+      <c r="J2" t="str">
+        <v>High</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M2" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-a8c93-harts-and-tables-displayed--local\test-finished-1.png</v>
+      </c>
+      <c r="N2" t="str">
+        <v>4.04s</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>DRR-002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Verify Today filter displays registration data for current day.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'Today' filter button
+2. Verify data updates and date range reflects today</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Filter: Today</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Today button is active and data shows current day registrations</v>
+      </c>
+      <c r="J3" t="str">
+        <v>High</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M3" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-33437-ation-data-for-current-day--local\test-finished-1.png</v>
+      </c>
+      <c r="N3" t="str">
+        <v>4.95s</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>DRR-003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Verify 7D filter displays registration data for last 7 days.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click '7D' filter button
+2. Verify data updates for last 7 days range</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Filter: 7D</v>
+      </c>
+      <c r="I4" t="str">
+        <v>7D button is active and data shows last 7 days registrations</v>
+      </c>
+      <c r="J4" t="str">
+        <v>High</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M4" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-4f84f-ation-data-for-last-7-days--local\test-finished-1.png</v>
+      </c>
+      <c r="N4" t="str">
+        <v>4.99s</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>DRR-004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Verify 30D filter displays registration data for last 30 days.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click '30D' filter button
+2. Verify data updates for last 30 days range</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Filter: 30D</v>
+      </c>
+      <c r="I5" t="str">
+        <v>30D button is active and data shows last 30 days registrations</v>
+      </c>
+      <c r="J5" t="str">
+        <v>High</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M5" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-646fb-tion-data-for-last-30-days--local\test-finished-1.png</v>
+      </c>
+      <c r="N5" t="str">
+        <v>4.80s</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>DRR-005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Verify Custom Date filter displays selected date range data.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'Custom' date picker
+2. Select start date and end date
+3. Verify data updates for selected range</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Start: 2026-06-01, End: 2026-06-15</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Page shows registrations for the custom date range selected</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M6" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-5253a-s-selected-date-range-data--local\test-finished-1.png</v>
+      </c>
+      <c r="N6" t="str">
+        <v>7.32s</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>DRR-006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Verify Refresh button reloads latest registration data.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Daily Registration Report page is open with data loaded</v>
+      </c>
+      <c r="G7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'Refresh' button
+2. Verify page reloads data without navigation</v>
+      </c>
+      <c r="H7" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Data refreshes successfully and page remains on report screen</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M7" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-4ce03-s-latest-registration-data--local\test-finished-1.png</v>
+      </c>
+      <c r="N7" t="str">
+        <v>5.33s</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>DRR-007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Verify Export CSV downloads registration report successfully.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Daily Registration Report page is open with data loaded</v>
+      </c>
+      <c r="G8" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Export CSV button
+2. Verify download initiates
+3. Verify file is not empty</v>
+      </c>
+      <c r="H8" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I8" t="str">
+        <v>CSV file downloads successfully and is not empty</v>
+      </c>
+      <c r="J8" t="str">
+        <v>High</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Blocked</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Not Available In Current Build</v>
+      </c>
+      <c r="M8" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-30294-ration-report-successfully--local\test-finished-1.png</v>
+      </c>
+      <c r="N8" t="str">
+        <v>2.93s</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>DRR-008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Verify PDF button downloads registration report successfully.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Daily Registration Report page is open with data loaded</v>
+      </c>
+      <c r="G9" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click PDF download button
+2. Verify download initiates
+3. Verify file exists and is valid</v>
+      </c>
+      <c r="H9" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I9" t="str">
+        <v>PDF file downloads successfully and is not empty</v>
+      </c>
+      <c r="J9" t="str">
+        <v>High</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Blocked</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Not Available In Current Build</v>
+      </c>
+      <c r="M9" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-e0951-ration-report-successfully--local\test-finished-1.png</v>
+      </c>
+      <c r="N9" t="str">
+        <v>2.95s</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>DRR-009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Verify View Download History navigation works correctly.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G10" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'View Download History' button
+2. Verify navigation to Download History page</v>
+      </c>
+      <c r="H10" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I10" t="str">
+        <v>User navigates to /analytics/history/CUSTOMER page successfully</v>
+      </c>
+      <c r="J10" t="str">
+        <v>High</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M10" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-0d6f9-navigation-works-correctly--local\test-finished-1.png</v>
+      </c>
+      <c r="N10" t="str">
+        <v>4.62s</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>DRR-010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Verify Schedule Report functionality opens successfully.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G11" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Schedule Report button if present
+2. Verify schedule dialog or page opens</v>
+      </c>
+      <c r="H11" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Schedule report dialog or page opens without error</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Blocked</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Feature Not Available In Current Build</v>
+      </c>
+      <c r="M11" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-cba3d-onality-opens-successfully--local\test-finished-1.png</v>
+      </c>
+      <c r="N11" t="str">
+        <v>3.02s</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>DRR-011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Verify Customer tab filters registration trend correctly.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G12" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'Customer' tab in Daily Registration Trend chart
+2. Verify chart updates to show only customer trend data</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Tab: Customer</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Trend chart filters to customer data only</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M12" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-7de73-gistration-trend-correctly--local\test-finished-1.png</v>
+      </c>
+      <c r="N12" t="str">
+        <v>4.24s</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>DRR-012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Verify Partner tab filters registration trend correctly.</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G13" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'Partner' tab in Daily Registration Trend chart
+2. Verify chart updates to show only partner trend data</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Tab: Partner</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Trend chart filters to partner data only</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M13" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-fcd59-gistration-trend-correctly--local\test-finished-1.png</v>
+      </c>
+      <c r="N13" t="str">
+        <v>4.61s</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>DRR-013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Verify Staff tab filters registration trend correctly.</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G14" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'Staff' tab in Daily Registration Trend chart
+2. Verify chart updates to show only staff trend data</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Tab: Staff</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Trend chart filters to staff data only</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M14" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-e6d0b-gistration-trend-correctly--local\test-finished-1.png</v>
+      </c>
+      <c r="N14" t="str">
+        <v>4.03s</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>DRR-014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Verify Registration Details search returns matching records.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Daily Registration Report page is open with Registration Detail table visible</v>
+      </c>
+      <c r="G15" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Type 'Raj Kumar' in search box and verify matching records
+2. Clear and type 'Priya Singh' and verify
+3. Clear and type 'Amir Khan' and verify</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Search: Raj Kumar, Priya Singh, Amir Khan</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Only matching records appear for each search term</v>
+      </c>
+      <c r="J15" t="str">
+        <v>High</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M15" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-5e805-h-returns-matching-records--local\test-finished-1.png</v>
+      </c>
+      <c r="N15" t="str">
+        <v>13.98s</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>DRR-015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Verify Role filter displays matching records for Customer, Partner and Staff.</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Daily Registration Report page is open with Registration Detail table visible</v>
+      </c>
+      <c r="G16" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Select 'Customer' from Role dropdown, click Apply, verify results
+2. Select 'Partner' from Role dropdown, click Apply, verify results
+3. Select 'Staff' from Role dropdown, click Apply, verify results</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Roles: Customer, Partner, Staff</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Only records matching selected role are displayed</v>
+      </c>
+      <c r="J16" t="str">
+        <v>High</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L16" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M16" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-5373e-Customer-Partner-and-Staff--local\test-finished-1.png</v>
+      </c>
+      <c r="N16" t="str">
+        <v>15.18s</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>DRR-016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Verify combined Search + Role + Source + Status filtering returns correct results.</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Enter search text, select Role, Source and Status, click Apply
+2. Verify only records matching all conditions appear</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Customer+Mobile App+Verified; Customer+Web+Pending; Partner+Social/Ads+Rejected; Staff+Referral+Verified</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Results match all selected filter conditions simultaneously</v>
+      </c>
+      <c r="J17" t="str">
+        <v>High</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M17" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-4f0b2-ng-returns-correct-results--local\test-finished-1.png</v>
+      </c>
+      <c r="N17" t="str">
+        <v>17.56s</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>DRR-017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Verify error when End Date is earlier than Start Date in Custom filter.</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Custom date picker
+2. Set End Date earlier than Start Date
+3. Verify validation error or no data shown</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Start: 2026-06-15, End: 2026-06-01</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Validation error shown or empty result returned for invalid date range</v>
+      </c>
+      <c r="J18" t="str">
+        <v>High</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M18" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-c63a3-tart-Date-in-Custom-filter--local\test-finished-1.png</v>
+      </c>
+      <c r="N18" t="str">
+        <v>7.15s</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>DRR-018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Verify page handles Registration Report API failure gracefully.</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Network is intercepted to simulate API failure</v>
+      </c>
+      <c r="G19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Intercept API call to registration report endpoint
+2. Return 500 error
+3. Verify page shows error state gracefully without crashing</v>
+      </c>
+      <c r="H19" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Page shows error message or empty state, does not crash</v>
+      </c>
+      <c r="J19" t="str">
+        <v>High</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M19" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-a77c3-ort-API-failure-gracefully--local\test-finished-1.png</v>
+      </c>
+      <c r="N19" t="str">
+        <v>6.99s</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>DRR-019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Verify KPI cards display default values when no data exists.</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Daily Registration Report open with empty dataset</v>
+      </c>
+      <c r="G20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Select a date range with no registrations
+2. Verify KPI cards show 0 or default state</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Future date range with no data</v>
+      </c>
+      <c r="I20" t="str">
+        <v>KPI cards display 0 or N/A gracefully without errors</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L20" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M20" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-c91d2-values-when-no-data-exists--local\test-finished-1.png</v>
+      </c>
+      <c r="N20" t="str">
+        <v>9.02s</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>DRR-020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Verify charts display empty state when dataset is unavailable.</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Daily Registration Report open with empty dataset</v>
+      </c>
+      <c r="G21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Select a date range with no data
+2. Verify trend charts show empty state message</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Future date with no data</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Charts show empty state or no-data message, not broken UI</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K21" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L21" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M21" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-86927-hen-dataset-is-unavailable--local\test-finished-1.png</v>
+      </c>
+      <c r="N21" t="str">
+        <v>8.73s</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>DRR-021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Verify Export CSV behavior when no records exist.</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Daily Registration Report open showing no records</v>
+      </c>
+      <c r="G22" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Ensure no records visible in table
+2. Click Export CSV
+3. Verify behavior (error message or empty file)</v>
+      </c>
+      <c r="H22" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Error message shown or empty CSV with headers only downloaded</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L22" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M22" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-7fb4c-vior-when-no-records-exist--local\test-finished-1.png</v>
+      </c>
+      <c r="N22" t="str">
+        <v>7.00s</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>DRR-022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Verify PDF export behavior when no records exist.</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Daily Registration Report open showing no records</v>
+      </c>
+      <c r="G23" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Ensure no records visible in table
+2. Click PDF button
+3. Verify behavior (error message or empty file)</v>
+      </c>
+      <c r="H23" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Error message shown or empty PDF downloaded without crash</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M23" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-c7401-vior-when-no-records-exist--local\test-finished-1.png</v>
+      </c>
+      <c r="N23" t="str">
+        <v>7.01s</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>DRR-023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Verify Refresh button during network failure handles error gracefully.</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Network is intercepted to simulate failure</v>
+      </c>
+      <c r="G24" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Intercept network
+2. Click Refresh button
+3. Verify page shows error or retains previous state gracefully</v>
+      </c>
+      <c r="H24" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Page does not crash and shows appropriate error state</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L24" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M24" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-0341f-e-handles-error-gracefully--local\test-finished-1.png</v>
+      </c>
+      <c r="N24" t="str">
+        <v>8.07s</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>DRR-024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Verify unauthorized user cannot access Daily Registration Report page.</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F25" t="str">
+        <v>User is not logged in or logged in as non-admin role</v>
+      </c>
+      <c r="G25" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate directly to /analytics/dailyRegistration without auth
+2. Verify redirect to login or access denied shown</v>
+      </c>
+      <c r="H25" t="str">
+        <v>URL: /analytics/dailyRegistration</v>
+      </c>
+      <c r="I25" t="str">
+        <v>User is redirected to login or shown access denied message</v>
+      </c>
+      <c r="J25" t="str">
+        <v>High</v>
+      </c>
+      <c r="K25" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L25" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M25" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-624ab-y-Registration-Report-page--local\test-finished-1.png</v>
+      </c>
+      <c r="N25" t="str">
+        <v>4.35s</v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>DRR-025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Verify random invalid search text returns no records.</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Daily Registration Report page is open with Registration Detail table visible</v>
+      </c>
+      <c r="G26" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Type '@@@@@' in search box, click Apply, verify empty state
+2. Type '123456789' in search box, verify empty state
+3. Type 'xyz_invalid_test', verify empty state</v>
+      </c>
+      <c r="H26" t="str">
+        <v>@@@@@, 123456789, xyz_invalid_test</v>
+      </c>
+      <c r="I26" t="str">
+        <v>No records found / empty state shown for each invalid search</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K26" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L26" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M26" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-26b10-ch-text-returns-no-records--local\test-finished-1.png</v>
+      </c>
+      <c r="N26" t="str">
+        <v>6.04s</v>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
+        <v>DRR-026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Verify filters returning no matching data show empty state in table.</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G27" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Select a Role+Source+Status combination that has no matching data
+2. Click Apply
+3. Verify empty state message shown</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Combination with no matches</v>
+      </c>
+      <c r="I27" t="str">
+        <v>Table shows empty state message, not broken layout</v>
+      </c>
+      <c r="J27" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K27" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L27" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M27" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-8549a--show-empty-state-in-table--local\test-finished-1.png</v>
+      </c>
+      <c r="N27" t="str">
+        <v>7.83s</v>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
+        <v>DRR-027</v>
+      </c>
+      <c r="B28" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Verify table handles null or missing values correctly without UI crash.</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G28" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Load Registration Detail table
+2. Verify null or empty cells render as dash or empty, not as errors</v>
+      </c>
+      <c r="H28" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Null/missing values shown as '-' or blank without crashing UI</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K28" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L28" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M28" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-6aef5-correctly-without-UI-crash--local\test-finished-1.png</v>
+      </c>
+      <c r="N28" t="str">
+        <v>2.94s</v>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
+        <v>DRR-028</v>
+      </c>
+      <c r="B29" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Verify pagination is hidden or disabled when no records are present.</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Daily Registration Report open showing no records</v>
+      </c>
+      <c r="G29" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Apply filters so no records appear
+2. Verify pagination controls are hidden or disabled</v>
+      </c>
+      <c r="H29" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Pagination hidden/disabled when table has no records</v>
+      </c>
+      <c r="J29" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K29" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L29" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M29" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-d3646-hen-no-records-are-present--local\test-finished-1.png</v>
+      </c>
+      <c r="N29" t="str">
+        <v>7.55s</v>
+      </c>
+    </row>
+    <row r="30" xml:space="preserve">
+      <c r="A30" t="str">
+        <v>DRR-029</v>
+      </c>
+      <c r="B30" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Verify rapid multiple CSV clicks do not create duplicate downloads.</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Daily Registration Report page is open with data</v>
+      </c>
+      <c r="G30" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Export CSV button rapidly 5 times
+2. Verify only one download is initiated</v>
+      </c>
+      <c r="H30" t="str">
+        <v>5 rapid clicks</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Only one valid CSV download is generated</v>
+      </c>
+      <c r="J30" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K30" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L30" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M30" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-70c1f-create-duplicate-downloads--local\test-finished-1.png</v>
+      </c>
+      <c r="N30" t="str">
+        <v>2.90s</v>
+      </c>
+    </row>
+    <row r="31" xml:space="preserve">
+      <c r="A31" t="str">
+        <v>DRR-030</v>
+      </c>
+      <c r="B31" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Verify rapid multiple PDF clicks do not create duplicate files.</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Daily Registration Report page is open with data</v>
+      </c>
+      <c r="G31" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click PDF button rapidly 5 times
+2. Verify only one download is initiated</v>
+      </c>
+      <c r="H31" t="str">
+        <v>5 rapid clicks</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Only one valid PDF download is generated</v>
+      </c>
+      <c r="J31" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K31" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L31" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M31" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-fc69e-not-create-duplicate-files--local\test-finished-1.png</v>
+      </c>
+      <c r="N31" t="str">
+        <v>2.84s</v>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
+      <c r="A32" t="str">
+        <v>DRR-031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Verify page performance with large registration dataset meets acceptable thresholds.</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Daily Registration Report page open with large dataset</v>
+      </c>
+      <c r="G32" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Record page load time
+2. Apply filter and record response time
+3. Perform search and record time
+4. Click export and record time</v>
+      </c>
+      <c r="H32" t="str">
+        <v>30D filter (largest dataset period)</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Page load &lt; 5s, filter response &lt; 3s, search response &lt; 2s, export &lt; 10s</v>
+      </c>
+      <c r="J32" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K32" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L32" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M32" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-2d476-eets-acceptable-thresholds--local\test-finished-1.png</v>
+      </c>
+      <c r="N32" t="str">
+        <v>7.29s</v>
+      </c>
+    </row>
+    <row r="33" xml:space="preserve">
+      <c r="A33" t="str">
+        <v>CDH-001</v>
+      </c>
+      <c r="B33" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Verify Customer Download History page loads successfully with all sections visible.</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F33" t="str">
+        <v>User is logged in as Tenant admin</v>
+      </c>
+      <c r="G33" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to BI &amp; Analytics &gt; Daily Registration Report
+2. Click 'View Download History'
+3. Verify Download History page heading visible</v>
+      </c>
+      <c r="H33" t="str">
+        <v>URL: /analytics/history/CUSTOMER</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Download History page loads with heading, filter, table and action buttons</v>
+      </c>
+      <c r="J33" t="str">
+        <v>High</v>
+      </c>
+      <c r="K33" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L33" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M33" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-5547c--with-all-sections-visible--local\test-finished-1.png</v>
+      </c>
+      <c r="N33" t="str">
+        <v>4.48s</v>
+      </c>
+    </row>
+    <row r="34" xml:space="preserve">
+      <c r="A34" t="str">
+        <v>CDH-002</v>
+      </c>
+      <c r="B34" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Verify Today filter works correctly on Download History page.</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Customer Download History page is open</v>
+      </c>
+      <c r="G34" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Select 'Today' from the date filter dropdown
+2. Verify table updates to show today's download requests</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Filter: Today</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Table refreshes showing download requests from today</v>
+      </c>
+      <c r="J34" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K34" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L34" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M34" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-7916c-y-on-Download-History-page--local\test-finished-1.png</v>
+      </c>
+      <c r="N34" t="str">
+        <v>2.71s</v>
+      </c>
+    </row>
+    <row r="35" xml:space="preserve">
+      <c r="A35" t="str">
+        <v>CDH-003</v>
+      </c>
+      <c r="B35" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Verify View Customer Report button navigates back to Customer Report correctly.</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Customer Download History page is open</v>
+      </c>
+      <c r="G35" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'VIEW CUSTOMER REPORT' button
+2. Verify navigation to Daily Registration Report page</v>
+      </c>
+      <c r="H35" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I35" t="str">
+        <v>User navigates to Daily Registration Report page successfully</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K35" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L35" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M35" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-f69a1--Customer-Report-correctly--local\test-finished-1.png</v>
+      </c>
+      <c r="N35" t="str">
+        <v>4.41s</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>CDH-004</v>
+      </c>
+      <c r="B36" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Verify Request Downloads table displays all required column headers correctly.</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Customer Download History page is open</v>
+      </c>
+      <c r="G36" t="str">
+        <v>1. Verify table column headers: REQUEST#, REQUEST DATE, REQUEST TYPE, REQUESTED BY, STATUS, ACTION</v>
+      </c>
+      <c r="H36" t="str">
+        <v>Columns: REQUEST#, REQUEST DATE, REQUEST TYPE, REQUESTED BY, STATUS, ACTION</v>
+      </c>
+      <c r="I36" t="str">
+        <v>All 6 column headers are visible and correctly labeled</v>
+      </c>
+      <c r="J36" t="str">
+        <v>High</v>
+      </c>
+      <c r="K36" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L36" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M36" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-21b1d-d-column-headers-correctly--local\test-finished-1.png</v>
+      </c>
+      <c r="N36" t="str">
+        <v>2.79s</v>
+      </c>
+    </row>
+    <row r="37" xml:space="preserve">
+      <c r="A37" t="str">
+        <v>CDH-005</v>
+      </c>
+      <c r="B37" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Verify pagination works correctly on Download History page when records exist.</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Customer Download History page has multiple pages of records</v>
+      </c>
+      <c r="G37" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Verify pagination controls visible
+2. Click Next page and verify next records load
+3. Click Previous and verify navigation works</v>
+      </c>
+      <c r="H37" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Pagination navigates between pages correctly</v>
+      </c>
+      <c r="J37" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K37" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L37" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M37" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-0f758-ry-page-when-records-exist--local\test-finished-1.png</v>
+      </c>
+      <c r="N37" t="str">
+        <v>4.79s</v>
+      </c>
+    </row>
+    <row r="38" xml:space="preserve">
+      <c r="A38" t="str">
+        <v>CDH-006</v>
+      </c>
+      <c r="B38" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Verify No Data Available message is displayed when no download records exist.</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Customer Download History page is open with no download records</v>
+      </c>
+      <c r="G38" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Verify table shows 'No data available' message
+2. Verify no action buttons are present</v>
+      </c>
+      <c r="H38" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Table shows 'No data available' message clearly</v>
+      </c>
+      <c r="J38" t="str">
+        <v>High</v>
+      </c>
+      <c r="K38" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L38" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M38" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-04fd2--no-download-records-exist--local\test-finished-1.png</v>
+      </c>
+      <c r="N38" t="str">
+        <v>3.08s</v>
+      </c>
+    </row>
+    <row r="39" xml:space="preserve">
+      <c r="A39" t="str">
+        <v>CDH-007</v>
+      </c>
+      <c r="B39" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Verify Download History page handles API failure gracefully.</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Network is intercepted to simulate API failure</v>
+      </c>
+      <c r="G39" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Intercept download history API call
+2. Return 500 error
+3. Verify page shows error state without crashing</v>
+      </c>
+      <c r="H39" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I39" t="str">
+        <v>Page shows error message or empty state gracefully</v>
+      </c>
+      <c r="J39" t="str">
+        <v>High</v>
+      </c>
+      <c r="K39" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L39" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M39" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-ed31f-les-API-failure-gracefully--local\test-finished-1.png</v>
+      </c>
+      <c r="N39" t="str">
+        <v>6.23s</v>
+      </c>
+    </row>
+    <row r="40" xml:space="preserve">
+      <c r="A40" t="str">
+        <v>CDH-008</v>
+      </c>
+      <c r="B40" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Verify invalid date filter does not return incorrect download history data.</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Customer Download History page is open</v>
+      </c>
+      <c r="G40" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Select an invalid or future date from filter
+2. Verify no incorrect records are returned</v>
+      </c>
+      <c r="H40" t="str">
+        <v>Future date with no records</v>
+      </c>
+      <c r="I40" t="str">
+        <v>Empty state shown or validation error — no incorrect data returned</v>
+      </c>
+      <c r="J40" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K40" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L40" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M40" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-a4379-rect-download-history-data--local\test-finished-1.png</v>
+      </c>
+      <c r="N40" t="str">
+        <v>2.92s</v>
+      </c>
+    </row>
+    <row r="41" xml:space="preserve">
+      <c r="A41" t="str">
+        <v>CDH-009</v>
+      </c>
+      <c r="B41" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Verify unauthorized users cannot access Download History page directly.</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F41" t="str">
+        <v>User is not logged in</v>
+      </c>
+      <c r="G41" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate directly to /analytics/history/CUSTOMER without authentication
+2. Verify redirect to login or access denied</v>
+      </c>
+      <c r="H41" t="str">
+        <v>URL: /analytics/history/CUSTOMER</v>
+      </c>
+      <c r="I41" t="str">
+        <v>User redirected to login page or access denied message shown</v>
+      </c>
+      <c r="J41" t="str">
+        <v>High</v>
+      </c>
+      <c r="K41" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L41" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M41" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-ac751-load-History-page-directly--local\test-finished-1.png</v>
+      </c>
+      <c r="N41" t="str">
+        <v>4.25s</v>
+      </c>
+    </row>
+    <row r="42" xml:space="preserve">
+      <c r="A42" t="str">
+        <v>CDH-010</v>
+      </c>
+      <c r="B42" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Verify Action buttons are disabled or absent when download file is unavailable.</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Customer Download History page is open with a failed download request</v>
+      </c>
+      <c r="G42" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Identify a record with failed/unavailable file
+2. Verify action button (download) is disabled or absent</v>
+      </c>
+      <c r="H42" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I42" t="str">
+        <v>Download action button is disabled or not shown for unavailable files</v>
+      </c>
+      <c r="J42" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K42" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L42" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M42" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-54118-wnload-file-is-unavailable--local\test-finished-1.png</v>
+      </c>
+      <c r="N42" t="str">
+        <v>3.19s</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:N42"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O3"/>

</xml_diff>

<commit_message>
fix: audit and update NotificationTemplateTest excel coverage
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -47,28 +47,6 @@
     <sheet name="StockPointSellerTest" sheetId="42" r:id="rId42"/>
   </sheets>
 </workbook>
-</file>
-
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -764,10 +742,10 @@
         <v>NotificationTemplateTest</v>
       </c>
       <c r="B30" t="str">
-        <v>NO</v>
+        <v>YES</v>
       </c>
       <c r="C30" t="str">
-        <v>parallel</v>
+        <v>serial</v>
       </c>
     </row>
     <row r="31">
@@ -14105,7 +14083,7 @@
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G26"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -14118,139 +14096,596 @@
         <v>Scenario</v>
       </c>
       <c r="D1" t="str">
-        <v>Search Type</v>
+        <v>Runnable</v>
       </c>
       <c r="E1" t="str">
+        <v>Priority</v>
+      </c>
+      <c r="F1" t="str">
         <v>Test Data</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Expected Result</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>TC01</v>
+        <v>TC_NT_01</v>
       </c>
       <c r="B2" t="str">
         <v>Notification Template</v>
       </c>
       <c r="C2" t="str">
-        <v>Search Concern Positive</v>
+        <v>Verify user can open the Notification Template page successfully</v>
       </c>
       <c r="D2" t="str">
-        <v>Concern</v>
+        <v>Yes</v>
       </c>
       <c r="E2" t="str">
-        <v>VERIFY_PHONE_CONCERN</v>
+        <v>High</v>
       </c>
       <c r="F2" t="str">
-        <v>Matching record displayed</v>
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>Action completes successfully</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>TC02</v>
+        <v>TC_NT_02</v>
       </c>
       <c r="B3" t="str">
         <v>Notification Template</v>
       </c>
       <c r="C3" t="str">
-        <v>Search Body Positive</v>
+        <v>Verify template list displays all existing templates correctly</v>
       </c>
       <c r="D3" t="str">
-        <v>Body</v>
+        <v>Yes</v>
       </c>
       <c r="E3" t="str">
-        <v>testing purpose</v>
+        <v>High</v>
       </c>
       <c r="F3" t="str">
-        <v>Matching record displayed</v>
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>Action completes successfully</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>TC03</v>
+        <v>TC_NT_03</v>
       </c>
       <c r="B4" t="str">
         <v>Notification Template</v>
       </c>
       <c r="C4" t="str">
-        <v>Search Concern Negative</v>
+        <v>Verify clicking Create Template opens the template creation screen</v>
       </c>
       <c r="D4" t="str">
-        <v>Concern</v>
+        <v>Yes</v>
       </c>
       <c r="E4" t="str">
-        <v>VERIFY_PHONE_CONCERN_XYZ</v>
+        <v>High</v>
       </c>
       <c r="F4" t="str">
-        <v>No matching record found</v>
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>Action completes successfully</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>TC04</v>
+        <v>TC_NT_04</v>
       </c>
       <c r="B5" t="str">
         <v>Notification Template</v>
       </c>
       <c r="C5" t="str">
-        <v>Search Body Negative</v>
+        <v>Verify system prevents template creation when Concern is not selected</v>
       </c>
       <c r="D5" t="str">
-        <v>Body</v>
+        <v>Yes</v>
       </c>
       <c r="E5" t="str">
-        <v>testing purpose XYZ</v>
+        <v>High</v>
       </c>
       <c r="F5" t="str">
-        <v>No matching record found</v>
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>Action completes successfully</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>TC05</v>
+        <v>TC_NT_05</v>
       </c>
       <c r="B6" t="str">
         <v>Notification Template</v>
       </c>
       <c r="C6" t="str">
-        <v>Create Template</v>
+        <v>Verify user can select a valid Concern from the dropdown list</v>
       </c>
       <c r="D6" t="str">
-        <v>Create</v>
+        <v>Yes</v>
       </c>
       <c r="E6" t="str">
-        <v>Subject=AUTO_TEMPLATE_, Body=Test notification body, From Name=Automation User, From Email=auto_@mailinator.com</v>
+        <v>High</v>
       </c>
       <c r="F6" t="str">
-        <v>Template created successfully</v>
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>Action completes successfully</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>TC06</v>
+        <v>TC_NT_06</v>
       </c>
       <c r="B7" t="str">
         <v>Notification Template</v>
       </c>
       <c r="C7" t="str">
-        <v>Delete Template</v>
+        <v>Verify user can switch between Email, SMS, WhatsApp, and InApp template types</v>
       </c>
       <c r="D7" t="str">
-        <v>Delete</v>
+        <v>Yes</v>
       </c>
       <c r="E7" t="str">
-        <v>Delete template created in TC05</v>
+        <v>High</v>
       </c>
       <c r="F7" t="str">
-        <v>Template removed successfully</v>
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TC_NT_07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Verify Email template is created successfully with all mandatory fields filled</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E8" t="str">
+        <v>High</v>
+      </c>
+      <c r="F8" t="str">
+        <v>{"type":"Email"}</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TC_NT_08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Verify Email template creation fails when mandatory fields are left blank</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E9" t="str">
+        <v>High</v>
+      </c>
+      <c r="F9" t="str">
+        <v>{"type":"Email"}</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TC_NT_09</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Verify Email template creation fails with an invalid From Email format</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E10" t="str">
+        <v>High</v>
+      </c>
+      <c r="F10" t="str">
+        <v>{"type":"Email"}</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TC_NT_10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Verify SMS template is created successfully with valid Body and Template ID</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E11" t="str">
+        <v>High</v>
+      </c>
+      <c r="F11" t="str">
+        <v>{"type":"SMS"}</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TC_NT_11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Verify SMS template creation fails when Template ID is empty</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E12" t="str">
+        <v>High</v>
+      </c>
+      <c r="F12" t="str">
+        <v>{"type":"SMS"}</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TC_NT_12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Verify WhatsApp template is created successfully with valid Header and Body details</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E13" t="str">
+        <v>High</v>
+      </c>
+      <c r="F13" t="str">
+        <v>{"type":"Whatsapp"}</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TC_NT_13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Verify WhatsApp template creation fails when mandatory Body field is blank</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E14" t="str">
+        <v>High</v>
+      </c>
+      <c r="F14" t="str">
+        <v>{"type":"Whatsapp"}</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TC_NT_14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Verify user can add WhatsApp message variables using the (+) button</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E15" t="str">
+        <v>High</v>
+      </c>
+      <c r="F15" t="str">
+        <v>{"type":"Whatsapp"}</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TC_NT_15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Verify InApp template is created successfully with Subject, Body, and image upload</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E16" t="str">
+        <v>High</v>
+      </c>
+      <c r="F16" t="str">
+        <v>{"type":"Inapp"}</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TC_NT_16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Verify InApp template creation fails when Subject or Body is empty</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E17" t="str">
+        <v>High</v>
+      </c>
+      <c r="F17" t="str">
+        <v>{"type":"Inapp"}</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TC_NT_17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Verify system accepts only supported file formats for InApp image upload</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E18" t="str">
+        <v>High</v>
+      </c>
+      <c r="F18" t="str">
+        <v>{"type":"Inapp"}</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TC_NT_18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Verify system rejects unsupported file formats during image upload</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E19" t="str">
+        <v>High</v>
+      </c>
+      <c r="F19" t="str">
+        <v>{"type":"Inapp"}</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TC_NT_19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Verify newly created template appears in the template list after successful submission</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E20" t="str">
+        <v>High</v>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TC_NT_20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Verify duplicate template creation for the same Concern and Template Type is not allowed</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E21" t="str">
+        <v>High</v>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>TC_NT_21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Verify search functionality returns matching templates for a valid keyword</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E22" t="str">
+        <v>High</v>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>TC_NT_22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Verify search functionality returns no records for an invalid keyword</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E23" t="str">
+        <v>High</v>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TC_NT_23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Verify user can delete an existing template successfully</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E24" t="str">
+        <v>High</v>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TC_NT_24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Verify template is not deleted when delete action is cancelled</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E25" t="str">
+        <v>High</v>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <v>Action completes successfully</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TC_NT_25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Notification Template</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Verify refresh button reloads the latest template data correctly</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E26" t="str">
+        <v>High</v>
+      </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
+      <c r="G26" t="str">
+        <v>Action completes successfully</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G26"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Merge testData.xlsx: keep all 46 sheets, add StockPointSellerTest and ItemTest to Regression
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -46,6 +46,9 @@
     <sheet name="CatalogTest" sheetId="41" r:id="rId41"/>
     <sheet name="Partner (Tenant)" sheetId="42" r:id="rId42"/>
     <sheet name="ItemTest" sheetId="43" r:id="rId43"/>
+    <sheet name="UserManagement" sheetId="44" r:id="rId46"/>
+    <sheet name="Daily Registration Regression" sheetId="45" r:id="rId47"/>
+    <sheet name="StockPointSellerTest" sheetId="46" r:id="rId48"/>
   </sheets>
 </workbook>
 </file>
@@ -18709,7 +18712,7 @@
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C45"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -19181,6 +19184,28 @@
         <v>YES</v>
       </c>
       <c r="C43" t="str">
+        <v>serial</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>StockPointSellerTest</v>
+      </c>
+      <c r="B44" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C44" t="str">
+        <v>serial</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>ItemTest</v>
+      </c>
+      <c r="B45" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C45" t="str">
         <v>serial</v>
       </c>
     </row>
@@ -37983,6 +38008,3278 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AC10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>TestID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Issue</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Description</v>
+      </c>
+      <c r="D1" t="str">
+        <v>UserName</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Password</v>
+      </c>
+      <c r="F1" t="str">
+        <v>persona</v>
+      </c>
+      <c r="G1" t="str">
+        <v>SearchText</v>
+      </c>
+      <c r="H1" t="str">
+        <v>UpdatedName</v>
+      </c>
+      <c r="I1" t="str">
+        <v>FullName</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="L1" t="str">
+        <v>DOB</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Gender</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Address</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Category</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Role</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Experience</v>
+      </c>
+      <c r="R1" t="str">
+        <v>UserLogin</v>
+      </c>
+      <c r="S1" t="str">
+        <v>UserPassword</v>
+      </c>
+      <c r="T1" t="str">
+        <v>ConfirmPassword</v>
+      </c>
+      <c r="U1" t="str">
+        <v>IDType</v>
+      </c>
+      <c r="V1" t="str">
+        <v>AddressType</v>
+      </c>
+      <c r="W1" t="str">
+        <v>IDNumber</v>
+      </c>
+      <c r="X1" t="str">
+        <v>AddressNumber</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>IDFrontPhoto</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>IDBackPhoto</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>AddressFrontPhoto</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>AddressBackPhoto</v>
+      </c>
+      <c r="AC1" t="str">
+        <v>ExpectedResult</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>TC01_PageLoad</v>
+      </c>
+      <c r="B2">
+        <v>7001</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Verify User Management page load</v>
+      </c>
+      <c r="D2" t="str">
+        <v>freshcart@gmail.com</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Welcome@123</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Tenant</v>
+      </c>
+      <c r="S2" t="str">
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>TC02_SearchUserPositive</v>
+      </c>
+      <c r="B3">
+        <v>7002</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Verify search by valid user name</v>
+      </c>
+      <c r="D3" t="str">
+        <v>freshcart@gmail.com</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Welcome@123</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Tenant</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Hari K</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TC03_SearchUserByEmail</v>
+      </c>
+      <c r="B4">
+        <v>7003</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Verify search by valid email</v>
+      </c>
+      <c r="D4" t="str">
+        <v>freshcart@gmail.com</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Welcome@123</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Tenant</v>
+      </c>
+      <c r="G4" t="str">
+        <v>asit@yopmail.com</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TC04_SearchUserNegative</v>
+      </c>
+      <c r="B5">
+        <v>7004</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Verify search by invalid value</v>
+      </c>
+      <c r="D5" t="str">
+        <v>freshcart@gmail.com</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Welcome@123</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Tenant</v>
+      </c>
+      <c r="G5" t="str">
+        <v>xyz123test</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TC06_VerifyTabs</v>
+      </c>
+      <c r="B6">
+        <v>7006</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Verify all user tabs</v>
+      </c>
+      <c r="D6" t="str">
+        <v>freshcart@gmail.com</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Welcome@123</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Tenant</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TC07_ViewUserDetails</v>
+      </c>
+      <c r="B7">
+        <v>7007</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Verify view user details</v>
+      </c>
+      <c r="D7" t="str">
+        <v>freshcart@gmail.com</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Welcome@123</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Tenant</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Don Samanta</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TC08_EditUser</v>
+      </c>
+      <c r="B8">
+        <v>7008</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Verify edit user details</v>
+      </c>
+      <c r="D8" t="str">
+        <v>freshcart@gmail.com</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Welcome@123</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Tenant</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Anik bhai</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Don</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TC09_DeleteUser</v>
+      </c>
+      <c r="B9">
+        <v>7009</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Verify delete user</v>
+      </c>
+      <c r="D9" t="str">
+        <v>freshcart@gmail.com</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Welcome@123</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Tenant</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Gopal yu</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TC10_CreateUser</v>
+      </c>
+      <c r="B10">
+        <v>7010</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Verify create user</v>
+      </c>
+      <c r="D10" t="str">
+        <v>freshcart@gmail.com</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Welcome@123</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Tenant</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Doli Sing</v>
+      </c>
+      <c r="J10" t="str">
+        <v>dilinsing781@yopmail.com</v>
+      </c>
+      <c r="K10">
+        <v>9999183910</v>
+      </c>
+      <c r="L10">
+        <v>34830</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Male</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Khirpai, West Bengal 721232, India</v>
+      </c>
+      <c r="O10" t="str">
+        <v>DELIVERY_AGENT</v>
+      </c>
+      <c r="P10" t="str">
+        <v>Agent_calonex</v>
+      </c>
+      <c r="Q10">
+        <v>4</v>
+      </c>
+      <c r="R10" t="str">
+        <v>Sing Dolin</v>
+      </c>
+      <c r="S10" t="str">
+        <v>Welcome@123</v>
+      </c>
+      <c r="T10" t="str">
+        <v>Welcome@123</v>
+      </c>
+      <c r="U10" t="str">
+        <v>Aadhaar Card</v>
+      </c>
+      <c r="V10" t="str">
+        <v>Aadhaar Card</v>
+      </c>
+      <c r="W10" t="str">
+        <v>RANDOM</v>
+      </c>
+      <c r="X10" t="str">
+        <v>RANDOM</v>
+      </c>
+      <c r="Y10" t="str">
+        <v>https://d3etdz0uek6d8j.cloudfront.net/payment_gatway_logos/pvc-aadhaar-card-500x500.jpg</v>
+      </c>
+      <c r="Z10" t="str">
+        <v>https://d3etdz0uek6d8j.cloudfront.net/payment_gatway_logos/20250404112835_Aadhaar-card-generated-using-AI.jpg</v>
+      </c>
+      <c r="AA10" t="str">
+        <v>https://d3etdz0uek6d8j.cloudfront.net/payment_gatway_logos/pvc-aadhaar-card-500x500.jpg</v>
+      </c>
+      <c r="AB10" t="str">
+        <v>https://d3etdz0uek6d8j.cloudfront.net/payment_gatway_logos/20250404112835_Aadhaar-card-generated-using-AI.jpg</v>
+      </c>
+      <c r="AC10" t="str">
+        <v>Created</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G4" r:id="rId1"/>
+    <hyperlink ref="J10" r:id="rId2"/>
+    <hyperlink ref="Y10" r:id="rId3"/>
+    <hyperlink ref="Z10" r:id="rId4"/>
+    <hyperlink ref="AA10" r:id="rId5"/>
+    <hyperlink ref="AB10" r:id="rId6"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC10"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N42"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Test Case ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Module</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Screen Name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Test Scenario</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Test Case Type</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Preconditions</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Test Steps</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Test Data</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Expected Result</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Priority</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Actual Result</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Screenshot Path</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Execution Time</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>DRR-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Verify Daily Registration Report page loads successfully with all KPI cards, charts and tables displayed.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F2" t="str">
+        <v>User is logged in as Tenant admin</v>
+      </c>
+      <c r="G2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to BI &amp; Analytics &gt; Daily Registration Report
+2. Verify page heading visible
+3. Verify KPI cards (Total, Customers, Partners, Staff, Verified Rate) visible
+4. Verify trend chart and Registration Detail table visible</v>
+      </c>
+      <c r="H2" t="str">
+        <v>URL: /analytics/dailyRegistration</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Page loads with heading, 5 KPI cards, trend chart, and detail table</v>
+      </c>
+      <c r="J2" t="str">
+        <v>High</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M2" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-a8c93-harts-and-tables-displayed--local\test-finished-1.png</v>
+      </c>
+      <c r="N2" t="str">
+        <v>5.74s</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>DRR-002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Verify Today filter displays registration data for current day.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'Today' filter button
+2. Verify data updates and date range reflects today</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Filter: Today</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Today button is active and data shows current day registrations</v>
+      </c>
+      <c r="J3" t="str">
+        <v>High</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M3" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-33437-ation-data-for-current-day--local\test-finished-1.png</v>
+      </c>
+      <c r="N3" t="str">
+        <v>5.24s</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>DRR-003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Verify 7D filter displays registration data for last 7 days.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click '7D' filter button
+2. Verify data updates for last 7 days range</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Filter: 7D</v>
+      </c>
+      <c r="I4" t="str">
+        <v>7D button is active and data shows last 7 days registrations</v>
+      </c>
+      <c r="J4" t="str">
+        <v>High</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M4" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-4f84f-ation-data-for-last-7-days--local\test-finished-1.png</v>
+      </c>
+      <c r="N4" t="str">
+        <v>5.27s</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>DRR-004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Verify 30D filter displays registration data for last 30 days.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click '30D' filter button
+2. Verify data updates for last 30 days range</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Filter: 30D</v>
+      </c>
+      <c r="I5" t="str">
+        <v>30D button is active and data shows last 30 days registrations</v>
+      </c>
+      <c r="J5" t="str">
+        <v>High</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M5" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-646fb-tion-data-for-last-30-days--local\test-finished-1.png</v>
+      </c>
+      <c r="N5" t="str">
+        <v>4.45s</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>DRR-005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Verify Custom Date filter displays selected date range data.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'Custom' date picker
+2. Select start date and end date
+3. Verify data updates for selected range</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Start: 2026-06-01, End: 2026-06-15</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Page shows registrations for the custom date range selected</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M6" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-5253a-s-selected-date-range-data--local\test-finished-1.png</v>
+      </c>
+      <c r="N6" t="str">
+        <v>7.89s</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>DRR-006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Verify Refresh button reloads latest registration data.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Daily Registration Report page is open with data loaded</v>
+      </c>
+      <c r="G7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'Refresh' button
+2. Verify page reloads data without navigation</v>
+      </c>
+      <c r="H7" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Data refreshes successfully and page remains on report screen</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M7" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-4ce03-s-latest-registration-data--local\test-finished-1.png</v>
+      </c>
+      <c r="N7" t="str">
+        <v>5.77s</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>DRR-007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Verify Export CSV downloads registration report successfully.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Daily Registration Report page is open with data loaded</v>
+      </c>
+      <c r="G8" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Export CSV button
+2. Verify download initiates
+3. Verify file is not empty</v>
+      </c>
+      <c r="H8" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I8" t="str">
+        <v>CSV file downloads successfully and is not empty</v>
+      </c>
+      <c r="J8" t="str">
+        <v>High</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Blocked</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Not Available In Current Build</v>
+      </c>
+      <c r="M8" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-30294-ration-report-successfully--local\test-finished-1.png</v>
+      </c>
+      <c r="N8" t="str">
+        <v>3.34s</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>DRR-008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Verify PDF button downloads registration report successfully.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Daily Registration Report page is open with data loaded</v>
+      </c>
+      <c r="G9" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click PDF download button
+2. Verify download initiates
+3. Verify file exists and is valid</v>
+      </c>
+      <c r="H9" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I9" t="str">
+        <v>PDF file downloads successfully and is not empty</v>
+      </c>
+      <c r="J9" t="str">
+        <v>High</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Blocked</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Not Available In Current Build</v>
+      </c>
+      <c r="M9" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-e0951-ration-report-successfully--local\test-finished-1.png</v>
+      </c>
+      <c r="N9" t="str">
+        <v>3.16s</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>DRR-009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Verify View Download History navigation works correctly.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G10" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'View Download History' button
+2. Verify navigation to Download History page</v>
+      </c>
+      <c r="H10" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I10" t="str">
+        <v>User navigates to /analytics/history/CUSTOMER page successfully</v>
+      </c>
+      <c r="J10" t="str">
+        <v>High</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M10" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-0d6f9-navigation-works-correctly--local\test-finished-1.png</v>
+      </c>
+      <c r="N10" t="str">
+        <v>5.39s</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>DRR-010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Verify Schedule Report functionality opens successfully.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G11" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Schedule Report button if present
+2. Verify schedule dialog or page opens</v>
+      </c>
+      <c r="H11" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Schedule report dialog or page opens without error</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Blocked</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Feature Not Available In Current Build</v>
+      </c>
+      <c r="M11" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-cba3d-onality-opens-successfully--local\test-finished-1.png</v>
+      </c>
+      <c r="N11" t="str">
+        <v>3.33s</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>DRR-011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Verify Customer tab filters registration trend correctly.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G12" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'Customer' tab in Daily Registration Trend chart
+2. Verify chart updates to show only customer trend data</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Tab: Customer</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Trend chart filters to customer data only</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M12" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-7de73-gistration-trend-correctly--local\test-finished-1.png</v>
+      </c>
+      <c r="N12" t="str">
+        <v>4.25s</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>DRR-012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Verify Partner tab filters registration trend correctly.</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G13" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'Partner' tab in Daily Registration Trend chart
+2. Verify chart updates to show only partner trend data</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Tab: Partner</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Trend chart filters to partner data only</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M13" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-fcd59-gistration-trend-correctly--local\test-finished-1.png</v>
+      </c>
+      <c r="N13" t="str">
+        <v>4.56s</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>DRR-013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Verify Staff tab filters registration trend correctly.</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G14" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'Staff' tab in Daily Registration Trend chart
+2. Verify chart updates to show only staff trend data</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Tab: Staff</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Trend chart filters to staff data only</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M14" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-e6d0b-gistration-trend-correctly--local\test-finished-1.png</v>
+      </c>
+      <c r="N14" t="str">
+        <v>4.29s</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>DRR-014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Verify Registration Details search returns matching records.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Daily Registration Report page is open with Registration Detail table visible</v>
+      </c>
+      <c r="G15" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Type 'Raj Kumar' in search box and verify matching records
+2. Clear and type 'Priya Singh' and verify
+3. Clear and type 'Amir Khan' and verify</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Search: Raj Kumar, Priya Singh, Amir Khan</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Only matching records appear for each search term</v>
+      </c>
+      <c r="J15" t="str">
+        <v>High</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M15" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-5e805-h-returns-matching-records--local\test-finished-1.png</v>
+      </c>
+      <c r="N15" t="str">
+        <v>25.82s</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>DRR-015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Verify Role filter displays matching records for Customer, Partner and Staff.</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Daily Registration Report page is open with Registration Detail table visible</v>
+      </c>
+      <c r="G16" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Select 'Customer' from Role dropdown, click Apply, verify results
+2. Select 'Partner' from Role dropdown, click Apply, verify results
+3. Select 'Staff' from Role dropdown, click Apply, verify results</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Roles: Customer, Partner, Staff</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Only records matching selected role are displayed</v>
+      </c>
+      <c r="J16" t="str">
+        <v>High</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L16" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M16" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-5373e-Customer-Partner-and-Staff--local\test-finished-1.png</v>
+      </c>
+      <c r="N16" t="str">
+        <v>40.33s</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>DRR-016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Verify combined Search + Role + Source + Status filtering returns correct results.</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Enter search text, select Role, Source and Status, click Apply
+2. Verify only records matching all conditions appear</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Customer+Mobile App+Verified; Customer+Web+Pending; Partner+Social/Ads+Rejected; Staff+Referral+Verified</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Results match all selected filter conditions simultaneously</v>
+      </c>
+      <c r="J17" t="str">
+        <v>High</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M17" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-4f0b2-ng-returns-correct-results--local\test-finished-1.png</v>
+      </c>
+      <c r="N17" t="str">
+        <v>48.42s</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>DRR-017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Verify error when End Date is earlier than Start Date in Custom filter.</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Custom date picker
+2. Set End Date earlier than Start Date
+3. Verify validation error or no data shown</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Start: 2026-06-15, End: 2026-06-01</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Validation error shown or empty result returned for invalid date range</v>
+      </c>
+      <c r="J18" t="str">
+        <v>High</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M18" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-c63a3-tart-Date-in-Custom-filter--local\test-finished-1.png</v>
+      </c>
+      <c r="N18" t="str">
+        <v>13.40s</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>DRR-018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Verify page handles Registration Report API failure gracefully.</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Network is intercepted to simulate API failure</v>
+      </c>
+      <c r="G19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Intercept API call to registration report endpoint
+2. Return 500 error
+3. Verify page shows error state gracefully without crashing</v>
+      </c>
+      <c r="H19" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Page shows error message or empty state, does not crash</v>
+      </c>
+      <c r="J19" t="str">
+        <v>High</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M19" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-a77c3-ort-API-failure-gracefully--local\test-finished-1.png</v>
+      </c>
+      <c r="N19" t="str">
+        <v>13.01s</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>DRR-019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Verify KPI cards display default values when no data exists.</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Daily Registration Report open with empty dataset</v>
+      </c>
+      <c r="G20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Select a date range with no registrations
+2. Verify KPI cards show 0 or default state</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Future date range with no data</v>
+      </c>
+      <c r="I20" t="str">
+        <v>KPI cards display 0 or N/A gracefully without errors</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L20" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M20" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-c91d2-values-when-no-data-exists--local\test-finished-1.png</v>
+      </c>
+      <c r="N20" t="str">
+        <v>15.49s</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>DRR-020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Verify charts display empty state when dataset is unavailable.</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Daily Registration Report open with empty dataset</v>
+      </c>
+      <c r="G21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Select a date range with no data
+2. Verify trend charts show empty state message</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Future date with no data</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Charts show empty state or no-data message, not broken UI</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K21" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L21" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M21" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-86927-hen-dataset-is-unavailable--local\test-finished-1.png</v>
+      </c>
+      <c r="N21" t="str">
+        <v>14.56s</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>DRR-021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Verify Export CSV behavior when no records exist.</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Daily Registration Report open showing no records</v>
+      </c>
+      <c r="G22" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Ensure no records visible in table
+2. Click Export CSV
+3. Verify behavior (error message or empty file)</v>
+      </c>
+      <c r="H22" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Error message shown or empty CSV with headers only downloaded</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L22" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M22" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-7fb4c-vior-when-no-records-exist--local\test-finished-1.png</v>
+      </c>
+      <c r="N22" t="str">
+        <v>7.55s</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>DRR-022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Verify PDF export behavior when no records exist.</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Daily Registration Report open showing no records</v>
+      </c>
+      <c r="G23" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Ensure no records visible in table
+2. Click PDF button
+3. Verify behavior (error message or empty file)</v>
+      </c>
+      <c r="H23" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Error message shown or empty PDF downloaded without crash</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M23" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-c7401-vior-when-no-records-exist--local\test-finished-1.png</v>
+      </c>
+      <c r="N23" t="str">
+        <v>7.37s</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>DRR-023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Verify Refresh button during network failure handles error gracefully.</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Network is intercepted to simulate failure</v>
+      </c>
+      <c r="G24" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Intercept network
+2. Click Refresh button
+3. Verify page shows error or retains previous state gracefully</v>
+      </c>
+      <c r="H24" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Page does not crash and shows appropriate error state</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L24" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M24" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-0341f-e-handles-error-gracefully--local\test-finished-1.png</v>
+      </c>
+      <c r="N24" t="str">
+        <v>15.61s</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>DRR-024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Verify unauthorized user cannot access Daily Registration Report page.</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F25" t="str">
+        <v>User is not logged in or logged in as non-admin role</v>
+      </c>
+      <c r="G25" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate directly to /analytics/dailyRegistration without auth
+2. Verify redirect to login or access denied shown</v>
+      </c>
+      <c r="H25" t="str">
+        <v>URL: /analytics/dailyRegistration</v>
+      </c>
+      <c r="I25" t="str">
+        <v>User is redirected to login or shown access denied message</v>
+      </c>
+      <c r="J25" t="str">
+        <v>High</v>
+      </c>
+      <c r="K25" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L25" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M25" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-624ab-y-Registration-Report-page--local\test-finished-1.png</v>
+      </c>
+      <c r="N25" t="str">
+        <v>5.86s</v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>DRR-025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Verify random invalid search text returns no records.</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Daily Registration Report page is open with Registration Detail table visible</v>
+      </c>
+      <c r="G26" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Type '@@@@@' in search box, click Apply, verify empty state
+2. Type '123456789' in search box, verify empty state
+3. Type 'xyz_invalid_test', verify empty state</v>
+      </c>
+      <c r="H26" t="str">
+        <v>@@@@@, 123456789, xyz_invalid_test</v>
+      </c>
+      <c r="I26" t="str">
+        <v>No records found / empty state shown for each invalid search</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K26" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L26" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M26" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-26b10-ch-text-returns-no-records--local\test-finished-1.png</v>
+      </c>
+      <c r="N26" t="str">
+        <v>6.34s</v>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
+        <v>DRR-026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Verify filters returning no matching data show empty state in table.</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G27" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Select a Role+Source+Status combination that has no matching data
+2. Click Apply
+3. Verify empty state message shown</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Combination with no matches</v>
+      </c>
+      <c r="I27" t="str">
+        <v>Table shows empty state message, not broken layout</v>
+      </c>
+      <c r="J27" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K27" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L27" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M27" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-8549a--show-empty-state-in-table--local\test-finished-1.png</v>
+      </c>
+      <c r="N27" t="str">
+        <v>8.14s</v>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
+        <v>DRR-027</v>
+      </c>
+      <c r="B28" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Verify table handles null or missing values correctly without UI crash.</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Daily Registration Report page is open</v>
+      </c>
+      <c r="G28" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Load Registration Detail table
+2. Verify null or empty cells render as dash or empty, not as errors</v>
+      </c>
+      <c r="H28" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Null/missing values shown as '-' or blank without crashing UI</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K28" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L28" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M28" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-6aef5-correctly-without-UI-crash--local\test-finished-1.png</v>
+      </c>
+      <c r="N28" t="str">
+        <v>3.19s</v>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
+        <v>DRR-028</v>
+      </c>
+      <c r="B29" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Verify pagination is hidden or disabled when no records are present.</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Daily Registration Report open showing no records</v>
+      </c>
+      <c r="G29" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Apply filters so no records appear
+2. Verify pagination controls are hidden or disabled</v>
+      </c>
+      <c r="H29" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Pagination hidden/disabled when table has no records</v>
+      </c>
+      <c r="J29" t="str">
+        <v>Low</v>
+      </c>
+      <c r="K29" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L29" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M29" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-d3646-hen-no-records-are-present--local\test-finished-1.png</v>
+      </c>
+      <c r="N29" t="str">
+        <v>7.78s</v>
+      </c>
+    </row>
+    <row r="30" xml:space="preserve">
+      <c r="A30" t="str">
+        <v>DRR-029</v>
+      </c>
+      <c r="B30" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Verify rapid multiple CSV clicks do not create duplicate downloads.</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Daily Registration Report page is open with data</v>
+      </c>
+      <c r="G30" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Export CSV button rapidly 5 times
+2. Verify only one download is initiated</v>
+      </c>
+      <c r="H30" t="str">
+        <v>5 rapid clicks</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Only one valid CSV download is generated</v>
+      </c>
+      <c r="J30" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K30" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L30" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M30" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-70c1f-create-duplicate-downloads--local\test-finished-1.png</v>
+      </c>
+      <c r="N30" t="str">
+        <v>3.06s</v>
+      </c>
+    </row>
+    <row r="31" xml:space="preserve">
+      <c r="A31" t="str">
+        <v>DRR-030</v>
+      </c>
+      <c r="B31" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Verify rapid multiple PDF clicks do not create duplicate files.</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Daily Registration Report page is open with data</v>
+      </c>
+      <c r="G31" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click PDF button rapidly 5 times
+2. Verify only one download is initiated</v>
+      </c>
+      <c r="H31" t="str">
+        <v>5 rapid clicks</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Only one valid PDF download is generated</v>
+      </c>
+      <c r="J31" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K31" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L31" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M31" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-fc69e-not-create-duplicate-files--local\test-finished-1.png</v>
+      </c>
+      <c r="N31" t="str">
+        <v>3.05s</v>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
+      <c r="A32" t="str">
+        <v>DRR-031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Daily Registration Report</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Verify page performance with large registration dataset meets acceptable thresholds.</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Daily Registration Report page open with large dataset</v>
+      </c>
+      <c r="G32" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Record page load time
+2. Apply filter and record response time
+3. Perform search and record time
+4. Click export and record time</v>
+      </c>
+      <c r="H32" t="str">
+        <v>30D filter (largest dataset period)</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Page load &lt; 5s, filter response &lt; 3s, search response &lt; 2s, export &lt; 10s</v>
+      </c>
+      <c r="J32" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K32" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L32" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M32" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-2d476-eets-acceptable-thresholds--local\test-finished-1.png</v>
+      </c>
+      <c r="N32" t="str">
+        <v>7.40s</v>
+      </c>
+    </row>
+    <row r="33" xml:space="preserve">
+      <c r="A33" t="str">
+        <v>CDH-001</v>
+      </c>
+      <c r="B33" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Verify Customer Download History page loads successfully with all sections visible.</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F33" t="str">
+        <v>User is logged in as Tenant admin</v>
+      </c>
+      <c r="G33" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to BI &amp; Analytics &gt; Daily Registration Report
+2. Click 'View Download History'
+3. Verify Download History page heading visible</v>
+      </c>
+      <c r="H33" t="str">
+        <v>URL: /analytics/history/CUSTOMER</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Download History page loads with heading, filter, table and action buttons</v>
+      </c>
+      <c r="J33" t="str">
+        <v>High</v>
+      </c>
+      <c r="K33" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L33" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M33" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-5547c--with-all-sections-visible--local\test-finished-1.png</v>
+      </c>
+      <c r="N33" t="str">
+        <v>4.71s</v>
+      </c>
+    </row>
+    <row r="34" xml:space="preserve">
+      <c r="A34" t="str">
+        <v>CDH-002</v>
+      </c>
+      <c r="B34" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Verify Today filter works correctly on Download History page.</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Customer Download History page is open</v>
+      </c>
+      <c r="G34" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Select 'Today' from the date filter dropdown
+2. Verify table updates to show today's download requests</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Filter: Today</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Table refreshes showing download requests from today</v>
+      </c>
+      <c r="J34" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K34" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L34" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M34" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-7916c-y-on-Download-History-page--local\test-finished-1.png</v>
+      </c>
+      <c r="N34" t="str">
+        <v>2.91s</v>
+      </c>
+    </row>
+    <row r="35" xml:space="preserve">
+      <c r="A35" t="str">
+        <v>CDH-003</v>
+      </c>
+      <c r="B35" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Verify View Customer Report button navigates back to Customer Report correctly.</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Customer Download History page is open</v>
+      </c>
+      <c r="G35" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click 'VIEW CUSTOMER REPORT' button
+2. Verify navigation to Daily Registration Report page</v>
+      </c>
+      <c r="H35" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I35" t="str">
+        <v>User navigates to Daily Registration Report page successfully</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K35" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L35" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M35" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-f69a1--Customer-Report-correctly--local\test-finished-1.png</v>
+      </c>
+      <c r="N35" t="str">
+        <v>4.69s</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>CDH-004</v>
+      </c>
+      <c r="B36" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Verify Request Downloads table displays all required column headers correctly.</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Customer Download History page is open</v>
+      </c>
+      <c r="G36" t="str">
+        <v>1. Verify table column headers: REQUEST#, REQUEST DATE, REQUEST TYPE, REQUESTED BY, STATUS, ACTION</v>
+      </c>
+      <c r="H36" t="str">
+        <v>Columns: REQUEST#, REQUEST DATE, REQUEST TYPE, REQUESTED BY, STATUS, ACTION</v>
+      </c>
+      <c r="I36" t="str">
+        <v>All 6 column headers are visible and correctly labeled</v>
+      </c>
+      <c r="J36" t="str">
+        <v>High</v>
+      </c>
+      <c r="K36" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L36" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M36" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-21b1d-d-column-headers-correctly--local\test-finished-1.png</v>
+      </c>
+      <c r="N36" t="str">
+        <v>3.00s</v>
+      </c>
+    </row>
+    <row r="37" xml:space="preserve">
+      <c r="A37" t="str">
+        <v>CDH-005</v>
+      </c>
+      <c r="B37" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Verify pagination works correctly on Download History page when records exist.</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Customer Download History page has multiple pages of records</v>
+      </c>
+      <c r="G37" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Verify pagination controls visible
+2. Click Next page and verify next records load
+3. Click Previous and verify navigation works</v>
+      </c>
+      <c r="H37" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Pagination navigates between pages correctly</v>
+      </c>
+      <c r="J37" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K37" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L37" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M37" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-0f758-ry-page-when-records-exist--local\test-finished-1.png</v>
+      </c>
+      <c r="N37" t="str">
+        <v>5.04s</v>
+      </c>
+    </row>
+    <row r="38" xml:space="preserve">
+      <c r="A38" t="str">
+        <v>CDH-006</v>
+      </c>
+      <c r="B38" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Verify No Data Available message is displayed when no download records exist.</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Customer Download History page is open with no download records</v>
+      </c>
+      <c r="G38" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Verify table shows 'No data available' message
+2. Verify no action buttons are present</v>
+      </c>
+      <c r="H38" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Table shows 'No data available' message clearly</v>
+      </c>
+      <c r="J38" t="str">
+        <v>High</v>
+      </c>
+      <c r="K38" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L38" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M38" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-04fd2--no-download-records-exist--local\test-finished-1.png</v>
+      </c>
+      <c r="N38" t="str">
+        <v>2.98s</v>
+      </c>
+    </row>
+    <row r="39" xml:space="preserve">
+      <c r="A39" t="str">
+        <v>CDH-007</v>
+      </c>
+      <c r="B39" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Verify Download History page handles API failure gracefully.</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Network is intercepted to simulate API failure</v>
+      </c>
+      <c r="G39" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Intercept download history API call
+2. Return 500 error
+3. Verify page shows error state without crashing</v>
+      </c>
+      <c r="H39" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I39" t="str">
+        <v>Page shows error message or empty state gracefully</v>
+      </c>
+      <c r="J39" t="str">
+        <v>High</v>
+      </c>
+      <c r="K39" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L39" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M39" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-ed31f-les-API-failure-gracefully--local\test-finished-1.png</v>
+      </c>
+      <c r="N39" t="str">
+        <v>6.27s</v>
+      </c>
+    </row>
+    <row r="40" xml:space="preserve">
+      <c r="A40" t="str">
+        <v>CDH-008</v>
+      </c>
+      <c r="B40" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Verify invalid date filter does not return incorrect download history data.</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Customer Download History page is open</v>
+      </c>
+      <c r="G40" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Select an invalid or future date from filter
+2. Verify no incorrect records are returned</v>
+      </c>
+      <c r="H40" t="str">
+        <v>Future date with no records</v>
+      </c>
+      <c r="I40" t="str">
+        <v>Empty state shown or validation error — no incorrect data returned</v>
+      </c>
+      <c r="J40" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K40" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L40" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M40" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-a4379-rect-download-history-data--local\test-finished-1.png</v>
+      </c>
+      <c r="N40" t="str">
+        <v>3.19s</v>
+      </c>
+    </row>
+    <row r="41" xml:space="preserve">
+      <c r="A41" t="str">
+        <v>CDH-009</v>
+      </c>
+      <c r="B41" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Verify unauthorized users cannot access Download History page directly.</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F41" t="str">
+        <v>User is not logged in</v>
+      </c>
+      <c r="G41" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate directly to /analytics/history/CUSTOMER without authentication
+2. Verify redirect to login or access denied</v>
+      </c>
+      <c r="H41" t="str">
+        <v>URL: /analytics/history/CUSTOMER</v>
+      </c>
+      <c r="I41" t="str">
+        <v>User redirected to login page or access denied message shown</v>
+      </c>
+      <c r="J41" t="str">
+        <v>High</v>
+      </c>
+      <c r="K41" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L41" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M41" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-ac751-load-History-page-directly--local\test-finished-1.png</v>
+      </c>
+      <c r="N41" t="str">
+        <v>4.61s</v>
+      </c>
+    </row>
+    <row r="42" xml:space="preserve">
+      <c r="A42" t="str">
+        <v>CDH-010</v>
+      </c>
+      <c r="B42" t="str">
+        <v>BI &amp; Analytics</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Customer Download History</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Verify Action buttons are disabled or absent when download file is unavailable.</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Customer Download History page is open with a failed download request</v>
+      </c>
+      <c r="G42" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Identify a record with failed/unavailable file
+2. Verify action button (download) is disabled or absent</v>
+      </c>
+      <c r="H42" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I42" t="str">
+        <v>Download action button is disabled or not shown for unavailable files</v>
+      </c>
+      <c r="J42" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K42" t="str">
+        <v>Passed</v>
+      </c>
+      <c r="L42" t="str">
+        <v>Test passed successfully.</v>
+      </c>
+      <c r="M42" t="str">
+        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-54118-wnload-file-is-unavailable--local\test-finished-1.png</v>
+      </c>
+      <c r="N42" t="str">
+        <v>3.18s</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:N42"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D69"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>TC_ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Module</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Scenario</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Type</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>TC_LIST_01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Verify the Stock Points page loads successfully with all summary cards, search box, and stock point records displayed.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>TC_LIST_02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Verify the Current Page Results count matches the number of records displayed in the table.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TC_LIST_03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Verify the Total Stock Points count displays the correct total number of stock points.</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TC_LIST_04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Verify searching with a valid Stock Point name returns the correct matching record.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TC_LIST_05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Verify searching with a valid Email ID returns the correct stock point record.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TC_LIST_06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Verify clicking the View (Eye) icon opens the selected Stock Point details page.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TC_LIST_07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Verify clicking Create Stock Point navigates to the Create Stock Point screen.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TC_LIST_08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Verify clicking the Refresh icon reloads the latest stock point data successfully.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TC_LIST_09</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Verify the correct Office Type badge (Branch Office, Head Office, Default) is displayed for each stock point.</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TC_LIST_10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Verify clicking the Back button navigates to the previous page successfully.</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TC_LIST_NEG_01</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Verify searching with a non-existent Stock Point name displays no records found.</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TC_LIST_NEG_02</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Verify searching with invalid special characters (@#$%^&amp;*) does not crash the application.</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TC_LIST_NEG_03</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Verify the page handles API failure gracefully while loading stock point records.</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TC_LIST_NEG_04</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Verify an appropriate error message is displayed when the stock point details API fails after clicking the View icon.</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TC_LIST_NEG_05</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Verify the table displays an empty-state message when no stock points exist.</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TC_LIST_NEG_06</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Verify incorrect or malformed email search values do not return unrelated records.</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TC_LIST_NEG_07</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Verify rapid multiple clicks on the Refresh button do not create duplicate API requests or UI issues.</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TC_LIST_NEG_08</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Verify clicking the View icon for a deleted/inactive stock point displays an appropriate error message.</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TC_LIST_NEG_09</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Verify unauthorized users cannot access the Stock Points page and receive an access denied message.</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TC_LIST_NEG_10</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Verify the summary cards do not display negative, null, or incorrect counts when API data is invalid.</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>TC_VIEW_01</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Verify the View Stock Point page loads successfully with all Stock Point details displayed.</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>TC_VIEW_02</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Verify Office information (Stock Point Name, Office Type, Email, Phone, City, State, Country, Zipcode) is displayed correctly.</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TC_VIEW_03</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Verify Organization details (Organization Name, Registration No, GST No, FSSAI No, Own Company) are displayed correctly.</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TC_VIEW_04</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Verify Bill To section displays the linked billing office information correctly.</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TC_VIEW_05</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Verify Authentication details (Username, Email, Phone, Security Question, Security Answer) are displayed correctly.</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TC_VIEW_06</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Verify the Office Type badge (e.g., Branch Office) matches the configured office type.</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TC_VIEW_07</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Verify clicking the Back button navigates to the Stock Point listing page.</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>TC_VIEW_08</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Verify clicking the Create button navigates to the Create Stock Point page.</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TC_VIEW_09</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Verify the Search box is displayed and accepts valid search input.</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TC_VIEW_10</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Verify the Refresh button reloads the latest stock point details successfully.</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>TC_VIEW_NEG_01</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Verify an appropriate error message is displayed when the Stock Point details API returns no data.</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>TC_VIEW_NEG_02</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Verify the page handles API/network failure gracefully while loading stock point details.</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TC_VIEW_NEG_03</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Verify accessing the page with an invalid Stock Point ID displays a Record Not Found message.</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>TC_VIEW_NEG_04</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Verify missing Organization information does not break the page layout and displays placeholders/default values.</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TC_VIEW_NEG_05</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Verify missing Bill To information is displayed as - or appropriate default values.</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TC_VIEW_NEG_06</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Verify missing Authentication details are handled gracefully without page crashes.</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>TC_VIEW_NEG_07</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Verify unauthorized users cannot access the View Stock Point page and receive an access denied message.</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>TC_VIEW_NEG_08</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Verify invalid search input (special characters only) does not cause application errors.</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>TC_VIEW_NEG_09</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Verify the Refresh button handles API timeout/failure scenarios correctly.</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>TC_VIEW_NEG_10</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Verify null or empty values in fields (Email, Phone, GST No, FSSAI No, Security Answer) are displayed properly without UI corruption.</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>TC_CR_OFF_01</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Verify user can create a Stock Point by entering all mandatory fields with valid data and click Next successfully.</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>TC_CR_OFF_02</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Verify valid email address can be added using the Add Email button.</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>TC_CR_OFF_03</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Verify valid phone number with country code can be added using the Add Phone button.</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>TC_CR_OFF_04</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Verify selecting a valid location from Google Search auto-populates Country, State, City, and Zipcode fields.</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>TC_CR_OFF_05</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Verify user can select different Office Types from the dropdown successfully.</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>TC_CR_OFF_06</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Verify map pin location is updated correctly when a valid address is searched and selected.</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>TC_CR_OFF_NEG_01</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Verify validation message appears when Stock Point Name is left blank and user clicks Next.</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>TC_CR_OFF_NEG_02</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Verify validation message appears when Email field contains an invalid email format.</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>TC_CR_OFF_NEG_03</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Verify validation message appears when Phone Number contains alphabets or special characters.</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>TC_CR_OFF_NEG_04</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Verify user cannot proceed when mandatory fields (Country, State, City, Zipcode) are empty.</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>TC_CR_OFF_NEG_05</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Verify Zipcode field rejects invalid formats (letters, special characters, insufficient digits).</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>TC_CR_OFF_NEG_06</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Verify user cannot proceed when Google location search returns no valid address or an invalid address is entered.</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>TC_CR_ORG_01</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Verify user can proceed to the next step by entering valid Organization Name, Logo, Registration No, GST/License No, and FSSAI No.</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>TC_CR_ORG_02</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Verify user can upload a valid logo file (JPG/PNG) successfully.</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>TC_CR_ORG_03</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Verify Organization Name uniqueness validation passes for a new unique organization name.</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>TC_CR_ORG_04</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Verify user can select the Own Company checkbox and continue successfully.</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>TC_CR_ORG_NEG_01</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Verify validation message appears when Organization Name is left blank and user clicks Next.</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>TC_CR_ORG_NEG_02</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Verify validation message appears when a duplicate Organization Name is entered.</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>TC_CR_ORG_NEG_03</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Verify user cannot proceed without uploading the mandatory Logo file.</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>TC_CR_ORG_NEG_04</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Verify validation message appears when Registration No, GST/License No, or FSSAI No is left empty and user clicks Next.</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>TC_CR_AUTH_01</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Verify user can proceed to the next step by entering valid Username, Email, Phone Number, and Password.</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>TC_CR_AUTH_02</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Verify system accepts a valid email format (e.g., user@example.com).</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>TC_CR_AUTH_03</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Verify system accepts a valid phone number with country code selected.</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>TC_CR_AUTH_04</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Verify password visibility toggle (eye icon) correctly shows and hides the password.</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Positive</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>TC_CR_AUTH_NEG_01</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Verify validation message appears when Username is left blank and user clicks Next.</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>TC_CR_AUTH_NEG_02</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Verify validation message appears when an invalid email format is entered (e.g., abc@com).</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>TC_CR_AUTH_NEG_03</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Verify validation message appears when Phone Number contains alphabets or special characters.</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>TC_CR_AUTH_NEG_04</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Stock Point (Seller)</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Verify user cannot proceed when Password field is empty or does not meet password policy requirements.</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Negative</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D69"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:O3"/>

</xml_diff>

<commit_message>
Return & Cancellation Policy
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -45,6 +45,7 @@
     <sheet name="Tenant super admin" sheetId="40" r:id="rId40"/>
     <sheet name="Partner (Tenant)" sheetId="41" r:id="rId41"/>
     <sheet name="StockPointSellerTest" sheetId="42" r:id="rId42"/>
+    <sheet name="Return Cancellation Regression" sheetId="43" r:id="rId43"/>
   </sheets>
 </workbook>
 </file>
@@ -5569,7 +5570,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-c91d2-values-when-no-data-exists--local\test-finished-1.png</v>
       </c>
       <c r="N20" t="str">
-        <v>15.49s</v>
+        <v>9.50s</v>
       </c>
     </row>
     <row r="21" xml:space="preserve">
@@ -5614,7 +5615,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-86927-hen-dataset-is-unavailable--local\test-finished-1.png</v>
       </c>
       <c r="N21" t="str">
-        <v>14.56s</v>
+        <v>9.39s</v>
       </c>
     </row>
     <row r="22" xml:space="preserve">
@@ -5660,7 +5661,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-7fb4c-vior-when-no-records-exist--local\test-finished-1.png</v>
       </c>
       <c r="N22" t="str">
-        <v>7.55s</v>
+        <v>8.49s</v>
       </c>
     </row>
     <row r="23" xml:space="preserve">
@@ -5706,7 +5707,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-c7401-vior-when-no-records-exist--local\test-finished-1.png</v>
       </c>
       <c r="N23" t="str">
-        <v>7.37s</v>
+        <v>7.83s</v>
       </c>
     </row>
     <row r="24" xml:space="preserve">
@@ -5752,7 +5753,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-0341f-e-handles-error-gracefully--local\test-finished-1.png</v>
       </c>
       <c r="N24" t="str">
-        <v>15.61s</v>
+        <v>8.39s</v>
       </c>
     </row>
     <row r="25" xml:space="preserve">
@@ -5797,7 +5798,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-624ab-y-Registration-Report-page--local\test-finished-1.png</v>
       </c>
       <c r="N25" t="str">
-        <v>5.86s</v>
+        <v>4.76s</v>
       </c>
     </row>
     <row r="26" xml:space="preserve">
@@ -5843,7 +5844,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-26b10-ch-text-returns-no-records--local\test-finished-1.png</v>
       </c>
       <c r="N26" t="str">
-        <v>6.34s</v>
+        <v>6.76s</v>
       </c>
     </row>
     <row r="27" xml:space="preserve">
@@ -5889,7 +5890,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-8549a--show-empty-state-in-table--local\test-finished-1.png</v>
       </c>
       <c r="N27" t="str">
-        <v>8.14s</v>
+        <v>8.35s</v>
       </c>
     </row>
     <row r="28" xml:space="preserve">
@@ -5934,7 +5935,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-6aef5-correctly-without-UI-crash--local\test-finished-1.png</v>
       </c>
       <c r="N28" t="str">
-        <v>3.19s</v>
+        <v>3.31s</v>
       </c>
     </row>
     <row r="29" xml:space="preserve">
@@ -5979,7 +5980,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-d3646-hen-no-records-are-present--local\test-finished-1.png</v>
       </c>
       <c r="N29" t="str">
-        <v>7.78s</v>
+        <v>8.20s</v>
       </c>
     </row>
     <row r="30" xml:space="preserve">
@@ -6024,7 +6025,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-70c1f-create-duplicate-downloads--local\test-finished-1.png</v>
       </c>
       <c r="N30" t="str">
-        <v>3.06s</v>
+        <v>3.52s</v>
       </c>
     </row>
     <row r="31" xml:space="preserve">
@@ -6069,7 +6070,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-fc69e-not-create-duplicate-files--local\test-finished-1.png</v>
       </c>
       <c r="N31" t="str">
-        <v>3.05s</v>
+        <v>3.42s</v>
       </c>
     </row>
     <row r="32" xml:space="preserve">
@@ -6116,7 +6117,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-2d476-eets-acceptable-thresholds--local\test-finished-1.png</v>
       </c>
       <c r="N32" t="str">
-        <v>7.40s</v>
+        <v>7.78s</v>
       </c>
     </row>
     <row r="33" xml:space="preserve">
@@ -6162,7 +6163,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-5547c--with-all-sections-visible--local\test-finished-1.png</v>
       </c>
       <c r="N33" t="str">
-        <v>4.71s</v>
+        <v>5.22s</v>
       </c>
     </row>
     <row r="34" xml:space="preserve">
@@ -6207,7 +6208,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-7916c-y-on-Download-History-page--local\test-finished-1.png</v>
       </c>
       <c r="N34" t="str">
-        <v>2.91s</v>
+        <v>3.02s</v>
       </c>
     </row>
     <row r="35" xml:space="preserve">
@@ -6252,7 +6253,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-f69a1--Customer-Report-correctly--local\test-finished-1.png</v>
       </c>
       <c r="N35" t="str">
-        <v>4.69s</v>
+        <v>4.94s</v>
       </c>
     </row>
     <row r="36">
@@ -6296,7 +6297,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-21b1d-d-column-headers-correctly--local\test-finished-1.png</v>
       </c>
       <c r="N36" t="str">
-        <v>3.00s</v>
+        <v>3.10s</v>
       </c>
     </row>
     <row r="37" xml:space="preserve">
@@ -6342,7 +6343,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-0f758-ry-page-when-records-exist--local\test-finished-1.png</v>
       </c>
       <c r="N37" t="str">
-        <v>5.04s</v>
+        <v>4.93s</v>
       </c>
     </row>
     <row r="38" xml:space="preserve">
@@ -6387,7 +6388,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-04fd2--no-download-records-exist--local\test-finished-1.png</v>
       </c>
       <c r="N38" t="str">
-        <v>2.98s</v>
+        <v>2.88s</v>
       </c>
     </row>
     <row r="39" xml:space="preserve">
@@ -6433,7 +6434,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-ed31f-les-API-failure-gracefully--local\test-finished-1.png</v>
       </c>
       <c r="N39" t="str">
-        <v>6.27s</v>
+        <v>6.37s</v>
       </c>
     </row>
     <row r="40" xml:space="preserve">
@@ -6478,7 +6479,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-a4379-rect-download-history-data--local\test-finished-1.png</v>
       </c>
       <c r="N40" t="str">
-        <v>3.19s</v>
+        <v>3.17s</v>
       </c>
     </row>
     <row r="41" xml:space="preserve">
@@ -6523,7 +6524,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-ac751-load-History-page-directly--local\test-finished-1.png</v>
       </c>
       <c r="N41" t="str">
-        <v>4.61s</v>
+        <v>4.80s</v>
       </c>
     </row>
     <row r="42" xml:space="preserve">
@@ -6568,7 +6569,7 @@
         <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\DailyRegistrationTest-Dail-54118-wnload-file-is-unavailable--local\test-finished-1.png</v>
       </c>
       <c r="N42" t="str">
-        <v>3.18s</v>
+        <v>3.02s</v>
       </c>
     </row>
   </sheetData>
@@ -24033,6 +24034,1722 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N36"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Test Case ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Module</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Screen Name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Test Scenario</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Test Case Type</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Preconditions</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Test Steps</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Test Data</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Expected Result</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Priority</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Actual Result</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Screenshot Path</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Execution Time</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>TC_RCP_001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Verify Return &amp; Cancellation Policy page loads via Setup sidebar with all 5 policy tabs visible.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F2" t="str">
+        <v>User is logged in as Tenant admin</v>
+      </c>
+      <c r="G2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. From Home page, expand Setup menu in sidebar
+2. Click 'Return &amp; Cancellation'
+3. Verify page heading visible
+4. Verify all 5 tabs (Cancellation, Return, Replacement, Refund, Market Policies) are present</v>
+      </c>
+      <c r="H2" t="str">
+        <v>URL: /setup/policy</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Page loads with heading and all 5 tabs visible</v>
+      </c>
+      <c r="J2" t="str">
+        <v>High</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>TC_RCP_002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Verify direct URL navigation to /setup/policy loads the Return &amp; Cancellation Policy page.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F3" t="str">
+        <v>User is logged in as Tenant admin</v>
+      </c>
+      <c r="G3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate directly to /setup/policy
+2. Verify page heading is visible
+3. Verify URL contains 'setup/policy'</v>
+      </c>
+      <c r="H3" t="str">
+        <v>URL: /setup/policy</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Page loads correctly with heading visible on direct navigation</v>
+      </c>
+      <c r="J3" t="str">
+        <v>High</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>TC_RCP_003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Verify Cancellation tab is active and displays all required fields.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F4" t="str">
+        <v>User is on Return &amp; Cancellation Policy page</v>
+      </c>
+      <c r="G4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to /setup/policy
+2. Click Cancellation tab
+3. Verify Window Minutes, Allowed Before Statuses, Free Cancellation Before Status, Fee Type, Cancellation Fee, Reasons fields are visible</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Tab: Cancellation</v>
+      </c>
+      <c r="I4" t="str">
+        <v>All Cancellation tab fields (Window Minutes, statuses, fee type, reasons) are visible</v>
+      </c>
+      <c r="J4" t="str">
+        <v>High</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>TC_RCP_004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Verify enabling Cancellation policy toggle and saving persists the enabled state.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Cancellation tab is active</v>
+      </c>
+      <c r="G5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Enable the Enabled toggle
+3. Click Save
+4. Re-navigate to page
+5. Verify toggle is still enabled</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Enabled: true</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Cancellation policy is enabled and persists after page reload</v>
+      </c>
+      <c r="J5" t="str">
+        <v>High</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>TC_RCP_005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Verify disabling Cancellation policy collapses conditional fields and saves.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Cancellation policy is currently enabled</v>
+      </c>
+      <c r="G6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Disable the Enabled toggle
+3. Click Save
+4. Verify save succeeds
+5. Re-enable for clean state</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Enabled: false</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Cancellation policy disabled state saves successfully; conditional fields hidden</v>
+      </c>
+      <c r="J6" t="str">
+        <v>High</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>TC_RCP_006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Verify Window Minutes accepts 0 (no time limit) and shows hint text.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Set Window Minutes to 0
+3. Verify '0 = no time limit' hint appears
+4. Click Save and verify success</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Window Minutes: 0</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Window Minutes 0 accepted, hint shown, save succeeds</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>TC_RCP_007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Verify Window Minutes accepts a valid positive value (60) and saves correctly.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G8" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Set Window Minutes to 60
+3. Click Save
+4. Verify success toast</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Window Minutes: 60</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Window Minutes 60 saved; success feedback displayed</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>TC_RCP_008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Verify Allowed Before Statuses multi-select adds PAYMENT_CONFIRMED and saves.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G9" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Open Allowed Before Statuses dropdown
+3. Select PAYMENT_CONFIRMED
+4. Click Save
+5. Verify success</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Status: PAYMENT_CONFIRMED</v>
+      </c>
+      <c r="I9" t="str">
+        <v>PAYMENT_CONFIRMED added to Allowed Before Statuses; saved successfully</v>
+      </c>
+      <c r="J9" t="str">
+        <v>High</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>TC_RCP_009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Verify Free Cancellation Before Status single-select selects INVENTORY_CONFIRMED and saves.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G10" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Open Free Cancellation Before Status dropdown
+3. Select INVENTORY_CONFIRMED
+4. Click Save
+5. Verify success</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Status: INVENTORY_CONFIRMED</v>
+      </c>
+      <c r="I10" t="str">
+        <v>INVENTORY_CONFIRMED selected and saved successfully</v>
+      </c>
+      <c r="J10" t="str">
+        <v>High</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>TC_RCP_010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Verify Fee Type FLAT with Cancellation Fee 50 saves correctly.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G11" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Select FLAT fee type
+3. Enter Cancellation Fee as 50
+4. Click Save
+5. Verify success</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Fee Type: FLAT, Fee: 50</v>
+      </c>
+      <c r="I11" t="str">
+        <v>FLAT fee type with 50 cancellation fee saved successfully</v>
+      </c>
+      <c r="J11" t="str">
+        <v>High</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>TC_RCP_011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Verify Fee Type PERCENTAGE with 10% saves correctly and resets to FLAT/0 afterwards.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G12" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Select PERCENTAGE fee type
+3. Enter 10 as fee
+4. Click Save
+5. Verify success
+6. Reset to FLAT/0</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Fee Type: PERCENTAGE, Fee: 10</v>
+      </c>
+      <c r="I12" t="str">
+        <v>PERCENTAGE fee type with 10% saved successfully; can be reset to FLAT/0</v>
+      </c>
+      <c r="J12" t="str">
+        <v>High</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>TC_RCP_012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Verify Auto Refund On Approval toggle saves and persists after reload.</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G13" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Enable Auto Refund On Approval toggle
+3. Click Save
+4. Re-navigate to page
+5. Verify toggle is still enabled</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Auto Refund On Approval: true</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Auto Refund On Approval toggle state persists after save and reload</v>
+      </c>
+      <c r="J13" t="str">
+        <v>High</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>TC_RCP_013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Verify COD Allowed toggle can be disabled and settings persist after save.</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G14" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Disable COD Allowed toggle
+3. Click Save
+4. Verify success
+5. Re-enable for clean state</v>
+      </c>
+      <c r="H14" t="str">
+        <v>COD Allowed: false</v>
+      </c>
+      <c r="I14" t="str">
+        <v>COD Allowed disabled state saves; re-enable restores default</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>TC_RCP_014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Verify adding a custom cancellation reason tag persists after save.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G15" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Type 'DAMAGED_PACKAGING' in Reasons input
+3. Press Enter to create tag
+4. Click Save
+5. Verify save succeeds</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Custom Reason: DAMAGED_PACKAGING</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Custom reason tag added and saved successfully</v>
+      </c>
+      <c r="J15" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>TC_RCP_015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Verify Return tab displays all required fields: Window Days, Item Types, Shipping Paid By, Restocking Fee.</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F16" t="str">
+        <v>User is on Return &amp; Cancellation Policy page</v>
+      </c>
+      <c r="G16" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Return &amp; Cancellation Policy
+2. Click Return tab
+3. Verify Window Days, Returnable Item Types, Non Returnable Item Types, Shipping Paid By, Restocking Fee fields are visible</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Tab: Return</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Return tab shows Window Days, item type fields, Shipping Paid By, Restocking Fee</v>
+      </c>
+      <c r="J16" t="str">
+        <v>High</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>TC_RCP_016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Verify enabling Return policy with Window Days 7 saves successfully.</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Return tab is active</v>
+      </c>
+      <c r="G17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Return tab
+2. Enable the Enabled toggle
+3. Set Window Days to 7
+4. Click Save
+5. Verify success</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Window Days: 7, Enabled: true</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Return policy enabled with 7-day window saves successfully</v>
+      </c>
+      <c r="J17" t="str">
+        <v>High</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>TC_RCP_017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Verify disabling Return policy toggle and saving succeeds.</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Return policy is currently enabled</v>
+      </c>
+      <c r="G18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Return tab
+2. Disable the Enabled toggle
+3. Click Save
+4. Verify save succeeds
+5. Re-enable for clean state</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Enabled: false</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Return policy disabled state saves; restore to enabled for clean state</v>
+      </c>
+      <c r="J18" t="str">
+        <v>High</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+      <c r="M18" t="str">
+        <v/>
+      </c>
+      <c r="N18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>TC_RCP_018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Verify adding returnable item type 'ELECTRONICS' as a tag and saving.</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Return tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Return tab
+2. Type 'ELECTRONICS' in Returnable Item Types input
+3. Press Enter
+4. Click Save
+5. Verify success</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Item Type: ELECTRONICS</v>
+      </c>
+      <c r="I19" t="str">
+        <v>ELECTRONICS tag added to Returnable Item Types and saved</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <v/>
+      </c>
+      <c r="N19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>TC_RCP_019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Verify enabling Require Images and setting Min Images to 2 saves correctly.</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Return tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Return tab
+2. Enable Require Images toggle
+3. Set Min Images to 2
+4. Click Save
+5. Verify success</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Require Images: true, Min Images: 2</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Require Images enabled with Min Images 2 saved successfully</v>
+      </c>
+      <c r="J20" t="str">
+        <v>High</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
+      <c r="M20" t="str">
+        <v/>
+      </c>
+      <c r="N20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>TC_RCP_020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Verify Restocking Fee (FLAT) set to 25 is saved correctly.</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Return tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Return tab
+2. Enter 25 in Restocking Fee field
+3. Click Save
+4. Verify success</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Restocking Fee: 25 (FLAT)</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Restocking Fee 25 saved; applied during return approval</v>
+      </c>
+      <c r="J21" t="str">
+        <v>High</v>
+      </c>
+      <c r="K21" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <v/>
+      </c>
+      <c r="N21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>TC_RCP_021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Verify Replacement tab displays Window Days, Shipping Paid By, Max Per Order, Require Original Return, Require Images fields.</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F22" t="str">
+        <v>User is on Return &amp; Cancellation Policy page</v>
+      </c>
+      <c r="G22" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Replacement tab
+2. Verify Window Days, Shipping Paid By, Max Per Order, Require Original Return, Require Images fields visible</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Tab: Replacement</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Replacement tab shows all expected fields</v>
+      </c>
+      <c r="J22" t="str">
+        <v>High</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L22" t="str">
+        <v/>
+      </c>
+      <c r="M22" t="str">
+        <v/>
+      </c>
+      <c r="N22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>TC_RCP_022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Verify enabling Replacement with Window Days 14 and Max Per Order 2 saves correctly.</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Replacement tab is active</v>
+      </c>
+      <c r="G23" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Replacement tab
+2. Enable Enabled toggle
+3. Set Window Days to 14
+4. Set Max Per Order to 2
+5. Click Save
+6. Verify success</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Enabled: true, Window Days: 14, Max Per Order: 2</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Replacement configured with 14-day window and max 2 per order saves successfully</v>
+      </c>
+      <c r="J23" t="str">
+        <v>High</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L23" t="str">
+        <v/>
+      </c>
+      <c r="M23" t="str">
+        <v/>
+      </c>
+      <c r="N23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>TC_RCP_023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Verify Require Original Return toggle saves and persists after reload.</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Replacement tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G24" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Replacement tab
+2. Enable Require Original Return toggle
+3. Click Save
+4. Re-navigate to page
+5. Verify Require Original Return is still enabled</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Require Original Return: true</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Require Original Return toggle persists after save and page reload</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
+      <c r="M24" t="str">
+        <v/>
+      </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>TC_RCP_024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Verify Require Images toggle on Replacement tab can be enabled and saved.</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Replacement tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G25" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Replacement tab
+2. Enable Require Images toggle
+3. Click Save
+4. Verify success</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Require Images: true (Replacement)</v>
+      </c>
+      <c r="I25" t="str">
+        <v>Require Images toggle enabled and saved on Replacement tab</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K25" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L25" t="str">
+        <v/>
+      </c>
+      <c r="M25" t="str">
+        <v/>
+      </c>
+      <c r="N25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>TC_RCP_025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Verify disabling Replacement policy saves and can be re-enabled for clean state.</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Replacement policy is currently enabled</v>
+      </c>
+      <c r="G26" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Replacement tab
+2. Disable Enabled toggle
+3. Click Save
+4. Verify success
+5. Re-enable for clean state</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Enabled: false (Replacement)</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Replacement disabled state saves; restore to enabled</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K26" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+      <c r="M26" t="str">
+        <v/>
+      </c>
+      <c r="N26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
+        <v>TC_RCP_026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Verify Refund tab displays Refund Method, COD Refund Method, Processing Days, and refund toggle fields.</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F27" t="str">
+        <v>User is on Return &amp; Cancellation Policy page</v>
+      </c>
+      <c r="G27" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Refund tab
+2. Verify Refund Method, COD Refund Method, Processing Days, Partial Refund Allowed, Shipping Refundable, Deduct Cancellation Fee, Deduct Restocking Fee fields are visible</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Tab: Refund</v>
+      </c>
+      <c r="I27" t="str">
+        <v>All Refund tab fields are visible</v>
+      </c>
+      <c r="J27" t="str">
+        <v>High</v>
+      </c>
+      <c r="K27" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
+      <c r="N27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
+        <v>TC_RCP_027</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Verify Refund Method (ORIGINAL_PAYMENT), COD Refund Method (WALLET), Processing Days 7 saves.</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Refund tab is active</v>
+      </c>
+      <c r="G28" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Refund tab
+2. Set Refund Method to ORIGINAL_PAYMENT
+3. Set COD Refund Method to WALLET
+4. Set Processing Days to 7
+5. Click Save
+6. Verify success</v>
+      </c>
+      <c r="H28" t="str">
+        <v>Refund: ORIGINAL_PAYMENT, COD: WALLET, Days: 7</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Refund configuration saves successfully</v>
+      </c>
+      <c r="J28" t="str">
+        <v>High</v>
+      </c>
+      <c r="K28" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L28" t="str">
+        <v/>
+      </c>
+      <c r="M28" t="str">
+        <v/>
+      </c>
+      <c r="N28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
+        <v>TC_RCP_028</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Verify Partial Refund Allowed and Shipping Refundable toggles save and Partial Refund Allowed persists.</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Refund tab is active</v>
+      </c>
+      <c r="G29" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Refund tab
+2. Enable Partial Refund Allowed toggle
+3. Enable Shipping Refundable toggle
+4. Click Save
+5. Re-navigate and verify Partial Refund Allowed is ON</v>
+      </c>
+      <c r="H29" t="str">
+        <v>Partial Refund: true, Shipping Refundable: true</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Both toggles enabled and Partial Refund Allowed persists after reload</v>
+      </c>
+      <c r="J29" t="str">
+        <v>High</v>
+      </c>
+      <c r="K29" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L29" t="str">
+        <v/>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
+      <c r="N29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30" xml:space="preserve">
+      <c r="A30" t="str">
+        <v>TC_RCP_029</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Verify Deduct Cancellation Fee and Deduct Restocking Fee toggles save and Deduct Cancellation Fee persists.</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Refund tab is active</v>
+      </c>
+      <c r="G30" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Refund tab
+2. Enable Deduct Cancellation Fee
+3. Enable Deduct Restocking Fee
+4. Click Save
+5. Re-navigate and verify Deduct Cancellation Fee is ON</v>
+      </c>
+      <c r="H30" t="str">
+        <v>Deduct Cancel Fee: true, Deduct Restocking Fee: true</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Both deduct toggles saved; Deduct Cancellation Fee persists after reload</v>
+      </c>
+      <c r="J30" t="str">
+        <v>High</v>
+      </c>
+      <c r="K30" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L30" t="str">
+        <v/>
+      </c>
+      <c r="M30" t="str">
+        <v/>
+      </c>
+      <c r="N30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31" xml:space="preserve">
+      <c r="A31" t="str">
+        <v>TC_RCP_030</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Verify Market Policies tab loads with Add Market button and empty-state or existing market list.</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F31" t="str">
+        <v>User is on Return &amp; Cancellation Policy page</v>
+      </c>
+      <c r="G31" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Market Policies tab
+2. Verify '+ Add Market' button is visible
+3. Verify empty state 'No market overrides configured' OR existing market rows are shown</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Tab: Market Policies</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Market Policies tab loads with Add Market button and empty state or market entries</v>
+      </c>
+      <c r="J31" t="str">
+        <v>High</v>
+      </c>
+      <c r="K31" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L31" t="str">
+        <v/>
+      </c>
+      <c r="M31" t="str">
+        <v/>
+      </c>
+      <c r="N31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
+      <c r="A32" t="str">
+        <v>TC_RCP_031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Verify clicking Add Market button opens Market Policy Override modal with all required fields.</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Market Policies tab is active</v>
+      </c>
+      <c r="G32" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Market Policies tab
+2. Click '+ Add Market'
+3. Verify modal opens with Market Name, Conditions fields
+4. Verify Override Cancellation/Return/Replacement/Refund toggles visible
+5. Click Cancel</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Modal: Market Policy Override</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Modal opens with all override fields; Cancel closes it without saving</v>
+      </c>
+      <c r="J32" t="str">
+        <v>High</v>
+      </c>
+      <c r="K32" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L32" t="str">
+        <v/>
+      </c>
+      <c r="M32" t="str">
+        <v/>
+      </c>
+      <c r="N32" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33" xml:space="preserve">
+      <c r="A33" t="str">
+        <v>TC_RCP_032</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Verify cancelling Market Policy modal discards changes without creating a new market override.</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Market Policies tab is active</v>
+      </c>
+      <c r="G33" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Market Policies tab
+2. Note current market count
+3. Click '+ Add Market'
+4. Click Cancel without filling any fields
+5. Verify modal is closed and no new market entry appeared</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Cancel without save</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Market modal closed; no new market override added on cancel</v>
+      </c>
+      <c r="J33" t="str">
+        <v>High</v>
+      </c>
+      <c r="K33" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L33" t="str">
+        <v/>
+      </c>
+      <c r="M33" t="str">
+        <v/>
+      </c>
+      <c r="N33" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34" xml:space="preserve">
+      <c r="A34" t="str">
+        <v>TC_RCP_033</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Verify unauthenticated user cannot access Return &amp; Cancellation Policy page directly.</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F34" t="str">
+        <v>User is NOT logged in</v>
+      </c>
+      <c r="G34" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open browser without authenticated session
+2. Navigate directly to /setup/policy
+3. Verify user is redirected to login page or access denied</v>
+      </c>
+      <c r="H34" t="str">
+        <v>URL: /setup/policy, No auth</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Unauthenticated access redirected to login page or access denied shown</v>
+      </c>
+      <c r="J34" t="str">
+        <v>High</v>
+      </c>
+      <c r="K34" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L34" t="str">
+        <v/>
+      </c>
+      <c r="M34" t="str">
+        <v/>
+      </c>
+      <c r="N34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35" xml:space="preserve">
+      <c r="A35" t="str">
+        <v>TC_RCP_034</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Verify API failure on Policy page load is handled gracefully without a JavaScript crash.</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F35" t="str">
+        <v>User is logged in as Tenant admin</v>
+      </c>
+      <c r="G35" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to /setup/policy
+2. Intercept and abort the policy API call
+3. Reload the page
+4. Verify app does not show uncaught JavaScript error</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Simulated API failure</v>
+      </c>
+      <c r="I35" t="str">
+        <v>App handles API failure gracefully — no uncaught JavaScript errors in page body</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K35" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L35" t="str">
+        <v/>
+      </c>
+      <c r="M35" t="str">
+        <v/>
+      </c>
+      <c r="N35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36" xml:space="preserve">
+      <c r="A36" t="str">
+        <v>TC_RCP_035</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Verify full cross-tab regression: configure and save Cancellation, Return, Replacement, and Refund tabs in sequence.</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F36" t="str">
+        <v>User is logged in as Tenant admin</v>
+      </c>
+      <c r="G36" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Configure Cancellation tab (Enabled, Window 0, FLAT 0) and Save
+2. Configure Return tab (Enabled, Window 7) and Save
+3. Configure Replacement tab (Enabled, Window 7, Max 1) and Save
+4. Configure Refund tab (ORIGINAL_PAYMENT, Days 7) and Save
+5. Verify each save succeeds</v>
+      </c>
+      <c r="H36" t="str">
+        <v>All tabs default/baseline values</v>
+      </c>
+      <c r="I36" t="str">
+        <v>All 4 policy tabs configured and saved in sequence without errors</v>
+      </c>
+      <c r="J36" t="str">
+        <v>High</v>
+      </c>
+      <c r="K36" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L36" t="str">
+        <v/>
+      </c>
+      <c r="M36" t="str">
+        <v/>
+      </c>
+      <c r="N36" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:N36"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K4"/>

</xml_diff>

<commit_message>
feat: add CustomerReportSuperAdmin automation and excel coverage
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -47,13 +47,14 @@
     <sheet sheetId="43" name="Permission( Super admin)" state="visible" r:id="rId44"/>
     <sheet sheetId="32" name="Subscription plans( Super admin" state="visible" r:id="rId45"/>
     <sheet sheetId="37" name="FeaturesSuperAdminTest" state="visible" r:id="rId46"/>
+    <sheet sheetId="44" name="Customer Report (Super Admin)" state="visible" r:id="rId47"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7481" uniqueCount="3503">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7763" uniqueCount="3610">
   <si>
     <t>TestName</t>
   </si>
@@ -10623,6 +10624,327 @@
   </si>
   <si>
     <t>Verify the application handles API/network failure gracefully during feature creation and displays an appropriate error message.</t>
+  </si>
+  <si>
+    <t>Search_Keyword</t>
+  </si>
+  <si>
+    <t>Report_Count</t>
+  </si>
+  <si>
+    <t>TC_CR_01</t>
+  </si>
+  <si>
+    <t>Verify Customer Report page loads successfully with customer records displayed.</t>
+  </si>
+  <si>
+    <t>TC_CR_02</t>
+  </si>
+  <si>
+    <t>Verify customer records are displayed with correct columns (Customer No, Name, Phone, Category).</t>
+  </si>
+  <si>
+    <t>TC_CR_03</t>
+  </si>
+  <si>
+    <t>Verify search functionality returns matching customer records for a valid Customer Number.</t>
+  </si>
+  <si>
+    <t>CCUZ0002</t>
+  </si>
+  <si>
+    <t>TC_CR_04</t>
+  </si>
+  <si>
+    <t>Verify search functionality returns matching customer records for a valid Customer Name.</t>
+  </si>
+  <si>
+    <t>Chetan Budhalakoti</t>
+  </si>
+  <si>
+    <t>TC_CR_05</t>
+  </si>
+  <si>
+    <t>Verify search functionality returns matching customer records for a valid Phone Number.</t>
+  </si>
+  <si>
+    <t>8279633139</t>
+  </si>
+  <si>
+    <t>TC_CR_06</t>
+  </si>
+  <si>
+    <t>Verify partial keyword search returns relevant customer records.</t>
+  </si>
+  <si>
+    <t>Chetan</t>
+  </si>
+  <si>
+    <t>TC_CR_07</t>
+  </si>
+  <si>
+    <t>Verify clicking Download Report downloads the customer report successfully.</t>
+  </si>
+  <si>
+    <t>TC_CR_08</t>
+  </si>
+  <si>
+    <t>Verify downloaded report contains all displayed customer data.</t>
+  </si>
+  <si>
+    <t>TC_CR_09</t>
+  </si>
+  <si>
+    <t>Verify Refresh button reloads the latest customer records.</t>
+  </si>
+  <si>
+    <t>TC_CR_10</t>
+  </si>
+  <si>
+    <t>Verify pagination displays records for the selected page correctly.</t>
+  </si>
+  <si>
+    <t>TC_CR_11</t>
+  </si>
+  <si>
+    <t>Verify clicking Next navigates to the next page of records.</t>
+  </si>
+  <si>
+    <t>TC_CR_12</t>
+  </si>
+  <si>
+    <t>Verify clicking a specific page number loads corresponding records.</t>
+  </si>
+  <si>
+    <t>TC_CR_13</t>
+  </si>
+  <si>
+    <t>Verify customer category is displayed correctly for all records.</t>
+  </si>
+  <si>
+    <t>TC_CR_14</t>
+  </si>
+  <si>
+    <t>Verify table data remains intact after page refresh.</t>
+  </si>
+  <si>
+    <t>TC_CR_15</t>
+  </si>
+  <si>
+    <t>Verify search results are updated correctly after clearing and entering new search criteria.</t>
+  </si>
+  <si>
+    <t>CHTQ0006</t>
+  </si>
+  <si>
+    <t>TC_CR_NEG_01</t>
+  </si>
+  <si>
+    <t>Verify search with invalid Customer Number returns no records found.</t>
+  </si>
+  <si>
+    <t>INVALID999</t>
+  </si>
+  <si>
+    <t>TC_CR_NEG_02</t>
+  </si>
+  <si>
+    <t>Verify search with non-existing Customer Name returns no records found.</t>
+  </si>
+  <si>
+    <t>NonExistingUser</t>
+  </si>
+  <si>
+    <t>TC_CR_NEG_03</t>
+  </si>
+  <si>
+    <t>Verify search with invalid Phone Number returns no records found.</t>
+  </si>
+  <si>
+    <t>0000000000</t>
+  </si>
+  <si>
+    <t>TC_CR_NEG_04</t>
+  </si>
+  <si>
+    <t>Verify search field accepts special characters without causing application errors.</t>
+  </si>
+  <si>
+    <t>TC_CR_NEG_05</t>
+  </si>
+  <si>
+    <t>Verify SQL injection strings entered in search field do not affect application behavior.</t>
+  </si>
+  <si>
+    <t>TC_CR_NEG_06</t>
+  </si>
+  <si>
+    <t>Verify XSS payloads entered in search field are sanitized and not executed.</t>
+  </si>
+  <si>
+    <t>TC_CR_NEG_07</t>
+  </si>
+  <si>
+    <t>Verify search with only blank spaces does not return incorrect results.</t>
+  </si>
+  <si>
+    <t>TC_CR_NEG_08</t>
+  </si>
+  <si>
+    <t>Verify extremely long search input is handled without UI breakage.</t>
+  </si>
+  <si>
+    <t>TC_CR_NEG_09</t>
+  </si>
+  <si>
+    <t>Verify Download Report handles API failure gracefully with an error message.</t>
+  </si>
+  <si>
+    <t>TC_CR_NEG_10</t>
+  </si>
+  <si>
+    <t>Verify Refresh button handles backend service failure correctly.</t>
+  </si>
+  <si>
+    <t>TC_CR_NEG_11</t>
+  </si>
+  <si>
+    <t>Verify pagination controls are disabled when only one page of records exists.</t>
+  </si>
+  <si>
+    <t>TC_CR_NEG_12</t>
+  </si>
+  <si>
+    <t>TC_CR_NEG_13</t>
+  </si>
+  <si>
+    <t>Verify invalid page number manipulation via URL does not break the page.</t>
+  </si>
+  <si>
+    <t>TC_CR_NEG_14</t>
+  </si>
+  <si>
+    <t>Verify empty customer dataset displays appropriate 'No Records Found' message.</t>
+  </si>
+  <si>
+    <t>XYZZY123</t>
+  </si>
+  <si>
+    <t>TC_CR_NEG_15</t>
+  </si>
+  <si>
+    <t>Verify unauthorized users cannot access the Customer Report page directly.</t>
+  </si>
+  <si>
+    <t>TC_CR_DL_01</t>
+  </si>
+  <si>
+    <t>Verify the Download Report popup opens successfully when the user clicks Download Report.</t>
+  </si>
+  <si>
+    <t>TC_CR_DL_02</t>
+  </si>
+  <si>
+    <t>Verify the user can enter a valid report count (e.g., 10) and download starts successfully.</t>
+  </si>
+  <si>
+    <t>TC_CR_DL_03</t>
+  </si>
+  <si>
+    <t>Verify the minimum allowed report count (e.g., 1) is accepted and downloaded correctly.</t>
+  </si>
+  <si>
+    <t>TC_CR_DL_04</t>
+  </si>
+  <si>
+    <t>Verify the maximum allowed report count is accepted and report generation completes successfully.</t>
+  </si>
+  <si>
+    <t>9999</t>
+  </si>
+  <si>
+    <t>TC_CR_DL_05</t>
+  </si>
+  <si>
+    <t>Verify the Download button downloads the exact number of reports entered.</t>
+  </si>
+  <si>
+    <t>TC_CR_DL_06</t>
+  </si>
+  <si>
+    <t>Verify clicking Cancel closes the popup without downloading any report.</t>
+  </si>
+  <si>
+    <t>TC_CR_DL_07</t>
+  </si>
+  <si>
+    <t>Verify the numeric input field accepts only numeric values.</t>
+  </si>
+  <si>
+    <t>123</t>
+  </si>
+  <si>
+    <t>TC_CR_DL_08</t>
+  </si>
+  <si>
+    <t>Verify the downloaded file is generated successfully and contains valid customer report data.</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>TC_CR_DL_NEG_01</t>
+  </si>
+  <si>
+    <t>Verify clicking Download without entering a report count displays a validation error.</t>
+  </si>
+  <si>
+    <t>TC_CR_DL_NEG_02</t>
+  </si>
+  <si>
+    <t>Verify entering 0 as the report count is rejected.</t>
+  </si>
+  <si>
+    <t>TC_CR_DL_NEG_03</t>
+  </si>
+  <si>
+    <t>Verify entering a negative value (e.g., -5) is not accepted.</t>
+  </si>
+  <si>
+    <t>TC_CR_DL_NEG_04</t>
+  </si>
+  <si>
+    <t>Verify entering alphabetic characters (e.g., 'ABC') in the report count field is prevented.</t>
+  </si>
+  <si>
+    <t>TC_CR_DL_NEG_05</t>
+  </si>
+  <si>
+    <t>Verify entering special characters (e.g., @#$%) in the report count field is rejected.</t>
+  </si>
+  <si>
+    <t>TC_CR_DL_NEG_06</t>
+  </si>
+  <si>
+    <t>Verify entering decimal values (e.g., 5.5) is not accepted if only integers are allowed.</t>
+  </si>
+  <si>
+    <t>5.5</t>
+  </si>
+  <si>
+    <t>TC_CR_DL_NEG_07</t>
+  </si>
+  <si>
+    <t>Verify entering a value greater than the allowed maximum limit displays an error message.</t>
+  </si>
+  <si>
+    <t>10001</t>
+  </si>
+  <si>
+    <t>TC_CR_DL_NEG_08</t>
+  </si>
+  <si>
+    <t>Verify clicking Download during API/report generation failure displays an appropriate error message without crashing the application.</t>
   </si>
 </sst>
 </file>
@@ -10666,9 +10988,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -27255,7 +27578,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -36406,6 +36729,965 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F47"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="50" customWidth="1"/>
+    <col min="4" max="4" width="25" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="50" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>1198</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1050</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3503</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3504</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>1203</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3505</v>
+      </c>
+      <c r="B2" t="s">
+        <v>761</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3506</v>
+      </c>
+      <c r="D2" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F2" t="s">
+        <v>3506</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3507</v>
+      </c>
+      <c r="B3" t="s">
+        <v>761</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3508</v>
+      </c>
+      <c r="D3" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E3" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F3" t="s">
+        <v>3508</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3509</v>
+      </c>
+      <c r="B4" t="s">
+        <v>761</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3510</v>
+      </c>
+      <c r="D4" t="s">
+        <v>3511</v>
+      </c>
+      <c r="E4" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F4" t="s">
+        <v>3510</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3512</v>
+      </c>
+      <c r="B5" t="s">
+        <v>761</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3513</v>
+      </c>
+      <c r="D5" t="s">
+        <v>3514</v>
+      </c>
+      <c r="E5" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F5" t="s">
+        <v>3513</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3515</v>
+      </c>
+      <c r="B6" t="s">
+        <v>761</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3516</v>
+      </c>
+      <c r="D6" t="s">
+        <v>3517</v>
+      </c>
+      <c r="E6" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F6" t="s">
+        <v>3516</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3518</v>
+      </c>
+      <c r="B7" t="s">
+        <v>761</v>
+      </c>
+      <c r="C7" t="s">
+        <v>3519</v>
+      </c>
+      <c r="D7" t="s">
+        <v>3520</v>
+      </c>
+      <c r="E7" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F7" t="s">
+        <v>3519</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3521</v>
+      </c>
+      <c r="B8" t="s">
+        <v>761</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3522</v>
+      </c>
+      <c r="D8" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E8" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F8" t="s">
+        <v>3522</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3523</v>
+      </c>
+      <c r="B9" t="s">
+        <v>761</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3524</v>
+      </c>
+      <c r="D9" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E9" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F9" t="s">
+        <v>3524</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3525</v>
+      </c>
+      <c r="B10" t="s">
+        <v>761</v>
+      </c>
+      <c r="C10" t="s">
+        <v>3526</v>
+      </c>
+      <c r="D10" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E10" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F10" t="s">
+        <v>3526</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3527</v>
+      </c>
+      <c r="B11" t="s">
+        <v>761</v>
+      </c>
+      <c r="C11" t="s">
+        <v>3528</v>
+      </c>
+      <c r="D11" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E11" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F11" t="s">
+        <v>3528</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3529</v>
+      </c>
+      <c r="B12" t="s">
+        <v>761</v>
+      </c>
+      <c r="C12" t="s">
+        <v>3530</v>
+      </c>
+      <c r="D12" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E12" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F12" t="s">
+        <v>3530</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3531</v>
+      </c>
+      <c r="B13" t="s">
+        <v>761</v>
+      </c>
+      <c r="C13" t="s">
+        <v>3532</v>
+      </c>
+      <c r="D13" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E13" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F13" t="s">
+        <v>3532</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3533</v>
+      </c>
+      <c r="B14" t="s">
+        <v>761</v>
+      </c>
+      <c r="C14" t="s">
+        <v>3534</v>
+      </c>
+      <c r="D14" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E14" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F14" t="s">
+        <v>3534</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>3535</v>
+      </c>
+      <c r="B15" t="s">
+        <v>761</v>
+      </c>
+      <c r="C15" t="s">
+        <v>3536</v>
+      </c>
+      <c r="D15" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E15" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F15" t="s">
+        <v>3536</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>3537</v>
+      </c>
+      <c r="B16" t="s">
+        <v>761</v>
+      </c>
+      <c r="C16" t="s">
+        <v>3538</v>
+      </c>
+      <c r="D16" t="s">
+        <v>3539</v>
+      </c>
+      <c r="E16" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F16" t="s">
+        <v>3538</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>3540</v>
+      </c>
+      <c r="B17" t="s">
+        <v>879</v>
+      </c>
+      <c r="C17" t="s">
+        <v>3541</v>
+      </c>
+      <c r="D17" t="s">
+        <v>3542</v>
+      </c>
+      <c r="E17" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F17" t="s">
+        <v>3541</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>3543</v>
+      </c>
+      <c r="B18" t="s">
+        <v>879</v>
+      </c>
+      <c r="C18" t="s">
+        <v>3544</v>
+      </c>
+      <c r="D18" t="s">
+        <v>3545</v>
+      </c>
+      <c r="E18" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F18" t="s">
+        <v>3544</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>3546</v>
+      </c>
+      <c r="B19" t="s">
+        <v>879</v>
+      </c>
+      <c r="C19" t="s">
+        <v>3547</v>
+      </c>
+      <c r="D19" t="s">
+        <v>3548</v>
+      </c>
+      <c r="E19" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F19" t="s">
+        <v>3547</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>3549</v>
+      </c>
+      <c r="B20" t="s">
+        <v>879</v>
+      </c>
+      <c r="C20" t="s">
+        <v>3550</v>
+      </c>
+      <c r="D20" t="s">
+        <v>441</v>
+      </c>
+      <c r="E20" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F20" t="s">
+        <v>3550</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>3551</v>
+      </c>
+      <c r="B21" t="s">
+        <v>879</v>
+      </c>
+      <c r="C21" t="s">
+        <v>3552</v>
+      </c>
+      <c r="D21" t="s">
+        <v>3292</v>
+      </c>
+      <c r="E21" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F21" t="s">
+        <v>3552</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>3553</v>
+      </c>
+      <c r="B22" t="s">
+        <v>879</v>
+      </c>
+      <c r="C22" t="s">
+        <v>3554</v>
+      </c>
+      <c r="D22" t="s">
+        <v>3117</v>
+      </c>
+      <c r="E22" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F22" t="s">
+        <v>3554</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>3555</v>
+      </c>
+      <c r="B23" t="s">
+        <v>879</v>
+      </c>
+      <c r="C23" t="s">
+        <v>3556</v>
+      </c>
+      <c r="D23" t="s">
+        <v>2075</v>
+      </c>
+      <c r="E23" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F23" t="s">
+        <v>3556</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>3557</v>
+      </c>
+      <c r="B24" t="s">
+        <v>879</v>
+      </c>
+      <c r="C24" t="s">
+        <v>3558</v>
+      </c>
+      <c r="D24" t="s">
+        <v>3120</v>
+      </c>
+      <c r="E24" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F24" t="s">
+        <v>3558</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>3559</v>
+      </c>
+      <c r="B25" t="s">
+        <v>879</v>
+      </c>
+      <c r="C25" t="s">
+        <v>3560</v>
+      </c>
+      <c r="D25" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E25" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F25" t="s">
+        <v>3560</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>3561</v>
+      </c>
+      <c r="B26" t="s">
+        <v>879</v>
+      </c>
+      <c r="C26" t="s">
+        <v>3562</v>
+      </c>
+      <c r="D26" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E26" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F26" t="s">
+        <v>3562</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>3563</v>
+      </c>
+      <c r="B27" t="s">
+        <v>879</v>
+      </c>
+      <c r="C27" t="s">
+        <v>3564</v>
+      </c>
+      <c r="D27" t="s">
+        <v>3511</v>
+      </c>
+      <c r="E27" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F27" t="s">
+        <v>3564</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>3565</v>
+      </c>
+      <c r="B28" t="s">
+        <v>879</v>
+      </c>
+      <c r="C28" t="s">
+        <v>2363</v>
+      </c>
+      <c r="D28" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E28" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F28" t="s">
+        <v>2363</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>3566</v>
+      </c>
+      <c r="B29" t="s">
+        <v>879</v>
+      </c>
+      <c r="C29" t="s">
+        <v>3567</v>
+      </c>
+      <c r="D29" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E29" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F29" t="s">
+        <v>3567</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>3568</v>
+      </c>
+      <c r="B30" t="s">
+        <v>879</v>
+      </c>
+      <c r="C30" t="s">
+        <v>3569</v>
+      </c>
+      <c r="D30" t="s">
+        <v>3570</v>
+      </c>
+      <c r="E30" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F30" t="s">
+        <v>3569</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>3571</v>
+      </c>
+      <c r="B31" t="s">
+        <v>879</v>
+      </c>
+      <c r="C31" t="s">
+        <v>3572</v>
+      </c>
+      <c r="D31" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E31" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F31" t="s">
+        <v>3572</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>3573</v>
+      </c>
+      <c r="B32" t="s">
+        <v>761</v>
+      </c>
+      <c r="C32" t="s">
+        <v>3574</v>
+      </c>
+      <c r="D32" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E32" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F32" t="s">
+        <v>3574</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>3575</v>
+      </c>
+      <c r="B33" t="s">
+        <v>761</v>
+      </c>
+      <c r="C33" t="s">
+        <v>3576</v>
+      </c>
+      <c r="D33" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E33" t="s">
+        <v>504</v>
+      </c>
+      <c r="F33" t="s">
+        <v>3576</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>3577</v>
+      </c>
+      <c r="B34" t="s">
+        <v>761</v>
+      </c>
+      <c r="C34" t="s">
+        <v>3578</v>
+      </c>
+      <c r="D34" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E34" t="s">
+        <v>2910</v>
+      </c>
+      <c r="F34" t="s">
+        <v>3578</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>3579</v>
+      </c>
+      <c r="B35" t="s">
+        <v>761</v>
+      </c>
+      <c r="C35" t="s">
+        <v>3580</v>
+      </c>
+      <c r="D35" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E35" t="s">
+        <v>3581</v>
+      </c>
+      <c r="F35" t="s">
+        <v>3580</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>3582</v>
+      </c>
+      <c r="B36" t="s">
+        <v>761</v>
+      </c>
+      <c r="C36" t="s">
+        <v>3583</v>
+      </c>
+      <c r="D36" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E36" t="s">
+        <v>1168</v>
+      </c>
+      <c r="F36" t="s">
+        <v>3583</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>3584</v>
+      </c>
+      <c r="B37" t="s">
+        <v>761</v>
+      </c>
+      <c r="C37" t="s">
+        <v>3585</v>
+      </c>
+      <c r="D37" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E37" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F37" t="s">
+        <v>3585</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>3586</v>
+      </c>
+      <c r="B38" t="s">
+        <v>761</v>
+      </c>
+      <c r="C38" t="s">
+        <v>3587</v>
+      </c>
+      <c r="D38" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E38" t="s">
+        <v>3588</v>
+      </c>
+      <c r="F38" t="s">
+        <v>3587</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>3589</v>
+      </c>
+      <c r="B39" t="s">
+        <v>761</v>
+      </c>
+      <c r="C39" t="s">
+        <v>3590</v>
+      </c>
+      <c r="D39" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E39" t="s">
+        <v>3591</v>
+      </c>
+      <c r="F39" t="s">
+        <v>3590</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>3592</v>
+      </c>
+      <c r="B40" t="s">
+        <v>879</v>
+      </c>
+      <c r="C40" t="s">
+        <v>3593</v>
+      </c>
+      <c r="D40" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E40" t="s">
+        <v>3095</v>
+      </c>
+      <c r="F40" t="s">
+        <v>3593</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>3594</v>
+      </c>
+      <c r="B41" t="s">
+        <v>879</v>
+      </c>
+      <c r="C41" t="s">
+        <v>3595</v>
+      </c>
+      <c r="D41" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E41" t="s">
+        <v>1171</v>
+      </c>
+      <c r="F41" t="s">
+        <v>3595</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>3596</v>
+      </c>
+      <c r="B42" t="s">
+        <v>879</v>
+      </c>
+      <c r="C42" t="s">
+        <v>3597</v>
+      </c>
+      <c r="D42" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E42" t="s">
+        <v>2988</v>
+      </c>
+      <c r="F42" t="s">
+        <v>3597</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>3598</v>
+      </c>
+      <c r="B43" t="s">
+        <v>879</v>
+      </c>
+      <c r="C43" t="s">
+        <v>3599</v>
+      </c>
+      <c r="D43" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E43" t="s">
+        <v>2984</v>
+      </c>
+      <c r="F43" t="s">
+        <v>3599</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>3600</v>
+      </c>
+      <c r="B44" t="s">
+        <v>879</v>
+      </c>
+      <c r="C44" t="s">
+        <v>3601</v>
+      </c>
+      <c r="D44" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E44" t="s">
+        <v>441</v>
+      </c>
+      <c r="F44" t="s">
+        <v>3601</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>3602</v>
+      </c>
+      <c r="B45" t="s">
+        <v>879</v>
+      </c>
+      <c r="C45" t="s">
+        <v>3603</v>
+      </c>
+      <c r="D45" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E45" t="s">
+        <v>3604</v>
+      </c>
+      <c r="F45" t="s">
+        <v>3603</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>3605</v>
+      </c>
+      <c r="B46" t="s">
+        <v>879</v>
+      </c>
+      <c r="C46" t="s">
+        <v>3606</v>
+      </c>
+      <c r="D46" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E46" t="s">
+        <v>3607</v>
+      </c>
+      <c r="F46" t="s">
+        <v>3606</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>3608</v>
+      </c>
+      <c r="B47" t="s">
+        <v>879</v>
+      </c>
+      <c r="C47" t="s">
+        <v>3609</v>
+      </c>
+      <c r="D47" t="s">
+        <v>3095</v>
+      </c>
+      <c r="E47" t="s">
+        <v>504</v>
+      </c>
+      <c r="F47" t="s">
+        <v>3609</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K4"/>

</xml_diff>

<commit_message>
fix: restore PaymentHistory, ReturnCancellation and OfficeManagement sheets
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -56,6 +56,10 @@
     <sheet name="Subscription plans( Super admin" sheetId="51" r:id="rId51"/>
     <sheet name="Customer Report (Super Admin)" sheetId="52" r:id="rId52"/>
     <sheet name="FAQ (Tenant)" sheetId="53" r:id="rId53"/>
+    <sheet name="PaymentHistory" sheetId="54" r:id="rId54"/>
+    <sheet name="Payment History Regression" sheetId="55" r:id="rId55"/>
+    <sheet name="Return Cancellation Regression" sheetId="56" r:id="rId56"/>
+    <sheet name="OfficeManagement" sheetId="57" r:id="rId57"/>
   </sheets>
 </workbook>
 </file>
@@ -19151,7 +19155,7 @@
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -19670,10 +19674,20 @@
         <v>serial</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>OfficeManagementTest</v>
+      </c>
+      <c r="B48" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C48" t="str">
+        <v>serial</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C48"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -57473,6 +57487,4643 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H51"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>TestID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Description</v>
+      </c>
+      <c r="C1" t="str">
+        <v>TimePeriod</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Provider</v>
+      </c>
+      <c r="E1" t="str">
+        <v>PaymentStatus</v>
+      </c>
+      <c r="F1" t="str">
+        <v>TransactionID</v>
+      </c>
+      <c r="G1" t="str">
+        <v>ExpectedResult</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Run</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>TC_PH_001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Verify Payment History page loads successfully</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>Page heading visible</v>
+      </c>
+      <c r="H2" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>TC_PH_002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Verify Time Period dropdown displays all available options</v>
+      </c>
+      <c r="C3" t="str">
+        <v>All</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>5 options visible</v>
+      </c>
+      <c r="H3" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TC_PH_003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Verify user can select Last 7 Days filter</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Last 7 days</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>Filter applied, page stable</v>
+      </c>
+      <c r="H4" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TC_PH_004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Verify user can select Last 15 Days filter</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Last 15 days</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>Filter applied, page stable</v>
+      </c>
+      <c r="H5" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TC_PH_005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Verify user can select Last 30 Days filter</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Last 30 days</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>Filter applied, page stable</v>
+      </c>
+      <c r="H6" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TC_PH_006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Verify user can select Last 3 Months filter</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Last 3 Months</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v>Filter applied, page stable</v>
+      </c>
+      <c r="H7" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TC_PH_007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Verify user can select Last 6 Months filter</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Last 6 Months</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v>Filter applied, page stable</v>
+      </c>
+      <c r="H8" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TC_PH_008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Verify Provider dropdown displays all providers</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v>All</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v>5 provider options visible</v>
+      </c>
+      <c r="H9" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TC_PH_009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Verify user can select Branch Office provider</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v>Branch Office</v>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v>Filter applied, page stable</v>
+      </c>
+      <c r="H10" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TC_PH_010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Verify user can select Fresh Market provider</v>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v>Fresh Market</v>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v>Filter applied, page stable</v>
+      </c>
+      <c r="H11" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TC_PH_011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Verify user can select Fresh Town Market provider</v>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v>Fresh Town Market</v>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v>Filter applied, page stable</v>
+      </c>
+      <c r="H12" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TC_PH_012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Verify user can select Green Market provider</v>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v>Green Market</v>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v>Filter applied, page stable</v>
+      </c>
+      <c r="H13" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TC_PH_013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Verify Payment Status dropdown displays all status values</v>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v>All</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v>5 status options visible</v>
+      </c>
+      <c r="H14" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TC_PH_014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Verify user can select Pending status</v>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v>PENDING</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v>Filter applied, page stable</v>
+      </c>
+      <c r="H15" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TC_PH_015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Verify user can select Refunded status</v>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v>REFUNDED</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v>Filter applied, page stable</v>
+      </c>
+      <c r="H16" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TC_PH_016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Verify user can select Paid status</v>
+      </c>
+      <c r="C17" t="str">
+        <v/>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v>PAID</v>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v>Filter applied, page stable</v>
+      </c>
+      <c r="H17" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TC_PH_017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Verify user can select Cancelled status</v>
+      </c>
+      <c r="C18" t="str">
+        <v/>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+      <c r="E18" t="str">
+        <v>CANCELLED</v>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v>Filter applied, page stable</v>
+      </c>
+      <c r="H18" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TC_PH_018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Verify user can select Failed status</v>
+      </c>
+      <c r="C19" t="str">
+        <v/>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v>FAILED</v>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v>Filter applied, page stable</v>
+      </c>
+      <c r="H19" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TC_PH_019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Verify Search works using valid Transaction ID</v>
+      </c>
+      <c r="C20" t="str">
+        <v/>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v>ORD-</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Page stable, results shown</v>
+      </c>
+      <c r="H20" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TC_PH_020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Verify Search returns matching transaction details</v>
+      </c>
+      <c r="C21" t="str">
+        <v/>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v>first-row-dynamic</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Matching row shown</v>
+      </c>
+      <c r="H21" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>TC_PH_021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Verify Refresh button reloads latest data</v>
+      </c>
+      <c r="C22" t="str">
+        <v/>
+      </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v>Page reloads, table loaded</v>
+      </c>
+      <c r="H22" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>TC_PH_022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Verify KPI cards display values</v>
+      </c>
+      <c r="C23" t="str">
+        <v/>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <v>All 3 KPI cards visible</v>
+      </c>
+      <c r="H23" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TC_PH_023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Verify Visible Transactions count is displayed</v>
+      </c>
+      <c r="C24" t="str">
+        <v/>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v>Non-empty numeric value</v>
+      </c>
+      <c r="H24" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TC_PH_024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Verify Visible Amount is displayed</v>
+      </c>
+      <c r="C25" t="str">
+        <v/>
+      </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <v>Non-empty currency value</v>
+      </c>
+      <c r="H25" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TC_PH_025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Verify Paid Transactions count is displayed</v>
+      </c>
+      <c r="C26" t="str">
+        <v/>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
+      <c r="G26" t="str">
+        <v>Non-empty numeric value</v>
+      </c>
+      <c r="H26" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TC_PH_026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Verify table loads transaction records</v>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v>Table with column headers shown</v>
+      </c>
+      <c r="H27" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TC_PH_027</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Verify Transaction ID column displays values</v>
+      </c>
+      <c r="C28" t="str">
+        <v/>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v>Column header &amp; values present</v>
+      </c>
+      <c r="H28" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>TC_PH_028</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Verify Customer column displays values</v>
+      </c>
+      <c r="C29" t="str">
+        <v/>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v>Column header &amp; values present</v>
+      </c>
+      <c r="H29" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TC_PH_029</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Verify Payment Type column displays values</v>
+      </c>
+      <c r="C30" t="str">
+        <v/>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
+      <c r="G30" t="str">
+        <v>Column header &amp; values present</v>
+      </c>
+      <c r="H30" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TC_PH_030</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Verify Amount column displays values</v>
+      </c>
+      <c r="C31" t="str">
+        <v/>
+      </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
+      <c r="F31" t="str">
+        <v/>
+      </c>
+      <c r="G31" t="str">
+        <v>Column header &amp; values present</v>
+      </c>
+      <c r="H31" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>TC_PH_031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Verify Payment Status column displays values</v>
+      </c>
+      <c r="C32" t="str">
+        <v/>
+      </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
+      <c r="F32" t="str">
+        <v/>
+      </c>
+      <c r="G32" t="str">
+        <v>Column header &amp; values present</v>
+      </c>
+      <c r="H32" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>TC_PH_032</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Verify Date column displays values</v>
+      </c>
+      <c r="C33" t="str">
+        <v/>
+      </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
+      <c r="G33" t="str">
+        <v>Column header &amp; values present</v>
+      </c>
+      <c r="H33" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TC_PH_033</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Verify filtered records update after Time Period selection</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Last 30 days</v>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34" t="str">
+        <v>Table refreshes after filter</v>
+      </c>
+      <c r="H34" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>TC_PH_034</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Verify filtered records update after Provider selection</v>
+      </c>
+      <c r="C35" t="str">
+        <v/>
+      </c>
+      <c r="D35" t="str">
+        <v>All Providers</v>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35" t="str">
+        <v>Table refreshes after filter</v>
+      </c>
+      <c r="H35" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TC_PH_035</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Verify filtered records update after Payment Status selection</v>
+      </c>
+      <c r="C36" t="str">
+        <v/>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v>PAID</v>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <v>Table refreshes after filter</v>
+      </c>
+      <c r="H36" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TC_PH_036</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Verify Search with invalid Transaction ID shows no records found</v>
+      </c>
+      <c r="C37" t="str">
+        <v/>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v>INVALID-TXN-XYZ999999</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Empty state / no-results msg</v>
+      </c>
+      <c r="H37" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>TC_PH_037</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Verify Search with special characters is handled properly</v>
+      </c>
+      <c r="C38" t="str">
+        <v/>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
+      <c r="F38" t="str">
+        <v>!@#$%^&amp;*()</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Page remains stable</v>
+      </c>
+      <c r="H38" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>TC_PH_038</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Verify Search with blank value does not break the page</v>
+      </c>
+      <c r="C39" t="str">
+        <v/>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
+      <c r="F39" t="str">
+        <v xml:space="preserve">   </v>
+      </c>
+      <c r="G39" t="str">
+        <v>Page remains stable</v>
+      </c>
+      <c r="H39" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>TC_PH_039</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Verify page handles API failure gracefully</v>
+      </c>
+      <c r="C40" t="str">
+        <v/>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+      <c r="G40" t="str">
+        <v>No crash, graceful degradation</v>
+      </c>
+      <c r="H40" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>TC_PH_040</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Verify KPI cards show zero/default values when no data exists</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Last 7 days</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Branch Office</v>
+      </c>
+      <c r="E41" t="str">
+        <v>FAILED</v>
+      </c>
+      <c r="F41" t="str">
+        <v/>
+      </c>
+      <c r="G41" t="str">
+        <v>KPI cards visible, page stable</v>
+      </c>
+      <c r="H41" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>TC_PH_041</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Verify table handles empty dataset correctly</v>
+      </c>
+      <c r="C42" t="str">
+        <v/>
+      </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
+      <c r="F42" t="str">
+        <v>EMPTY-DATASET-TEST-99999</v>
+      </c>
+      <c r="G42" t="str">
+        <v>Page stable</v>
+      </c>
+      <c r="H42" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>TC_PH_042</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Verify Provider filter handles no matching records</v>
+      </c>
+      <c r="C43" t="str">
+        <v/>
+      </c>
+      <c r="D43" t="str">
+        <v>Green Market</v>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
+      <c r="G43" t="str">
+        <v>Page stable, empty or few rows</v>
+      </c>
+      <c r="H43" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>TC_PH_043</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Verify Payment Status filter handles no matching records</v>
+      </c>
+      <c r="C44" t="str">
+        <v/>
+      </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
+      <c r="E44" t="str">
+        <v>REFUNDED</v>
+      </c>
+      <c r="F44" t="str">
+        <v/>
+      </c>
+      <c r="G44" t="str">
+        <v>Page stable, empty or few rows</v>
+      </c>
+      <c r="H44" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>TC_PH_044</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Verify Time Period filter handles no data scenario</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Last 7 days</v>
+      </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
+      <c r="F45" t="str">
+        <v/>
+      </c>
+      <c r="G45" t="str">
+        <v>Page stable</v>
+      </c>
+      <c r="H45" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>TC_PH_045</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Verify rapid clicks on Refresh do not crash the application</v>
+      </c>
+      <c r="C46" t="str">
+        <v/>
+      </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
+      <c r="F46" t="str">
+        <v/>
+      </c>
+      <c r="G46" t="str">
+        <v>Page reloads, no crash</v>
+      </c>
+      <c r="H46" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>TC_PH_046</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Verify unauthorized user cannot access Payment History page</v>
+      </c>
+      <c r="C47" t="str">
+        <v/>
+      </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+      <c r="G47" t="str">
+        <v>Redirect to login page</v>
+      </c>
+      <c r="H47" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>TC_PH_047</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Verify application remains responsive with large datasets</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Last 6 Months</v>
+      </c>
+      <c r="D48" t="str">
+        <v/>
+      </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
+      <c r="F48" t="str">
+        <v/>
+      </c>
+      <c r="G48" t="str">
+        <v>Page stable, KPIs visible</v>
+      </c>
+      <c r="H48" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>TC_PH_048</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Verify dropdown selections persist correctly after refresh</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Last 30 days</v>
+      </c>
+      <c r="D49" t="str">
+        <v/>
+      </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
+      <c r="F49" t="str">
+        <v/>
+      </c>
+      <c r="G49" t="str">
+        <v>Filters present after reload</v>
+      </c>
+      <c r="H49" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>TC_PH_049</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Verify search field rejects excessively long input values</v>
+      </c>
+      <c r="C50" t="str">
+        <v/>
+      </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
+      <c r="F50" t="str">
+        <v>A×500</v>
+      </c>
+      <c r="G50" t="str">
+        <v>Page stable, no crash</v>
+      </c>
+      <c r="H50" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>TC_PH_050</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Verify application handles network timeout gracefully</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Last 3 Months</v>
+      </c>
+      <c r="D51" t="str">
+        <v>All Providers</v>
+      </c>
+      <c r="E51" t="str">
+        <v>PENDING</v>
+      </c>
+      <c r="F51" t="str">
+        <v/>
+      </c>
+      <c r="G51" t="str">
+        <v>Graceful handling, no crash</v>
+      </c>
+      <c r="H51" t="str">
+        <v>YES</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H51"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>TestName</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Run</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Mode</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>PaymentHistoryTest</v>
+      </c>
+      <c r="B2" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C2" t="str">
+        <v>serial</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N36"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Test Case ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Module</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Screen Name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Test Scenario</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Test Case Type</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Preconditions</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Test Steps</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Test Data</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Expected Result</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Priority</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Actual Result</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Screenshot Path</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Execution Time</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>TC_RCP_001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Verify Return &amp; Cancellation Policy page loads via Setup sidebar with all 5 policy tabs visible.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F2" t="str">
+        <v>User is logged in as Tenant admin</v>
+      </c>
+      <c r="G2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. From Home page, expand Setup menu in sidebar
+2. Click 'Return &amp; Cancellation'
+3. Verify page heading visible
+4. Verify all 5 tabs (Cancellation, Return, Replacement, Refund, Market Policies) are present</v>
+      </c>
+      <c r="H2" t="str">
+        <v>URL: /setup/policy</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Page loads with heading and all 5 tabs visible</v>
+      </c>
+      <c r="J2" t="str">
+        <v>High</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>TC_RCP_002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Verify direct URL navigation to /setup/policy loads the Return &amp; Cancellation Policy page.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F3" t="str">
+        <v>User is logged in as Tenant admin</v>
+      </c>
+      <c r="G3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate directly to /setup/policy
+2. Verify page heading is visible
+3. Verify URL contains 'setup/policy'</v>
+      </c>
+      <c r="H3" t="str">
+        <v>URL: /setup/policy</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Page loads correctly with heading visible on direct navigation</v>
+      </c>
+      <c r="J3" t="str">
+        <v>High</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>TC_RCP_003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Verify Cancellation tab is active and displays all required fields.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F4" t="str">
+        <v>User is on Return &amp; Cancellation Policy page</v>
+      </c>
+      <c r="G4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to /setup/policy
+2. Click Cancellation tab
+3. Verify Window Minutes, Allowed Before Statuses, Free Cancellation Before Status, Fee Type, Cancellation Fee, Reasons fields are visible</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Tab: Cancellation</v>
+      </c>
+      <c r="I4" t="str">
+        <v>All Cancellation tab fields (Window Minutes, statuses, fee type, reasons) are visible</v>
+      </c>
+      <c r="J4" t="str">
+        <v>High</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>TC_RCP_004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Verify enabling Cancellation policy toggle and saving persists the enabled state.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Cancellation tab is active</v>
+      </c>
+      <c r="G5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Enable the Enabled toggle
+3. Click Save
+4. Re-navigate to page
+5. Verify toggle is still enabled</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Enabled: true</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Cancellation policy is enabled and persists after page reload</v>
+      </c>
+      <c r="J5" t="str">
+        <v>High</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>TC_RCP_005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Verify disabling Cancellation policy collapses conditional fields and saves.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Cancellation policy is currently enabled</v>
+      </c>
+      <c r="G6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Disable the Enabled toggle
+3. Click Save
+4. Verify save succeeds
+5. Re-enable for clean state</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Enabled: false</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Cancellation policy disabled state saves successfully; conditional fields hidden</v>
+      </c>
+      <c r="J6" t="str">
+        <v>High</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>TC_RCP_006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Verify Window Minutes accepts 0 (no time limit) and shows hint text.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Set Window Minutes to 0
+3. Verify '0 = no time limit' hint appears
+4. Click Save and verify success</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Window Minutes: 0</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Window Minutes 0 accepted, hint shown, save succeeds</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>TC_RCP_007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Verify Window Minutes accepts a valid positive value (60) and saves correctly.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G8" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Set Window Minutes to 60
+3. Click Save
+4. Verify success toast</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Window Minutes: 60</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Window Minutes 60 saved; success feedback displayed</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>TC_RCP_008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Verify Allowed Before Statuses multi-select adds PAYMENT_CONFIRMED and saves.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G9" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Open Allowed Before Statuses dropdown
+3. Select PAYMENT_CONFIRMED
+4. Click Save
+5. Verify success</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Status: PAYMENT_CONFIRMED</v>
+      </c>
+      <c r="I9" t="str">
+        <v>PAYMENT_CONFIRMED added to Allowed Before Statuses; saved successfully</v>
+      </c>
+      <c r="J9" t="str">
+        <v>High</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>TC_RCP_009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Verify Free Cancellation Before Status single-select selects INVENTORY_CONFIRMED and saves.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G10" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Open Free Cancellation Before Status dropdown
+3. Select INVENTORY_CONFIRMED
+4. Click Save
+5. Verify success</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Status: INVENTORY_CONFIRMED</v>
+      </c>
+      <c r="I10" t="str">
+        <v>INVENTORY_CONFIRMED selected and saved successfully</v>
+      </c>
+      <c r="J10" t="str">
+        <v>High</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>TC_RCP_010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Verify Fee Type FLAT with Cancellation Fee 50 saves correctly.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G11" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Select FLAT fee type
+3. Enter Cancellation Fee as 50
+4. Click Save
+5. Verify success</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Fee Type: FLAT, Fee: 50</v>
+      </c>
+      <c r="I11" t="str">
+        <v>FLAT fee type with 50 cancellation fee saved successfully</v>
+      </c>
+      <c r="J11" t="str">
+        <v>High</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>TC_RCP_011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Verify Fee Type PERCENTAGE with 10% saves correctly and resets to FLAT/0 afterwards.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G12" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Select PERCENTAGE fee type
+3. Enter 10 as fee
+4. Click Save
+5. Verify success
+6. Reset to FLAT/0</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Fee Type: PERCENTAGE, Fee: 10</v>
+      </c>
+      <c r="I12" t="str">
+        <v>PERCENTAGE fee type with 10% saved successfully; can be reset to FLAT/0</v>
+      </c>
+      <c r="J12" t="str">
+        <v>High</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>TC_RCP_012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Verify Auto Refund On Approval toggle saves and persists after reload.</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G13" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Enable Auto Refund On Approval toggle
+3. Click Save
+4. Re-navigate to page
+5. Verify toggle is still enabled</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Auto Refund On Approval: true</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Auto Refund On Approval toggle state persists after save and reload</v>
+      </c>
+      <c r="J13" t="str">
+        <v>High</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>TC_RCP_013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Verify COD Allowed toggle can be disabled and settings persist after save.</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G14" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Disable COD Allowed toggle
+3. Click Save
+4. Verify success
+5. Re-enable for clean state</v>
+      </c>
+      <c r="H14" t="str">
+        <v>COD Allowed: false</v>
+      </c>
+      <c r="I14" t="str">
+        <v>COD Allowed disabled state saves; re-enable restores default</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>TC_RCP_014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Verify adding a custom cancellation reason tag persists after save.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Cancellation tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G15" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Cancellation tab
+2. Type 'DAMAGED_PACKAGING' in Reasons input
+3. Press Enter to create tag
+4. Click Save
+5. Verify save succeeds</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Custom Reason: DAMAGED_PACKAGING</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Custom reason tag added and saved successfully</v>
+      </c>
+      <c r="J15" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>TC_RCP_015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Verify Return tab displays all required fields: Window Days, Item Types, Shipping Paid By, Restocking Fee.</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F16" t="str">
+        <v>User is on Return &amp; Cancellation Policy page</v>
+      </c>
+      <c r="G16" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to Return &amp; Cancellation Policy
+2. Click Return tab
+3. Verify Window Days, Returnable Item Types, Non Returnable Item Types, Shipping Paid By, Restocking Fee fields are visible</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Tab: Return</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Return tab shows Window Days, item type fields, Shipping Paid By, Restocking Fee</v>
+      </c>
+      <c r="J16" t="str">
+        <v>High</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>TC_RCP_016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Verify enabling Return policy with Window Days 7 saves successfully.</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Return tab is active</v>
+      </c>
+      <c r="G17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Return tab
+2. Enable the Enabled toggle
+3. Set Window Days to 7
+4. Click Save
+5. Verify success</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Window Days: 7, Enabled: true</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Return policy enabled with 7-day window saves successfully</v>
+      </c>
+      <c r="J17" t="str">
+        <v>High</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>TC_RCP_017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Verify disabling Return policy toggle and saving succeeds.</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Return policy is currently enabled</v>
+      </c>
+      <c r="G18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Return tab
+2. Disable the Enabled toggle
+3. Click Save
+4. Verify save succeeds
+5. Re-enable for clean state</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Enabled: false</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Return policy disabled state saves; restore to enabled for clean state</v>
+      </c>
+      <c r="J18" t="str">
+        <v>High</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+      <c r="M18" t="str">
+        <v/>
+      </c>
+      <c r="N18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>TC_RCP_018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Verify adding returnable item type 'ELECTRONICS' as a tag and saving.</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Return tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Return tab
+2. Type 'ELECTRONICS' in Returnable Item Types input
+3. Press Enter
+4. Click Save
+5. Verify success</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Item Type: ELECTRONICS</v>
+      </c>
+      <c r="I19" t="str">
+        <v>ELECTRONICS tag added to Returnable Item Types and saved</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <v/>
+      </c>
+      <c r="N19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>TC_RCP_019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Verify enabling Require Images and setting Min Images to 2 saves correctly.</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Return tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Return tab
+2. Enable Require Images toggle
+3. Set Min Images to 2
+4. Click Save
+5. Verify success</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Require Images: true, Min Images: 2</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Require Images enabled with Min Images 2 saved successfully</v>
+      </c>
+      <c r="J20" t="str">
+        <v>High</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
+      <c r="M20" t="str">
+        <v/>
+      </c>
+      <c r="N20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>TC_RCP_020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Verify Restocking Fee (FLAT) set to 25 is saved correctly.</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Return tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Return tab
+2. Enter 25 in Restocking Fee field
+3. Click Save
+4. Verify success</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Restocking Fee: 25 (FLAT)</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Restocking Fee 25 saved; applied during return approval</v>
+      </c>
+      <c r="J21" t="str">
+        <v>High</v>
+      </c>
+      <c r="K21" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <v/>
+      </c>
+      <c r="N21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>TC_RCP_021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Verify Replacement tab displays Window Days, Shipping Paid By, Max Per Order, Require Original Return, Require Images fields.</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F22" t="str">
+        <v>User is on Return &amp; Cancellation Policy page</v>
+      </c>
+      <c r="G22" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Replacement tab
+2. Verify Window Days, Shipping Paid By, Max Per Order, Require Original Return, Require Images fields visible</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Tab: Replacement</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Replacement tab shows all expected fields</v>
+      </c>
+      <c r="J22" t="str">
+        <v>High</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L22" t="str">
+        <v/>
+      </c>
+      <c r="M22" t="str">
+        <v/>
+      </c>
+      <c r="N22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>TC_RCP_022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Verify enabling Replacement with Window Days 14 and Max Per Order 2 saves correctly.</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Replacement tab is active</v>
+      </c>
+      <c r="G23" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Replacement tab
+2. Enable Enabled toggle
+3. Set Window Days to 14
+4. Set Max Per Order to 2
+5. Click Save
+6. Verify success</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Enabled: true, Window Days: 14, Max Per Order: 2</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Replacement configured with 14-day window and max 2 per order saves successfully</v>
+      </c>
+      <c r="J23" t="str">
+        <v>High</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L23" t="str">
+        <v/>
+      </c>
+      <c r="M23" t="str">
+        <v/>
+      </c>
+      <c r="N23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>TC_RCP_023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Verify Require Original Return toggle saves and persists after reload.</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Replacement tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G24" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Replacement tab
+2. Enable Require Original Return toggle
+3. Click Save
+4. Re-navigate to page
+5. Verify Require Original Return is still enabled</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Require Original Return: true</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Require Original Return toggle persists after save and page reload</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
+      <c r="M24" t="str">
+        <v/>
+      </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>TC_RCP_024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Verify Require Images toggle on Replacement tab can be enabled and saved.</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Replacement tab is active and Enabled toggle is ON</v>
+      </c>
+      <c r="G25" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Replacement tab
+2. Enable Require Images toggle
+3. Click Save
+4. Verify success</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Require Images: true (Replacement)</v>
+      </c>
+      <c r="I25" t="str">
+        <v>Require Images toggle enabled and saved on Replacement tab</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K25" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L25" t="str">
+        <v/>
+      </c>
+      <c r="M25" t="str">
+        <v/>
+      </c>
+      <c r="N25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>TC_RCP_025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Verify disabling Replacement policy saves and can be re-enabled for clean state.</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Replacement policy is currently enabled</v>
+      </c>
+      <c r="G26" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Replacement tab
+2. Disable Enabled toggle
+3. Click Save
+4. Verify success
+5. Re-enable for clean state</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Enabled: false (Replacement)</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Replacement disabled state saves; restore to enabled</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K26" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+      <c r="M26" t="str">
+        <v/>
+      </c>
+      <c r="N26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
+        <v>TC_RCP_026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Verify Refund tab displays Refund Method, COD Refund Method, Processing Days, and refund toggle fields.</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F27" t="str">
+        <v>User is on Return &amp; Cancellation Policy page</v>
+      </c>
+      <c r="G27" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Refund tab
+2. Verify Refund Method, COD Refund Method, Processing Days, Partial Refund Allowed, Shipping Refundable, Deduct Cancellation Fee, Deduct Restocking Fee fields are visible</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Tab: Refund</v>
+      </c>
+      <c r="I27" t="str">
+        <v>All Refund tab fields are visible</v>
+      </c>
+      <c r="J27" t="str">
+        <v>High</v>
+      </c>
+      <c r="K27" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
+      <c r="N27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
+        <v>TC_RCP_027</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Verify Refund Method (ORIGINAL_PAYMENT), COD Refund Method (WALLET), Processing Days 7 saves.</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Refund tab is active</v>
+      </c>
+      <c r="G28" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Refund tab
+2. Set Refund Method to ORIGINAL_PAYMENT
+3. Set COD Refund Method to WALLET
+4. Set Processing Days to 7
+5. Click Save
+6. Verify success</v>
+      </c>
+      <c r="H28" t="str">
+        <v>Refund: ORIGINAL_PAYMENT, COD: WALLET, Days: 7</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Refund configuration saves successfully</v>
+      </c>
+      <c r="J28" t="str">
+        <v>High</v>
+      </c>
+      <c r="K28" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L28" t="str">
+        <v/>
+      </c>
+      <c r="M28" t="str">
+        <v/>
+      </c>
+      <c r="N28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
+        <v>TC_RCP_028</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Verify Partial Refund Allowed and Shipping Refundable toggles save and Partial Refund Allowed persists.</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Refund tab is active</v>
+      </c>
+      <c r="G29" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Refund tab
+2. Enable Partial Refund Allowed toggle
+3. Enable Shipping Refundable toggle
+4. Click Save
+5. Re-navigate and verify Partial Refund Allowed is ON</v>
+      </c>
+      <c r="H29" t="str">
+        <v>Partial Refund: true, Shipping Refundable: true</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Both toggles enabled and Partial Refund Allowed persists after reload</v>
+      </c>
+      <c r="J29" t="str">
+        <v>High</v>
+      </c>
+      <c r="K29" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L29" t="str">
+        <v/>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
+      <c r="N29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30" xml:space="preserve">
+      <c r="A30" t="str">
+        <v>TC_RCP_029</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Verify Deduct Cancellation Fee and Deduct Restocking Fee toggles save and Deduct Cancellation Fee persists.</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Refund tab is active</v>
+      </c>
+      <c r="G30" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Refund tab
+2. Enable Deduct Cancellation Fee
+3. Enable Deduct Restocking Fee
+4. Click Save
+5. Re-navigate and verify Deduct Cancellation Fee is ON</v>
+      </c>
+      <c r="H30" t="str">
+        <v>Deduct Cancel Fee: true, Deduct Restocking Fee: true</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Both deduct toggles saved; Deduct Cancellation Fee persists after reload</v>
+      </c>
+      <c r="J30" t="str">
+        <v>High</v>
+      </c>
+      <c r="K30" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L30" t="str">
+        <v/>
+      </c>
+      <c r="M30" t="str">
+        <v/>
+      </c>
+      <c r="N30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31" xml:space="preserve">
+      <c r="A31" t="str">
+        <v>TC_RCP_030</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Verify Market Policies tab loads with Add Market button and empty-state or existing market list.</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F31" t="str">
+        <v>User is on Return &amp; Cancellation Policy page</v>
+      </c>
+      <c r="G31" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Market Policies tab
+2. Verify '+ Add Market' button is visible
+3. Verify empty state 'No market overrides configured' OR existing market rows are shown</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Tab: Market Policies</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Market Policies tab loads with Add Market button and empty state or market entries</v>
+      </c>
+      <c r="J31" t="str">
+        <v>High</v>
+      </c>
+      <c r="K31" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L31" t="str">
+        <v/>
+      </c>
+      <c r="M31" t="str">
+        <v/>
+      </c>
+      <c r="N31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
+      <c r="A32" t="str">
+        <v>TC_RCP_031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Verify clicking Add Market button opens Market Policy Override modal with all required fields.</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Market Policies tab is active</v>
+      </c>
+      <c r="G32" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Market Policies tab
+2. Click '+ Add Market'
+3. Verify modal opens with Market Name, Conditions fields
+4. Verify Override Cancellation/Return/Replacement/Refund toggles visible
+5. Click Cancel</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Modal: Market Policy Override</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Modal opens with all override fields; Cancel closes it without saving</v>
+      </c>
+      <c r="J32" t="str">
+        <v>High</v>
+      </c>
+      <c r="K32" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L32" t="str">
+        <v/>
+      </c>
+      <c r="M32" t="str">
+        <v/>
+      </c>
+      <c r="N32" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33" xml:space="preserve">
+      <c r="A33" t="str">
+        <v>TC_RCP_032</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Verify cancelling Market Policy modal discards changes without creating a new market override.</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Market Policies tab is active</v>
+      </c>
+      <c r="G33" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click Market Policies tab
+2. Note current market count
+3. Click '+ Add Market'
+4. Click Cancel without filling any fields
+5. Verify modal is closed and no new market entry appeared</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Cancel without save</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Market modal closed; no new market override added on cancel</v>
+      </c>
+      <c r="J33" t="str">
+        <v>High</v>
+      </c>
+      <c r="K33" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L33" t="str">
+        <v/>
+      </c>
+      <c r="M33" t="str">
+        <v/>
+      </c>
+      <c r="N33" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34" xml:space="preserve">
+      <c r="A34" t="str">
+        <v>TC_RCP_033</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Verify unauthenticated user cannot access Return &amp; Cancellation Policy page directly.</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F34" t="str">
+        <v>User is NOT logged in</v>
+      </c>
+      <c r="G34" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open browser without authenticated session
+2. Navigate directly to /setup/policy
+3. Verify user is redirected to login page or access denied</v>
+      </c>
+      <c r="H34" t="str">
+        <v>URL: /setup/policy, No auth</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Unauthenticated access redirected to login page or access denied shown</v>
+      </c>
+      <c r="J34" t="str">
+        <v>High</v>
+      </c>
+      <c r="K34" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L34" t="str">
+        <v/>
+      </c>
+      <c r="M34" t="str">
+        <v/>
+      </c>
+      <c r="N34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35" xml:space="preserve">
+      <c r="A35" t="str">
+        <v>TC_RCP_034</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Verify API failure on Policy page load is handled gracefully without a JavaScript crash.</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F35" t="str">
+        <v>User is logged in as Tenant admin</v>
+      </c>
+      <c r="G35" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to /setup/policy
+2. Intercept and abort the policy API call
+3. Reload the page
+4. Verify app does not show uncaught JavaScript error</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Simulated API failure</v>
+      </c>
+      <c r="I35" t="str">
+        <v>App handles API failure gracefully — no uncaught JavaScript errors in page body</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="K35" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L35" t="str">
+        <v/>
+      </c>
+      <c r="M35" t="str">
+        <v/>
+      </c>
+      <c r="N35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36" xml:space="preserve">
+      <c r="A36" t="str">
+        <v>TC_RCP_035</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Setup</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Return &amp; Cancellation Policy</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Verify full cross-tab regression: configure and save Cancellation, Return, Replacement, and Refund tabs in sequence.</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F36" t="str">
+        <v>User is logged in as Tenant admin</v>
+      </c>
+      <c r="G36" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Configure Cancellation tab (Enabled, Window 0, FLAT 0) and Save
+2. Configure Return tab (Enabled, Window 7) and Save
+3. Configure Replacement tab (Enabled, Window 7, Max 1) and Save
+4. Configure Refund tab (ORIGINAL_PAYMENT, Days 7) and Save
+5. Verify each save succeeds</v>
+      </c>
+      <c r="H36" t="str">
+        <v>All tabs default/baseline values</v>
+      </c>
+      <c r="I36" t="str">
+        <v>All 4 policy tabs configured and saved in sequence without errors</v>
+      </c>
+      <c r="J36" t="str">
+        <v>High</v>
+      </c>
+      <c r="K36" t="str">
+        <v>Not Executed</v>
+      </c>
+      <c r="L36" t="str">
+        <v/>
+      </c>
+      <c r="M36" t="str">
+        <v/>
+      </c>
+      <c r="N36" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:N36"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F77"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Test Case ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Description</v>
+      </c>
+      <c r="C1" t="str">
+        <v>persona</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Type</v>
+      </c>
+      <c r="E1" t="str">
+        <v>ExpectedMessage</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Issue</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>TC_OM_001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Verify user can create an Office successfully with all mandatory fields populated with valid data.</v>
+      </c>
+      <c r="C2" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Partner details submitted successfully!</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>TC_OM_002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Verify office type dropdown displays all available office types and allows selection.</v>
+      </c>
+      <c r="C3" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Dropdown has options</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TC_OM_003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Verify user can add multiple valid email addresses using the Add New button.</v>
+      </c>
+      <c r="C4" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Email inputs/tags visible</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TC_OM_004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Verify Google address selection auto-populates City, State, Country, and Zip Code fields correctly.</v>
+      </c>
+      <c r="C5" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Address fields auto-populated</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TC_OM_005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Verify clicking Next navigates to the Organization step when all required fields are valid.</v>
+      </c>
+      <c r="C6" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Step 2 Organization visible</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TC_OM_006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Verify validation error is displayed when Email field contains an invalid email format.</v>
+      </c>
+      <c r="C7" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Email validation error</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TC_OM_007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Verify validation error is displayed when Phone field contains invalid or insufficient digits.</v>
+      </c>
+      <c r="C8" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Phone validation error</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TC_OM_008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Verify user cannot proceed to the next step when mandatory fields are left blank.</v>
+      </c>
+      <c r="C9" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Mandatory field validation shown</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TC_OM_009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Verify duplicate email address addition is prevented and appropriate error message is shown.</v>
+      </c>
+      <c r="C10" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Duplicate email rejected</v>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TC_OM_010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Verify system prevents submission when an invalid or unsupported office type value is selected through manipulation.</v>
+      </c>
+      <c r="C11" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Office Type required validation</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TC_OM_011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Verify user can proceed to the next step with valid Organization Name, Logo, Registration No, GST/License No, and FSSAI No.</v>
+      </c>
+      <c r="C12" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Step 3 Authentication visible</v>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TC_OM_012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Verify a valid logo file (PNG/JPG) uploads successfully and preview is displayed.</v>
+      </c>
+      <c r="C13" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Logo uploaded or preview visible</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TC_OM_013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Verify the Own Company checkbox can be selected and retained after clicking Next.</v>
+      </c>
+      <c r="C14" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Checkbox state changes</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TC_OM_014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Verify the Back button navigates to the previous onboarding step without data loss.</v>
+      </c>
+      <c r="C15" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Step 1 data retained after Back</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TC_OM_015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Verify validation error is displayed when Organization Name is left blank and user clicks Next.</v>
+      </c>
+      <c r="C16" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Organisation name required</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TC_OM_016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Verify system prevents upload of unsupported file formats (e.g., .exe, .zip) in the Logo field.</v>
+      </c>
+      <c r="C17" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Unsupported file type error</v>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TC_OM_017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Verify validation error is displayed when Registration No, GST/License No, or FSSAI No contains invalid characters.</v>
+      </c>
+      <c r="C18" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Registration/GST/FSSAI validation error</v>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TC_OM_018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Verify user cannot proceed when mandatory fields or logo upload are missing.</v>
+      </c>
+      <c r="C19" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Mandatory field validation shown</v>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TC_OM_019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Verify user can proceed to the next step with valid Username, Email, Phone Number, and Password.</v>
+      </c>
+      <c r="C20" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Step 4 Agreement visible</v>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TC_OM_020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Verify password visibility toggle correctly shows and hides the entered password.</v>
+      </c>
+      <c r="C21" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Password input type changes</v>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>TC_OM_021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Verify country code dropdown allows selecting a valid country code and updates the phone field accordingly.</v>
+      </c>
+      <c r="C22" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Country code selectable</v>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>TC_OM_022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Verify clicking Back navigates to the Organization step while retaining previously entered data.</v>
+      </c>
+      <c r="C23" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Step 2 data retained after Back</v>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>TC_OM_023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Verify validation error is displayed when Username is left blank and user clicks Next.</v>
+      </c>
+      <c r="C24" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Username required validation</v>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>TC_OM_024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Verify validation error is displayed when an invalid email format is entered (e.g., abc@com).</v>
+      </c>
+      <c r="C25" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Email format validation error</v>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>TC_OM_025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Verify validation error is displayed when Phone Number contains alphabetic or special characters.</v>
+      </c>
+      <c r="C26" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Phone validation error</v>
+      </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>TC_OM_026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Verify user cannot proceed when Password does not meet the minimum security requirements or is left empty.</v>
+      </c>
+      <c r="C27" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Password strength validation error</v>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>TC_OM_027</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Verify user can upload a valid agreement document and proceed to the next step successfully.</v>
+      </c>
+      <c r="C28" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Agreement URL generated</v>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>TC_OM_028</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Verify user can select a valid Catalog Option and corresponding Market from the dropdowns.</v>
+      </c>
+      <c r="C29" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Catalog and Market selected</v>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>TC_OM_029</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Verify Select All Market checkbox selects all available markets correctly.</v>
+      </c>
+      <c r="C30" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E30" t="str">
+        <v>All markets selected</v>
+      </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TC_OM_030</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Verify user can select a valid Mode of Sale and save the selection.</v>
+      </c>
+      <c r="C31" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Mode of Sale selected</v>
+      </c>
+      <c r="F31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>TC_OM_031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Verify Agreement Start Date and End Date can be selected using the date picker.</v>
+      </c>
+      <c r="C32" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Start and End dates set</v>
+      </c>
+      <c r="F32" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>TC_OM_032</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Verify user can proceed to the Done step when all mandatory fields are completed with valid data.</v>
+      </c>
+      <c r="C33" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Step 5 Done indicator visible</v>
+      </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>TC_OM_033</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Verify validation error is displayed when Agreement document is not uploaded and user clicks Next.</v>
+      </c>
+      <c r="C34" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Agreement file required validation</v>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>TC_OM_034</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Verify system rejects unsupported agreement file formats (e.g., .exe, .bat, .zip).</v>
+      </c>
+      <c r="C35" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Unsupported file type error</v>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>TC_OM_035</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Verify validation error is displayed when Catalog Option is not selected.</v>
+      </c>
+      <c r="C36" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Catalog required validation</v>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>TC_OM_036</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Verify validation error is displayed when Market is not selected while Select All Market is unchecked.</v>
+      </c>
+      <c r="C37" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Market required validation</v>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>TC_OM_037</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Verify system prevents proceeding when Agreement End Date is earlier than Agreement Start Date.</v>
+      </c>
+      <c r="C38" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E38" t="str">
+        <v>End date before start date validation</v>
+      </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>TC_OM_038</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Verify user cannot proceed when any mandatory field marked with (*) is left blank.</v>
+      </c>
+      <c r="C39" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Mandatory field validation shown</v>
+      </c>
+      <c r="F39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>TC_OM_039</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Verify success message "Partner details submitted successfully!" is displayed after completing all onboarding steps with valid data.</v>
+      </c>
+      <c r="C40" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Partner details submitted successfully!</v>
+      </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>TC_OM_040</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Verify clicking the Done button redirects the user to the Office Management list page successfully.</v>
+      </c>
+      <c r="C41" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Office Registry heading visible</v>
+      </c>
+      <c r="F41" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>TC_OM_041</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Verify the success screen is not displayed if any previous onboarding step contains invalid or incomplete mandatory data.</v>
+      </c>
+      <c r="C42" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Success message not shown</v>
+      </c>
+      <c r="F42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>TC_OM_042</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Verify clicking the Done button when the backend submission fails displays an appropriate error message and prevents redirection.</v>
+      </c>
+      <c r="C43" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Error shown or wizard not advanced</v>
+      </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>TC_OM_043</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Verify Office Registry page loads successfully and displays all office records with correct details.</v>
+      </c>
+      <c r="C44" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Office Registry heading visible</v>
+      </c>
+      <c r="F44" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>TC_OM_044</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Verify user can search an existing office using the search box and matching results are displayed.</v>
+      </c>
+      <c r="C45" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Search result visible in table</v>
+      </c>
+      <c r="F45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>TC_OM_045</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Verify clicking the View icon opens the selected office details page successfully.</v>
+      </c>
+      <c r="C46" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E46" t="str">
+        <v>View page loaded</v>
+      </c>
+      <c r="F46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>TC_OM_046</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Verify clicking the Edit icon opens the selected office record in edit mode with pre-filled data.</v>
+      </c>
+      <c r="C47" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Edit URL shown</v>
+      </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>TC_OM_047</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Verify clicking Create Office navigates the user to the Office Onboarding/Create Office page.</v>
+      </c>
+      <c r="C48" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Step 1 Office indicator visible</v>
+      </c>
+      <c r="F48" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>TC_OM_048</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Verify "No records found" message is displayed when searching with a non-existing office name.</v>
+      </c>
+      <c r="C49" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E49" t="str">
+        <v>No Records Found message visible</v>
+      </c>
+      <c r="F49" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>TC_OM_049</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Verify special characters or invalid input in the search field do not break the search functionality.</v>
+      </c>
+      <c r="C50" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Page remains stable</v>
+      </c>
+      <c r="F50" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>TC_OM_050</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Verify user without view permission cannot access office details through the View icon.</v>
+      </c>
+      <c r="C51" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Listing accessible or icons hidden</v>
+      </c>
+      <c r="F51" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>TC_OM_051</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Verify user without edit permission cannot modify office details through the Edit icon.</v>
+      </c>
+      <c r="C52" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Listing accessible or edit icons hidden</v>
+      </c>
+      <c r="F52" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>TC_OM_052</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Verify deleting an office that is linked to active records displays an appropriate error message and prevents deletion.</v>
+      </c>
+      <c r="C53" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Error toast or record retained</v>
+      </c>
+      <c r="F53" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>TC_OM_053</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Verify View Office page loads successfully and displays all office details correctly for a valid office record.</v>
+      </c>
+      <c r="C54" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E54" t="str">
+        <v>View page heading visible</v>
+      </c>
+      <c r="F54" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>TC_OM_054</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Verify Office Details, Organization Details, and Authentication Details sections display accurate data matching the created office.</v>
+      </c>
+      <c r="C55" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E55" t="str">
+        <v>All 3 detail sections visible</v>
+      </c>
+      <c r="F55" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>TC_OM_055</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Verify logo URL is displayed correctly and opens/downloads the associated logo when accessed.</v>
+      </c>
+      <c r="C56" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Logo visible or URL accessible</v>
+      </c>
+      <c r="F56" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>TC_OM_056</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Verify the Office Type badge (e.g., Branch Office) is displayed correctly on the page.</v>
+      </c>
+      <c r="C57" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Office type badge visible</v>
+      </c>
+      <c r="F57" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>TC_OM_057</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Verify clicking the Back button returns the user to the Office Registry page successfully.</v>
+      </c>
+      <c r="C58" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Office Registry heading visible</v>
+      </c>
+      <c r="F58" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>TC_OM_058</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Verify an appropriate error message is displayed when attempting to view a non-existent office record.</v>
+      </c>
+      <c r="C59" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Error or redirect shown</v>
+      </c>
+      <c r="F59" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>TC_OM_059</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Verify the page handles missing organization details gracefully without UI breakage.</v>
+      </c>
+      <c r="C60" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Page stable with no crash</v>
+      </c>
+      <c r="F60" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>TC_OM_060</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Verify invalid or broken logo URLs do not crash the page and display a fallback message/image.</v>
+      </c>
+      <c r="C61" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Page stable or fallback shown</v>
+      </c>
+      <c r="F61" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>TC_OM_061</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Verify unauthorized users cannot access the View Office page directly via URL manipulation.</v>
+      </c>
+      <c r="C62" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Redirect or access denied</v>
+      </c>
+      <c r="F62" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>TC_OM_062</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Verify null or missing authentication fields are displayed safely without exposing system errors or sensitive data.</v>
+      </c>
+      <c r="C63" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Page stable no system errors</v>
+      </c>
+      <c r="F63" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>TC_OM_063</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Verify user can successfully update office details with valid data in all mandatory fields and save changes.</v>
+      </c>
+      <c r="C64" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Office updated successfully</v>
+      </c>
+      <c r="F64" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>TC_OM_064</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Verify user can modify Office Type and the updated value is reflected after saving.</v>
+      </c>
+      <c r="C65" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E65" t="str">
+        <v>Updated office type reflected</v>
+      </c>
+      <c r="F65" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>TC_OM_065</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Verify user can update Email, Phone, and Address information successfully.</v>
+      </c>
+      <c r="C66" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E66" t="str">
+        <v>Updated email/phone/address reflected</v>
+      </c>
+      <c r="F66" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>TC_OM_066</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Verify user can change Security Question and Security Answer and save the updated values.</v>
+      </c>
+      <c r="C67" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Security fields updated</v>
+      </c>
+      <c r="F67" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>TC_OM_067</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Verify clicking Update Office displays a success message and persists the updated data.</v>
+      </c>
+      <c r="C68" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Update success toast visible and data persists</v>
+      </c>
+      <c r="F68" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>TC_OM_068</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Verify validation error is displayed when mandatory fields (Office Name, Email, Phone, etc.) are left blank and Update Office is clicked.</v>
+      </c>
+      <c r="C69" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E69" t="str">
+        <v>Mandatory field validation shown</v>
+      </c>
+      <c r="F69" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>TC_OM_069</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Verify validation error is displayed when an invalid email format is entered in the Email field.</v>
+      </c>
+      <c r="C70" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Email format validation error</v>
+      </c>
+      <c r="F70" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>TC_OM_070</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Verify validation error is displayed when Phone Number contains invalid characters or exceeds allowed length.</v>
+      </c>
+      <c r="C71" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Phone validation error</v>
+      </c>
+      <c r="F71" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>TC_OM_071</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Verify system prevents saving when Registration No, GST No, or FSSAI No contains invalid data formats.</v>
+      </c>
+      <c r="C72" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Registration/GST/FSSAI validation error</v>
+      </c>
+      <c r="F72" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>TC_OM_072</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Verify unauthorized users cannot update office details and receive an appropriate access denied message.</v>
+      </c>
+      <c r="C73" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Access denied or not editable</v>
+      </c>
+      <c r="F73" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>TC_OM_073</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Verify clicking Cancel closes the delete confirmation popup and retains the office record in the registry.</v>
+      </c>
+      <c r="C74" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Office record retained in listing</v>
+      </c>
+      <c r="F74" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>TC_OM_074</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Verify clicking Delete successfully removes the selected office and displays a success message.</v>
+      </c>
+      <c r="C75" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Office removed from listing</v>
+      </c>
+      <c r="F75" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>TC_OM_075</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Verify office is not deleted when the delete API returns an error and an appropriate error message is displayed.</v>
+      </c>
+      <c r="C76" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Error toast shown and record retained</v>
+      </c>
+      <c r="F76" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>TC_OM_076</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Verify unauthorized users cannot delete an office and receive an access denied message when clicking Delete.</v>
+      </c>
+      <c r="C77" t="str">
+        <v>tenant</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Access denied message shown</v>
+      </c>
+      <c r="F77" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F77"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F6"/>

</xml_diff>

<commit_message>
fix: update regression sheet with correct spec names
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -19155,7 +19155,7 @@
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C54"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -19685,9 +19685,75 @@
         <v>serial</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>FAQMasterConfigTest</v>
+      </c>
+      <c r="B49" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C49" t="str">
+        <v>serial</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>PaymentHistoryTest</v>
+      </c>
+      <c r="B50" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C50" t="str">
+        <v>serial</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>ReturnCancellationPolicyTest</v>
+      </c>
+      <c r="B51" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C51" t="str">
+        <v>serial</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>FeaturesSuperAdminTest</v>
+      </c>
+      <c r="B52" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C52" t="str">
+        <v>serial</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>PartnerReportTest</v>
+      </c>
+      <c r="B53" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C53" t="str">
+        <v>serial</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>AdminDashboardTest</v>
+      </c>
+      <c r="B54" t="str">
+        <v>YES</v>
+      </c>
+      <c r="C54" t="str">
+        <v>serial</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C54"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: restore AdminDashboardTest sheet to testData.xlsx
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -60,6 +60,7 @@
     <sheet name="Payment History Regression" sheetId="55" r:id="rId55"/>
     <sheet name="Return Cancellation Regression" sheetId="56" r:id="rId56"/>
     <sheet name="OfficeManagement" sheetId="57" r:id="rId57"/>
+    <sheet name="AdminDashboardTest" sheetId="58" r:id="rId58"/>
   </sheets>
 </workbook>
 </file>
@@ -62190,6 +62191,147 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>TestID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Issue</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Description</v>
+      </c>
+      <c r="D1" t="str">
+        <v>UserName</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Password</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Persona</v>
+      </c>
+      <c r="G1" t="str">
+        <v>FromDate</v>
+      </c>
+      <c r="H1" t="str">
+        <v>ToDate</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>TC01_AdminDashboardLoad</v>
+      </c>
+      <c r="B2" t="str">
+        <v>4001</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Verify Admin Dashboard Load</v>
+      </c>
+      <c r="D2" t="str">
+        <v>nipigev2@yopmail.com</v>
+      </c>
+      <c r="E2" t="str">
+        <v>admin@123</v>
+      </c>
+      <c r="F2" t="str">
+        <v>admin</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>TC02_AdminDashboardFilters</v>
+      </c>
+      <c r="B3" t="str">
+        <v>4002</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Verify Admin Dashboard Filters</v>
+      </c>
+      <c r="D3" t="str">
+        <v>nipigev2@yopmail.com</v>
+      </c>
+      <c r="E3" t="str">
+        <v>admin@123</v>
+      </c>
+      <c r="F3" t="str">
+        <v>admin</v>
+      </c>
+      <c r="G3" t="str">
+        <v>6/1/25</v>
+      </c>
+      <c r="H3" t="str">
+        <v>6/10/26</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TC03_AdminOrderChartDropdown</v>
+      </c>
+      <c r="B4" t="str">
+        <v>4003</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Verify Admin Order Chart</v>
+      </c>
+      <c r="D4" t="str">
+        <v>nipigev2@yopmail.com</v>
+      </c>
+      <c r="E4" t="str">
+        <v>admin@123</v>
+      </c>
+      <c r="F4" t="str">
+        <v>admin</v>
+      </c>
+      <c r="G4" t="str">
+        <v>6/1/25</v>
+      </c>
+      <c r="H4" t="str">
+        <v>6/10/26</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TC04_AdminRevenueDropdown</v>
+      </c>
+      <c r="B5" t="str">
+        <v>4004</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Verify Admin Revenue Dropdown</v>
+      </c>
+      <c r="D5" t="str">
+        <v>nipigev2@yopmail.com</v>
+      </c>
+      <c r="E5" t="str">
+        <v>admin@123</v>
+      </c>
+      <c r="F5" t="str">
+        <v>admin</v>
+      </c>
+      <c r="G5" t="str">
+        <v>6/1/25</v>
+      </c>
+      <c r="H5" t="str">
+        <v>6/10/26</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F6"/>

</xml_diff>

<commit_message>
perf: optimize parallel execution on CI with 6 workers and 90m timeout
</commit_message>
<xml_diff>
--- a/src/resources/data/testData.xlsx
+++ b/src/resources/data/testData.xlsx
@@ -45562,10 +45562,10 @@
         <v>Test passed successfully.</v>
       </c>
       <c r="I2" t="str">
-        <v>54.06s</v>
+        <v>104.52s</v>
       </c>
       <c r="J2" t="str">
-        <v>D:\Trigital poject\nipige_qa_automation\test-results\failure\OfficeManagementTest-Offic-0aad2--populated-with-valid-data--local\test-finished-1.png</v>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-3ca3c--populated-with-valid-data--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="3">
@@ -45588,16 +45588,16 @@
         <v/>
       </c>
       <c r="G3" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H3" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I3" t="str">
-        <v>0.00s</v>
+        <v>4.29s</v>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-003c6-types-and-allows-selection--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="4">
@@ -45620,16 +45620,16 @@
         <v/>
       </c>
       <c r="G4" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H4" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I4" t="str">
-        <v>0.00s</v>
+        <v>6.21s</v>
       </c>
       <c r="J4" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-10db6-s-using-the-Add-New-button--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="5">
@@ -45652,16 +45652,16 @@
         <v/>
       </c>
       <c r="G5" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H5" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I5" t="str">
-        <v>0.00s</v>
+        <v>8.63s</v>
       </c>
       <c r="J5" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-06924--Zip-Code-fields-correctly--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="6">
@@ -45684,16 +45684,16 @@
         <v/>
       </c>
       <c r="G6" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H6" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I6" t="str">
-        <v>0.00s</v>
+        <v>13.05s</v>
       </c>
       <c r="J6" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-014f9--required-fields-are-valid--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="7">
@@ -45716,16 +45716,16 @@
         <v/>
       </c>
       <c r="G7" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H7" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I7" t="str">
-        <v>0.00s</v>
+        <v>6.24s</v>
       </c>
       <c r="J7" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-b23a4-ns-an-invalid-email-format--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="8">
@@ -45748,16 +45748,16 @@
         <v/>
       </c>
       <c r="G8" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H8" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I8" t="str">
-        <v>0.00s</v>
+        <v>7.22s</v>
       </c>
       <c r="J8" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-343fd-lid-or-insufficient-digits--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="9">
@@ -45780,16 +45780,16 @@
         <v/>
       </c>
       <c r="G9" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H9" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I9" t="str">
-        <v>0.00s</v>
+        <v>5.14s</v>
       </c>
       <c r="J9" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-3aee9-tory-fields-are-left-blank--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="10">
@@ -45812,16 +45812,16 @@
         <v/>
       </c>
       <c r="G10" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H10" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I10" t="str">
-        <v>0.00s</v>
+        <v>7.14s</v>
       </c>
       <c r="J10" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-0ddd8-ate-error-message-is-shown--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="11">
@@ -45844,16 +45844,16 @@
         <v/>
       </c>
       <c r="G11" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H11" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I11" t="str">
-        <v>0.00s</v>
+        <v>6.56s</v>
       </c>
       <c r="J11" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-b33d1-ected-through-manipulation--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="12">
@@ -45876,16 +45876,16 @@
         <v/>
       </c>
       <c r="G12" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H12" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I12" t="str">
-        <v>0.00s</v>
+        <v>17.11s</v>
       </c>
       <c r="J12" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-9c22c-ST-License-No-and-FSSAI-No--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="13">
@@ -45908,16 +45908,16 @@
         <v/>
       </c>
       <c r="G13" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H13" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I13" t="str">
-        <v>0.00s</v>
+        <v>13.71s</v>
       </c>
       <c r="J13" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-96a46-y-and-preview-is-displayed--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="14">
@@ -45940,16 +45940,16 @@
         <v/>
       </c>
       <c r="G14" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H14" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I14" t="str">
-        <v>0.00s</v>
+        <v>13.36s</v>
       </c>
       <c r="J14" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-f7d2b-tained-after-clicking-Next--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="15">
@@ -45972,16 +45972,16 @@
         <v/>
       </c>
       <c r="G15" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H15" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I15" t="str">
-        <v>0.00s</v>
+        <v>74.61s</v>
       </c>
       <c r="J15" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-7ac8c-ing-step-without-data-loss--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="16">
@@ -46004,16 +46004,16 @@
         <v/>
       </c>
       <c r="G16" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H16" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I16" t="str">
-        <v>0.00s</v>
+        <v>13.03s</v>
       </c>
       <c r="J16" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-09b82-blank-and-user-clicks-Next--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="17">
@@ -46036,16 +46036,16 @@
         <v/>
       </c>
       <c r="G17" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H17" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I17" t="str">
-        <v>0.00s</v>
+        <v>72.73s</v>
       </c>
       <c r="J17" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-e6bf4--exe-zip-in-the-Logo-field--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="18">
@@ -46068,16 +46068,16 @@
         <v/>
       </c>
       <c r="G18" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H18" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I18" t="str">
-        <v>0.00s</v>
+        <v>74.69s</v>
       </c>
       <c r="J18" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-7536a-ontains-invalid-characters--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="19">
@@ -46100,16 +46100,16 @@
         <v/>
       </c>
       <c r="G19" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H19" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I19" t="str">
-        <v>0.00s</v>
+        <v>73.15s</v>
       </c>
       <c r="J19" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-f8178-or-logo-upload-are-missing--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="20">
@@ -46132,16 +46132,16 @@
         <v/>
       </c>
       <c r="G20" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H20" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I20" t="str">
-        <v>0.00s</v>
+        <v>20.19s</v>
       </c>
       <c r="J20" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-c81a4--Phone-Number-and-Password--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="21">
@@ -46164,16 +46164,16 @@
         <v/>
       </c>
       <c r="G21" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H21" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I21" t="str">
-        <v>0.00s</v>
+        <v>17.08s</v>
       </c>
       <c r="J21" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-33330-hides-the-entered-password--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="22">
@@ -46196,16 +46196,16 @@
         <v/>
       </c>
       <c r="G22" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H22" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I22" t="str">
-        <v>0.00s</v>
+        <v>16.75s</v>
       </c>
       <c r="J22" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-3567f-he-phone-field-accordingly--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="23">
@@ -46228,16 +46228,16 @@
         <v/>
       </c>
       <c r="G23" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H23" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I23" t="str">
-        <v>0.00s</v>
+        <v>19.74s</v>
       </c>
       <c r="J23" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-b3ad1-ng-previously-entered-data--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="24">
@@ -46260,16 +46260,16 @@
         <v/>
       </c>
       <c r="G24" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H24" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I24" t="str">
-        <v>0.00s</v>
+        <v>18.55s</v>
       </c>
       <c r="J24" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-3403c-blank-and-user-clicks-Next--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="25">
@@ -46292,16 +46292,16 @@
         <v/>
       </c>
       <c r="G25" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H25" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I25" t="str">
-        <v>0.00s</v>
+        <v>78.06s</v>
       </c>
       <c r="J25" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-ced58-mat-is-entered-e-g-abc-com--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="26">
@@ -46324,16 +46324,16 @@
         <v/>
       </c>
       <c r="G26" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H26" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I26" t="str">
-        <v>0.00s</v>
+        <v>19.42s</v>
       </c>
       <c r="J26" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-de608-etic-or-special-characters--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="27">
@@ -46356,16 +46356,16 @@
         <v/>
       </c>
       <c r="G27" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H27" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I27" t="str">
-        <v>0.00s</v>
+        <v>78.65s</v>
       </c>
       <c r="J27" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-47893-uirements-or-is-left-empty--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="28">
@@ -46388,16 +46388,16 @@
         <v/>
       </c>
       <c r="G28" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H28" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I28" t="str">
-        <v>0.00s</v>
+        <v>21.45s</v>
       </c>
       <c r="J28" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-c982b-the-next-step-successfully--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="29">
@@ -46420,16 +46420,16 @@
         <v/>
       </c>
       <c r="G29" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H29" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I29" t="str">
-        <v>0.00s</v>
+        <v>24.75s</v>
       </c>
       <c r="J29" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-b422c--Market-from-the-dropdowns--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="30">
@@ -46452,16 +46452,16 @@
         <v/>
       </c>
       <c r="G30" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H30" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I30" t="str">
-        <v>0.00s</v>
+        <v>22.38s</v>
       </c>
       <c r="J30" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-530a1-vailable-markets-correctly--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="31">
@@ -46484,16 +46484,16 @@
         <v/>
       </c>
       <c r="G31" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H31" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I31" t="str">
-        <v>0.00s</v>
+        <v>21.03s</v>
       </c>
       <c r="J31" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-0bab7-ale-and-save-the-selection--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="32">
@@ -46516,16 +46516,16 @@
         <v/>
       </c>
       <c r="G32" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H32" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I32" t="str">
-        <v>0.00s</v>
+        <v>21.29s</v>
       </c>
       <c r="J32" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-8cd57-cted-using-the-date-picker--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="33">
@@ -46548,16 +46548,16 @@
         <v/>
       </c>
       <c r="G33" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H33" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I33" t="str">
-        <v>0.00s</v>
+        <v>28.64s</v>
       </c>
       <c r="J33" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-d3722--completed-with-valid-data--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="34">
@@ -46580,16 +46580,16 @@
         <v/>
       </c>
       <c r="G34" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H34" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I34" t="str">
-        <v>0.00s</v>
+        <v>84.50s</v>
       </c>
       <c r="J34" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-e87e3-oaded-and-user-clicks-Next--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="35">
@@ -46612,16 +46612,16 @@
         <v/>
       </c>
       <c r="G35" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H35" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I35" t="str">
-        <v>0.00s</v>
+        <v>21.45s</v>
       </c>
       <c r="J35" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-ccbd7-le-formats-e-g-exe-bat-zip--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="36">
@@ -46644,16 +46644,16 @@
         <v/>
       </c>
       <c r="G36" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H36" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I36" t="str">
-        <v>0.00s</v>
+        <v>25.98s</v>
       </c>
       <c r="J36" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-11e59-log-Option-is-not-selected--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="37">
@@ -46676,16 +46676,16 @@
         <v/>
       </c>
       <c r="G37" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H37" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I37" t="str">
-        <v>0.00s</v>
+        <v>84.51s</v>
       </c>
       <c r="J37" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-69355-ct-All-Market-is-unchecked--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="38">
@@ -46708,16 +46708,16 @@
         <v/>
       </c>
       <c r="G38" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H38" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I38" t="str">
-        <v>0.00s</v>
+        <v>86.21s</v>
       </c>
       <c r="J38" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-1ca75--than-Agreement-Start-Date--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="39">
@@ -46740,16 +46740,16 @@
         <v/>
       </c>
       <c r="G39" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H39" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I39" t="str">
-        <v>0.00s</v>
+        <v>80.40s</v>
       </c>
       <c r="J39" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-baf2d--marked-with-is-left-blank--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="40">
@@ -46772,16 +46772,16 @@
         <v/>
       </c>
       <c r="G40" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H40" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I40" t="str">
-        <v>0.00s</v>
+        <v>44.94s</v>
       </c>
       <c r="J40" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-0f168-ding-steps-with-valid-data--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="41">
@@ -46804,16 +46804,16 @@
         <v/>
       </c>
       <c r="G41" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H41" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I41" t="str">
-        <v>0.00s</v>
+        <v>2.98s</v>
       </c>
       <c r="J41" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-f5dea-ent-list-page-successfully--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="42">
@@ -46836,16 +46836,16 @@
         <v/>
       </c>
       <c r="G42" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H42" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I42" t="str">
-        <v>0.00s</v>
+        <v>4.00s</v>
       </c>
       <c r="J42" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-b7878--incomplete-mandatory-data--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="43">
@@ -46868,16 +46868,16 @@
         <v/>
       </c>
       <c r="G43" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H43" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I43" t="str">
-        <v>0.00s</v>
+        <v>12.87s</v>
       </c>
       <c r="J43" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-539b3-e-and-prevents-redirection--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="44">
@@ -46900,16 +46900,16 @@
         <v/>
       </c>
       <c r="G44" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H44" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I44" t="str">
-        <v>0.00s</v>
+        <v>3.03s</v>
       </c>
       <c r="J44" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-a3f96-cords-with-correct-details--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="45">
@@ -46932,16 +46932,16 @@
         <v/>
       </c>
       <c r="G45" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H45" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I45" t="str">
-        <v>0.00s</v>
+        <v>8.69s</v>
       </c>
       <c r="J45" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-46f45-hing-results-are-displayed--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="46">
@@ -46964,16 +46964,16 @@
         <v/>
       </c>
       <c r="G46" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H46" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I46" t="str">
-        <v>0.00s</v>
+        <v>10.36s</v>
       </c>
       <c r="J46" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-865b6--details-page-successfully--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="47">
@@ -46996,16 +46996,16 @@
         <v/>
       </c>
       <c r="G47" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H47" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I47" t="str">
-        <v>0.00s</v>
+        <v>10.24s</v>
       </c>
       <c r="J47" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-bb980--mode-with-pre-filled-data--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="48">
@@ -47028,16 +47028,16 @@
         <v/>
       </c>
       <c r="G48" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H48" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I48" t="str">
-        <v>0.00s</v>
+        <v>4.21s</v>
       </c>
       <c r="J48" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-638ae-oarding-Create-Office-page--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="49">
@@ -47060,16 +47060,16 @@
         <v/>
       </c>
       <c r="G49" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H49" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I49" t="str">
-        <v>0.00s</v>
+        <v>17.36s</v>
       </c>
       <c r="J49" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-47cf9-a-non-existing-office-name--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="50">
@@ -47092,16 +47092,16 @@
         <v/>
       </c>
       <c r="G50" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H50" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I50" t="str">
-        <v>0.00s</v>
+        <v>18.88s</v>
       </c>
       <c r="J50" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-35ae0-k-the-search-functionality--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="51">
@@ -47124,16 +47124,16 @@
         <v/>
       </c>
       <c r="G51" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H51" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I51" t="str">
-        <v>0.00s</v>
+        <v>3.27s</v>
       </c>
       <c r="J51" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-05b75-ails-through-the-View-icon--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="52">
@@ -47156,16 +47156,16 @@
         <v/>
       </c>
       <c r="G52" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H52" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I52" t="str">
-        <v>0.00s</v>
+        <v>3.86s</v>
       </c>
       <c r="J52" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-4f546-ails-through-the-Edit-icon--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="53">
@@ -47188,16 +47188,16 @@
         <v/>
       </c>
       <c r="G53" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H53" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I53" t="str">
-        <v>0.00s</v>
+        <v>5.83s</v>
       </c>
       <c r="J53" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-5c6bc-sage-and-prevents-deletion--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="54">
@@ -47220,16 +47220,16 @@
         <v/>
       </c>
       <c r="G54" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H54" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I54" t="str">
-        <v>0.00s</v>
+        <v>10.41s</v>
       </c>
       <c r="J54" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-06c40--for-a-valid-office-record--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="55">
@@ -47252,16 +47252,16 @@
         <v/>
       </c>
       <c r="G55" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H55" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I55" t="str">
-        <v>0.00s</v>
+        <v>10.69s</v>
       </c>
       <c r="J55" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-5f06d-atching-the-created-office--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="56">
@@ -47284,16 +47284,16 @@
         <v/>
       </c>
       <c r="G56" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H56" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I56" t="str">
-        <v>0.00s</v>
+        <v>10.41s</v>
       </c>
       <c r="J56" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-97fbd-ociated-logo-when-accessed--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="57">
@@ -47316,16 +47316,16 @@
         <v/>
       </c>
       <c r="G57" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H57" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I57" t="str">
-        <v>0.00s</v>
+        <v>10.56s</v>
       </c>
       <c r="J57" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-92567-ayed-correctly-on-the-page--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="58">
@@ -47348,16 +47348,16 @@
         <v/>
       </c>
       <c r="G58" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H58" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I58" t="str">
-        <v>0.00s</v>
+        <v>11.30s</v>
       </c>
       <c r="J58" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-aab39-Registry-page-successfully--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="59">
@@ -47380,16 +47380,16 @@
         <v/>
       </c>
       <c r="G59" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H59" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I59" t="str">
-        <v>0.00s</v>
+        <v>3.20s</v>
       </c>
       <c r="J59" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-9a348-non-existent-office-record--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="60">
@@ -47412,16 +47412,16 @@
         <v/>
       </c>
       <c r="G60" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H60" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I60" t="str">
-        <v>0.00s</v>
+        <v>10.69s</v>
       </c>
       <c r="J60" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-b58fa-efully-without-UI-breakage--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="61">
@@ -47444,16 +47444,16 @@
         <v/>
       </c>
       <c r="G61" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H61" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I61" t="str">
-        <v>0.00s</v>
+        <v>10.56s</v>
       </c>
       <c r="J61" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-72690-y-a-fallback-message-image--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="62">
@@ -47476,16 +47476,16 @@
         <v/>
       </c>
       <c r="G62" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H62" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I62" t="str">
-        <v>0.00s</v>
+        <v>2.46s</v>
       </c>
       <c r="J62" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-069e7-ectly-via-URL-manipulation--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="63">
@@ -47508,16 +47508,16 @@
         <v/>
       </c>
       <c r="G63" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H63" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I63" t="str">
-        <v>0.00s</v>
+        <v>10.86s</v>
       </c>
       <c r="J63" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-81f65-m-errors-or-sensitive-data--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="64">
@@ -47540,16 +47540,16 @@
         <v/>
       </c>
       <c r="G64" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H64" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I64" t="str">
-        <v>0.00s</v>
+        <v>14.18s</v>
       </c>
       <c r="J64" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-4682f-ry-fields-and-save-changes--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="65">
@@ -47572,16 +47572,16 @@
         <v/>
       </c>
       <c r="G65" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H65" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I65" t="str">
-        <v>0.00s</v>
+        <v>15.58s</v>
       </c>
       <c r="J65" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-3c097--is-reflected-after-saving--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="66">
@@ -47604,16 +47604,16 @@
         <v/>
       </c>
       <c r="G66" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H66" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I66" t="str">
-        <v>0.00s</v>
+        <v>14.49s</v>
       </c>
       <c r="J66" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-58dd7-s-information-successfully--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="67">
@@ -47636,16 +47636,16 @@
         <v/>
       </c>
       <c r="G67" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H67" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I67" t="str">
-        <v>0.00s</v>
+        <v>14.39s</v>
       </c>
       <c r="J67" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-f8e11-nd-save-the-updated-values--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="68">
@@ -47668,16 +47668,16 @@
         <v/>
       </c>
       <c r="G68" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H68" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I68" t="str">
-        <v>0.00s</v>
+        <v>20.95s</v>
       </c>
       <c r="J68" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-e529a--persists-the-updated-data--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="69">
@@ -47700,16 +47700,16 @@
         <v/>
       </c>
       <c r="G69" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H69" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I69" t="str">
-        <v>0.00s</v>
+        <v>13.79s</v>
       </c>
       <c r="J69" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-68ec7-d-Update-Office-is-clicked--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="70">
@@ -47732,16 +47732,16 @@
         <v/>
       </c>
       <c r="G70" t="str">
-        <v>Skipped</v>
+        <v>Pass</v>
       </c>
       <c r="H70" t="str">
-        <v>Test was skipped.</v>
+        <v>Test passed successfully.</v>
       </c>
       <c r="I70" t="str">
-        <v>0.00s</v>
+        <v>15.92s</v>
       </c>
       <c r="J70" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-dea18-entered-in-the-Email-field--suite\test-finished-1.png</v>
       </c>
     </row>
     <row r="71">
@@ -47770,10 +47770,10 @@
         <v>Test was skipped.</v>
       </c>
       <c r="I71" t="str">
-        <v>0.00s</v>
+        <v>9.02s</v>
       </c>
       <c r="J71" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-OfficeManagemen-942b6--or-exceeds-allowed-length--suite\test-failed-1.png</v>
       </c>
     </row>
     <row r="72">
@@ -47969,7 +47969,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:J77"/>
   </ignoredErrors>
@@ -60755,16 +60754,16 @@
         <v>High</v>
       </c>
       <c r="K2" t="str">
-        <v>Not Executed</v>
+        <v>Failed</v>
       </c>
       <c r="L2" t="str">
-        <v/>
+        <v>Error: Login failed for '': Please enter email/username/phone</v>
       </c>
       <c r="M2" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N2" t="str">
-        <v/>
+        <v>C:\Users\sriro\Music\nipige_qa_automation\test-results\failure\Regression-FAQMasterConfig-137a5-oads-via-sidebar-navigation-suite\test-failed-1.png</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -60800,13 +60799,13 @@
         <v>Medium</v>
       </c>
       <c r="K3" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L3" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M3" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N3" t="str">
         <v/>
@@ -60844,13 +60843,13 @@
         <v>High</v>
       </c>
       <c r="K4" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L4" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M4" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N4" t="str">
         <v/>
@@ -60889,13 +60888,13 @@
         <v>High</v>
       </c>
       <c r="K5" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L5" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M5" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N5" t="str">
         <v/>
@@ -60934,13 +60933,13 @@
         <v>Medium</v>
       </c>
       <c r="K6" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L6" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M6" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N6" t="str">
         <v/>
@@ -60979,13 +60978,13 @@
         <v>Medium</v>
       </c>
       <c r="K7" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L7" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M7" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N7" t="str">
         <v/>
@@ -61024,13 +61023,13 @@
         <v>Medium</v>
       </c>
       <c r="K8" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L8" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M8" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N8" t="str">
         <v/>
@@ -61070,13 +61069,13 @@
         <v>Medium</v>
       </c>
       <c r="K9" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L9" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M9" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N9" t="str">
         <v/>
@@ -61116,13 +61115,13 @@
         <v>Medium</v>
       </c>
       <c r="K10" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L10" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M10" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N10" t="str">
         <v/>
@@ -61161,13 +61160,13 @@
         <v>High</v>
       </c>
       <c r="K11" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L11" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M11" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N11" t="str">
         <v/>
@@ -61210,13 +61209,13 @@
         <v>High</v>
       </c>
       <c r="K12" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L12" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M12" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N12" t="str">
         <v/>
@@ -61256,13 +61255,13 @@
         <v>Medium</v>
       </c>
       <c r="K13" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L13" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M13" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N13" t="str">
         <v/>
@@ -61301,13 +61300,13 @@
         <v>Medium</v>
       </c>
       <c r="K14" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L14" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M14" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N14" t="str">
         <v/>
@@ -61348,13 +61347,13 @@
         <v>High</v>
       </c>
       <c r="K15" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L15" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M15" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N15" t="str">
         <v/>
@@ -61395,13 +61394,13 @@
         <v>Medium</v>
       </c>
       <c r="K16" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L16" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M16" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N16" t="str">
         <v/>
@@ -61440,13 +61439,13 @@
         <v>Medium</v>
       </c>
       <c r="K17" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L17" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M17" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N17" t="str">
         <v/>
@@ -61486,13 +61485,13 @@
         <v>High</v>
       </c>
       <c r="K18" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L18" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M18" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N18" t="str">
         <v/>
@@ -61531,13 +61530,13 @@
         <v>Medium</v>
       </c>
       <c r="K19" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L19" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M19" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N19" t="str">
         <v/>
@@ -61577,13 +61576,13 @@
         <v>High</v>
       </c>
       <c r="K20" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L20" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M20" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N20" t="str">
         <v/>
@@ -61623,13 +61622,13 @@
         <v>High</v>
       </c>
       <c r="K21" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L21" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M21" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N21" t="str">
         <v/>
@@ -61669,13 +61668,13 @@
         <v>Medium</v>
       </c>
       <c r="K22" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L22" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M22" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N22" t="str">
         <v/>
@@ -61715,13 +61714,13 @@
         <v>Medium</v>
       </c>
       <c r="K23" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L23" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M23" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N23" t="str">
         <v/>
@@ -61761,13 +61760,13 @@
         <v>Medium</v>
       </c>
       <c r="K24" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L24" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M24" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N24" t="str">
         <v/>
@@ -61808,13 +61807,13 @@
         <v>High</v>
       </c>
       <c r="K25" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L25" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M25" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N25" t="str">
         <v/>
@@ -61854,13 +61853,13 @@
         <v>Medium</v>
       </c>
       <c r="K26" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L26" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M26" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N26" t="str">
         <v/>
@@ -61899,13 +61898,13 @@
         <v>Medium</v>
       </c>
       <c r="K27" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L27" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M27" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N27" t="str">
         <v/>
@@ -61945,13 +61944,13 @@
         <v>High</v>
       </c>
       <c r="K28" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L28" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M28" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N28" t="str">
         <v/>
@@ -61992,13 +61991,13 @@
         <v>Medium</v>
       </c>
       <c r="K29" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L29" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M29" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N29" t="str">
         <v/>
@@ -62037,13 +62036,13 @@
         <v>Medium</v>
       </c>
       <c r="K30" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L30" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M30" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N30" t="str">
         <v/>
@@ -62082,13 +62081,13 @@
         <v>Medium</v>
       </c>
       <c r="K31" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L31" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M31" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N31" t="str">
         <v/>
@@ -62128,13 +62127,13 @@
         <v>High</v>
       </c>
       <c r="K32" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L32" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M32" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N32" t="str">
         <v/>
@@ -62174,13 +62173,13 @@
         <v>High</v>
       </c>
       <c r="K33" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L33" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M33" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N33" t="str">
         <v/>
@@ -62220,13 +62219,13 @@
         <v>High</v>
       </c>
       <c r="K34" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L34" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M34" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N34" t="str">
         <v/>
@@ -62266,13 +62265,13 @@
         <v>High</v>
       </c>
       <c r="K35" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L35" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M35" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N35" t="str">
         <v/>
@@ -62311,13 +62310,13 @@
         <v>Medium</v>
       </c>
       <c r="K36" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L36" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M36" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N36" t="str">
         <v/>
@@ -62356,13 +62355,13 @@
         <v>Medium</v>
       </c>
       <c r="K37" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L37" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M37" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N37" t="str">
         <v/>
@@ -62401,13 +62400,13 @@
         <v>Low</v>
       </c>
       <c r="K38" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L38" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M38" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N38" t="str">
         <v/>
@@ -62446,13 +62445,13 @@
         <v>Medium</v>
       </c>
       <c r="K39" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L39" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M39" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N39" t="str">
         <v/>
@@ -62491,13 +62490,13 @@
         <v>Medium</v>
       </c>
       <c r="K40" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L40" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M40" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N40" t="str">
         <v/>
@@ -62536,20 +62535,19 @@
         <v>Medium</v>
       </c>
       <c r="K41" t="str">
-        <v>Not Executed</v>
+        <v>Blocked</v>
       </c>
       <c r="L41" t="str">
-        <v/>
+        <v>Test was skipped.</v>
       </c>
       <c r="M41" t="str">
-        <v/>
+        <v>0.00s</v>
       </c>
       <c r="N41" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:N41"/>
   </ignoredErrors>

</xml_diff>